<commit_message>
Atualização automática - 2026-09-15
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3702</v>
+        <v>13.3665</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149649.93</v>
+        <v>149801.03</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151536.58</v>
+        <v>151689.59</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150593.25</v>
+        <v>150745.31</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3702</v>
+        <v>13.3665</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114547.28</v>
+        <v>114662.94</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115326.1</v>
+        <v>115442.54</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114936.69</v>
+        <v>115052.74</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3702</v>
+        <v>13.3665</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81674.89999999999</v>
+        <v>81757.36</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82183.83</v>
+        <v>82266.81</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81929.36</v>
+        <v>82012.09</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3702</v>
+        <v>13.3665</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57874.81</v>
+        <v>57933.25</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57436.19</v>
+        <v>57494.18</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57655.5</v>
+        <v>57713.71</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3702</v>
+        <v>13.3665</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37384.83</v>
+        <v>37422.58</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37690.65</v>
+        <v>37728.71</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37537.74</v>
+        <v>37575.64</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3702</v>
+        <v>13.3665</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17003.32</v>
+        <v>17020.49</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16891.66</v>
+        <v>16908.72</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16947.49</v>
+        <v>16964.6</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3481</v>
+        <v>13.3503</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162600.21</v>
+        <v>162760.42</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161727.72</v>
+        <v>161887.07</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162163.96</v>
+        <v>162323.74</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3481</v>
+        <v>13.3503</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122113.25</v>
+        <v>122233.57</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120388.58</v>
+        <v>120507.19</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121250.91</v>
+        <v>121370.38</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3481</v>
+        <v>13.3503</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87242.33</v>
+        <v>87328.28999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86162</v>
+        <v>86246.89999999999</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86702.17</v>
+        <v>86787.59</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3481</v>
+        <v>13.3503</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66456.78999999999</v>
+        <v>66522.27</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65989.61</v>
+        <v>66054.63</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66223.2</v>
+        <v>66288.45</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3481</v>
+        <v>13.3503</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51917.12</v>
+        <v>51968.27</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50051.27</v>
+        <v>50100.58</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50984.19</v>
+        <v>51034.43</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3481</v>
+        <v>13.3503</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39355.99</v>
+        <v>39394.77</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40328.49</v>
+        <v>40368.23</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39842.24</v>
+        <v>39881.5</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3707</v>
+        <v>13.3703</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167400.72</v>
+        <v>167567.86</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168942.76</v>
+        <v>169111.44</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168171.74</v>
+        <v>168339.65</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3707</v>
+        <v>13.3703</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120672.6</v>
+        <v>120793.09</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119230.31</v>
+        <v>119349.35</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119951.45</v>
+        <v>120071.22</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3707</v>
+        <v>13.3703</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82662.64</v>
+        <v>82745.17</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82350.42</v>
+        <v>82432.64</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82506.53</v>
+        <v>82588.91</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3707</v>
+        <v>13.3703</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55073.82</v>
+        <v>55128.81</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55377.69</v>
+        <v>55432.99</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55225.76</v>
+        <v>55280.9</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3707</v>
+        <v>13.3703</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33239.86</v>
+        <v>33273.05</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32850.8</v>
+        <v>32883.6</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33045.33</v>
+        <v>33078.32</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3707</v>
+        <v>13.3703</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17256.72</v>
+        <v>17273.95</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17940.86</v>
+        <v>17958.78</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17598.79</v>
+        <v>17616.36</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3956</v>
+        <v>13.3963</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129359.05</v>
+        <v>129487.63</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129453.83</v>
+        <v>129582.5</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129406.44</v>
+        <v>129535.07</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3956</v>
+        <v>13.3963</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89587.92</v>
+        <v>89676.96000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88197.77</v>
+        <v>88285.44</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88892.84</v>
+        <v>88981.2</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3956</v>
+        <v>13.3963</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56311.04</v>
+        <v>56367.01</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56598.41</v>
+        <v>56654.67</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56454.72</v>
+        <v>56510.84</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3956</v>
+        <v>13.3963</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29811.1</v>
+        <v>29840.74</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30011.76</v>
+        <v>30041.59</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29911.43</v>
+        <v>29941.16</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3956</v>
+        <v>13.3963</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6837.42</v>
+        <v>6844.22</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6836.12</v>
+        <v>6842.91</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6836.77</v>
+        <v>6843.56</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3956</v>
+        <v>13.3963</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3799.17</v>
+        <v>3802.95</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3709.56</v>
+        <v>3713.25</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3754.37</v>
+        <v>3758.1</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.4211</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109206.37</v>
+        <v>109314.27</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109685.46</v>
+        <v>109793.84</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109445.91</v>
+        <v>109554.06</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.4211</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76584.97</v>
+        <v>76660.64999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76040.10000000001</v>
+        <v>76115.24000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76312.53999999999</v>
+        <v>76387.94</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.4211</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46341.66</v>
+        <v>46387.45</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47449.63</v>
+        <v>47496.52</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46895.65</v>
+        <v>46941.99</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.4211</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28790.17</v>
+        <v>28818.62</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28682.88</v>
+        <v>28711.22</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28736.53</v>
+        <v>28764.92</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.4211</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14123.19</v>
+        <v>14137.15</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14245.64</v>
+        <v>14259.71</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14184.41</v>
+        <v>14198.43</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.4211</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6547.52</v>
+        <v>6553.99</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6385.76</v>
+        <v>6392.07</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6466.64</v>
+        <v>6473.03</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4441</v>
+        <v>13.447</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49698.93</v>
+        <v>49747.64</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49366.2</v>
+        <v>49414.59</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49532.56</v>
+        <v>49581.12</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4441</v>
+        <v>13.447</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43721.78</v>
+        <v>43764.64</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43915.89</v>
+        <v>43958.94</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43818.84</v>
+        <v>43861.79</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4441</v>
+        <v>13.447</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31997.77</v>
+        <v>32029.13</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32338.53</v>
+        <v>32370.23</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32168.15</v>
+        <v>32199.68</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4441</v>
+        <v>13.447</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22498.55</v>
+        <v>22520.6</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22653.06</v>
+        <v>22675.26</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22575.8</v>
+        <v>22597.93</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4441</v>
+        <v>13.447</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14460.53</v>
+        <v>14474.71</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14666.31</v>
+        <v>14680.69</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14563.42</v>
+        <v>14577.7</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4441</v>
+        <v>13.447</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8310.48</v>
+        <v>8318.629999999999</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8365.540000000001</v>
+        <v>8373.74</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8338.01</v>
+        <v>8346.18</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4701</v>
+        <v>13.4742</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48888.64</v>
+        <v>48936.07</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48169.13</v>
+        <v>48215.86</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48528.89</v>
+        <v>48575.97</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4701</v>
+        <v>13.4742</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43780.47</v>
+        <v>43822.94</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43444.15</v>
+        <v>43486.3</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43612.31</v>
+        <v>43654.62</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4701</v>
+        <v>13.4742</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31618.27</v>
+        <v>31648.95</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31049.88</v>
+        <v>31080</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31334.08</v>
+        <v>31364.48</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4701</v>
+        <v>13.4742</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23566.1</v>
+        <v>23588.96</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23461.03</v>
+        <v>23483.79</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23513.56</v>
+        <v>23536.38</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4701</v>
+        <v>13.4742</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18487.3</v>
+        <v>18505.24</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18301.52</v>
+        <v>18319.27</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18394.41</v>
+        <v>18412.26</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4701</v>
+        <v>13.4742</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15549.08</v>
+        <v>15564.17</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15493.57</v>
+        <v>15508.6</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15521.33</v>
+        <v>15536.39</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4942</v>
+        <v>13.4991</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108597.01</v>
+        <v>108701.39</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109146.97</v>
+        <v>109251.87</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>108871.99</v>
+        <v>108976.63</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4942</v>
+        <v>13.4991</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77875.67999999999</v>
+        <v>77950.52</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78190.49000000001</v>
+        <v>78265.64</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78033.08</v>
+        <v>78108.08</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4942</v>
+        <v>13.4991</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50871.72</v>
+        <v>50920.61</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50439.67</v>
+        <v>50488.15</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50655.7</v>
+        <v>50704.38</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4942</v>
+        <v>13.4991</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29247.78</v>
+        <v>29275.89</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29037.04</v>
+        <v>29064.94</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29142.41</v>
+        <v>29170.42</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4942</v>
+        <v>13.4991</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16621.22</v>
+        <v>16637.19</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16555.54</v>
+        <v>16571.45</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16588.38</v>
+        <v>16604.32</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4942</v>
+        <v>13.4991</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6738.86</v>
+        <v>6745.33</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6525.62</v>
+        <v>6531.89</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6632.24</v>
+        <v>6638.61</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.68</v>
+        <v>13.6625</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>402865.22</v>
+        <v>403279.08</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>397880.78</v>
+        <v>398289.52</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>400373</v>
+        <v>400784.3</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.68</v>
+        <v>13.6625</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>302442.81</v>
+        <v>302753.5</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>303423.69</v>
+        <v>303735.4</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302933.25</v>
+        <v>303244.45</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.68</v>
+        <v>13.6625</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211620.16</v>
+        <v>211837.56</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211492.5</v>
+        <v>211709.76</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211556.33</v>
+        <v>211773.66</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.68</v>
+        <v>13.6625</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128652.74</v>
+        <v>128784.9</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128936.31</v>
+        <v>129068.76</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128794.52</v>
+        <v>128926.83</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.68</v>
+        <v>13.6625</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62359.65</v>
+        <v>62423.71</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62068.32</v>
+        <v>62132.09</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62213.99</v>
+        <v>62277.9</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.68</v>
+        <v>13.6625</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31848.1</v>
+        <v>31880.82</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31872.15</v>
+        <v>31904.9</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31860.13</v>
+        <v>31892.86</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5288</v>
+        <v>13.5233</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>406414.54</v>
+        <v>406827.02</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>406960.81</v>
+        <v>407373.84</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>406687.67</v>
+        <v>407100.43</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5288</v>
+        <v>13.5233</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>301677.19</v>
+        <v>301983.37</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>299793.55</v>
+        <v>300097.81</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>300735.37</v>
+        <v>301040.59</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5288</v>
+        <v>13.5233</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204627.91</v>
+        <v>204835.59</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204697.91</v>
+        <v>204905.66</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204662.91</v>
+        <v>204870.63</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5288</v>
+        <v>13.5233</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123827.46</v>
+        <v>123953.13</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124343.75</v>
+        <v>124469.95</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124085.6</v>
+        <v>124211.54</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5288</v>
+        <v>13.5233</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49451.17</v>
+        <v>49501.36</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49392.24</v>
+        <v>49442.37</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49421.7</v>
+        <v>49471.86</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5288</v>
+        <v>13.5233</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5439.47</v>
+        <v>5444.99</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5475.34</v>
+        <v>5480.9</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5457.4</v>
+        <v>5462.94</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4304</v>
+        <v>13.4207</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169752.1</v>
+        <v>169925.29</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169779.25</v>
+        <v>169952.47</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169765.67</v>
+        <v>169938.88</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4304</v>
+        <v>13.4207</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111555.32</v>
+        <v>111669.13</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111167.24</v>
+        <v>111280.66</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111361.28</v>
+        <v>111474.89</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4304</v>
+        <v>13.4207</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62475.9</v>
+        <v>62539.64</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62830.27</v>
+        <v>62894.37</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62653.08</v>
+        <v>62717.01</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4304</v>
+        <v>13.4207</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26746.54</v>
+        <v>26773.83</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26945.8</v>
+        <v>26973.29</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26846.17</v>
+        <v>26873.56</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4304</v>
+        <v>13.4207</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6295.85</v>
+        <v>6302.27</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6447.19</v>
+        <v>6453.77</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6371.52</v>
+        <v>6378.02</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4304</v>
+        <v>13.4207</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3728.73</v>
+        <v>3732.54</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3722.26</v>
+        <v>3726.06</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3725.5</v>
+        <v>3729.3</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.3843</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189879.67</v>
+        <v>190074.68</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190806.83</v>
+        <v>191002.79</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190343.25</v>
+        <v>190538.74</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.3843</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137666.78</v>
+        <v>137808.16</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138627.46</v>
+        <v>138769.84</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138147.12</v>
+        <v>138289</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.3843</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87019.2</v>
+        <v>87108.57000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87723.41</v>
+        <v>87813.5</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87371.3</v>
+        <v>87461.03999999999</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.3843</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41565.8</v>
+        <v>41608.49</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41499.14</v>
+        <v>41541.76</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41532.47</v>
+        <v>41575.12</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.3843</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12961.62</v>
+        <v>12974.93</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12818.85</v>
+        <v>12832.01</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12890.23</v>
+        <v>12903.47</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.3843</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4498.49</v>
+        <v>4503.11</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4388.68</v>
+        <v>4393.19</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4443.59</v>
+        <v>4448.15</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-16
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3665</v>
+        <v>13.3724</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149801.03</v>
+        <v>149872.48</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151689.59</v>
+        <v>151761.94</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150745.31</v>
+        <v>150817.21</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3665</v>
+        <v>13.3724</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114662.94</v>
+        <v>114717.63</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115442.54</v>
+        <v>115497.6</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115052.74</v>
+        <v>115107.62</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3665</v>
+        <v>13.3724</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81757.36</v>
+        <v>81796.36</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82266.81</v>
+        <v>82306.05</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82012.09</v>
+        <v>82051.2</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3665</v>
+        <v>13.3724</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57933.25</v>
+        <v>57960.88</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57494.18</v>
+        <v>57521.6</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57713.71</v>
+        <v>57741.24</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3665</v>
+        <v>13.3724</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37422.58</v>
+        <v>37440.43</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37728.71</v>
+        <v>37746.7</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37575.64</v>
+        <v>37593.57</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3665</v>
+        <v>13.3724</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17020.49</v>
+        <v>17028.61</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16908.72</v>
+        <v>16916.78</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16964.6</v>
+        <v>16972.69</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3503</v>
+        <v>13.3575</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162760.42</v>
+        <v>162836.4</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161887.07</v>
+        <v>161962.65</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162323.74</v>
+        <v>162399.52</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3503</v>
+        <v>13.3575</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122233.57</v>
+        <v>122290.63</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120507.19</v>
+        <v>120563.45</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121370.38</v>
+        <v>121427.04</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3503</v>
+        <v>13.3575</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87328.28999999999</v>
+        <v>87369.05</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86246.89999999999</v>
+        <v>86287.16</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86787.59</v>
+        <v>86828.11</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3503</v>
+        <v>13.3575</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66522.27</v>
+        <v>66553.32000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66054.63</v>
+        <v>66085.46000000001</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66288.45</v>
+        <v>66319.39</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3503</v>
+        <v>13.3575</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51968.27</v>
+        <v>51992.53</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50100.58</v>
+        <v>50123.97</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51034.43</v>
+        <v>51058.25</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3503</v>
+        <v>13.3575</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39394.77</v>
+        <v>39413.16</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40368.23</v>
+        <v>40387.08</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39881.5</v>
+        <v>39900.12</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3703</v>
+        <v>13.3773</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167567.86</v>
+        <v>167645.42</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169111.44</v>
+        <v>169189.71</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168339.65</v>
+        <v>168417.57</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3703</v>
+        <v>13.3773</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120793.09</v>
+        <v>120849</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119349.35</v>
+        <v>119404.59</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120071.22</v>
+        <v>120126.8</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3703</v>
+        <v>13.3773</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82745.17</v>
+        <v>82783.47</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82432.64</v>
+        <v>82470.8</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82588.91</v>
+        <v>82627.13</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3703</v>
+        <v>13.3773</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55128.81</v>
+        <v>55154.32</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55432.99</v>
+        <v>55458.64</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55280.9</v>
+        <v>55306.48</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3703</v>
+        <v>13.3773</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33273.05</v>
+        <v>33288.45</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32883.6</v>
+        <v>32898.82</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33078.32</v>
+        <v>33093.63</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3703</v>
+        <v>13.3773</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17273.95</v>
+        <v>17281.95</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17958.78</v>
+        <v>17967.09</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17616.36</v>
+        <v>17624.52</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3963</v>
+        <v>13.4052</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129487.63</v>
+        <v>129545.53</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129582.5</v>
+        <v>129640.46</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129535.07</v>
+        <v>129593</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3963</v>
+        <v>13.4052</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89676.96000000001</v>
+        <v>89717.07000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88285.44</v>
+        <v>88324.92</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88981.2</v>
+        <v>89020.99000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3963</v>
+        <v>13.4052</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56367.01</v>
+        <v>56392.22</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56654.67</v>
+        <v>56680.01</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56510.84</v>
+        <v>56536.11</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3963</v>
+        <v>13.4052</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29840.74</v>
+        <v>29854.08</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30041.59</v>
+        <v>30055.03</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29941.16</v>
+        <v>29954.55</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3963</v>
+        <v>13.4052</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6844.22</v>
+        <v>6847.28</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6842.91</v>
+        <v>6845.97</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6843.56</v>
+        <v>6846.62</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3963</v>
+        <v>13.4052</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3802.95</v>
+        <v>3804.65</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3713.25</v>
+        <v>3714.91</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3758.1</v>
+        <v>3759.78</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4211</v>
+        <v>13.4318</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109314.27</v>
+        <v>109361.23</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109793.84</v>
+        <v>109841</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109554.06</v>
+        <v>109601.12</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4211</v>
+        <v>13.4318</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76660.64999999999</v>
+        <v>76693.57000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76115.24000000001</v>
+        <v>76147.92999999999</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76387.94</v>
+        <v>76420.75</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4211</v>
+        <v>13.4318</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46387.45</v>
+        <v>46407.38</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47496.52</v>
+        <v>47516.92</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46941.99</v>
+        <v>46962.15</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4211</v>
+        <v>13.4318</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28818.62</v>
+        <v>28831</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28711.22</v>
+        <v>28723.55</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28764.92</v>
+        <v>28777.28</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4211</v>
+        <v>13.4318</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14137.15</v>
+        <v>14143.22</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14259.71</v>
+        <v>14265.84</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14198.43</v>
+        <v>14204.53</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4211</v>
+        <v>13.4318</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6553.99</v>
+        <v>6556.8</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6392.07</v>
+        <v>6394.82</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6473.03</v>
+        <v>6475.81</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.447</v>
+        <v>13.4597</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49747.64</v>
+        <v>49767.95</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49414.59</v>
+        <v>49434.76</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49581.12</v>
+        <v>49601.35</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.447</v>
+        <v>13.4597</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43764.64</v>
+        <v>43782.5</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43958.94</v>
+        <v>43976.88</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43861.79</v>
+        <v>43879.69</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.447</v>
+        <v>13.4597</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32029.13</v>
+        <v>32042.21</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32370.23</v>
+        <v>32383.45</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32199.68</v>
+        <v>32212.83</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.447</v>
+        <v>13.4597</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22520.6</v>
+        <v>22529.79</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22675.26</v>
+        <v>22684.52</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22597.93</v>
+        <v>22607.16</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.447</v>
+        <v>13.4597</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14474.71</v>
+        <v>14480.61</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14680.69</v>
+        <v>14686.68</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14577.7</v>
+        <v>14583.65</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.447</v>
+        <v>13.4597</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8318.629999999999</v>
+        <v>8322.02</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8373.74</v>
+        <v>8377.16</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8346.18</v>
+        <v>8349.59</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4742</v>
+        <v>13.4889</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48936.07</v>
+        <v>48954.8</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48215.86</v>
+        <v>48234.31</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48575.97</v>
+        <v>48594.55</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4742</v>
+        <v>13.4889</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43822.94</v>
+        <v>43839.71</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43486.3</v>
+        <v>43502.94</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43654.62</v>
+        <v>43671.32</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4742</v>
+        <v>13.4889</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31648.95</v>
+        <v>31661.06</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31080</v>
+        <v>31091.9</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31364.48</v>
+        <v>31376.48</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4742</v>
+        <v>13.4889</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23588.96</v>
+        <v>23597.99</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23483.79</v>
+        <v>23492.78</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23536.38</v>
+        <v>23545.38</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4742</v>
+        <v>13.4889</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18505.24</v>
+        <v>18512.32</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18319.27</v>
+        <v>18326.28</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18412.26</v>
+        <v>18419.3</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4742</v>
+        <v>13.4889</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15564.17</v>
+        <v>15570.13</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15508.6</v>
+        <v>15514.53</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15536.39</v>
+        <v>15542.33</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.5156</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108701.39</v>
+        <v>108740.18</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109251.87</v>
+        <v>109290.87</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>108976.63</v>
+        <v>109015.52</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.5156</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77950.52</v>
+        <v>77978.34</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78265.64</v>
+        <v>78293.57000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78108.08</v>
+        <v>78135.96000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.5156</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50920.61</v>
+        <v>50938.79</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50488.15</v>
+        <v>50506.17</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50704.38</v>
+        <v>50722.48</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.5156</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29275.89</v>
+        <v>29286.34</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29064.94</v>
+        <v>29075.32</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29170.42</v>
+        <v>29180.83</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.5156</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16637.19</v>
+        <v>16643.13</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16571.45</v>
+        <v>16577.36</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16604.32</v>
+        <v>16610.25</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.5156</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6745.33</v>
+        <v>6747.74</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6531.89</v>
+        <v>6534.22</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6638.61</v>
+        <v>6640.98</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6625</v>
+        <v>13.6413</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>403279.08</v>
+        <v>403488.25</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>398289.52</v>
+        <v>398496.11</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>400784.3</v>
+        <v>400992.18</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6625</v>
+        <v>13.6413</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>302753.5</v>
+        <v>302910.54</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>303735.4</v>
+        <v>303892.94</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>303244.45</v>
+        <v>303401.74</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6625</v>
+        <v>13.6413</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211837.56</v>
+        <v>211947.44</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211709.76</v>
+        <v>211819.57</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211773.66</v>
+        <v>211883.5</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6625</v>
+        <v>13.6413</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128784.9</v>
+        <v>128851.7</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129068.76</v>
+        <v>129135.71</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128926.83</v>
+        <v>128993.71</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6625</v>
+        <v>13.6413</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62423.71</v>
+        <v>62456.09</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62132.09</v>
+        <v>62164.31</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62277.9</v>
+        <v>62310.2</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6625</v>
+        <v>13.6413</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31880.82</v>
+        <v>31897.35</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31904.9</v>
+        <v>31921.44</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31892.86</v>
+        <v>31909.4</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5233</v>
+        <v>13.5231</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>406827.02</v>
+        <v>407031.91</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>407373.84</v>
+        <v>407579.01</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>407100.43</v>
+        <v>407305.46</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5233</v>
+        <v>13.5231</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>301983.37</v>
+        <v>302135.45</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>300097.81</v>
+        <v>300248.95</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>301040.59</v>
+        <v>301192.2</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5233</v>
+        <v>13.5231</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204835.59</v>
+        <v>204938.75</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204905.66</v>
+        <v>205008.86</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204870.63</v>
+        <v>204973.8</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5233</v>
+        <v>13.5231</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123953.13</v>
+        <v>124015.56</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124469.95</v>
+        <v>124532.63</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124211.54</v>
+        <v>124274.1</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5233</v>
+        <v>13.5231</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49501.36</v>
+        <v>49526.29</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49442.37</v>
+        <v>49467.27</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49471.86</v>
+        <v>49496.78</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5233</v>
+        <v>13.5231</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5444.99</v>
+        <v>5447.73</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5480.9</v>
+        <v>5483.66</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5462.94</v>
+        <v>5465.69</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4207</v>
+        <v>13.4257</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169925.29</v>
+        <v>170008.54</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169952.47</v>
+        <v>170035.73</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169938.88</v>
+        <v>170022.13</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4207</v>
+        <v>13.4257</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111669.13</v>
+        <v>111723.84</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111280.66</v>
+        <v>111335.18</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111474.89</v>
+        <v>111529.51</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4207</v>
+        <v>13.4257</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62539.64</v>
+        <v>62570.28</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62894.37</v>
+        <v>62925.18</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62717.01</v>
+        <v>62747.73</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4207</v>
+        <v>13.4257</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26773.83</v>
+        <v>26786.94</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26973.29</v>
+        <v>26986.51</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26873.56</v>
+        <v>26886.72</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4207</v>
+        <v>13.4257</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6302.27</v>
+        <v>6305.36</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6453.77</v>
+        <v>6456.93</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6378.02</v>
+        <v>6381.15</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4207</v>
+        <v>13.4257</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3732.54</v>
+        <v>3734.37</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3726.06</v>
+        <v>3727.89</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3729.3</v>
+        <v>3731.13</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3843</v>
+        <v>13.3888</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190074.68</v>
+        <v>190167.06</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191002.79</v>
+        <v>191095.62</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190538.74</v>
+        <v>190631.34</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3843</v>
+        <v>13.3888</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137808.16</v>
+        <v>137875.14</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138769.84</v>
+        <v>138837.28</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138289</v>
+        <v>138356.21</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3843</v>
+        <v>13.3888</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87108.57000000001</v>
+        <v>87150.89999999999</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87813.5</v>
+        <v>87856.17999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87461.03999999999</v>
+        <v>87503.53999999999</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3843</v>
+        <v>13.3888</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41608.49</v>
+        <v>41628.71</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41541.76</v>
+        <v>41561.95</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41575.12</v>
+        <v>41595.33</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3843</v>
+        <v>13.3888</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12974.93</v>
+        <v>12981.24</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12832.01</v>
+        <v>12838.25</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12903.47</v>
+        <v>12909.74</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3843</v>
+        <v>13.3888</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4503.11</v>
+        <v>4505.3</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4393.19</v>
+        <v>4395.32</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4448.15</v>
+        <v>4450.31</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-17
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3724</v>
+        <v>13.4005</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149872.48</v>
+        <v>149932.23</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151761.94</v>
+        <v>151822.44</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150817.21</v>
+        <v>150877.33</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3724</v>
+        <v>13.4005</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114717.63</v>
+        <v>114763.37</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115497.6</v>
+        <v>115543.65</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115107.62</v>
+        <v>115153.51</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3724</v>
+        <v>13.4005</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81796.36</v>
+        <v>81828.97</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82306.05</v>
+        <v>82338.86</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82051.2</v>
+        <v>82083.92</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3724</v>
+        <v>13.4005</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57960.88</v>
+        <v>57983.98</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57521.6</v>
+        <v>57544.53</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57741.24</v>
+        <v>57764.26</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3724</v>
+        <v>13.4005</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37440.43</v>
+        <v>37455.35</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37746.7</v>
+        <v>37761.75</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37593.57</v>
+        <v>37608.55</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3724</v>
+        <v>13.4005</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17028.61</v>
+        <v>17035.39</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16916.78</v>
+        <v>16923.53</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16972.69</v>
+        <v>16979.46</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3575</v>
+        <v>13.3927</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162836.4</v>
+        <v>162893.16</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161962.65</v>
+        <v>162019.1</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162399.52</v>
+        <v>162456.13</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3575</v>
+        <v>13.3927</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122290.63</v>
+        <v>122333.26</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120563.45</v>
+        <v>120605.48</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121427.04</v>
+        <v>121469.37</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3575</v>
+        <v>13.3927</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87369.05</v>
+        <v>87399.50999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86287.16</v>
+        <v>86317.24000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86828.11</v>
+        <v>86858.37</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3575</v>
+        <v>13.3927</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66553.32000000001</v>
+        <v>66576.52</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66085.46000000001</v>
+        <v>66108.5</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66319.39</v>
+        <v>66342.50999999999</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3575</v>
+        <v>13.3927</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51992.53</v>
+        <v>52010.66</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50123.97</v>
+        <v>50141.44</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51058.25</v>
+        <v>51076.05</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3575</v>
+        <v>13.3927</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39413.16</v>
+        <v>39426.9</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40387.08</v>
+        <v>40401.15</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39900.12</v>
+        <v>39914.02</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3773</v>
+        <v>13.4122</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167645.42</v>
+        <v>167699.66</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169189.71</v>
+        <v>169244.45</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168417.57</v>
+        <v>168472.05</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3773</v>
+        <v>13.4122</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120849</v>
+        <v>120888.1</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119404.59</v>
+        <v>119443.22</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120126.8</v>
+        <v>120165.66</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3773</v>
+        <v>13.4122</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82783.47</v>
+        <v>82810.25</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82470.8</v>
+        <v>82497.48</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82627.13</v>
+        <v>82653.87</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3773</v>
+        <v>13.4122</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55154.32</v>
+        <v>55172.17</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55458.64</v>
+        <v>55476.59</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55306.48</v>
+        <v>55324.38</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3773</v>
+        <v>13.4122</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33288.45</v>
+        <v>33299.22</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32898.82</v>
+        <v>32909.46</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33093.63</v>
+        <v>33104.34</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3773</v>
+        <v>13.4122</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17281.95</v>
+        <v>17287.54</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17967.09</v>
+        <v>17972.9</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17624.52</v>
+        <v>17630.22</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.4052</v>
+        <v>13.4401</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129545.53</v>
+        <v>129584.11</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129640.46</v>
+        <v>129679.06</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129593</v>
+        <v>129631.58</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.4052</v>
+        <v>13.4401</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89717.07000000001</v>
+        <v>89743.78</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88324.92</v>
+        <v>88351.22</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89020.99000000001</v>
+        <v>89047.5</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.4052</v>
+        <v>13.4401</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56392.22</v>
+        <v>56409.01</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56680.01</v>
+        <v>56696.88</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56536.11</v>
+        <v>56552.95</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.4052</v>
+        <v>13.4401</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29854.08</v>
+        <v>29862.97</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30055.03</v>
+        <v>30063.98</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29954.55</v>
+        <v>29963.47</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.4052</v>
+        <v>13.4401</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6847.28</v>
+        <v>6849.32</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6845.97</v>
+        <v>6848.01</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6846.62</v>
+        <v>6848.66</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.4052</v>
+        <v>13.4401</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3804.65</v>
+        <v>3805.78</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3714.91</v>
+        <v>3716.02</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3759.78</v>
+        <v>3760.9</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4318</v>
+        <v>13.4667</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109361.23</v>
+        <v>109391.11</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109841</v>
+        <v>109871.01</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109601.12</v>
+        <v>109631.06</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4318</v>
+        <v>13.4667</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76693.57000000001</v>
+        <v>76714.53</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76147.92999999999</v>
+        <v>76168.74000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76420.75</v>
+        <v>76441.63</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4318</v>
+        <v>13.4667</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46407.38</v>
+        <v>46420.06</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47516.92</v>
+        <v>47529.9</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46962.15</v>
+        <v>46974.98</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4318</v>
+        <v>13.4667</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28831</v>
+        <v>28838.88</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28723.55</v>
+        <v>28731.4</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28777.28</v>
+        <v>28785.14</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4318</v>
+        <v>13.4667</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14143.22</v>
+        <v>14147.08</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14265.84</v>
+        <v>14269.74</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14204.53</v>
+        <v>14208.41</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4318</v>
+        <v>13.4667</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6556.8</v>
+        <v>6558.59</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6394.82</v>
+        <v>6396.57</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6475.81</v>
+        <v>6477.58</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4597</v>
+        <v>13.4946</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49767.95</v>
+        <v>49780.27</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49434.76</v>
+        <v>49447</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49601.35</v>
+        <v>49613.63</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4597</v>
+        <v>13.4946</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43782.5</v>
+        <v>43793.34</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43976.88</v>
+        <v>43987.76</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43879.69</v>
+        <v>43890.55</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4597</v>
+        <v>13.4946</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32042.21</v>
+        <v>32050.14</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32383.45</v>
+        <v>32391.46</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32212.83</v>
+        <v>32220.8</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4597</v>
+        <v>13.4946</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22529.79</v>
+        <v>22535.37</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22684.52</v>
+        <v>22690.13</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22607.16</v>
+        <v>22612.75</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4597</v>
+        <v>13.4946</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14480.61</v>
+        <v>14484.2</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14686.68</v>
+        <v>14690.32</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14583.65</v>
+        <v>14587.26</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4597</v>
+        <v>13.4946</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8322.02</v>
+        <v>8324.08</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8377.16</v>
+        <v>8379.23</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8349.59</v>
+        <v>8351.66</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4889</v>
+        <v>13.5237</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48954.8</v>
+        <v>48965.6</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48234.31</v>
+        <v>48244.96</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48594.55</v>
+        <v>48605.28</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4889</v>
+        <v>13.5237</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43839.71</v>
+        <v>43849.39</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43502.94</v>
+        <v>43512.54</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43671.32</v>
+        <v>43680.96</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4889</v>
+        <v>13.5237</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31661.06</v>
+        <v>31668.05</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31091.9</v>
+        <v>31098.76</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31376.48</v>
+        <v>31383.4</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4889</v>
+        <v>13.5237</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23597.99</v>
+        <v>23603.2</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23492.78</v>
+        <v>23497.96</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23545.38</v>
+        <v>23550.58</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4889</v>
+        <v>13.5237</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18512.32</v>
+        <v>18516.41</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18326.28</v>
+        <v>18330.33</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18419.3</v>
+        <v>18423.37</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4889</v>
+        <v>13.5237</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15570.13</v>
+        <v>15573.56</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15514.53</v>
+        <v>15517.96</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15542.33</v>
+        <v>15545.76</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.5156</v>
+        <v>13.5503</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108740.18</v>
+        <v>108761.64</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109290.87</v>
+        <v>109312.43</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109015.52</v>
+        <v>109037.03</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.5156</v>
+        <v>13.5503</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77978.34</v>
+        <v>77993.73</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78293.57000000001</v>
+        <v>78309.02</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78135.96000000001</v>
+        <v>78151.37</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.5156</v>
+        <v>13.5503</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50938.79</v>
+        <v>50948.84</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50506.17</v>
+        <v>50516.14</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50722.48</v>
+        <v>50732.49</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.5156</v>
+        <v>13.5503</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29286.34</v>
+        <v>29292.12</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29075.32</v>
+        <v>29081.05</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29180.83</v>
+        <v>29186.58</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.5156</v>
+        <v>13.5503</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16643.13</v>
+        <v>16646.41</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16577.36</v>
+        <v>16580.63</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16610.25</v>
+        <v>16613.52</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.5156</v>
+        <v>13.5503</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6747.74</v>
+        <v>6749.07</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6534.22</v>
+        <v>6535.51</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6640.98</v>
+        <v>6642.29</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6174</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>403488.25</v>
+        <v>403697.44</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>398496.11</v>
+        <v>398702.7</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>400992.18</v>
+        <v>401200.07</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6174</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>302910.54</v>
+        <v>303067.57</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>303892.94</v>
+        <v>304050.49</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>303401.74</v>
+        <v>303559.03</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6174</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211947.44</v>
+        <v>212057.32</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211819.57</v>
+        <v>211929.39</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211883.5</v>
+        <v>211993.35</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6174</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128851.7</v>
+        <v>128918.5</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129135.71</v>
+        <v>129202.66</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128993.71</v>
+        <v>129060.58</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6174</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62456.09</v>
+        <v>62488.47</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62164.31</v>
+        <v>62196.54</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62310.2</v>
+        <v>62342.5</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6174</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31897.35</v>
+        <v>31913.89</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31921.44</v>
+        <v>31937.99</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31909.4</v>
+        <v>31925.94</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5231</v>
+        <v>13.5228</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>407031.91</v>
+        <v>407237.02</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>407579.01</v>
+        <v>407784.39</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>407305.46</v>
+        <v>407510.7</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5231</v>
+        <v>13.5228</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>302135.45</v>
+        <v>302287.7</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>300248.95</v>
+        <v>300400.25</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>301192.2</v>
+        <v>301343.98</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5231</v>
+        <v>13.5228</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204938.75</v>
+        <v>205042.02</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205008.86</v>
+        <v>205112.16</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204973.8</v>
+        <v>205077.09</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5231</v>
+        <v>13.5228</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124015.56</v>
+        <v>124078.05</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124532.63</v>
+        <v>124595.39</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124274.1</v>
+        <v>124336.72</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5231</v>
+        <v>13.5228</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49526.29</v>
+        <v>49551.24</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49467.27</v>
+        <v>49492.2</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49496.78</v>
+        <v>49521.72</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5231</v>
+        <v>13.5228</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5447.73</v>
+        <v>5450.48</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5483.66</v>
+        <v>5486.42</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5465.69</v>
+        <v>5468.45</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4257</v>
+        <v>13.4386</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170008.54</v>
+        <v>170089.24</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170035.73</v>
+        <v>170116.44</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170022.13</v>
+        <v>170102.84</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4257</v>
+        <v>13.4386</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111723.84</v>
+        <v>111776.87</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111335.18</v>
+        <v>111388.02</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111529.51</v>
+        <v>111582.45</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4257</v>
+        <v>13.4386</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62570.28</v>
+        <v>62599.98</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62925.18</v>
+        <v>62955.05</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62747.73</v>
+        <v>62777.52</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4257</v>
+        <v>13.4386</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26786.94</v>
+        <v>26799.66</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26986.51</v>
+        <v>26999.32</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26886.72</v>
+        <v>26899.49</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4257</v>
+        <v>13.4386</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6305.36</v>
+        <v>6308.36</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6456.93</v>
+        <v>6460</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6381.15</v>
+        <v>6384.18</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4257</v>
+        <v>13.4386</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3734.37</v>
+        <v>3736.14</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3727.89</v>
+        <v>3729.66</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3731.13</v>
+        <v>3732.9</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3888</v>
+        <v>13.4092</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190167.06</v>
+        <v>190251.18</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191095.62</v>
+        <v>191180.15</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190631.34</v>
+        <v>190715.67</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3888</v>
+        <v>13.4092</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137875.14</v>
+        <v>137936.13</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138837.28</v>
+        <v>138898.7</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138356.21</v>
+        <v>138417.41</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3888</v>
+        <v>13.4092</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87150.89999999999</v>
+        <v>87189.46000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87856.17999999999</v>
+        <v>87895.05</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87503.53999999999</v>
+        <v>87542.25</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3888</v>
+        <v>13.4092</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41628.71</v>
+        <v>41647.12</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41561.95</v>
+        <v>41580.33</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41595.33</v>
+        <v>41613.73</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3888</v>
+        <v>13.4092</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12981.24</v>
+        <v>12986.98</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12838.25</v>
+        <v>12843.93</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12909.74</v>
+        <v>12915.45</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3888</v>
+        <v>13.4092</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4505.3</v>
+        <v>4507.29</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4395.32</v>
+        <v>4397.27</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4450.31</v>
+        <v>4452.28</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-18
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.4005</v>
+        <v>13.3575</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149932.23</v>
+        <v>150029.65</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151822.44</v>
+        <v>151921.1</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150877.33</v>
+        <v>150975.37</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.4005</v>
+        <v>13.3575</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114763.37</v>
+        <v>114837.94</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115543.65</v>
+        <v>115618.73</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115153.51</v>
+        <v>115228.33</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.4005</v>
+        <v>13.3575</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81828.97</v>
+        <v>81882.14</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82338.86</v>
+        <v>82392.37</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82083.92</v>
+        <v>82137.25</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.4005</v>
+        <v>13.3575</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57983.98</v>
+        <v>58021.66</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57544.53</v>
+        <v>57581.93</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57764.26</v>
+        <v>57801.79</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.4005</v>
+        <v>13.3575</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37455.35</v>
+        <v>37479.69</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37761.75</v>
+        <v>37786.29</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37608.55</v>
+        <v>37632.99</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.4005</v>
+        <v>13.3575</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17035.39</v>
+        <v>17046.46</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16923.53</v>
+        <v>16934.53</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16979.46</v>
+        <v>16990.49</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3927</v>
+        <v>13.3474</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162893.16</v>
+        <v>163005.39</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162019.1</v>
+        <v>162130.74</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162456.13</v>
+        <v>162568.06</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3927</v>
+        <v>13.3474</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122333.26</v>
+        <v>122417.55</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120605.48</v>
+        <v>120688.57</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121469.37</v>
+        <v>121553.06</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3927</v>
+        <v>13.3474</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87399.50999999999</v>
+        <v>87459.73</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86317.24000000001</v>
+        <v>86376.71000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86858.37</v>
+        <v>86918.22</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3927</v>
+        <v>13.3474</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66576.52</v>
+        <v>66622.39</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66108.5</v>
+        <v>66154.05</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66342.50999999999</v>
+        <v>66388.22</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3927</v>
+        <v>13.3474</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52010.66</v>
+        <v>52046.49</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50141.44</v>
+        <v>50175.99</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51076.05</v>
+        <v>51111.24</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3927</v>
+        <v>13.3474</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39426.9</v>
+        <v>39454.06</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40401.15</v>
+        <v>40428.99</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39914.02</v>
+        <v>39941.53</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.4122</v>
+        <v>13.3629</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167699.66</v>
+        <v>167824.59</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169244.45</v>
+        <v>169370.54</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168472.05</v>
+        <v>168597.57</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.4122</v>
+        <v>13.3629</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120888.1</v>
+        <v>120978.16</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119443.22</v>
+        <v>119532.21</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120165.66</v>
+        <v>120255.18</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.4122</v>
+        <v>13.3629</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82810.25</v>
+        <v>82871.95</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82497.48</v>
+        <v>82558.94</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82653.87</v>
+        <v>82715.44</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.4122</v>
+        <v>13.3629</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55172.17</v>
+        <v>55213.27</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55476.59</v>
+        <v>55517.92</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55324.38</v>
+        <v>55365.59</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.4122</v>
+        <v>13.3629</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33299.22</v>
+        <v>33324.02</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32909.46</v>
+        <v>32933.98</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33104.34</v>
+        <v>33129</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.4122</v>
+        <v>13.3629</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17287.54</v>
+        <v>17300.42</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17972.9</v>
+        <v>17986.29</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17630.22</v>
+        <v>17643.35</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.4401</v>
+        <v>13.3883</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129584.11</v>
+        <v>129687.53</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129679.06</v>
+        <v>129782.55</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129631.58</v>
+        <v>129735.04</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.4401</v>
+        <v>13.3883</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89743.78</v>
+        <v>89815.41</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88351.22</v>
+        <v>88421.73</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89047.5</v>
+        <v>89118.57000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.4401</v>
+        <v>13.3883</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56409.01</v>
+        <v>56454.03</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56696.88</v>
+        <v>56742.13</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56552.95</v>
+        <v>56598.08</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.4401</v>
+        <v>13.3883</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29862.97</v>
+        <v>29886.8</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30063.98</v>
+        <v>30087.97</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29963.47</v>
+        <v>29987.39</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.4401</v>
+        <v>13.3883</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6849.32</v>
+        <v>6854.78</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6848.01</v>
+        <v>6853.48</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6848.66</v>
+        <v>6854.13</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.4401</v>
+        <v>13.3883</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3805.78</v>
+        <v>3808.82</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3716.02</v>
+        <v>3718.98</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3760.9</v>
+        <v>3763.9</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4667</v>
+        <v>13.4125</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109391.11</v>
+        <v>109484.34</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109871.01</v>
+        <v>109964.65</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109631.06</v>
+        <v>109724.49</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4667</v>
+        <v>13.4125</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76714.53</v>
+        <v>76779.91</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76168.74000000001</v>
+        <v>76233.64999999999</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76441.63</v>
+        <v>76506.78</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4667</v>
+        <v>13.4125</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46420.06</v>
+        <v>46459.62</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47529.9</v>
+        <v>47570.41</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46974.98</v>
+        <v>47015.01</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4667</v>
+        <v>13.4125</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28838.88</v>
+        <v>28863.45</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28731.4</v>
+        <v>28755.89</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28785.14</v>
+        <v>28809.67</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4667</v>
+        <v>13.4125</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14147.08</v>
+        <v>14159.14</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14269.74</v>
+        <v>14281.9</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14208.41</v>
+        <v>14220.52</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4667</v>
+        <v>13.4125</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6558.59</v>
+        <v>6564.18</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6396.57</v>
+        <v>6402.02</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6477.58</v>
+        <v>6483.1</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4946</v>
+        <v>13.4379</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49780.27</v>
+        <v>49825.7</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49447</v>
+        <v>49492.13</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49613.63</v>
+        <v>49658.91</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4946</v>
+        <v>13.4379</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43793.34</v>
+        <v>43833.31</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43987.76</v>
+        <v>44027.91</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43890.55</v>
+        <v>43930.61</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4946</v>
+        <v>13.4379</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32050.14</v>
+        <v>32079.39</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32391.46</v>
+        <v>32421.03</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32220.8</v>
+        <v>32250.21</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4946</v>
+        <v>13.4379</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22535.37</v>
+        <v>22555.94</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22690.13</v>
+        <v>22710.84</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22612.75</v>
+        <v>22633.39</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4946</v>
+        <v>13.4379</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14484.2</v>
+        <v>14497.42</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14690.32</v>
+        <v>14703.72</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14587.26</v>
+        <v>14600.57</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4946</v>
+        <v>13.4379</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8324.08</v>
+        <v>8331.68</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8379.23</v>
+        <v>8386.879999999999</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8351.66</v>
+        <v>8359.280000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.5237</v>
+        <v>13.4645</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48965.6</v>
+        <v>49013.59</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48244.96</v>
+        <v>48292.23</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48605.28</v>
+        <v>48652.91</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.5237</v>
+        <v>13.4645</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43849.39</v>
+        <v>43892.36</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43512.54</v>
+        <v>43555.18</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43680.96</v>
+        <v>43723.77</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.5237</v>
+        <v>13.4645</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31668.05</v>
+        <v>31699.08</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31098.76</v>
+        <v>31129.23</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31383.4</v>
+        <v>31414.16</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.5237</v>
+        <v>13.4645</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23603.2</v>
+        <v>23626.33</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23497.96</v>
+        <v>23520.99</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23550.58</v>
+        <v>23573.66</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.5237</v>
+        <v>13.4645</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18516.41</v>
+        <v>18534.55</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18330.33</v>
+        <v>18348.29</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18423.37</v>
+        <v>18441.42</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.5237</v>
+        <v>13.4645</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15573.56</v>
+        <v>15588.82</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15517.96</v>
+        <v>15533.16</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15545.76</v>
+        <v>15560.99</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.5503</v>
+        <v>13.4887</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108761.64</v>
+        <v>108875.28</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109312.43</v>
+        <v>109426.65</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109037.03</v>
+        <v>109150.97</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.5503</v>
+        <v>13.4887</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77993.73</v>
+        <v>78075.23</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78309.02</v>
+        <v>78390.84</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78151.37</v>
+        <v>78233.03</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.5503</v>
+        <v>13.4887</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50948.84</v>
+        <v>51002.08</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50516.14</v>
+        <v>50568.92</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50732.49</v>
+        <v>50785.5</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.5503</v>
+        <v>13.4887</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29292.12</v>
+        <v>29322.72</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29081.05</v>
+        <v>29111.44</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29186.58</v>
+        <v>29217.08</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.5503</v>
+        <v>13.4887</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16646.41</v>
+        <v>16663.81</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16580.63</v>
+        <v>16597.96</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16613.52</v>
+        <v>16630.88</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.5503</v>
+        <v>13.4887</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6749.07</v>
+        <v>6756.12</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6535.51</v>
+        <v>6542.34</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6642.29</v>
+        <v>6649.23</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6174</v>
+        <v>13.5705</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>403697.44</v>
+        <v>403909.95</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>398702.7</v>
+        <v>398912.58</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>401200.07</v>
+        <v>401411.26</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6174</v>
+        <v>13.5705</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>303067.57</v>
+        <v>303227.11</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>304050.49</v>
+        <v>304210.54</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>303559.03</v>
+        <v>303718.83</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6174</v>
+        <v>13.5705</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212057.32</v>
+        <v>212168.95</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211929.39</v>
+        <v>212040.95</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211993.35</v>
+        <v>212104.95</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6174</v>
+        <v>13.5705</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128918.5</v>
+        <v>128986.37</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129202.66</v>
+        <v>129270.67</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129060.58</v>
+        <v>129128.52</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6174</v>
+        <v>13.5705</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62488.47</v>
+        <v>62521.36</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62196.54</v>
+        <v>62229.28</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62342.5</v>
+        <v>62375.32</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6174</v>
+        <v>13.5705</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31913.89</v>
+        <v>31930.69</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31937.99</v>
+        <v>31954.81</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31925.94</v>
+        <v>31942.75</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5228</v>
+        <v>13.4863</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>407237.02</v>
+        <v>407460.21</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>407784.39</v>
+        <v>408007.88</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>407510.7</v>
+        <v>407734.05</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5228</v>
+        <v>13.4863</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>302287.7</v>
+        <v>302453.38</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>300400.25</v>
+        <v>300564.89</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>301343.98</v>
+        <v>301509.13</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5228</v>
+        <v>13.4863</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205042.02</v>
+        <v>205154.4</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205112.16</v>
+        <v>205224.58</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205077.09</v>
+        <v>205189.49</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5228</v>
+        <v>13.4863</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124078.05</v>
+        <v>124146.05</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124595.39</v>
+        <v>124663.67</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124336.72</v>
+        <v>124404.86</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5228</v>
+        <v>13.4863</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49551.24</v>
+        <v>49578.4</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49492.2</v>
+        <v>49519.32</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49521.72</v>
+        <v>49548.86</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5228</v>
+        <v>13.4863</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5450.48</v>
+        <v>5453.46</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5486.42</v>
+        <v>5489.43</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5468.45</v>
+        <v>5471.44</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4386</v>
+        <v>13.4021</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170089.24</v>
+        <v>170186.33</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170116.44</v>
+        <v>170213.55</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170102.84</v>
+        <v>170199.94</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4386</v>
+        <v>13.4021</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111776.87</v>
+        <v>111840.68</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111388.02</v>
+        <v>111451.61</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111582.45</v>
+        <v>111646.14</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4386</v>
+        <v>13.4021</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62599.98</v>
+        <v>62635.71</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62955.05</v>
+        <v>62990.99</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62777.52</v>
+        <v>62813.35</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4386</v>
+        <v>13.4021</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26799.66</v>
+        <v>26814.96</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26999.32</v>
+        <v>27014.73</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26899.49</v>
+        <v>26914.84</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4386</v>
+        <v>13.4021</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6308.36</v>
+        <v>6311.96</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6460</v>
+        <v>6463.69</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6384.18</v>
+        <v>6387.82</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4386</v>
+        <v>13.4021</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3736.14</v>
+        <v>3738.27</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3729.66</v>
+        <v>3731.79</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3732.9</v>
+        <v>3735.03</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4092</v>
+        <v>13.3686</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190251.18</v>
+        <v>190367.29</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191180.15</v>
+        <v>191296.83</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190715.67</v>
+        <v>190832.06</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4092</v>
+        <v>13.3686</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137936.13</v>
+        <v>138020.31</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138898.7</v>
+        <v>138983.46</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138417.41</v>
+        <v>138501.89</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4092</v>
+        <v>13.3686</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87189.46000000001</v>
+        <v>87242.67</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87895.05</v>
+        <v>87948.69</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87542.25</v>
+        <v>87595.67999999999</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4092</v>
+        <v>13.3686</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41647.12</v>
+        <v>41672.54</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41580.33</v>
+        <v>41605.71</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41613.73</v>
+        <v>41639.12</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4092</v>
+        <v>13.3686</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12986.98</v>
+        <v>12994.9</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12843.93</v>
+        <v>12851.77</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12915.45</v>
+        <v>12923.34</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4092</v>
+        <v>13.3686</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4507.29</v>
+        <v>4510.04</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4397.27</v>
+        <v>4399.95</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4452.28</v>
+        <v>4455</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-19
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3575</v>
+        <v>13.3632</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150029.65</v>
+        <v>150026.68</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151921.1</v>
+        <v>151918.09</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150975.37</v>
+        <v>150972.39</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3575</v>
+        <v>13.3632</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114837.94</v>
+        <v>114835.67</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115618.73</v>
+        <v>115616.44</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115228.33</v>
+        <v>115226.05</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3575</v>
+        <v>13.3632</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81882.14</v>
+        <v>81880.52</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82392.37</v>
+        <v>82390.74000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82137.25</v>
+        <v>82135.63</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3575</v>
+        <v>13.3632</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58021.66</v>
+        <v>58020.51</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57581.93</v>
+        <v>57580.79</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57801.79</v>
+        <v>57800.65</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3575</v>
+        <v>13.3632</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37479.69</v>
+        <v>37478.95</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37786.29</v>
+        <v>37785.54</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37632.99</v>
+        <v>37632.25</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3575</v>
+        <v>13.3632</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17046.46</v>
+        <v>17046.13</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16934.53</v>
+        <v>16934.19</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16990.49</v>
+        <v>16990.16</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3474</v>
+        <v>13.3567</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163005.39</v>
+        <v>162999.02</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162130.74</v>
+        <v>162124.4</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162568.06</v>
+        <v>162561.71</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3474</v>
+        <v>13.3567</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122417.55</v>
+        <v>122412.76</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120688.57</v>
+        <v>120683.86</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121553.06</v>
+        <v>121548.31</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3474</v>
+        <v>13.3567</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87459.73</v>
+        <v>87456.31</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86376.71000000001</v>
+        <v>86373.34</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86918.22</v>
+        <v>86914.82000000001</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3474</v>
+        <v>13.3567</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66622.39</v>
+        <v>66619.78999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66154.05</v>
+        <v>66151.46000000001</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66388.22</v>
+        <v>66385.62</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3474</v>
+        <v>13.3567</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52046.49</v>
+        <v>52044.46</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50175.99</v>
+        <v>50174.03</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51111.24</v>
+        <v>51109.24</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3474</v>
+        <v>13.3567</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39454.06</v>
+        <v>39452.52</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40428.99</v>
+        <v>40427.41</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39941.53</v>
+        <v>39939.96</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3629</v>
+        <v>13.3735</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167824.59</v>
+        <v>167815.77</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169370.54</v>
+        <v>169361.63</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168597.57</v>
+        <v>168588.7</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3629</v>
+        <v>13.3735</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120978.16</v>
+        <v>120971.8</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119532.21</v>
+        <v>119525.93</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120255.18</v>
+        <v>120248.86</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3629</v>
+        <v>13.3735</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82871.95</v>
+        <v>82867.59</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82558.94</v>
+        <v>82554.60000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82715.44</v>
+        <v>82711.09</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3629</v>
+        <v>13.3735</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55213.27</v>
+        <v>55210.37</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55517.92</v>
+        <v>55515</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55365.59</v>
+        <v>55362.68</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3629</v>
+        <v>13.3735</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33324.02</v>
+        <v>33322.27</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32933.98</v>
+        <v>32932.25</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33129</v>
+        <v>33127.26</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3629</v>
+        <v>13.3735</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17300.42</v>
+        <v>17299.51</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17986.29</v>
+        <v>17985.35</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17643.35</v>
+        <v>17642.43</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3883</v>
+        <v>13.3991</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129687.53</v>
+        <v>129679.47</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129782.55</v>
+        <v>129774.49</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129735.04</v>
+        <v>129726.98</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3883</v>
+        <v>13.3991</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89815.41</v>
+        <v>89809.83</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88421.73</v>
+        <v>88416.24000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89118.57000000001</v>
+        <v>89113.03</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3883</v>
+        <v>13.3991</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56454.03</v>
+        <v>56450.52</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56742.13</v>
+        <v>56738.61</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56598.08</v>
+        <v>56594.56</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3883</v>
+        <v>13.3991</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29886.8</v>
+        <v>29884.95</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30087.97</v>
+        <v>30086.1</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29987.39</v>
+        <v>29985.52</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3883</v>
+        <v>13.3991</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6854.78</v>
+        <v>6854.36</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6853.48</v>
+        <v>6853.05</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6854.13</v>
+        <v>6853.7</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3883</v>
+        <v>13.3991</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3808.82</v>
+        <v>3808.58</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3718.98</v>
+        <v>3718.75</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3763.9</v>
+        <v>3763.67</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4125</v>
+        <v>13.4236</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109484.34</v>
+        <v>109476.5</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109964.65</v>
+        <v>109956.78</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109724.49</v>
+        <v>109716.64</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4125</v>
+        <v>13.4236</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76779.91</v>
+        <v>76774.41</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76233.64999999999</v>
+        <v>76228.2</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76506.78</v>
+        <v>76501.31</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4125</v>
+        <v>13.4236</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46459.62</v>
+        <v>46456.3</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47570.41</v>
+        <v>47567.01</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47015.01</v>
+        <v>47011.65</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4125</v>
+        <v>13.4236</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28863.45</v>
+        <v>28861.39</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28755.89</v>
+        <v>28753.83</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28809.67</v>
+        <v>28807.61</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4125</v>
+        <v>13.4236</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14159.14</v>
+        <v>14158.13</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14281.9</v>
+        <v>14280.87</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14220.52</v>
+        <v>14219.5</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4125</v>
+        <v>13.4236</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6564.18</v>
+        <v>6563.71</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6402.02</v>
+        <v>6401.56</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6483.1</v>
+        <v>6482.64</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4379</v>
+        <v>13.4492</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49825.7</v>
+        <v>49821.62</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49492.13</v>
+        <v>49488.08</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49658.91</v>
+        <v>49654.85</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4379</v>
+        <v>13.4492</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43833.31</v>
+        <v>43829.72</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44027.91</v>
+        <v>44024.31</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43930.61</v>
+        <v>43927.02</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4379</v>
+        <v>13.4492</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32079.39</v>
+        <v>32076.77</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32421.03</v>
+        <v>32418.37</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32250.21</v>
+        <v>32247.57</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4379</v>
+        <v>13.4492</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22555.94</v>
+        <v>22554.09</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22710.84</v>
+        <v>22708.99</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22633.39</v>
+        <v>22631.54</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4379</v>
+        <v>13.4492</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14497.42</v>
+        <v>14496.23</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14703.72</v>
+        <v>14702.52</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14600.57</v>
+        <v>14599.38</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4379</v>
+        <v>13.4492</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8331.68</v>
+        <v>8331</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8386.879999999999</v>
+        <v>8386.190000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8359.280000000001</v>
+        <v>8358.59</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4645</v>
+        <v>13.4761</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49013.59</v>
+        <v>49009.03</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48292.23</v>
+        <v>48287.74</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48652.91</v>
+        <v>48648.39</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4645</v>
+        <v>13.4761</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43892.36</v>
+        <v>43888.28</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43555.18</v>
+        <v>43551.13</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43723.77</v>
+        <v>43719.7</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4645</v>
+        <v>13.4761</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31699.08</v>
+        <v>31696.13</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31129.23</v>
+        <v>31126.34</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31414.16</v>
+        <v>31411.24</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4645</v>
+        <v>13.4761</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23626.33</v>
+        <v>23624.13</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23520.99</v>
+        <v>23518.8</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23573.66</v>
+        <v>23571.47</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4645</v>
+        <v>13.4761</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18534.55</v>
+        <v>18532.83</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18348.29</v>
+        <v>18346.59</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18441.42</v>
+        <v>18439.71</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4645</v>
+        <v>13.4761</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15588.82</v>
+        <v>15587.37</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15533.16</v>
+        <v>15531.72</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15560.99</v>
+        <v>15559.55</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4887</v>
+        <v>13.5005</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108875.28</v>
+        <v>108864.02</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109426.65</v>
+        <v>109415.33</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109150.97</v>
+        <v>109139.67</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4887</v>
+        <v>13.5005</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78075.23</v>
+        <v>78067.14999999999</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78390.84</v>
+        <v>78382.73</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78233.03</v>
+        <v>78224.94</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4887</v>
+        <v>13.5005</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51002.08</v>
+        <v>50996.8</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50568.92</v>
+        <v>50563.69</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50785.5</v>
+        <v>50780.24</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4887</v>
+        <v>13.5005</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29322.72</v>
+        <v>29319.69</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29111.44</v>
+        <v>29108.43</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29217.08</v>
+        <v>29214.06</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4887</v>
+        <v>13.5005</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16663.81</v>
+        <v>16662.08</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16597.96</v>
+        <v>16596.24</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16630.88</v>
+        <v>16629.16</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4887</v>
+        <v>13.5005</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6756.12</v>
+        <v>6755.42</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6542.34</v>
+        <v>6541.66</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6649.23</v>
+        <v>6648.54</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.5705</v>
+        <v>13.5585</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>403909.95</v>
+        <v>403911.98</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>398912.58</v>
+        <v>398914.59</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>401411.26</v>
+        <v>401413.28</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.5705</v>
+        <v>13.5585</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>303227.11</v>
+        <v>303228.64</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>304210.54</v>
+        <v>304212.07</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>303718.83</v>
+        <v>303720.36</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.5705</v>
+        <v>13.5585</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212168.95</v>
+        <v>212170.01</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212040.95</v>
+        <v>212042.02</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212104.95</v>
+        <v>212106.01</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.5705</v>
+        <v>13.5585</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128986.37</v>
+        <v>128987.02</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129270.67</v>
+        <v>129271.32</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129128.52</v>
+        <v>129129.17</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.5705</v>
+        <v>13.5585</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62521.36</v>
+        <v>62521.68</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62229.28</v>
+        <v>62229.59</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62375.32</v>
+        <v>62375.64</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.5705</v>
+        <v>13.5585</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31930.69</v>
+        <v>31930.85</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31954.81</v>
+        <v>31954.97</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31942.75</v>
+        <v>31942.91</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4863</v>
+        <v>13.4777</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>407460.21</v>
+        <v>407464.5</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>408007.88</v>
+        <v>408012.18</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>407734.05</v>
+        <v>407738.34</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4863</v>
+        <v>13.4777</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>302453.38</v>
+        <v>302456.56</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>300564.89</v>
+        <v>300568.05</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>301509.13</v>
+        <v>301512.31</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4863</v>
+        <v>13.4777</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205154.4</v>
+        <v>205156.56</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205224.58</v>
+        <v>205226.74</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205189.49</v>
+        <v>205191.65</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4863</v>
+        <v>13.4777</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124146.05</v>
+        <v>124147.36</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124663.67</v>
+        <v>124664.99</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124404.86</v>
+        <v>124406.17</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4863</v>
+        <v>13.4777</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49578.4</v>
+        <v>49578.92</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49519.32</v>
+        <v>49519.84</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49548.86</v>
+        <v>49549.38</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4863</v>
+        <v>13.4777</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5453.46</v>
+        <v>5453.52</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5489.43</v>
+        <v>5489.48</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5471.44</v>
+        <v>5471.5</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4021</v>
+        <v>13.3988</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170186.33</v>
+        <v>170187.41</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170213.55</v>
+        <v>170214.63</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170199.94</v>
+        <v>170201.02</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4021</v>
+        <v>13.3988</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111840.68</v>
+        <v>111841.39</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111451.61</v>
+        <v>111452.32</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111646.14</v>
+        <v>111646.85</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4021</v>
+        <v>13.3988</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62635.71</v>
+        <v>62636.11</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62990.99</v>
+        <v>62991.39</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62813.35</v>
+        <v>62813.75</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4021</v>
+        <v>13.3988</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26814.96</v>
+        <v>26815.13</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27014.73</v>
+        <v>27014.9</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26914.84</v>
+        <v>26915.01</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4021</v>
+        <v>13.3988</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6311.96</v>
+        <v>6312</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6463.69</v>
+        <v>6463.73</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6387.82</v>
+        <v>6387.86</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4021</v>
+        <v>13.3988</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3738.27</v>
+        <v>3738.3</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3731.79</v>
+        <v>3731.81</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3735.03</v>
+        <v>3735.05</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3686</v>
+        <v>13.3703</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190367.29</v>
+        <v>190366.44</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191296.83</v>
+        <v>191295.97</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190832.06</v>
+        <v>190831.2</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3686</v>
+        <v>13.3703</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138020.31</v>
+        <v>138019.69</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138983.46</v>
+        <v>138982.84</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138501.89</v>
+        <v>138501.27</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3686</v>
+        <v>13.3703</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87242.67</v>
+        <v>87242.27</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87948.69</v>
+        <v>87948.28999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87595.67999999999</v>
+        <v>87595.28</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3686</v>
+        <v>13.3703</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41672.54</v>
+        <v>41672.35</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41605.71</v>
+        <v>41605.52</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41639.12</v>
+        <v>41638.94</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3686</v>
+        <v>13.3703</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12994.9</v>
+        <v>12994.85</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12851.77</v>
+        <v>12851.71</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12923.34</v>
+        <v>12923.28</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3686</v>
+        <v>13.3703</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4510.04</v>
+        <v>4510.02</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4399.95</v>
+        <v>4399.93</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4455</v>
+        <v>4454.98</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-22
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3632</v>
+        <v>13.361</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150026.68</v>
+        <v>150177.23</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151918.09</v>
+        <v>152070.53</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150972.39</v>
+        <v>151123.88</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3632</v>
+        <v>13.361</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114835.67</v>
+        <v>114950.9</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115616.44</v>
+        <v>115732.46</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115226.05</v>
+        <v>115341.68</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3632</v>
+        <v>13.361</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81880.52</v>
+        <v>81962.67999999999</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82390.74000000001</v>
+        <v>82473.41</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82135.63</v>
+        <v>82218.05</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3632</v>
+        <v>13.361</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58020.51</v>
+        <v>58078.74</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57580.79</v>
+        <v>57638.57</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57800.65</v>
+        <v>57858.65</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3632</v>
+        <v>13.361</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37478.95</v>
+        <v>37516.56</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37785.54</v>
+        <v>37823.46</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37632.25</v>
+        <v>37670.01</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3632</v>
+        <v>13.361</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17046.13</v>
+        <v>17063.23</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16934.19</v>
+        <v>16951.18</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16990.16</v>
+        <v>17007.21</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3567</v>
+        <v>13.3432</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162999.02</v>
+        <v>163170.4</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162124.4</v>
+        <v>162294.86</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162561.71</v>
+        <v>162732.63</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3567</v>
+        <v>13.3432</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122412.76</v>
+        <v>122541.47</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120683.86</v>
+        <v>120810.75</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121548.31</v>
+        <v>121676.11</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3567</v>
+        <v>13.3432</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87456.31</v>
+        <v>87548.25999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86373.34</v>
+        <v>86464.14999999999</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86914.82000000001</v>
+        <v>87006.21000000001</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3567</v>
+        <v>13.3432</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66619.78999999999</v>
+        <v>66689.83</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66151.46000000001</v>
+        <v>66221.00999999999</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66385.62</v>
+        <v>66455.42</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3567</v>
+        <v>13.3432</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52044.46</v>
+        <v>52099.18</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50174.03</v>
+        <v>50226.78</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51109.24</v>
+        <v>51162.98</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3567</v>
+        <v>13.3432</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39452.52</v>
+        <v>39494</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40427.41</v>
+        <v>40469.92</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39939.96</v>
+        <v>39981.96</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3735</v>
+        <v>13.3457</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167815.77</v>
+        <v>168005.88</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169361.63</v>
+        <v>169553.49</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168588.7</v>
+        <v>168779.68</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3735</v>
+        <v>13.3457</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120971.8</v>
+        <v>121108.84</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119525.93</v>
+        <v>119661.33</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120248.86</v>
+        <v>120385.08</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3735</v>
+        <v>13.3457</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82867.59</v>
+        <v>82961.47</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82554.60000000001</v>
+        <v>82648.12</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82711.09</v>
+        <v>82804.78999999999</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3735</v>
+        <v>13.3457</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55210.37</v>
+        <v>55272.91</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55515</v>
+        <v>55577.89</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55362.68</v>
+        <v>55425.4</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3735</v>
+        <v>13.3457</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33322.27</v>
+        <v>33360.02</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32932.25</v>
+        <v>32969.55</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33127.26</v>
+        <v>33164.79</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3735</v>
+        <v>13.3457</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17299.51</v>
+        <v>17319.1</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17985.35</v>
+        <v>18005.72</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17642.43</v>
+        <v>17662.41</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3991</v>
+        <v>13.3608</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129679.47</v>
+        <v>129837.16</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129774.49</v>
+        <v>129932.29</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129726.98</v>
+        <v>129884.72</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3991</v>
+        <v>13.3608</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89809.83</v>
+        <v>89919.03</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88416.24000000001</v>
+        <v>88523.75</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89113.03</v>
+        <v>89221.39</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3991</v>
+        <v>13.3608</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56450.52</v>
+        <v>56519.16</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56738.61</v>
+        <v>56807.6</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56594.56</v>
+        <v>56663.38</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3991</v>
+        <v>13.3608</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29884.95</v>
+        <v>29921.29</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30086.1</v>
+        <v>30122.69</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29985.52</v>
+        <v>30021.99</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3991</v>
+        <v>13.3608</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6854.36</v>
+        <v>6862.69</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6853.05</v>
+        <v>6861.38</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6853.7</v>
+        <v>6862.04</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3991</v>
+        <v>13.3608</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3808.58</v>
+        <v>3813.22</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3718.75</v>
+        <v>3723.27</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3763.67</v>
+        <v>3768.24</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4236</v>
+        <v>13.3752</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109476.5</v>
+        <v>109619.97</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109956.78</v>
+        <v>110100.88</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109716.64</v>
+        <v>109860.42</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4236</v>
+        <v>13.3752</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76774.41</v>
+        <v>76875.03</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76228.2</v>
+        <v>76328.09</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76501.31</v>
+        <v>76601.56</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4236</v>
+        <v>13.3752</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46456.3</v>
+        <v>46517.18</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47567.01</v>
+        <v>47629.34</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47011.65</v>
+        <v>47073.26</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4236</v>
+        <v>13.3752</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28861.39</v>
+        <v>28899.21</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28753.83</v>
+        <v>28791.51</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28807.61</v>
+        <v>28845.36</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4236</v>
+        <v>13.3752</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14158.13</v>
+        <v>14176.68</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14280.87</v>
+        <v>14299.59</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14219.5</v>
+        <v>14238.14</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4236</v>
+        <v>13.3752</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6563.71</v>
+        <v>6572.32</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6401.56</v>
+        <v>6409.95</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6482.64</v>
+        <v>6491.13</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4492</v>
+        <v>13.3903</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49821.62</v>
+        <v>49892.64</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49488.08</v>
+        <v>49558.62</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49654.85</v>
+        <v>49725.63</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4492</v>
+        <v>13.3903</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43829.72</v>
+        <v>43892.2</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44024.31</v>
+        <v>44087.06</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43927.02</v>
+        <v>43989.63</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4492</v>
+        <v>13.3903</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32076.77</v>
+        <v>32122.49</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32418.37</v>
+        <v>32464.58</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32247.57</v>
+        <v>32293.54</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4492</v>
+        <v>13.3903</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22554.09</v>
+        <v>22586.24</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22708.99</v>
+        <v>22741.35</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22631.54</v>
+        <v>22663.8</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4492</v>
+        <v>13.3903</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14496.23</v>
+        <v>14516.9</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14702.52</v>
+        <v>14723.48</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14599.38</v>
+        <v>14620.19</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4492</v>
+        <v>13.3903</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8331</v>
+        <v>8342.870000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8386.190000000001</v>
+        <v>8398.15</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8358.59</v>
+        <v>8370.51</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4761</v>
+        <v>13.406</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49009.03</v>
+        <v>49085.63</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48287.74</v>
+        <v>48363.21</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48648.39</v>
+        <v>48724.42</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4761</v>
+        <v>13.406</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43888.28</v>
+        <v>43956.87</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43551.13</v>
+        <v>43619.2</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43719.7</v>
+        <v>43788.03</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4761</v>
+        <v>13.406</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31696.13</v>
+        <v>31745.67</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31126.34</v>
+        <v>31174.99</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31411.24</v>
+        <v>31460.33</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4761</v>
+        <v>13.406</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23624.13</v>
+        <v>23661.05</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23518.8</v>
+        <v>23555.56</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23571.47</v>
+        <v>23608.31</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4761</v>
+        <v>13.406</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18532.83</v>
+        <v>18561.79</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18346.59</v>
+        <v>18375.26</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18439.71</v>
+        <v>18468.53</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4761</v>
+        <v>13.406</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15587.37</v>
+        <v>15611.74</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15531.72</v>
+        <v>15556</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15559.55</v>
+        <v>15583.87</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.5005</v>
+        <v>13.4204</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108864.02</v>
+        <v>109049.52</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109415.33</v>
+        <v>109601.77</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109139.67</v>
+        <v>109325.65</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.5005</v>
+        <v>13.4204</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78067.14999999999</v>
+        <v>78200.17</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78382.73</v>
+        <v>78516.3</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78224.94</v>
+        <v>78358.24000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.5005</v>
+        <v>13.4204</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50996.8</v>
+        <v>51083.7</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50563.69</v>
+        <v>50649.85</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50780.24</v>
+        <v>50866.77</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.5005</v>
+        <v>13.4204</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29319.69</v>
+        <v>29369.65</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29108.43</v>
+        <v>29158.03</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29214.06</v>
+        <v>29263.84</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.5005</v>
+        <v>13.4204</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16662.08</v>
+        <v>16690.48</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16596.24</v>
+        <v>16624.52</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16629.16</v>
+        <v>16657.5</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.5005</v>
+        <v>13.4204</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6755.42</v>
+        <v>6766.94</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6541.66</v>
+        <v>6552.81</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6648.54</v>
+        <v>6659.87</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.5585</v>
+        <v>13.5566</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>403911.98</v>
+        <v>404320.05</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>398914.59</v>
+        <v>399317.61</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>401413.28</v>
+        <v>401818.83</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.5585</v>
+        <v>13.5566</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>303228.64</v>
+        <v>303534.99</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>304212.07</v>
+        <v>304519.42</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>303720.36</v>
+        <v>304027.2</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.5585</v>
+        <v>13.5566</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212170.01</v>
+        <v>212384.37</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212042.02</v>
+        <v>212256.24</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212106.01</v>
+        <v>212320.3</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.5585</v>
+        <v>13.5566</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128987.02</v>
+        <v>129117.33</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129271.32</v>
+        <v>129401.92</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129129.17</v>
+        <v>129259.63</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.5585</v>
+        <v>13.5566</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62521.68</v>
+        <v>62584.84</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62229.59</v>
+        <v>62292.46</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62375.64</v>
+        <v>62438.65</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.5585</v>
+        <v>13.5566</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31930.85</v>
+        <v>31963.11</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31954.97</v>
+        <v>31987.25</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31942.91</v>
+        <v>31975.18</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4777</v>
+        <v>13.4981</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>407464.5</v>
+        <v>407863.98</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>408012.18</v>
+        <v>408412.2</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>407738.34</v>
+        <v>408138.09</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4777</v>
+        <v>13.4981</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>302456.56</v>
+        <v>302753.1</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>300568.05</v>
+        <v>300862.74</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>301512.31</v>
+        <v>301807.92</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4777</v>
+        <v>13.4981</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205156.56</v>
+        <v>205357.7</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205226.74</v>
+        <v>205427.95</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205191.65</v>
+        <v>205392.82</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4777</v>
+        <v>13.4981</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124147.36</v>
+        <v>124269.08</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124664.99</v>
+        <v>124787.21</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124406.17</v>
+        <v>124528.14</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4777</v>
+        <v>13.4981</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49578.92</v>
+        <v>49627.53</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49519.84</v>
+        <v>49568.39</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49549.38</v>
+        <v>49597.96</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4777</v>
+        <v>13.4981</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5453.52</v>
+        <v>5458.87</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5489.48</v>
+        <v>5494.87</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5471.5</v>
+        <v>5476.87</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3988</v>
+        <v>13.4217</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170187.41</v>
+        <v>170350.11</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170214.63</v>
+        <v>170377.35</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170201.02</v>
+        <v>170363.73</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3988</v>
+        <v>13.4217</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111841.39</v>
+        <v>111948.31</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111452.32</v>
+        <v>111558.86</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111646.85</v>
+        <v>111753.58</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3988</v>
+        <v>13.4217</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62636.11</v>
+        <v>62695.99</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62991.39</v>
+        <v>63051.61</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62813.75</v>
+        <v>62873.8</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3988</v>
+        <v>13.4217</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26815.13</v>
+        <v>26840.76</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27014.9</v>
+        <v>27040.73</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26915.01</v>
+        <v>26940.74</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3988</v>
+        <v>13.4217</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6312</v>
+        <v>6318.03</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6463.73</v>
+        <v>6469.91</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6387.86</v>
+        <v>6393.97</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3988</v>
+        <v>13.4217</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3738.3</v>
+        <v>3741.87</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3731.81</v>
+        <v>3735.38</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3735.05</v>
+        <v>3738.62</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3703</v>
+        <v>13.3805</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190366.44</v>
+        <v>190550.92</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191295.97</v>
+        <v>191481.35</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190831.2</v>
+        <v>191016.13</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3703</v>
+        <v>13.3805</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138019.69</v>
+        <v>138153.44</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138982.84</v>
+        <v>139117.53</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138501.27</v>
+        <v>138635.49</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3703</v>
+        <v>13.3805</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87242.27</v>
+        <v>87326.82000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87948.28999999999</v>
+        <v>88033.52</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87595.28</v>
+        <v>87680.17</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3703</v>
+        <v>13.3805</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41672.35</v>
+        <v>41712.74</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41605.52</v>
+        <v>41645.84</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41638.94</v>
+        <v>41679.29</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3703</v>
+        <v>13.3805</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12994.85</v>
+        <v>13007.44</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12851.71</v>
+        <v>12864.17</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12923.28</v>
+        <v>12935.8</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3703</v>
+        <v>13.3805</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4510.02</v>
+        <v>4514.4</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4399.93</v>
+        <v>4404.19</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4454.98</v>
+        <v>4459.29</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-23
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.361</v>
+        <v>13.3421</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150177.23</v>
+        <v>150261.61</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152070.53</v>
+        <v>152155.98</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151123.88</v>
+        <v>151208.79</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.361</v>
+        <v>13.3421</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114950.9</v>
+        <v>115015.49</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115732.46</v>
+        <v>115797.48</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115341.68</v>
+        <v>115406.49</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.361</v>
+        <v>13.3421</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81962.67999999999</v>
+        <v>82008.74000000001</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82473.41</v>
+        <v>82519.75</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82218.05</v>
+        <v>82264.24000000001</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.361</v>
+        <v>13.3421</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58078.74</v>
+        <v>58111.37</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57638.57</v>
+        <v>57670.95</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57858.65</v>
+        <v>57891.16</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.361</v>
+        <v>13.3421</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37516.56</v>
+        <v>37537.64</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37823.46</v>
+        <v>37844.71</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37670.01</v>
+        <v>37691.17</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.361</v>
+        <v>13.3421</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17063.23</v>
+        <v>17072.82</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16951.18</v>
+        <v>16960.71</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17007.21</v>
+        <v>17016.76</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3432</v>
+        <v>13.3219</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163170.4</v>
+        <v>163265.77</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162294.86</v>
+        <v>162389.72</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162732.63</v>
+        <v>162827.75</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3432</v>
+        <v>13.3219</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122541.47</v>
+        <v>122613.09</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120810.75</v>
+        <v>120881.36</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121676.11</v>
+        <v>121747.23</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3432</v>
+        <v>13.3219</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87548.25999999999</v>
+        <v>87599.42999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86464.14999999999</v>
+        <v>86514.69</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87006.21000000001</v>
+        <v>87057.06</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3432</v>
+        <v>13.3219</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66689.83</v>
+        <v>66728.81</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66221.00999999999</v>
+        <v>66259.72</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66455.42</v>
+        <v>66494.27</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3432</v>
+        <v>13.3219</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52099.18</v>
+        <v>52129.63</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50226.78</v>
+        <v>50256.14</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51162.98</v>
+        <v>51192.89</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3432</v>
+        <v>13.3219</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39494</v>
+        <v>39517.08</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40469.92</v>
+        <v>40493.57</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39981.96</v>
+        <v>40005.33</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3457</v>
+        <v>13.3209</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168005.88</v>
+        <v>168109.67</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169553.49</v>
+        <v>169658.24</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168779.68</v>
+        <v>168883.96</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3457</v>
+        <v>13.3209</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121108.84</v>
+        <v>121183.66</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119661.33</v>
+        <v>119735.25</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120385.08</v>
+        <v>120459.46</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3457</v>
+        <v>13.3209</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82961.47</v>
+        <v>83012.72</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82648.12</v>
+        <v>82699.17999999999</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82804.78999999999</v>
+        <v>82855.95</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3457</v>
+        <v>13.3209</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55272.91</v>
+        <v>55307.06</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55577.89</v>
+        <v>55612.22</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55425.4</v>
+        <v>55459.64</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3457</v>
+        <v>13.3209</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33360.02</v>
+        <v>33380.63</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32969.55</v>
+        <v>32989.92</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33164.79</v>
+        <v>33185.28</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3457</v>
+        <v>13.3209</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17319.1</v>
+        <v>17329.8</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18005.72</v>
+        <v>18016.85</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17662.41</v>
+        <v>17673.32</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3608</v>
+        <v>13.3347</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129837.16</v>
+        <v>129920.87</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129932.29</v>
+        <v>130016.07</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129884.72</v>
+        <v>129968.47</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3608</v>
+        <v>13.3347</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89919.03</v>
+        <v>89977.00999999999</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88523.75</v>
+        <v>88580.83</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89221.39</v>
+        <v>89278.92</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3608</v>
+        <v>13.3347</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56519.16</v>
+        <v>56555.6</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56807.6</v>
+        <v>56844.23</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56663.38</v>
+        <v>56699.92</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3608</v>
+        <v>13.3347</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29921.29</v>
+        <v>29940.58</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30122.69</v>
+        <v>30142.11</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30021.99</v>
+        <v>30041.34</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3608</v>
+        <v>13.3347</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6862.69</v>
+        <v>6867.12</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6861.38</v>
+        <v>6865.81</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6862.04</v>
+        <v>6866.46</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3608</v>
+        <v>13.3347</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3813.22</v>
+        <v>3815.67</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3723.27</v>
+        <v>3725.68</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3768.24</v>
+        <v>3770.67</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3752</v>
+        <v>13.3479</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109619.97</v>
+        <v>109693.68</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110100.88</v>
+        <v>110174.91</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109860.42</v>
+        <v>109934.3</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3752</v>
+        <v>13.3479</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76875.03</v>
+        <v>76926.72</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76328.09</v>
+        <v>76379.42</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76601.56</v>
+        <v>76653.07000000001</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3752</v>
+        <v>13.3479</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46517.18</v>
+        <v>46548.45</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47629.34</v>
+        <v>47661.37</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47073.26</v>
+        <v>47104.91</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3752</v>
+        <v>13.3479</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28899.21</v>
+        <v>28918.64</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28791.51</v>
+        <v>28810.87</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28845.36</v>
+        <v>28864.76</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3752</v>
+        <v>13.3479</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14176.68</v>
+        <v>14186.21</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14299.59</v>
+        <v>14309.21</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14238.14</v>
+        <v>14247.71</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3752</v>
+        <v>13.3479</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6572.32</v>
+        <v>6576.74</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6409.95</v>
+        <v>6414.26</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6491.13</v>
+        <v>6495.5</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.3903</v>
+        <v>13.3616</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49892.64</v>
+        <v>49927.73</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49558.62</v>
+        <v>49593.47</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49725.63</v>
+        <v>49760.6</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.3903</v>
+        <v>13.3616</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43892.2</v>
+        <v>43923.07</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44087.06</v>
+        <v>44118.07</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43989.63</v>
+        <v>44020.57</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.3903</v>
+        <v>13.3616</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32122.49</v>
+        <v>32145.08</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32464.58</v>
+        <v>32487.42</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32293.54</v>
+        <v>32316.25</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.3903</v>
+        <v>13.3616</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22586.24</v>
+        <v>22602.13</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22741.35</v>
+        <v>22757.35</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22663.8</v>
+        <v>22679.74</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.3903</v>
+        <v>13.3616</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14516.9</v>
+        <v>14527.11</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14723.48</v>
+        <v>14733.83</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14620.19</v>
+        <v>14630.47</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.3903</v>
+        <v>13.3616</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8342.870000000001</v>
+        <v>8348.74</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8398.15</v>
+        <v>8404.049999999999</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8370.51</v>
+        <v>8376.4</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.406</v>
+        <v>13.376</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49085.63</v>
+        <v>49121.84</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48363.21</v>
+        <v>48398.9</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48724.42</v>
+        <v>48760.37</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.406</v>
+        <v>13.376</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43956.87</v>
+        <v>43989.3</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43619.2</v>
+        <v>43651.38</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43788.03</v>
+        <v>43820.34</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.406</v>
+        <v>13.376</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31745.67</v>
+        <v>31769.09</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31174.99</v>
+        <v>31197.99</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31460.33</v>
+        <v>31483.54</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.406</v>
+        <v>13.376</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23661.05</v>
+        <v>23678.51</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23555.56</v>
+        <v>23572.94</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23608.31</v>
+        <v>23625.73</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.406</v>
+        <v>13.376</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18561.79</v>
+        <v>18575.49</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18375.26</v>
+        <v>18388.82</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18468.53</v>
+        <v>18482.15</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.406</v>
+        <v>13.376</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15611.74</v>
+        <v>15623.25</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15556</v>
+        <v>15567.47</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15583.87</v>
+        <v>15595.36</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4204</v>
+        <v>13.3892</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109049.52</v>
+        <v>109133.62</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109601.77</v>
+        <v>109686.3</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109325.65</v>
+        <v>109409.96</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4204</v>
+        <v>13.3892</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78200.17</v>
+        <v>78260.48</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78516.3</v>
+        <v>78576.85000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78358.24000000001</v>
+        <v>78418.67</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4204</v>
+        <v>13.3892</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51083.7</v>
+        <v>51123.09</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50649.85</v>
+        <v>50688.91</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50866.77</v>
+        <v>50906</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4204</v>
+        <v>13.3892</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29369.65</v>
+        <v>29392.3</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29158.03</v>
+        <v>29180.52</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29263.84</v>
+        <v>29286.41</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4204</v>
+        <v>13.3892</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16690.48</v>
+        <v>16703.35</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16624.52</v>
+        <v>16637.34</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16657.5</v>
+        <v>16670.34</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4204</v>
+        <v>13.3892</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6766.94</v>
+        <v>6772.15</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6552.81</v>
+        <v>6557.86</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6659.87</v>
+        <v>6665.01</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.5566</v>
+        <v>13.55</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>404320.05</v>
+        <v>404524.91</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>399317.61</v>
+        <v>399519.94</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>401818.83</v>
+        <v>402022.42</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.5566</v>
+        <v>13.55</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>303534.99</v>
+        <v>303688.79</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>304519.42</v>
+        <v>304673.71</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>304027.2</v>
+        <v>304181.25</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.5566</v>
+        <v>13.55</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212384.37</v>
+        <v>212491.98</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212256.24</v>
+        <v>212363.79</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212320.3</v>
+        <v>212427.88</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.5566</v>
+        <v>13.55</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129117.33</v>
+        <v>129182.75</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129401.92</v>
+        <v>129467.49</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129259.63</v>
+        <v>129325.12</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.5566</v>
+        <v>13.55</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62584.84</v>
+        <v>62616.55</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62292.46</v>
+        <v>62324.03</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62438.65</v>
+        <v>62470.29</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.5566</v>
+        <v>13.55</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31963.11</v>
+        <v>31979.31</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31987.25</v>
+        <v>32003.46</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31975.18</v>
+        <v>31991.38</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4981</v>
+        <v>13.4937</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>407863.98</v>
+        <v>408070.97</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>408412.2</v>
+        <v>408619.47</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>408138.09</v>
+        <v>408345.22</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4981</v>
+        <v>13.4937</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>302753.1</v>
+        <v>302906.74</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>300862.74</v>
+        <v>301015.42</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>301807.92</v>
+        <v>301961.08</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4981</v>
+        <v>13.4937</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205357.7</v>
+        <v>205461.91</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205427.95</v>
+        <v>205532.2</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205392.82</v>
+        <v>205497.06</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4981</v>
+        <v>13.4937</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124269.08</v>
+        <v>124332.14</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124787.21</v>
+        <v>124850.54</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124528.14</v>
+        <v>124591.34</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4981</v>
+        <v>13.4937</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49627.53</v>
+        <v>49652.72</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49568.39</v>
+        <v>49593.55</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49597.96</v>
+        <v>49623.13</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4981</v>
+        <v>13.4937</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5458.87</v>
+        <v>5461.64</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5494.87</v>
+        <v>5497.66</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5476.87</v>
+        <v>5479.65</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4217</v>
+        <v>13.4111</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170350.11</v>
+        <v>170438.55</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170377.35</v>
+        <v>170465.81</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170363.73</v>
+        <v>170452.18</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4217</v>
+        <v>13.4111</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111948.31</v>
+        <v>112006.43</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111558.86</v>
+        <v>111616.78</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111753.58</v>
+        <v>111811.61</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4217</v>
+        <v>13.4111</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62695.99</v>
+        <v>62728.54</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63051.61</v>
+        <v>63084.34</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62873.8</v>
+        <v>62906.44</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4217</v>
+        <v>13.4111</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26840.76</v>
+        <v>26854.7</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27040.73</v>
+        <v>27054.76</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26940.74</v>
+        <v>26954.73</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4217</v>
+        <v>13.4111</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6318.03</v>
+        <v>6321.31</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6469.91</v>
+        <v>6473.27</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6393.97</v>
+        <v>6397.29</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4217</v>
+        <v>13.4111</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3741.87</v>
+        <v>3743.81</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3735.38</v>
+        <v>3737.32</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3738.62</v>
+        <v>3740.56</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3805</v>
+        <v>13.3644</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190550.92</v>
+        <v>190654</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191481.35</v>
+        <v>191584.93</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191016.13</v>
+        <v>191119.46</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3805</v>
+        <v>13.3644</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138153.44</v>
+        <v>138228.18</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139117.53</v>
+        <v>139192.78</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138635.49</v>
+        <v>138710.48</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3805</v>
+        <v>13.3644</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87326.82000000001</v>
+        <v>87374.06</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88033.52</v>
+        <v>88081.14</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87680.17</v>
+        <v>87727.60000000001</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3805</v>
+        <v>13.3644</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41712.74</v>
+        <v>41735.3</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41645.84</v>
+        <v>41668.37</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41679.29</v>
+        <v>41701.83</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3805</v>
+        <v>13.3644</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13007.44</v>
+        <v>13014.47</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12864.17</v>
+        <v>12871.12</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12935.8</v>
+        <v>12942.8</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3805</v>
+        <v>13.3644</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4514.4</v>
+        <v>4516.84</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4404.19</v>
+        <v>4406.58</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4459.29</v>
+        <v>4461.71</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-24
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3421</v>
+        <v>13.3587</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150261.61</v>
+        <v>150327.95</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152155.98</v>
+        <v>152223.16</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151208.79</v>
+        <v>151275.55</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3421</v>
+        <v>13.3587</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115015.49</v>
+        <v>115066.27</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115797.48</v>
+        <v>115848.61</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115406.49</v>
+        <v>115457.44</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3421</v>
+        <v>13.3587</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82008.74000000001</v>
+        <v>82044.94</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82519.75</v>
+        <v>82556.19</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82264.24000000001</v>
+        <v>82300.56</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3421</v>
+        <v>13.3587</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58111.37</v>
+        <v>58137.02</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57670.95</v>
+        <v>57696.41</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57891.16</v>
+        <v>57916.72</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3421</v>
+        <v>13.3587</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37537.64</v>
+        <v>37554.21</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37844.71</v>
+        <v>37861.42</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37691.17</v>
+        <v>37707.81</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3421</v>
+        <v>13.3587</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17072.82</v>
+        <v>17080.36</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16960.71</v>
+        <v>16968.2</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17016.76</v>
+        <v>17024.28</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3219</v>
+        <v>13.3495</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163265.77</v>
+        <v>163328.52</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162389.72</v>
+        <v>162452.13</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162827.75</v>
+        <v>162890.32</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3219</v>
+        <v>13.3495</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122613.09</v>
+        <v>122660.21</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120881.36</v>
+        <v>120927.81</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121747.23</v>
+        <v>121794.01</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3219</v>
+        <v>13.3495</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87599.42999999999</v>
+        <v>87633.10000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86514.69</v>
+        <v>86547.94</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87057.06</v>
+        <v>87090.52</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3219</v>
+        <v>13.3495</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66728.81</v>
+        <v>66754.46000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66259.72</v>
+        <v>66285.17999999999</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66494.27</v>
+        <v>66519.82000000001</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3219</v>
+        <v>13.3495</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52129.63</v>
+        <v>52149.66</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50256.14</v>
+        <v>50275.45</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51192.89</v>
+        <v>51212.56</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3219</v>
+        <v>13.3495</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39517.08</v>
+        <v>39532.27</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40493.57</v>
+        <v>40509.13</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40005.33</v>
+        <v>40020.7</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3209</v>
+        <v>13.3565</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168109.67</v>
+        <v>168164.25</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169658.24</v>
+        <v>169713.33</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168883.96</v>
+        <v>168938.79</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3209</v>
+        <v>13.3565</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121183.66</v>
+        <v>121223</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119735.25</v>
+        <v>119774.13</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120459.46</v>
+        <v>120498.57</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3209</v>
+        <v>13.3565</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83012.72</v>
+        <v>83039.67</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82699.17999999999</v>
+        <v>82726.03</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82855.95</v>
+        <v>82882.85000000001</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3209</v>
+        <v>13.3565</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55307.06</v>
+        <v>55325.01</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55612.22</v>
+        <v>55630.28</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55459.64</v>
+        <v>55477.65</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3209</v>
+        <v>13.3565</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33380.63</v>
+        <v>33391.47</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32989.92</v>
+        <v>33000.63</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33185.28</v>
+        <v>33196.05</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3209</v>
+        <v>13.3565</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17329.8</v>
+        <v>17335.43</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18016.85</v>
+        <v>18022.69</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17673.32</v>
+        <v>17679.06</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3347</v>
+        <v>13.3777</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129920.87</v>
+        <v>129954.17</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130016.07</v>
+        <v>130049.39</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129968.47</v>
+        <v>130001.78</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3347</v>
+        <v>13.3777</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89977.00999999999</v>
+        <v>90000.07000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88580.83</v>
+        <v>88603.52</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89278.92</v>
+        <v>89301.8</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3347</v>
+        <v>13.3777</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56555.6</v>
+        <v>56570.1</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56844.23</v>
+        <v>56858.8</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56699.92</v>
+        <v>56714.45</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3347</v>
+        <v>13.3777</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29940.58</v>
+        <v>29948.25</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30142.11</v>
+        <v>30149.83</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30041.34</v>
+        <v>30049.04</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3347</v>
+        <v>13.3777</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6867.12</v>
+        <v>6868.88</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6865.81</v>
+        <v>6867.57</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6866.46</v>
+        <v>6868.22</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3347</v>
+        <v>13.3777</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3815.67</v>
+        <v>3816.65</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3725.68</v>
+        <v>3726.63</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3770.67</v>
+        <v>3771.64</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3479</v>
+        <v>13.3979</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109693.68</v>
+        <v>109713.46</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110174.91</v>
+        <v>110194.77</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109934.3</v>
+        <v>109954.11</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3479</v>
+        <v>13.3979</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76926.72</v>
+        <v>76940.59</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76379.42</v>
+        <v>76393.19</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76653.07000000001</v>
+        <v>76666.89</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3479</v>
+        <v>13.3979</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46548.45</v>
+        <v>46556.85</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47661.37</v>
+        <v>47669.96</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47104.91</v>
+        <v>47113.4</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3479</v>
+        <v>13.3979</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28918.64</v>
+        <v>28923.86</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28810.87</v>
+        <v>28816.06</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28864.76</v>
+        <v>28869.96</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3479</v>
+        <v>13.3979</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14186.21</v>
+        <v>14188.77</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14309.21</v>
+        <v>14311.78</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14247.71</v>
+        <v>14250.28</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3479</v>
+        <v>13.3979</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6576.74</v>
+        <v>6577.92</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6414.26</v>
+        <v>6415.42</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6495.5</v>
+        <v>6496.67</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.4191</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49927.73</v>
+        <v>49932.2</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49593.47</v>
+        <v>49597.92</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49760.6</v>
+        <v>49765.06</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.4191</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43923.07</v>
+        <v>43927</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44118.07</v>
+        <v>44122.02</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44020.57</v>
+        <v>44024.51</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.4191</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32145.08</v>
+        <v>32147.96</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32487.42</v>
+        <v>32490.32</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32316.25</v>
+        <v>32319.14</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.4191</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22602.13</v>
+        <v>22604.15</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22757.35</v>
+        <v>22759.39</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22679.74</v>
+        <v>22681.77</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.4191</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14527.11</v>
+        <v>14528.41</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14733.83</v>
+        <v>14735.15</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14630.47</v>
+        <v>14631.78</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.4191</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8348.74</v>
+        <v>8349.49</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8404.049999999999</v>
+        <v>8404.799999999999</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8376.4</v>
+        <v>8377.15</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.376</v>
+        <v>13.4412</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49121.84</v>
+        <v>49120.99</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48398.9</v>
+        <v>48398.05</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48760.37</v>
+        <v>48759.52</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.376</v>
+        <v>13.4412</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43989.3</v>
+        <v>43988.54</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43651.38</v>
+        <v>43650.62</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43820.34</v>
+        <v>43819.58</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.376</v>
+        <v>13.4412</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31769.09</v>
+        <v>31768.54</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31197.99</v>
+        <v>31197.44</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31483.54</v>
+        <v>31482.99</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.376</v>
+        <v>13.4412</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23678.51</v>
+        <v>23678.1</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23572.94</v>
+        <v>23572.53</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23625.73</v>
+        <v>23625.31</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.376</v>
+        <v>13.4412</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18575.49</v>
+        <v>18575.16</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18388.82</v>
+        <v>18388.5</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18482.15</v>
+        <v>18481.83</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.376</v>
+        <v>13.4412</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15623.25</v>
+        <v>15622.98</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15567.47</v>
+        <v>15567.2</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15595.36</v>
+        <v>15595.09</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.4615</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109133.62</v>
+        <v>109119.87</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109686.3</v>
+        <v>109672.47</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109409.96</v>
+        <v>109396.17</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.4615</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78260.48</v>
+        <v>78250.62</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78576.85000000001</v>
+        <v>78566.95</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78418.67</v>
+        <v>78408.78</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.4615</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51123.09</v>
+        <v>51116.65</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50688.91</v>
+        <v>50682.52</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50906</v>
+        <v>50899.59</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.4615</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29392.3</v>
+        <v>29388.6</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29180.52</v>
+        <v>29176.84</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29286.41</v>
+        <v>29282.72</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.4615</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16703.35</v>
+        <v>16701.24</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16637.34</v>
+        <v>16635.25</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16670.34</v>
+        <v>16668.24</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.4615</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6772.15</v>
+        <v>6771.3</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6557.86</v>
+        <v>6557.03</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6665.01</v>
+        <v>6664.17</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.55</v>
+        <v>13.492</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>404524.91</v>
+        <v>404735.51</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>399519.94</v>
+        <v>399727.93</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>402022.42</v>
+        <v>402231.72</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.55</v>
+        <v>13.492</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>303688.79</v>
+        <v>303846.89</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>304673.71</v>
+        <v>304832.33</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>304181.25</v>
+        <v>304339.61</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.55</v>
+        <v>13.492</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212491.98</v>
+        <v>212602.61</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212363.79</v>
+        <v>212474.35</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212427.88</v>
+        <v>212538.48</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.55</v>
+        <v>13.492</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129182.75</v>
+        <v>129250.01</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129467.49</v>
+        <v>129534.89</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129325.12</v>
+        <v>129392.45</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.55</v>
+        <v>13.492</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62616.55</v>
+        <v>62649.15</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62324.03</v>
+        <v>62356.47</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62470.29</v>
+        <v>62502.81</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.55</v>
+        <v>13.492</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31979.31</v>
+        <v>31995.95</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32003.46</v>
+        <v>32020.12</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31991.38</v>
+        <v>32008.04</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4937</v>
+        <v>13.457</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>408070.97</v>
+        <v>408292.23</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>408619.47</v>
+        <v>408841.02</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>408345.22</v>
+        <v>408566.63</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4937</v>
+        <v>13.457</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>302906.74</v>
+        <v>303070.98</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>301015.42</v>
+        <v>301178.63</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>301961.08</v>
+        <v>302124.81</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4937</v>
+        <v>13.457</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205461.91</v>
+        <v>205573.32</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205532.2</v>
+        <v>205643.64</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205497.06</v>
+        <v>205608.48</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4937</v>
+        <v>13.457</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124332.14</v>
+        <v>124399.56</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124850.54</v>
+        <v>124918.23</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124591.34</v>
+        <v>124658.9</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4937</v>
+        <v>13.457</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49652.72</v>
+        <v>49679.64</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49593.55</v>
+        <v>49620.44</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49623.13</v>
+        <v>49650.04</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4937</v>
+        <v>13.457</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5461.64</v>
+        <v>5464.6</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5497.66</v>
+        <v>5500.64</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5479.65</v>
+        <v>5482.62</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4111</v>
+        <v>13.3993</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170438.55</v>
+        <v>170527.26</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170465.81</v>
+        <v>170554.53</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170452.18</v>
+        <v>170540.89</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4111</v>
+        <v>13.3993</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112006.43</v>
+        <v>112064.72</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111616.78</v>
+        <v>111674.88</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111811.61</v>
+        <v>111869.8</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4111</v>
+        <v>13.3993</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62728.54</v>
+        <v>62761.19</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63084.34</v>
+        <v>63117.18</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62906.44</v>
+        <v>62939.18</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4111</v>
+        <v>13.3993</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26854.7</v>
+        <v>26868.67</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27054.76</v>
+        <v>27068.85</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26954.73</v>
+        <v>26968.76</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4111</v>
+        <v>13.3993</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6321.31</v>
+        <v>6324.6</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6473.27</v>
+        <v>6476.64</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6397.29</v>
+        <v>6400.62</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4111</v>
+        <v>13.3993</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3743.81</v>
+        <v>3745.76</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3737.32</v>
+        <v>3739.26</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3740.56</v>
+        <v>3742.51</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3644</v>
+        <v>13.3688</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190654</v>
+        <v>190746.75</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191584.93</v>
+        <v>191678.14</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191119.46</v>
+        <v>191212.45</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3644</v>
+        <v>13.3688</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138228.18</v>
+        <v>138295.43</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139192.78</v>
+        <v>139260.5</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138710.48</v>
+        <v>138777.97</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3644</v>
+        <v>13.3688</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87374.06</v>
+        <v>87416.57000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88081.14</v>
+        <v>88124</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87727.60000000001</v>
+        <v>87770.28</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3644</v>
+        <v>13.3688</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41735.3</v>
+        <v>41755.61</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41668.37</v>
+        <v>41688.64</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41701.83</v>
+        <v>41722.12</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3644</v>
+        <v>13.3688</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13014.47</v>
+        <v>13020.81</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12871.12</v>
+        <v>12877.39</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12942.8</v>
+        <v>12949.1</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3644</v>
+        <v>13.3688</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4516.84</v>
+        <v>4519.03</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4406.58</v>
+        <v>4408.72</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4461.71</v>
+        <v>4463.88</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-25
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3587</v>
+        <v>13.3722</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150327.95</v>
+        <v>150396.02</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152223.16</v>
+        <v>152292.08</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151275.55</v>
+        <v>151344.05</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3587</v>
+        <v>13.3722</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115066.27</v>
+        <v>115118.37</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115848.61</v>
+        <v>115901.06</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115457.44</v>
+        <v>115509.72</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3587</v>
+        <v>13.3722</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82044.94</v>
+        <v>82082.09</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82556.19</v>
+        <v>82593.57000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82300.56</v>
+        <v>82337.83</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3587</v>
+        <v>13.3722</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58137.02</v>
+        <v>58163.35</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57696.41</v>
+        <v>57722.54</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57916.72</v>
+        <v>57942.94</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3587</v>
+        <v>13.3722</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37554.21</v>
+        <v>37571.22</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37861.42</v>
+        <v>37878.56</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37707.81</v>
+        <v>37724.89</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3587</v>
+        <v>13.3722</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17080.36</v>
+        <v>17088.09</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16968.2</v>
+        <v>16975.88</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17024.28</v>
+        <v>17031.98</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3495</v>
+        <v>13.3784</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163328.52</v>
+        <v>163390.75</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162452.13</v>
+        <v>162514.02</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162890.32</v>
+        <v>162952.39</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3495</v>
+        <v>13.3784</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122660.21</v>
+        <v>122706.95</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120927.81</v>
+        <v>120973.89</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121794.01</v>
+        <v>121840.42</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3495</v>
+        <v>13.3784</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87633.10000000001</v>
+        <v>87666.49000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86547.94</v>
+        <v>86580.91</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87090.52</v>
+        <v>87123.7</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3495</v>
+        <v>13.3784</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66754.46000000001</v>
+        <v>66779.89</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66285.17999999999</v>
+        <v>66310.44</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66519.82000000001</v>
+        <v>66545.16</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3495</v>
+        <v>13.3784</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52149.66</v>
+        <v>52169.53</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50275.45</v>
+        <v>50294.61</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51212.56</v>
+        <v>51232.07</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3495</v>
+        <v>13.3784</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39532.27</v>
+        <v>39547.33</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40509.13</v>
+        <v>40524.57</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40020.7</v>
+        <v>40035.95</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3565</v>
+        <v>13.3966</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168164.25</v>
+        <v>168215.58</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169713.33</v>
+        <v>169765.13</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168938.79</v>
+        <v>168990.36</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3565</v>
+        <v>13.3966</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121223</v>
+        <v>121260.01</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119774.13</v>
+        <v>119810.69</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120498.57</v>
+        <v>120535.35</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3565</v>
+        <v>13.3966</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83039.67</v>
+        <v>83065.02</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82726.03</v>
+        <v>82751.28</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82882.85000000001</v>
+        <v>82908.14999999999</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3565</v>
+        <v>13.3966</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55325.01</v>
+        <v>55341.9</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55630.28</v>
+        <v>55647.26</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55477.65</v>
+        <v>55494.58</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3565</v>
+        <v>13.3966</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33391.47</v>
+        <v>33401.66</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33000.63</v>
+        <v>33010.71</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33196.05</v>
+        <v>33206.18</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3565</v>
+        <v>13.3966</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17335.43</v>
+        <v>17340.72</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18022.69</v>
+        <v>18028.2</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17679.06</v>
+        <v>17684.46</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3777</v>
+        <v>13.4261</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129954.17</v>
+        <v>129983.9</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130049.39</v>
+        <v>130079.14</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130001.78</v>
+        <v>130031.52</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3777</v>
+        <v>13.4261</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90000.07000000001</v>
+        <v>90020.66</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88603.52</v>
+        <v>88623.8</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89301.8</v>
+        <v>89322.23</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3777</v>
+        <v>13.4261</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56570.1</v>
+        <v>56583.04</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56858.8</v>
+        <v>56871.81</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56714.45</v>
+        <v>56727.42</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3777</v>
+        <v>13.4261</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29948.25</v>
+        <v>29955.1</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30149.83</v>
+        <v>30156.73</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30049.04</v>
+        <v>30055.92</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3777</v>
+        <v>13.4261</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6868.88</v>
+        <v>6870.45</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6867.57</v>
+        <v>6869.14</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6868.22</v>
+        <v>6869.79</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3777</v>
+        <v>13.4261</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3816.65</v>
+        <v>3817.52</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3726.63</v>
+        <v>3727.48</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3771.64</v>
+        <v>3772.5</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3979</v>
+        <v>13.4543</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109713.46</v>
+        <v>109729.24</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110194.77</v>
+        <v>110210.63</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109954.11</v>
+        <v>109969.94</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3979</v>
+        <v>13.4543</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76940.59</v>
+        <v>76951.66</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76393.19</v>
+        <v>76404.17999999999</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76666.89</v>
+        <v>76677.92</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3979</v>
+        <v>13.4543</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46556.85</v>
+        <v>46563.55</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47669.96</v>
+        <v>47676.82</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47113.4</v>
+        <v>47120.18</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3979</v>
+        <v>13.4543</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28923.86</v>
+        <v>28928.02</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28816.06</v>
+        <v>28820.21</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28869.96</v>
+        <v>28874.11</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3979</v>
+        <v>13.4543</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14188.77</v>
+        <v>14190.81</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14311.78</v>
+        <v>14313.84</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14250.28</v>
+        <v>14252.33</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3979</v>
+        <v>13.4543</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6577.92</v>
+        <v>6578.87</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6415.42</v>
+        <v>6416.34</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6496.67</v>
+        <v>6497.6</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4191</v>
+        <v>13.4838</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49932.2</v>
+        <v>49934.32</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49597.92</v>
+        <v>49600.02</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49765.06</v>
+        <v>49767.17</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4191</v>
+        <v>13.4838</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43927</v>
+        <v>43928.87</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44122.02</v>
+        <v>44123.9</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44024.51</v>
+        <v>44026.38</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4191</v>
+        <v>13.4838</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32147.96</v>
+        <v>32149.33</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32490.32</v>
+        <v>32491.71</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32319.14</v>
+        <v>32320.52</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4191</v>
+        <v>13.4838</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22604.15</v>
+        <v>22605.11</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22759.39</v>
+        <v>22760.35</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22681.77</v>
+        <v>22682.73</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4191</v>
+        <v>13.4838</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14528.41</v>
+        <v>14529.02</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14735.15</v>
+        <v>14735.78</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14631.78</v>
+        <v>14632.4</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4191</v>
+        <v>13.4838</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8349.49</v>
+        <v>8349.84</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8404.799999999999</v>
+        <v>8405.16</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8377.15</v>
+        <v>8377.5</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4412</v>
+        <v>13.5147</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49120.99</v>
+        <v>49117.2</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48398.05</v>
+        <v>48394.32</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48759.52</v>
+        <v>48755.76</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4412</v>
+        <v>13.5147</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43988.54</v>
+        <v>43985.14</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43650.62</v>
+        <v>43647.25</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43819.58</v>
+        <v>43816.19</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4412</v>
+        <v>13.5147</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31768.54</v>
+        <v>31766.09</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31197.44</v>
+        <v>31195.04</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31482.99</v>
+        <v>31480.56</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4412</v>
+        <v>13.5147</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23678.1</v>
+        <v>23676.27</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23572.53</v>
+        <v>23570.71</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23625.31</v>
+        <v>23623.49</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4412</v>
+        <v>13.5147</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18575.16</v>
+        <v>18573.73</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18388.5</v>
+        <v>18387.08</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18481.83</v>
+        <v>18480.4</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4412</v>
+        <v>13.5147</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15622.98</v>
+        <v>15621.78</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15567.2</v>
+        <v>15566</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15595.09</v>
+        <v>15593.89</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4615</v>
+        <v>13.5428</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109119.87</v>
+        <v>109098.2</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109672.47</v>
+        <v>109650.69</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109396.17</v>
+        <v>109374.44</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4615</v>
+        <v>13.5428</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78250.62</v>
+        <v>78235.08</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78566.95</v>
+        <v>78551.34</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78408.78</v>
+        <v>78393.21000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4615</v>
+        <v>13.5428</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51116.65</v>
+        <v>51106.5</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50682.52</v>
+        <v>50672.46</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50899.59</v>
+        <v>50889.48</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4615</v>
+        <v>13.5428</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29388.6</v>
+        <v>29382.76</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29176.84</v>
+        <v>29171.04</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29282.72</v>
+        <v>29276.9</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4615</v>
+        <v>13.5428</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16701.24</v>
+        <v>16697.92</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16635.25</v>
+        <v>16631.94</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16668.24</v>
+        <v>16664.93</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4615</v>
+        <v>13.5428</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6771.3</v>
+        <v>6769.96</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6557.03</v>
+        <v>6555.73</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6664.17</v>
+        <v>6662.84</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.492</v>
+        <v>13.4642</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>404735.51</v>
+        <v>404941.59</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>399727.93</v>
+        <v>399931.46</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>402231.72</v>
+        <v>402436.53</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.492</v>
+        <v>13.4642</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>303846.89</v>
+        <v>304001.6</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>304832.33</v>
+        <v>304987.54</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>304339.61</v>
+        <v>304494.57</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.492</v>
+        <v>13.4642</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212602.61</v>
+        <v>212710.85</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212474.35</v>
+        <v>212582.53</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212538.48</v>
+        <v>212646.69</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.492</v>
+        <v>13.4642</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129250.01</v>
+        <v>129315.82</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129534.89</v>
+        <v>129600.84</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129392.45</v>
+        <v>129458.33</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.492</v>
+        <v>13.4642</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62649.15</v>
+        <v>62681.05</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62356.47</v>
+        <v>62388.22</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62502.81</v>
+        <v>62534.64</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.492</v>
+        <v>13.4642</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31995.95</v>
+        <v>32012.25</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32020.12</v>
+        <v>32036.42</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>32008.04</v>
+        <v>32024.33</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.457</v>
+        <v>13.4341</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>408292.23</v>
+        <v>408506.67</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>408841.02</v>
+        <v>409055.75</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>408566.63</v>
+        <v>408781.21</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.457</v>
+        <v>13.4341</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>303070.98</v>
+        <v>303230.15</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>301178.63</v>
+        <v>301336.81</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>302124.81</v>
+        <v>302283.48</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.457</v>
+        <v>13.4341</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205573.32</v>
+        <v>205681.29</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205643.64</v>
+        <v>205751.65</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205608.48</v>
+        <v>205716.47</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.457</v>
+        <v>13.4341</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124399.56</v>
+        <v>124464.89</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124918.23</v>
+        <v>124983.84</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124658.9</v>
+        <v>124724.37</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.457</v>
+        <v>13.4341</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49679.64</v>
+        <v>49705.73</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49620.44</v>
+        <v>49646.5</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49650.04</v>
+        <v>49676.12</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.457</v>
+        <v>13.4341</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5464.6</v>
+        <v>5467.47</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5500.64</v>
+        <v>5503.52</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5482.62</v>
+        <v>5485.5</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3993</v>
+        <v>13.3818</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170527.26</v>
+        <v>170617.6</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170554.53</v>
+        <v>170644.89</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170540.89</v>
+        <v>170631.24</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3993</v>
+        <v>13.3818</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112064.72</v>
+        <v>112124.09</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111674.88</v>
+        <v>111734.04</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111869.8</v>
+        <v>111929.07</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3993</v>
+        <v>13.3818</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62761.19</v>
+        <v>62794.44</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63117.18</v>
+        <v>63150.62</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62939.18</v>
+        <v>62972.53</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3993</v>
+        <v>13.3818</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26868.67</v>
+        <v>26882.91</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27068.85</v>
+        <v>27083.19</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26968.76</v>
+        <v>26983.05</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3993</v>
+        <v>13.3818</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6324.6</v>
+        <v>6327.95</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6476.64</v>
+        <v>6480.07</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6400.62</v>
+        <v>6404.01</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3993</v>
+        <v>13.3818</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3745.76</v>
+        <v>3747.75</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3739.26</v>
+        <v>3741.24</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3742.51</v>
+        <v>3744.49</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3688</v>
+        <v>13.3653</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190746.75</v>
+        <v>190843.43</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191678.14</v>
+        <v>191775.29</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191212.45</v>
+        <v>191309.36</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3688</v>
+        <v>13.3653</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138295.43</v>
+        <v>138365.52</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139260.5</v>
+        <v>139331.09</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138777.97</v>
+        <v>138848.3</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3688</v>
+        <v>13.3653</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87416.57000000001</v>
+        <v>87460.87</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88124</v>
+        <v>88168.66</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87770.28</v>
+        <v>87814.77</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3688</v>
+        <v>13.3653</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41755.61</v>
+        <v>41776.77</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41688.64</v>
+        <v>41709.77</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41722.12</v>
+        <v>41743.27</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3688</v>
+        <v>13.3653</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13020.81</v>
+        <v>13027.41</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12877.39</v>
+        <v>12883.91</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12949.1</v>
+        <v>12955.66</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3688</v>
+        <v>13.3653</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4519.03</v>
+        <v>4521.33</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4408.72</v>
+        <v>4410.95</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4463.88</v>
+        <v>4466.14</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-26
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3722</v>
+        <v>13.3367</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150396.02</v>
+        <v>150413.77</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152292.08</v>
+        <v>152310.06</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151344.05</v>
+        <v>151361.91</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3722</v>
+        <v>13.3367</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115118.37</v>
+        <v>115131.96</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115901.06</v>
+        <v>115914.74</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115509.72</v>
+        <v>115523.35</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3722</v>
+        <v>13.3367</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82082.09</v>
+        <v>82091.78</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82593.57000000001</v>
+        <v>82603.32000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82337.83</v>
+        <v>82347.55</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3722</v>
+        <v>13.3367</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58163.35</v>
+        <v>58170.21</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57722.54</v>
+        <v>57729.35</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57942.94</v>
+        <v>57949.78</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3722</v>
+        <v>13.3367</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37571.22</v>
+        <v>37575.65</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37878.56</v>
+        <v>37883.03</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37724.89</v>
+        <v>37729.34</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3722</v>
+        <v>13.3367</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17088.09</v>
+        <v>17090.11</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16975.88</v>
+        <v>16977.88</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17031.98</v>
+        <v>17033.99</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3784</v>
+        <v>13.3413</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163390.75</v>
+        <v>163415.16</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162514.02</v>
+        <v>162538.3</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162952.39</v>
+        <v>162976.73</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3784</v>
+        <v>13.3413</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122706.95</v>
+        <v>122725.28</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120973.89</v>
+        <v>120991.96</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121840.42</v>
+        <v>121858.62</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3784</v>
+        <v>13.3413</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87666.49000000001</v>
+        <v>87679.59</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86580.91</v>
+        <v>86593.85000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87123.7</v>
+        <v>87136.72</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3784</v>
+        <v>13.3413</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66779.89</v>
+        <v>66789.87</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66310.44</v>
+        <v>66320.35000000001</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66545.16</v>
+        <v>66555.11</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3784</v>
+        <v>13.3413</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52169.53</v>
+        <v>52177.33</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50294.61</v>
+        <v>50302.12</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51232.07</v>
+        <v>51239.73</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3784</v>
+        <v>13.3413</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39547.33</v>
+        <v>39553.24</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40524.57</v>
+        <v>40530.62</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40035.95</v>
+        <v>40041.93</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3966</v>
+        <v>13.3589</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168215.58</v>
+        <v>168245.94</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169765.13</v>
+        <v>169795.76</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168990.36</v>
+        <v>169020.85</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3966</v>
+        <v>13.3589</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121260.01</v>
+        <v>121281.89</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119810.69</v>
+        <v>119832.31</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120535.35</v>
+        <v>120557.1</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3966</v>
+        <v>13.3589</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83065.02</v>
+        <v>83080.00999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82751.28</v>
+        <v>82766.21000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82908.14999999999</v>
+        <v>82923.11</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3966</v>
+        <v>13.3589</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55341.9</v>
+        <v>55351.89</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55647.26</v>
+        <v>55657.3</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55494.58</v>
+        <v>55504.59</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3966</v>
+        <v>13.3589</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33401.66</v>
+        <v>33407.69</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33010.71</v>
+        <v>33016.66</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33206.18</v>
+        <v>33212.17</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3966</v>
+        <v>13.3589</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17340.72</v>
+        <v>17343.85</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18028.2</v>
+        <v>18031.45</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17684.46</v>
+        <v>17687.65</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.4261</v>
+        <v>13.3892</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129983.9</v>
+        <v>130010.57</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130079.14</v>
+        <v>130105.83</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130031.52</v>
+        <v>130058.2</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.4261</v>
+        <v>13.3892</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90020.66</v>
+        <v>90039.13</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88623.8</v>
+        <v>88641.98</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89322.23</v>
+        <v>89340.55</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.4261</v>
+        <v>13.3892</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56583.04</v>
+        <v>56594.65</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56871.81</v>
+        <v>56883.47</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56727.42</v>
+        <v>56739.06</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.4261</v>
+        <v>13.3892</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29955.1</v>
+        <v>29961.25</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30156.73</v>
+        <v>30162.92</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30055.92</v>
+        <v>30062.08</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.4261</v>
+        <v>13.3892</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6870.45</v>
+        <v>6871.86</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6869.14</v>
+        <v>6870.55</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6869.79</v>
+        <v>6871.2</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.4261</v>
+        <v>13.3892</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3817.52</v>
+        <v>3818.31</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3727.48</v>
+        <v>3728.25</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3772.5</v>
+        <v>3773.28</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4543</v>
+        <v>13.4181</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109729.24</v>
+        <v>109754.23</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110210.63</v>
+        <v>110235.73</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109969.94</v>
+        <v>109994.98</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4543</v>
+        <v>13.4181</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76951.66</v>
+        <v>76969.17999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76404.17999999999</v>
+        <v>76421.58</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76677.92</v>
+        <v>76695.38</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4543</v>
+        <v>13.4181</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46563.55</v>
+        <v>46574.15</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47676.82</v>
+        <v>47687.68</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47120.18</v>
+        <v>47130.91</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4543</v>
+        <v>13.4181</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28928.02</v>
+        <v>28934.61</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28820.21</v>
+        <v>28826.77</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28874.11</v>
+        <v>28880.69</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4543</v>
+        <v>13.4181</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14190.81</v>
+        <v>14194.04</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14313.84</v>
+        <v>14317.1</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14252.33</v>
+        <v>14255.57</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4543</v>
+        <v>13.4181</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6578.87</v>
+        <v>6580.37</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6416.34</v>
+        <v>6417.8</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6497.6</v>
+        <v>6499.08</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4838</v>
+        <v>13.4484</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49934.32</v>
+        <v>49946.82</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49600.02</v>
+        <v>49612.43</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49767.17</v>
+        <v>49779.62</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4838</v>
+        <v>13.4484</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43928.87</v>
+        <v>43939.86</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44123.9</v>
+        <v>44134.93</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44026.38</v>
+        <v>44037.4</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4838</v>
+        <v>13.4484</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32149.33</v>
+        <v>32157.37</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32491.71</v>
+        <v>32499.83</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32320.52</v>
+        <v>32328.6</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4838</v>
+        <v>13.4484</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22605.11</v>
+        <v>22610.77</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22760.35</v>
+        <v>22766.05</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22682.73</v>
+        <v>22688.41</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4838</v>
+        <v>13.4484</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14529.02</v>
+        <v>14532.66</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14735.78</v>
+        <v>14739.46</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14632.4</v>
+        <v>14636.06</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4838</v>
+        <v>13.4484</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8349.84</v>
+        <v>8351.93</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8405.16</v>
+        <v>8407.26</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8377.5</v>
+        <v>8379.6</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.5147</v>
+        <v>13.48</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49117.2</v>
+        <v>49130.57</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48394.32</v>
+        <v>48407.5</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48755.76</v>
+        <v>48769.04</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.5147</v>
+        <v>13.48</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43985.14</v>
+        <v>43997.12</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43647.25</v>
+        <v>43659.14</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43816.19</v>
+        <v>43828.13</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.5147</v>
+        <v>13.48</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31766.09</v>
+        <v>31774.74</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31195.04</v>
+        <v>31203.53</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31480.56</v>
+        <v>31489.14</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.5147</v>
+        <v>13.48</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23676.27</v>
+        <v>23682.72</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23570.71</v>
+        <v>23577.13</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23623.49</v>
+        <v>23629.92</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.5147</v>
+        <v>13.48</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18573.73</v>
+        <v>18578.79</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18387.08</v>
+        <v>18392.09</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18480.4</v>
+        <v>18485.44</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.5147</v>
+        <v>13.48</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15621.78</v>
+        <v>15626.03</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15566</v>
+        <v>15570.24</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15593.89</v>
+        <v>15598.14</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.5428</v>
+        <v>13.5089</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109098.2</v>
+        <v>109130.01</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109650.69</v>
+        <v>109682.66</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109374.44</v>
+        <v>109406.34</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.5428</v>
+        <v>13.5089</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78235.08</v>
+        <v>78257.89</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78551.34</v>
+        <v>78574.25</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78393.21000000001</v>
+        <v>78416.07000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.5428</v>
+        <v>13.5089</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51106.5</v>
+        <v>51121.4</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50672.46</v>
+        <v>50687.23</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50889.48</v>
+        <v>50904.32</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.5428</v>
+        <v>13.5089</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29382.76</v>
+        <v>29391.33</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29171.04</v>
+        <v>29179.55</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29276.9</v>
+        <v>29285.44</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.5428</v>
+        <v>13.5089</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16697.92</v>
+        <v>16702.79</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16631.94</v>
+        <v>16636.79</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16664.93</v>
+        <v>16669.79</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.5428</v>
+        <v>13.5089</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6769.96</v>
+        <v>6771.93</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6555.73</v>
+        <v>6557.64</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6662.84</v>
+        <v>6664.79</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.4642</v>
+        <v>13.4673</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>404941.59</v>
+        <v>404941.28</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>399931.46</v>
+        <v>399931.16</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>402436.53</v>
+        <v>402436.22</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.4642</v>
+        <v>13.4673</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>304001.6</v>
+        <v>304001.37</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>304987.54</v>
+        <v>304987.31</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>304494.57</v>
+        <v>304494.34</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.4642</v>
+        <v>13.4673</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212710.85</v>
+        <v>212710.69</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212582.53</v>
+        <v>212582.37</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212646.69</v>
+        <v>212646.53</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.4642</v>
+        <v>13.4673</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129315.82</v>
+        <v>129315.72</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129600.84</v>
+        <v>129600.75</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129458.33</v>
+        <v>129458.23</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.4642</v>
+        <v>13.4673</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62681.05</v>
+        <v>62681</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62388.22</v>
+        <v>62388.18</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62534.64</v>
+        <v>62534.59</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.4642</v>
+        <v>13.4673</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>32012.25</v>
+        <v>32012.22</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32036.42</v>
+        <v>32036.4</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>32024.33</v>
+        <v>32024.31</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4341</v>
+        <v>13.4267</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>408506.67</v>
+        <v>408509.82</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>409055.75</v>
+        <v>409058.91</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>408781.21</v>
+        <v>408784.37</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4341</v>
+        <v>13.4267</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>303230.15</v>
+        <v>303232.49</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>301336.81</v>
+        <v>301339.14</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>302283.48</v>
+        <v>302285.82</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4341</v>
+        <v>13.4267</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205681.29</v>
+        <v>205682.87</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205751.65</v>
+        <v>205753.24</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205716.47</v>
+        <v>205718.06</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4341</v>
+        <v>13.4267</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124464.89</v>
+        <v>124465.85</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124983.84</v>
+        <v>124984.81</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124724.37</v>
+        <v>124725.33</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4341</v>
+        <v>13.4267</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49705.73</v>
+        <v>49706.12</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49646.5</v>
+        <v>49646.88</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49676.12</v>
+        <v>49676.5</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4341</v>
+        <v>13.4267</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5467.47</v>
+        <v>5467.51</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5503.52</v>
+        <v>5503.57</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5485.5</v>
+        <v>5485.54</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3818</v>
+        <v>13.3561</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170617.6</v>
+        <v>170625.28</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170644.89</v>
+        <v>170652.57</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170631.24</v>
+        <v>170638.93</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3818</v>
+        <v>13.3561</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112124.09</v>
+        <v>112129.14</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111734.04</v>
+        <v>111739.07</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111929.07</v>
+        <v>111934.1</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3818</v>
+        <v>13.3561</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62794.44</v>
+        <v>62797.27</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63150.62</v>
+        <v>63153.46</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62972.53</v>
+        <v>62975.36</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3818</v>
+        <v>13.3561</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26882.91</v>
+        <v>26884.12</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27083.19</v>
+        <v>27084.41</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26983.05</v>
+        <v>26984.26</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3818</v>
+        <v>13.3561</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6327.95</v>
+        <v>6328.24</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6480.07</v>
+        <v>6480.36</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6404.01</v>
+        <v>6404.3</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3818</v>
+        <v>13.3561</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3747.75</v>
+        <v>3747.91</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3741.24</v>
+        <v>3741.41</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3744.49</v>
+        <v>3744.66</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3316</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190843.43</v>
+        <v>190859.87</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191775.29</v>
+        <v>191791.82</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191309.36</v>
+        <v>191325.84</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3316</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138365.52</v>
+        <v>138377.44</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139331.09</v>
+        <v>139343.09</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138848.3</v>
+        <v>138860.27</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3316</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87460.87</v>
+        <v>87468.41</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88168.66</v>
+        <v>88176.25999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87814.77</v>
+        <v>87822.33</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3316</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41776.77</v>
+        <v>41780.37</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41709.77</v>
+        <v>41713.36</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41743.27</v>
+        <v>41746.87</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3316</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13027.41</v>
+        <v>13028.53</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12883.91</v>
+        <v>12885.02</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12955.66</v>
+        <v>12956.78</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3316</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4521.33</v>
+        <v>4521.71</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4410.95</v>
+        <v>4411.33</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4466.14</v>
+        <v>4466.52</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-29
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3367</v>
+        <v>13.3423</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150413.77</v>
+        <v>150560.53</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152310.06</v>
+        <v>152458.67</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151361.91</v>
+        <v>151509.6</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3367</v>
+        <v>13.3423</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115131.96</v>
+        <v>115244.29</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115914.74</v>
+        <v>116027.84</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115523.35</v>
+        <v>115636.07</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3367</v>
+        <v>13.3423</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82091.78</v>
+        <v>82171.88</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82603.32000000001</v>
+        <v>82683.91</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82347.55</v>
+        <v>82427.89999999999</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3367</v>
+        <v>13.3423</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58170.21</v>
+        <v>58226.97</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57729.35</v>
+        <v>57785.68</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57949.78</v>
+        <v>58006.32</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3367</v>
+        <v>13.3423</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37575.65</v>
+        <v>37612.31</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37883.03</v>
+        <v>37919.99</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37729.34</v>
+        <v>37766.15</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3367</v>
+        <v>13.3423</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17090.11</v>
+        <v>17106.78</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16977.88</v>
+        <v>16994.45</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17033.99</v>
+        <v>17050.61</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3413</v>
+        <v>13.3416</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163415.16</v>
+        <v>163577.46</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162538.3</v>
+        <v>162699.73</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162976.73</v>
+        <v>163138.6</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3413</v>
+        <v>13.3416</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122725.28</v>
+        <v>122847.17</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120991.96</v>
+        <v>121112.13</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121858.62</v>
+        <v>121979.65</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3413</v>
+        <v>13.3416</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87679.59</v>
+        <v>87766.67</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86593.85000000001</v>
+        <v>86679.85000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87136.72</v>
+        <v>87223.25999999999</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3413</v>
+        <v>13.3416</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66789.87</v>
+        <v>66856.2</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66320.35000000001</v>
+        <v>66386.22</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66555.11</v>
+        <v>66621.21000000001</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3413</v>
+        <v>13.3416</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52177.33</v>
+        <v>52229.15</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50302.12</v>
+        <v>50352.08</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51239.73</v>
+        <v>51290.62</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3413</v>
+        <v>13.3416</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39553.24</v>
+        <v>39592.53</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40530.62</v>
+        <v>40570.88</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40041.93</v>
+        <v>40081.7</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.354</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168245.94</v>
+        <v>168417.4</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169795.76</v>
+        <v>169968.8</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>169020.85</v>
+        <v>169193.1</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.354</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121281.89</v>
+        <v>121405.49</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119832.31</v>
+        <v>119954.43</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120557.1</v>
+        <v>120679.96</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.354</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83080.00999999999</v>
+        <v>83164.67</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82766.21000000001</v>
+        <v>82850.56</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82923.11</v>
+        <v>83007.62</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.354</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55351.89</v>
+        <v>55408.3</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55657.3</v>
+        <v>55714.02</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55504.59</v>
+        <v>55561.16</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.354</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33407.69</v>
+        <v>33441.73</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33016.66</v>
+        <v>33050.31</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33212.17</v>
+        <v>33246.02</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.354</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17343.85</v>
+        <v>17361.53</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18031.45</v>
+        <v>18049.83</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17687.65</v>
+        <v>17705.68</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3855</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130010.57</v>
+        <v>130142.97</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130105.83</v>
+        <v>130238.33</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130058.2</v>
+        <v>130190.65</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3855</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90039.13</v>
+        <v>90130.83</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88641.98</v>
+        <v>88732.25999999999</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89340.55</v>
+        <v>89431.53999999999</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3855</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56594.65</v>
+        <v>56652.29</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56883.47</v>
+        <v>56941.4</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56739.06</v>
+        <v>56796.85</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3855</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29961.25</v>
+        <v>29991.76</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30162.92</v>
+        <v>30193.64</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30062.08</v>
+        <v>30092.7</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3855</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6871.86</v>
+        <v>6878.86</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6870.55</v>
+        <v>6877.54</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6871.2</v>
+        <v>6878.2</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3855</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3818.31</v>
+        <v>3822.2</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3728.25</v>
+        <v>3732.04</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3773.28</v>
+        <v>3777.12</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4181</v>
+        <v>13.4155</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109754.23</v>
+        <v>109865.74</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110235.73</v>
+        <v>110347.73</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109994.98</v>
+        <v>110106.74</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4181</v>
+        <v>13.4155</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76969.17999999999</v>
+        <v>77047.38</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76421.58</v>
+        <v>76499.22</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76695.38</v>
+        <v>76773.3</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4181</v>
+        <v>13.4155</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46574.15</v>
+        <v>46621.47</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47687.68</v>
+        <v>47736.13</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47130.91</v>
+        <v>47178.8</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4181</v>
+        <v>13.4155</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28934.61</v>
+        <v>28964</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28826.77</v>
+        <v>28856.06</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28880.69</v>
+        <v>28910.03</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4181</v>
+        <v>13.4155</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14194.04</v>
+        <v>14208.47</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14317.1</v>
+        <v>14331.65</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14255.57</v>
+        <v>14270.06</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4181</v>
+        <v>13.4155</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6580.37</v>
+        <v>6587.05</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6417.8</v>
+        <v>6424.32</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6499.08</v>
+        <v>6505.69</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4484</v>
+        <v>13.447</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49946.82</v>
+        <v>49997.35</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49612.43</v>
+        <v>49662.62</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49779.62</v>
+        <v>49829.99</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4484</v>
+        <v>13.447</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43939.86</v>
+        <v>43984.31</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44134.93</v>
+        <v>44179.59</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44037.4</v>
+        <v>44081.95</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4484</v>
+        <v>13.447</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32157.37</v>
+        <v>32189.9</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32499.83</v>
+        <v>32532.71</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32328.6</v>
+        <v>32361.31</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4484</v>
+        <v>13.447</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22610.77</v>
+        <v>22633.64</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22766.05</v>
+        <v>22789.08</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22688.41</v>
+        <v>22711.36</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4484</v>
+        <v>13.447</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14532.66</v>
+        <v>14547.36</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14739.46</v>
+        <v>14754.38</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14636.06</v>
+        <v>14650.87</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4484</v>
+        <v>13.447</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8351.93</v>
+        <v>8360.379999999999</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8407.26</v>
+        <v>8415.77</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8379.6</v>
+        <v>8388.08</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.48</v>
+        <v>13.4799</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49130.57</v>
+        <v>49179.96</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48407.5</v>
+        <v>48456.16</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48769.04</v>
+        <v>48818.06</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.48</v>
+        <v>13.4799</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43997.12</v>
+        <v>44041.35</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43659.14</v>
+        <v>43703.03</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43828.13</v>
+        <v>43872.19</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.48</v>
+        <v>13.4799</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31774.74</v>
+        <v>31806.68</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31203.53</v>
+        <v>31234.9</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31489.14</v>
+        <v>31520.79</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.48</v>
+        <v>13.4799</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23682.72</v>
+        <v>23706.53</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23577.13</v>
+        <v>23600.83</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23629.92</v>
+        <v>23653.68</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.48</v>
+        <v>13.4799</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18578.79</v>
+        <v>18597.47</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18392.09</v>
+        <v>18410.57</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18485.44</v>
+        <v>18504.02</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.48</v>
+        <v>13.4799</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15626.03</v>
+        <v>15641.74</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15570.24</v>
+        <v>15585.89</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15598.14</v>
+        <v>15613.82</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.5089</v>
+        <v>13.51</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109130.01</v>
+        <v>109238.87</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109682.66</v>
+        <v>109792.08</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109406.34</v>
+        <v>109515.47</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.5089</v>
+        <v>13.51</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78257.89</v>
+        <v>78335.95</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78574.25</v>
+        <v>78652.63</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78416.07000000001</v>
+        <v>78494.28999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.5089</v>
+        <v>13.51</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51121.4</v>
+        <v>51172.4</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50687.23</v>
+        <v>50737.79</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50904.32</v>
+        <v>50955.09</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.5089</v>
+        <v>13.51</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29391.33</v>
+        <v>29420.65</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29179.55</v>
+        <v>29208.66</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29285.44</v>
+        <v>29314.65</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.5089</v>
+        <v>13.51</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16702.79</v>
+        <v>16719.46</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16636.79</v>
+        <v>16653.39</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16669.79</v>
+        <v>16686.42</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.5089</v>
+        <v>13.51</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6771.93</v>
+        <v>6778.69</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6557.64</v>
+        <v>6564.19</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6664.79</v>
+        <v>6671.44</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.4673</v>
+        <v>13.4542</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>404941.28</v>
+        <v>405348.46</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>399931.16</v>
+        <v>400333.3</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>402436.22</v>
+        <v>402840.88</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.4673</v>
+        <v>13.4542</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>304001.37</v>
+        <v>304307.05</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>304987.31</v>
+        <v>305293.98</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>304494.34</v>
+        <v>304800.52</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.4673</v>
+        <v>13.4542</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212710.69</v>
+        <v>212924.58</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212582.37</v>
+        <v>212796.13</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212646.53</v>
+        <v>212860.35</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.4673</v>
+        <v>13.4542</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129315.72</v>
+        <v>129445.75</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129600.75</v>
+        <v>129731.06</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129458.23</v>
+        <v>129588.41</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.4673</v>
+        <v>13.4542</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62681</v>
+        <v>62744.03</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62388.18</v>
+        <v>62450.91</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62534.59</v>
+        <v>62597.47</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.4673</v>
+        <v>13.4542</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>32012.22</v>
+        <v>32044.41</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32036.4</v>
+        <v>32068.61</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>32024.31</v>
+        <v>32056.51</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4267</v>
+        <v>13.4304</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>408509.82</v>
+        <v>408917.02</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>409058.91</v>
+        <v>409466.65</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>408784.37</v>
+        <v>409191.83</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4267</v>
+        <v>13.4304</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>303232.49</v>
+        <v>303534.75</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>301339.14</v>
+        <v>301639.51</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>302285.82</v>
+        <v>302587.13</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4267</v>
+        <v>13.4304</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205682.87</v>
+        <v>205887.9</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205753.24</v>
+        <v>205958.33</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205718.06</v>
+        <v>205923.11</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4267</v>
+        <v>13.4304</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124465.85</v>
+        <v>124589.92</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124984.81</v>
+        <v>125109.39</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124725.33</v>
+        <v>124849.65</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4267</v>
+        <v>13.4304</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49706.12</v>
+        <v>49755.66</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49646.88</v>
+        <v>49696.37</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49676.5</v>
+        <v>49726.02</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4267</v>
+        <v>13.4304</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5467.51</v>
+        <v>5472.96</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5503.57</v>
+        <v>5509.05</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5485.54</v>
+        <v>5491.01</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3561</v>
+        <v>13.3715</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170625.28</v>
+        <v>170790.7</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170652.57</v>
+        <v>170818.02</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170638.93</v>
+        <v>170804.36</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3561</v>
+        <v>13.3715</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112129.14</v>
+        <v>112237.85</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111739.07</v>
+        <v>111847.4</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111934.1</v>
+        <v>112042.62</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3561</v>
+        <v>13.3715</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62797.27</v>
+        <v>62858.15</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63153.46</v>
+        <v>63214.68</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62975.36</v>
+        <v>63036.42</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3561</v>
+        <v>13.3715</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26884.12</v>
+        <v>26910.18</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27084.41</v>
+        <v>27110.66</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26984.26</v>
+        <v>27010.42</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3561</v>
+        <v>13.3715</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6328.24</v>
+        <v>6334.37</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6480.36</v>
+        <v>6486.64</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6404.3</v>
+        <v>6410.51</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3561</v>
+        <v>13.3715</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3747.91</v>
+        <v>3751.55</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3741.41</v>
+        <v>3745.04</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3744.66</v>
+        <v>3748.29</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3316</v>
+        <v>13.3431</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>190859.87</v>
+        <v>191044.07</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191791.82</v>
+        <v>191976.91</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191325.84</v>
+        <v>191510.49</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3316</v>
+        <v>13.3431</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138377.44</v>
+        <v>138510.99</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139343.09</v>
+        <v>139477.57</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138860.27</v>
+        <v>138994.28</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3316</v>
+        <v>13.3431</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87468.41</v>
+        <v>87552.82000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88176.25999999999</v>
+        <v>88261.36</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87822.33</v>
+        <v>87907.09</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3316</v>
+        <v>13.3431</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41780.37</v>
+        <v>41820.69</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41713.36</v>
+        <v>41753.62</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41746.87</v>
+        <v>41787.16</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3316</v>
+        <v>13.3431</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13028.53</v>
+        <v>13041.1</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12885.02</v>
+        <v>12897.46</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12956.78</v>
+        <v>12969.28</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3316</v>
+        <v>13.3431</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4521.71</v>
+        <v>4526.08</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4411.33</v>
+        <v>4415.59</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4466.52</v>
+        <v>4470.83</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-30
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3423</v>
+        <v>13.3217</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150560.53</v>
+        <v>150645.39</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152458.67</v>
+        <v>152544.6</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151509.6</v>
+        <v>151594.99</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3423</v>
+        <v>13.3217</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115244.29</v>
+        <v>115309.25</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116027.84</v>
+        <v>116093.24</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115636.07</v>
+        <v>115701.24</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3423</v>
+        <v>13.3217</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82171.88</v>
+        <v>82218.19</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82683.91</v>
+        <v>82730.52</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82427.89999999999</v>
+        <v>82474.35000000001</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3423</v>
+        <v>13.3217</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58226.97</v>
+        <v>58259.79</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57785.68</v>
+        <v>57818.25</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58006.32</v>
+        <v>58039.02</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3423</v>
+        <v>13.3217</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37612.31</v>
+        <v>37633.51</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37919.99</v>
+        <v>37941.37</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37766.15</v>
+        <v>37787.44</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3423</v>
+        <v>13.3217</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17106.78</v>
+        <v>17116.42</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16994.45</v>
+        <v>17004.03</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17050.61</v>
+        <v>17060.23</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3416</v>
+        <v>13.3247</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163577.46</v>
+        <v>163669.58</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162699.73</v>
+        <v>162791.36</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163138.6</v>
+        <v>163230.47</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3416</v>
+        <v>13.3247</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122847.17</v>
+        <v>122916.35</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121112.13</v>
+        <v>121180.33</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121979.65</v>
+        <v>122048.34</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3416</v>
+        <v>13.3247</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87766.67</v>
+        <v>87816.09</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86679.85000000001</v>
+        <v>86728.66</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87223.25999999999</v>
+        <v>87272.38</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3416</v>
+        <v>13.3247</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66856.2</v>
+        <v>66893.85000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66386.22</v>
+        <v>66423.60000000001</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66621.21000000001</v>
+        <v>66658.73</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3416</v>
+        <v>13.3247</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52229.15</v>
+        <v>52258.56</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50352.08</v>
+        <v>50380.44</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51290.62</v>
+        <v>51319.5</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3416</v>
+        <v>13.3247</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39592.53</v>
+        <v>39614.82</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40570.88</v>
+        <v>40593.72</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40081.7</v>
+        <v>40104.27</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.354</v>
+        <v>13.3344</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168417.4</v>
+        <v>168516.68</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>169968.8</v>
+        <v>170069</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>169193.1</v>
+        <v>169292.84</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.354</v>
+        <v>13.3344</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121405.49</v>
+        <v>121477.05</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119954.43</v>
+        <v>120025.14</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120679.96</v>
+        <v>120751.1</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.354</v>
+        <v>13.3344</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83164.67</v>
+        <v>83213.7</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82850.56</v>
+        <v>82899.39999999999</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83007.62</v>
+        <v>83056.55</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.354</v>
+        <v>13.3344</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55408.3</v>
+        <v>55440.96</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55714.02</v>
+        <v>55746.86</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55561.16</v>
+        <v>55593.91</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.354</v>
+        <v>13.3344</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33441.73</v>
+        <v>33461.45</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33050.31</v>
+        <v>33069.79</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33246.02</v>
+        <v>33265.62</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.354</v>
+        <v>13.3344</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17361.53</v>
+        <v>17371.76</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18049.83</v>
+        <v>18060.47</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17705.68</v>
+        <v>17716.11</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3855</v>
+        <v>13.355</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130142.97</v>
+        <v>130229.54</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130238.33</v>
+        <v>130324.97</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130190.65</v>
+        <v>130277.26</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3855</v>
+        <v>13.355</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90130.83</v>
+        <v>90190.78</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88732.25999999999</v>
+        <v>88791.28</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89431.53999999999</v>
+        <v>89491.03</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3855</v>
+        <v>13.355</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56652.29</v>
+        <v>56689.97</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56941.4</v>
+        <v>56979.28</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56796.85</v>
+        <v>56834.63</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3855</v>
+        <v>13.355</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29991.76</v>
+        <v>30011.71</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30193.64</v>
+        <v>30213.72</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30092.7</v>
+        <v>30112.72</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3855</v>
+        <v>13.355</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6878.86</v>
+        <v>6883.43</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6877.54</v>
+        <v>6882.12</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6878.2</v>
+        <v>6882.78</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3855</v>
+        <v>13.355</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3822.2</v>
+        <v>3824.74</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3732.04</v>
+        <v>3734.53</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3777.12</v>
+        <v>3779.63</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4155</v>
+        <v>13.3746</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109865.74</v>
+        <v>109948.48</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110347.73</v>
+        <v>110430.83</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110106.74</v>
+        <v>110189.66</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4155</v>
+        <v>13.3746</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77047.38</v>
+        <v>77105.41</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76499.22</v>
+        <v>76556.84</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76773.3</v>
+        <v>76831.12</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4155</v>
+        <v>13.3746</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46621.47</v>
+        <v>46656.58</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47736.13</v>
+        <v>47772.08</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47178.8</v>
+        <v>47214.33</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4155</v>
+        <v>13.3746</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28964</v>
+        <v>28985.82</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28856.06</v>
+        <v>28877.79</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28910.03</v>
+        <v>28931.81</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4155</v>
+        <v>13.3746</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14208.47</v>
+        <v>14219.17</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14331.65</v>
+        <v>14342.44</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14270.06</v>
+        <v>14280.81</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4155</v>
+        <v>13.3746</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6587.05</v>
+        <v>6592.01</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6424.32</v>
+        <v>6429.16</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6505.69</v>
+        <v>6510.59</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.447</v>
+        <v>13.3952</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49997.35</v>
+        <v>50040.42</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49662.62</v>
+        <v>49705.41</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49829.99</v>
+        <v>49872.92</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.447</v>
+        <v>13.3952</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43984.31</v>
+        <v>44022.21</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44179.59</v>
+        <v>44217.65</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44081.95</v>
+        <v>44119.93</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.447</v>
+        <v>13.3952</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32189.9</v>
+        <v>32217.64</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32532.71</v>
+        <v>32560.74</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32361.31</v>
+        <v>32389.19</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.447</v>
+        <v>13.3952</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22633.64</v>
+        <v>22653.14</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22789.08</v>
+        <v>22808.72</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22711.36</v>
+        <v>22730.93</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.447</v>
+        <v>13.3952</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14547.36</v>
+        <v>14559.9</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14754.38</v>
+        <v>14767.09</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14650.87</v>
+        <v>14663.49</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.447</v>
+        <v>13.3952</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8360.379999999999</v>
+        <v>8367.58</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8415.77</v>
+        <v>8423.02</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8388.08</v>
+        <v>8395.299999999999</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4799</v>
+        <v>13.4167</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49179.96</v>
+        <v>49228.79</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48456.16</v>
+        <v>48504.27</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48818.06</v>
+        <v>48866.53</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4799</v>
+        <v>13.4167</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44041.35</v>
+        <v>44085.08</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43703.03</v>
+        <v>43746.42</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43872.19</v>
+        <v>43915.75</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4799</v>
+        <v>13.4167</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31806.68</v>
+        <v>31838.26</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31234.9</v>
+        <v>31265.91</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31520.79</v>
+        <v>31552.09</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4799</v>
+        <v>13.4167</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23706.53</v>
+        <v>23730.06</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23600.83</v>
+        <v>23624.26</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23653.68</v>
+        <v>23677.16</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4799</v>
+        <v>13.4167</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18597.47</v>
+        <v>18615.93</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18410.57</v>
+        <v>18428.85</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18504.02</v>
+        <v>18522.39</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4799</v>
+        <v>13.4167</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15641.74</v>
+        <v>15657.27</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15585.89</v>
+        <v>15601.37</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15613.82</v>
+        <v>15629.32</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.51</v>
+        <v>13.4364</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109238.87</v>
+        <v>109362.17</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109792.08</v>
+        <v>109916</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109515.47</v>
+        <v>109639.08</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.51</v>
+        <v>13.4364</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78335.95</v>
+        <v>78424.37</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78652.63</v>
+        <v>78741.39999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78494.28999999999</v>
+        <v>78582.89</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.51</v>
+        <v>13.4364</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51172.4</v>
+        <v>51230.16</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50737.79</v>
+        <v>50795.06</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50955.09</v>
+        <v>51012.61</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.51</v>
+        <v>13.4364</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29420.65</v>
+        <v>29453.85</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29208.66</v>
+        <v>29241.63</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29314.65</v>
+        <v>29347.74</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.51</v>
+        <v>13.4364</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16719.46</v>
+        <v>16738.33</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16653.39</v>
+        <v>16672.18</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16686.42</v>
+        <v>16705.26</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.51</v>
+        <v>13.4364</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6778.69</v>
+        <v>6786.34</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6564.19</v>
+        <v>6571.59</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6671.44</v>
+        <v>6678.97</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.4542</v>
+        <v>13.345</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>405348.46</v>
+        <v>405557.76</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>400333.3</v>
+        <v>400540</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>402840.88</v>
+        <v>403048.88</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.4542</v>
+        <v>13.345</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>304307.05</v>
+        <v>304464.17</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>305293.98</v>
+        <v>305451.62</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>304800.52</v>
+        <v>304957.89</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.4542</v>
+        <v>13.345</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>212924.58</v>
+        <v>213034.52</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212796.13</v>
+        <v>212906</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212860.35</v>
+        <v>212970.26</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.4542</v>
+        <v>13.345</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129445.75</v>
+        <v>129512.59</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129731.06</v>
+        <v>129798.05</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129588.41</v>
+        <v>129655.32</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.4542</v>
+        <v>13.345</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62744.03</v>
+        <v>62776.43</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62450.91</v>
+        <v>62483.16</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62597.47</v>
+        <v>62629.79</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.4542</v>
+        <v>13.345</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>32044.41</v>
+        <v>32060.96</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32068.61</v>
+        <v>32085.17</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>32056.51</v>
+        <v>32073.06</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4304</v>
+        <v>13.3398</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>408917.02</v>
+        <v>409156.59</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>409466.65</v>
+        <v>409706.54</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>409191.83</v>
+        <v>409431.56</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4304</v>
+        <v>13.3398</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>303534.75</v>
+        <v>303712.58</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>301639.51</v>
+        <v>301816.23</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>302587.13</v>
+        <v>302764.4</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4304</v>
+        <v>13.3398</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>205887.9</v>
+        <v>206008.52</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>205958.33</v>
+        <v>206078.99</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>205923.11</v>
+        <v>206043.75</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4304</v>
+        <v>13.3398</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124589.92</v>
+        <v>124662.91</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125109.39</v>
+        <v>125182.69</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124849.65</v>
+        <v>124922.8</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4304</v>
+        <v>13.3398</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49755.66</v>
+        <v>49784.81</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49696.37</v>
+        <v>49725.49</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49726.02</v>
+        <v>49755.15</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4304</v>
+        <v>13.3398</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5472.96</v>
+        <v>5476.17</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5509.05</v>
+        <v>5512.28</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5491.01</v>
+        <v>5494.22</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3715</v>
+        <v>13.3245</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170790.7</v>
+        <v>170889</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170818.02</v>
+        <v>170916.33</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170804.36</v>
+        <v>170902.67</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3715</v>
+        <v>13.3245</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112237.85</v>
+        <v>112302.45</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111847.4</v>
+        <v>111911.77</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112042.62</v>
+        <v>112107.11</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3715</v>
+        <v>13.3245</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62858.15</v>
+        <v>62894.33</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63214.68</v>
+        <v>63251.07</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63036.42</v>
+        <v>63072.7</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3715</v>
+        <v>13.3245</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26910.18</v>
+        <v>26925.67</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27110.66</v>
+        <v>27126.27</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27010.42</v>
+        <v>27025.97</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3715</v>
+        <v>13.3245</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6334.37</v>
+        <v>6338.02</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6486.64</v>
+        <v>6490.37</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6410.51</v>
+        <v>6414.2</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3715</v>
+        <v>13.3245</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3751.55</v>
+        <v>3753.71</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3745.04</v>
+        <v>3747.19</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3748.29</v>
+        <v>3750.45</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3431</v>
+        <v>13.3183</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191044.07</v>
+        <v>191150.68</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>191976.91</v>
+        <v>192084.04</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191510.49</v>
+        <v>191617.36</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3431</v>
+        <v>13.3183</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138510.99</v>
+        <v>138588.29</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139477.57</v>
+        <v>139555.4</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138994.28</v>
+        <v>139071.84</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3431</v>
+        <v>13.3183</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87552.82000000001</v>
+        <v>87601.67999999999</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88261.36</v>
+        <v>88310.61</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87907.09</v>
+        <v>87956.14999999999</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3431</v>
+        <v>13.3183</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41820.69</v>
+        <v>41844.03</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41753.62</v>
+        <v>41776.92</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41787.16</v>
+        <v>41810.48</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3431</v>
+        <v>13.3183</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13041.1</v>
+        <v>13048.38</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12897.46</v>
+        <v>12904.66</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12969.28</v>
+        <v>12976.52</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3431</v>
+        <v>13.3183</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4526.08</v>
+        <v>4528.6</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4415.59</v>
+        <v>4418.06</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4470.83</v>
+        <v>4473.33</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-01
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3217</v>
+        <v>13.3231</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150645.39</v>
+        <v>150719.48</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152544.6</v>
+        <v>152619.62</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151594.99</v>
+        <v>151669.55</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3217</v>
+        <v>13.3231</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115309.25</v>
+        <v>115365.96</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116093.24</v>
+        <v>116150.34</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115701.24</v>
+        <v>115758.15</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3217</v>
+        <v>13.3231</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82218.19</v>
+        <v>82258.63</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82730.52</v>
+        <v>82771.2</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82474.35000000001</v>
+        <v>82514.92</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3217</v>
+        <v>13.3231</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58259.79</v>
+        <v>58288.44</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57818.25</v>
+        <v>57846.68</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58039.02</v>
+        <v>58067.56</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3217</v>
+        <v>13.3231</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37633.51</v>
+        <v>37652.02</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37941.37</v>
+        <v>37960.03</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37787.44</v>
+        <v>37806.03</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3217</v>
+        <v>13.3231</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17116.42</v>
+        <v>17124.84</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17004.03</v>
+        <v>17012.39</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17060.23</v>
+        <v>17068.62</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3247</v>
+        <v>13.3251</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163669.58</v>
+        <v>163750.61</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162791.36</v>
+        <v>162871.96</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163230.47</v>
+        <v>163311.29</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3247</v>
+        <v>13.3251</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122916.35</v>
+        <v>122977.21</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121180.33</v>
+        <v>121240.33</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122048.34</v>
+        <v>122108.77</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3247</v>
+        <v>13.3251</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87816.09</v>
+        <v>87859.57000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86728.66</v>
+        <v>86771.61</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87272.38</v>
+        <v>87315.59</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3247</v>
+        <v>13.3251</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66893.85000000001</v>
+        <v>66926.97</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66423.60000000001</v>
+        <v>66456.49000000001</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66658.73</v>
+        <v>66691.73</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3247</v>
+        <v>13.3251</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52258.56</v>
+        <v>52284.44</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50380.44</v>
+        <v>50405.38</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51319.5</v>
+        <v>51344.91</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3247</v>
+        <v>13.3251</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39614.82</v>
+        <v>39634.43</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40593.72</v>
+        <v>40613.82</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40104.27</v>
+        <v>40124.13</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3344</v>
+        <v>13.3327</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168516.68</v>
+        <v>168601.74</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170069</v>
+        <v>170154.84</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>169292.84</v>
+        <v>169378.29</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3344</v>
+        <v>13.3327</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121477.05</v>
+        <v>121538.37</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120025.14</v>
+        <v>120085.73</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120751.1</v>
+        <v>120812.05</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3344</v>
+        <v>13.3327</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83213.7</v>
+        <v>83255.7</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82899.39999999999</v>
+        <v>82941.24000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83056.55</v>
+        <v>83098.47</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3344</v>
+        <v>13.3327</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55440.96</v>
+        <v>55468.95</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55746.86</v>
+        <v>55775</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55593.91</v>
+        <v>55621.97</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3344</v>
+        <v>13.3327</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33461.45</v>
+        <v>33478.34</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33069.79</v>
+        <v>33086.49</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33265.62</v>
+        <v>33282.41</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3344</v>
+        <v>13.3327</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17371.76</v>
+        <v>17380.53</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18060.47</v>
+        <v>18069.58</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17716.11</v>
+        <v>17725.06</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.355</v>
+        <v>13.3518</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130229.54</v>
+        <v>130296.58</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130324.97</v>
+        <v>130392.05</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130277.26</v>
+        <v>130344.32</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.355</v>
+        <v>13.3518</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90190.78</v>
+        <v>90237.21000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88791.28</v>
+        <v>88836.99000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89491.03</v>
+        <v>89537.10000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.355</v>
+        <v>13.3518</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56689.97</v>
+        <v>56719.15</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56979.28</v>
+        <v>57008.61</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56834.63</v>
+        <v>56863.88</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.355</v>
+        <v>13.3518</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30011.71</v>
+        <v>30027.16</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30213.72</v>
+        <v>30229.27</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30112.72</v>
+        <v>30128.22</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.355</v>
+        <v>13.3518</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6883.43</v>
+        <v>6886.98</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6882.12</v>
+        <v>6885.66</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6882.78</v>
+        <v>6886.32</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.355</v>
+        <v>13.3518</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3824.74</v>
+        <v>3826.71</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3734.53</v>
+        <v>3736.45</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3779.63</v>
+        <v>3781.58</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3746</v>
+        <v>13.3701</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109948.48</v>
+        <v>110006.36</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110430.83</v>
+        <v>110488.96</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110189.66</v>
+        <v>110247.66</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3746</v>
+        <v>13.3701</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77105.41</v>
+        <v>77146</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76556.84</v>
+        <v>76597.14</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76831.12</v>
+        <v>76871.57000000001</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3746</v>
+        <v>13.3701</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46656.58</v>
+        <v>46681.14</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47772.08</v>
+        <v>47797.23</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47214.33</v>
+        <v>47239.18</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3746</v>
+        <v>13.3701</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28985.82</v>
+        <v>29001.08</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28877.79</v>
+        <v>28893</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28931.81</v>
+        <v>28947.04</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3746</v>
+        <v>13.3701</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14219.17</v>
+        <v>14226.65</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14342.44</v>
+        <v>14349.99</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14280.81</v>
+        <v>14288.32</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3746</v>
+        <v>13.3701</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6592.01</v>
+        <v>6595.48</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6429.16</v>
+        <v>6432.54</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6510.59</v>
+        <v>6514.01</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.3952</v>
+        <v>13.3892</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50040.42</v>
+        <v>50067.49</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49705.41</v>
+        <v>49732.29</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49872.92</v>
+        <v>49899.89</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.3952</v>
+        <v>13.3892</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44022.21</v>
+        <v>44046.02</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44217.65</v>
+        <v>44241.56</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44119.93</v>
+        <v>44143.79</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.3952</v>
+        <v>13.3892</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32217.64</v>
+        <v>32235.06</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32560.74</v>
+        <v>32578.35</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32389.19</v>
+        <v>32406.71</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.3952</v>
+        <v>13.3892</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22653.14</v>
+        <v>22665.39</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22808.72</v>
+        <v>22821.05</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22730.93</v>
+        <v>22743.22</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.3952</v>
+        <v>13.3892</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14559.9</v>
+        <v>14567.77</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14767.09</v>
+        <v>14775.07</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14663.49</v>
+        <v>14671.42</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.3952</v>
+        <v>13.3892</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8367.58</v>
+        <v>8372.110000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8423.02</v>
+        <v>8427.58</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8395.299999999999</v>
+        <v>8399.84</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4167</v>
+        <v>13.4092</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49228.79</v>
+        <v>49256.27</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48504.27</v>
+        <v>48531.35</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48866.53</v>
+        <v>48893.81</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4167</v>
+        <v>13.4092</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44085.08</v>
+        <v>44109.69</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43746.42</v>
+        <v>43770.84</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43915.75</v>
+        <v>43940.26</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4167</v>
+        <v>13.4092</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31838.26</v>
+        <v>31856.03</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31265.91</v>
+        <v>31283.37</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31552.09</v>
+        <v>31569.7</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4167</v>
+        <v>13.4092</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23730.06</v>
+        <v>23743.31</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23624.26</v>
+        <v>23637.45</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23677.16</v>
+        <v>23690.38</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4167</v>
+        <v>13.4092</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18615.93</v>
+        <v>18626.32</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18428.85</v>
+        <v>18439.14</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18522.39</v>
+        <v>18532.73</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4167</v>
+        <v>13.4092</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15657.27</v>
+        <v>15666.01</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15601.37</v>
+        <v>15610.08</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15629.32</v>
+        <v>15638.04</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4364</v>
+        <v>13.4274</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109362.17</v>
+        <v>109425.2</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109916</v>
+        <v>109979.35</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109639.08</v>
+        <v>109702.28</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4364</v>
+        <v>13.4274</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78424.37</v>
+        <v>78469.58</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78741.39999999999</v>
+        <v>78786.78999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78582.89</v>
+        <v>78628.17999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4364</v>
+        <v>13.4274</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51230.16</v>
+        <v>51259.68</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50795.06</v>
+        <v>50824.34</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51012.61</v>
+        <v>51042.01</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4364</v>
+        <v>13.4274</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29453.85</v>
+        <v>29470.83</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29241.63</v>
+        <v>29258.48</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29347.74</v>
+        <v>29364.66</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4364</v>
+        <v>13.4274</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16738.33</v>
+        <v>16747.97</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16672.18</v>
+        <v>16681.79</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16705.26</v>
+        <v>16714.88</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4364</v>
+        <v>13.4274</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6786.34</v>
+        <v>6790.25</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6571.59</v>
+        <v>6575.38</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6678.97</v>
+        <v>6682.82</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.345</v>
+        <v>13.3498</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>405557.76</v>
+        <v>405759.2</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>400540</v>
+        <v>400738.95</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>403048.88</v>
+        <v>403249.08</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.345</v>
+        <v>13.3498</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>304464.17</v>
+        <v>304615.4</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>305451.62</v>
+        <v>305603.33</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>304957.89</v>
+        <v>305109.37</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.345</v>
+        <v>13.3498</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>213034.52</v>
+        <v>213140.33</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>212906</v>
+        <v>213011.75</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>212970.26</v>
+        <v>213076.04</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.345</v>
+        <v>13.3498</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129512.59</v>
+        <v>129576.92</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129798.05</v>
+        <v>129862.52</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129655.32</v>
+        <v>129719.72</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.345</v>
+        <v>13.3498</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62776.43</v>
+        <v>62807.61</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62483.16</v>
+        <v>62514.19</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62629.79</v>
+        <v>62660.9</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.345</v>
+        <v>13.3498</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>32060.96</v>
+        <v>32076.88</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32085.17</v>
+        <v>32101.11</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>32073.06</v>
+        <v>32088.99</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.3398</v>
+        <v>13.3453</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>409156.59</v>
+        <v>409357.9</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>409706.54</v>
+        <v>409908.12</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>409431.56</v>
+        <v>409633.01</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.3398</v>
+        <v>13.3453</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>303712.58</v>
+        <v>303862.01</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>301816.23</v>
+        <v>301964.73</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>302764.4</v>
+        <v>302913.37</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.3398</v>
+        <v>13.3453</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206008.52</v>
+        <v>206109.88</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206078.99</v>
+        <v>206180.39</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206043.75</v>
+        <v>206145.13</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.3398</v>
+        <v>13.3453</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124662.91</v>
+        <v>124724.25</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125182.69</v>
+        <v>125244.28</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124922.8</v>
+        <v>124984.26</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.3398</v>
+        <v>13.3453</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49784.81</v>
+        <v>49809.31</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49725.49</v>
+        <v>49749.95</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49755.15</v>
+        <v>49779.63</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.3398</v>
+        <v>13.3453</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5476.17</v>
+        <v>5478.86</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5512.28</v>
+        <v>5514.99</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5494.22</v>
+        <v>5496.93</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3245</v>
+        <v>13.3289</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170889</v>
+        <v>170972.64</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170916.33</v>
+        <v>170999.99</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170902.67</v>
+        <v>170986.32</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3245</v>
+        <v>13.3289</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112302.45</v>
+        <v>112357.42</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111911.77</v>
+        <v>111966.55</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112107.11</v>
+        <v>112161.98</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3245</v>
+        <v>13.3289</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62894.33</v>
+        <v>62925.11</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63251.07</v>
+        <v>63282.03</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63072.7</v>
+        <v>63103.57</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3245</v>
+        <v>13.3289</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26925.67</v>
+        <v>26938.85</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27126.27</v>
+        <v>27139.54</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27025.97</v>
+        <v>27039.2</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3245</v>
+        <v>13.3289</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6338.02</v>
+        <v>6341.12</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6490.37</v>
+        <v>6493.55</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6414.2</v>
+        <v>6417.34</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3245</v>
+        <v>13.3289</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3753.71</v>
+        <v>3755.54</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3747.19</v>
+        <v>3749.03</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3750.45</v>
+        <v>3752.29</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3183</v>
+        <v>13.3209</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191150.68</v>
+        <v>191244.33</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192084.04</v>
+        <v>192178.15</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191617.36</v>
+        <v>191711.24</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3183</v>
+        <v>13.3209</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138588.29</v>
+        <v>138656.19</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139555.4</v>
+        <v>139623.78</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139071.84</v>
+        <v>139139.98</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3183</v>
+        <v>13.3209</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87601.67999999999</v>
+        <v>87644.60000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88310.61</v>
+        <v>88353.88</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87956.14999999999</v>
+        <v>87999.24000000001</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3183</v>
+        <v>13.3209</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41844.03</v>
+        <v>41864.53</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41776.92</v>
+        <v>41797.39</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41810.48</v>
+        <v>41830.96</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3183</v>
+        <v>13.3209</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13048.38</v>
+        <v>13054.77</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12904.66</v>
+        <v>12910.98</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12976.52</v>
+        <v>12982.88</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3183</v>
+        <v>13.3209</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4528.6</v>
+        <v>4530.82</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4418.06</v>
+        <v>4420.22</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4473.33</v>
+        <v>4475.52</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-02
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3231</v>
+        <v>13.3532</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150719.48</v>
+        <v>150780.02</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152619.62</v>
+        <v>152680.92</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151669.55</v>
+        <v>151730.47</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3231</v>
+        <v>13.3532</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115365.96</v>
+        <v>115412.3</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116150.34</v>
+        <v>116196.99</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115758.15</v>
+        <v>115804.64</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3231</v>
+        <v>13.3532</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82258.63</v>
+        <v>82291.67</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82771.2</v>
+        <v>82804.45</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82514.92</v>
+        <v>82548.06</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3231</v>
+        <v>13.3532</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58288.44</v>
+        <v>58311.85</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57846.68</v>
+        <v>57869.92</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58067.56</v>
+        <v>58090.89</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3231</v>
+        <v>13.3532</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37652.02</v>
+        <v>37667.15</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37960.03</v>
+        <v>37975.27</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37806.03</v>
+        <v>37821.21</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3231</v>
+        <v>13.3532</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17124.84</v>
+        <v>17131.72</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17012.39</v>
+        <v>17019.22</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17068.62</v>
+        <v>17075.47</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3251</v>
+        <v>13.3471</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163750.61</v>
+        <v>163818.05</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162871.96</v>
+        <v>162939.03</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163311.29</v>
+        <v>163378.54</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3251</v>
+        <v>13.3471</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122977.21</v>
+        <v>123027.86</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121240.33</v>
+        <v>121290.26</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122108.77</v>
+        <v>122159.06</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3251</v>
+        <v>13.3471</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87859.57000000001</v>
+        <v>87895.75999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86771.61</v>
+        <v>86807.34</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87315.59</v>
+        <v>87351.55</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3251</v>
+        <v>13.3471</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66926.97</v>
+        <v>66954.53</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66456.49000000001</v>
+        <v>66483.86</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66691.73</v>
+        <v>66719.2</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3251</v>
+        <v>13.3471</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52284.44</v>
+        <v>52305.97</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50405.38</v>
+        <v>50426.14</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51344.91</v>
+        <v>51366.06</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3251</v>
+        <v>13.3471</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39634.43</v>
+        <v>39650.76</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40613.82</v>
+        <v>40630.55</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40124.13</v>
+        <v>40140.65</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3327</v>
+        <v>13.347</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168601.74</v>
+        <v>168674.32</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170154.84</v>
+        <v>170228.09</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>169378.29</v>
+        <v>169451.21</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3327</v>
+        <v>13.347</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121538.37</v>
+        <v>121590.69</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120085.73</v>
+        <v>120137.42</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120812.05</v>
+        <v>120864.06</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3327</v>
+        <v>13.347</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83255.7</v>
+        <v>83291.53999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82941.24000000001</v>
+        <v>82976.95</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83098.47</v>
+        <v>83134.25</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3327</v>
+        <v>13.347</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55468.95</v>
+        <v>55492.82</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55775</v>
+        <v>55799.01</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55621.97</v>
+        <v>55645.92</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3327</v>
+        <v>13.347</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33478.34</v>
+        <v>33492.75</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33086.49</v>
+        <v>33100.73</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33282.41</v>
+        <v>33296.74</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3327</v>
+        <v>13.347</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17380.53</v>
+        <v>17388.01</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18069.58</v>
+        <v>18077.36</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17725.06</v>
+        <v>17732.69</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3518</v>
+        <v>13.3647</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130296.58</v>
+        <v>130352.34</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130392.05</v>
+        <v>130447.85</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130344.32</v>
+        <v>130400.1</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3518</v>
+        <v>13.3647</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90237.21000000001</v>
+        <v>90275.83</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88836.99000000001</v>
+        <v>88875</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89537.10000000001</v>
+        <v>89575.42</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3518</v>
+        <v>13.3647</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56719.15</v>
+        <v>56743.43</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57008.61</v>
+        <v>57033.01</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56863.88</v>
+        <v>56888.22</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3518</v>
+        <v>13.3647</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30027.16</v>
+        <v>30040.01</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30229.27</v>
+        <v>30242.21</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30128.22</v>
+        <v>30141.11</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3518</v>
+        <v>13.3647</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6886.98</v>
+        <v>6889.92</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6885.66</v>
+        <v>6888.61</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6886.32</v>
+        <v>6889.27</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3518</v>
+        <v>13.3647</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3826.71</v>
+        <v>3828.35</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3736.45</v>
+        <v>3738.05</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3781.58</v>
+        <v>3783.2</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3701</v>
+        <v>13.3816</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110006.36</v>
+        <v>110053.4</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110488.96</v>
+        <v>110536.21</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110247.66</v>
+        <v>110294.8</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3701</v>
+        <v>13.3816</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77146</v>
+        <v>77178.99000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76597.14</v>
+        <v>76629.89</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76871.57000000001</v>
+        <v>76904.44</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3701</v>
+        <v>13.3816</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46681.14</v>
+        <v>46701.1</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47797.23</v>
+        <v>47817.66</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47239.18</v>
+        <v>47259.38</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3701</v>
+        <v>13.3816</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29001.08</v>
+        <v>29013.48</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28893</v>
+        <v>28905.35</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28947.04</v>
+        <v>28959.41</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3701</v>
+        <v>13.3816</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14226.65</v>
+        <v>14232.74</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14349.99</v>
+        <v>14356.13</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14288.32</v>
+        <v>14294.43</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3701</v>
+        <v>13.3816</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6595.48</v>
+        <v>6598.3</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6432.54</v>
+        <v>6435.29</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6514.01</v>
+        <v>6516.8</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3992</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50067.49</v>
+        <v>50088.99</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49732.29</v>
+        <v>49753.65</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49899.89</v>
+        <v>49921.32</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3992</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44046.02</v>
+        <v>44064.93</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44241.56</v>
+        <v>44260.56</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44143.79</v>
+        <v>44162.75</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3992</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32235.06</v>
+        <v>32248.9</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32578.35</v>
+        <v>32592.34</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32406.71</v>
+        <v>32420.62</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3992</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22665.39</v>
+        <v>22675.13</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22821.05</v>
+        <v>22830.85</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22743.22</v>
+        <v>22752.99</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3992</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14567.77</v>
+        <v>14574.02</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14775.07</v>
+        <v>14781.42</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14671.42</v>
+        <v>14677.72</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.3892</v>
+        <v>13.3992</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8372.110000000001</v>
+        <v>8375.700000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8427.58</v>
+        <v>8431.200000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8399.84</v>
+        <v>8403.450000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4092</v>
+        <v>13.4177</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49256.27</v>
+        <v>49277.64</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48531.35</v>
+        <v>48552.4</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48893.81</v>
+        <v>48915.02</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4092</v>
+        <v>13.4177</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44109.69</v>
+        <v>44128.82</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43770.84</v>
+        <v>43789.82</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43940.26</v>
+        <v>43959.32</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4092</v>
+        <v>13.4177</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31856.03</v>
+        <v>31869.85</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31283.37</v>
+        <v>31296.94</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31569.7</v>
+        <v>31583.39</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4092</v>
+        <v>13.4177</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23743.31</v>
+        <v>23753.61</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23637.45</v>
+        <v>23647.7</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23690.38</v>
+        <v>23700.66</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4092</v>
+        <v>13.4177</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18626.32</v>
+        <v>18634.4</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18439.14</v>
+        <v>18447.14</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18532.73</v>
+        <v>18540.77</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4092</v>
+        <v>13.4177</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15666.01</v>
+        <v>15672.8</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15610.08</v>
+        <v>15616.85</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15638.04</v>
+        <v>15644.83</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4274</v>
+        <v>13.4346</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109425.2</v>
+        <v>109473.32</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109979.35</v>
+        <v>110027.72</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109702.28</v>
+        <v>109750.52</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4274</v>
+        <v>13.4346</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78469.58</v>
+        <v>78504.08</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78786.78999999999</v>
+        <v>78821.42999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78628.17999999999</v>
+        <v>78662.75999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4274</v>
+        <v>13.4346</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51259.68</v>
+        <v>51282.22</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50824.34</v>
+        <v>50846.69</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51042.01</v>
+        <v>51064.46</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4274</v>
+        <v>13.4346</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29470.83</v>
+        <v>29483.79</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29258.48</v>
+        <v>29271.35</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29364.66</v>
+        <v>29377.57</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4274</v>
+        <v>13.4346</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16747.97</v>
+        <v>16755.34</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16681.79</v>
+        <v>16689.13</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16714.88</v>
+        <v>16722.23</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4274</v>
+        <v>13.4346</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6790.25</v>
+        <v>6793.23</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6575.38</v>
+        <v>6578.27</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6682.82</v>
+        <v>6685.75</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.3498</v>
+        <v>13.4219</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>405759.2</v>
+        <v>405958.97</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>400738.95</v>
+        <v>400936.25</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>403249.08</v>
+        <v>403447.61</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.3498</v>
+        <v>13.4219</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>304615.4</v>
+        <v>304765.37</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>305603.33</v>
+        <v>305753.79</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>305109.37</v>
+        <v>305259.58</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.3498</v>
+        <v>13.4219</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>213140.33</v>
+        <v>213245.27</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>213011.75</v>
+        <v>213116.62</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>213076.04</v>
+        <v>213180.95</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.3498</v>
+        <v>13.4219</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129576.92</v>
+        <v>129640.71</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129862.52</v>
+        <v>129926.45</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129719.72</v>
+        <v>129783.58</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.3498</v>
+        <v>13.4219</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62807.61</v>
+        <v>62838.53</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62514.19</v>
+        <v>62544.97</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62660.9</v>
+        <v>62691.75</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.3498</v>
+        <v>13.4219</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>32076.88</v>
+        <v>32092.67</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32101.11</v>
+        <v>32116.91</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>32088.99</v>
+        <v>32104.79</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.3453</v>
+        <v>13.415</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>409357.9</v>
+        <v>409536.45</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>409908.12</v>
+        <v>410086.92</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>409633.01</v>
+        <v>409811.69</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.3453</v>
+        <v>13.415</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>303862.01</v>
+        <v>303994.55</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>301964.73</v>
+        <v>302096.44</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>302913.37</v>
+        <v>303045.5</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.3453</v>
+        <v>13.415</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206109.88</v>
+        <v>206199.78</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206180.39</v>
+        <v>206270.32</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206145.13</v>
+        <v>206235.05</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.3453</v>
+        <v>13.415</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124724.25</v>
+        <v>124778.65</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125244.28</v>
+        <v>125298.91</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124984.26</v>
+        <v>125038.78</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.3453</v>
+        <v>13.415</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49809.31</v>
+        <v>49831.03</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49749.95</v>
+        <v>49771.65</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49779.63</v>
+        <v>49801.34</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.3453</v>
+        <v>13.415</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5478.86</v>
+        <v>5481.25</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5514.99</v>
+        <v>5517.4</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5496.93</v>
+        <v>5499.33</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3289</v>
+        <v>13.3823</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>170972.64</v>
+        <v>171043.16</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>170999.99</v>
+        <v>171070.51</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>170986.32</v>
+        <v>171056.84</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3289</v>
+        <v>13.3823</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112357.42</v>
+        <v>112403.76</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111966.55</v>
+        <v>112012.73</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112161.98</v>
+        <v>112208.24</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3289</v>
+        <v>13.3823</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62925.11</v>
+        <v>62951.06</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63282.03</v>
+        <v>63308.13</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63103.57</v>
+        <v>63129.6</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3289</v>
+        <v>13.3823</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26938.85</v>
+        <v>26949.96</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27139.54</v>
+        <v>27150.74</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27039.2</v>
+        <v>27050.35</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3289</v>
+        <v>13.3823</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6341.12</v>
+        <v>6343.73</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6493.55</v>
+        <v>6496.23</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6417.34</v>
+        <v>6419.98</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3289</v>
+        <v>13.3823</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3755.54</v>
+        <v>3757.09</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3749.03</v>
+        <v>3750.57</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3752.29</v>
+        <v>3753.83</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3209</v>
+        <v>13.3599</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191244.33</v>
+        <v>191321.51</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192178.15</v>
+        <v>192255.7</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191711.24</v>
+        <v>191788.6</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3209</v>
+        <v>13.3599</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138656.19</v>
+        <v>138712.14</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139623.78</v>
+        <v>139680.12</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139139.98</v>
+        <v>139196.13</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3209</v>
+        <v>13.3599</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87644.60000000001</v>
+        <v>87679.97</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88353.88</v>
+        <v>88389.53</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87999.24000000001</v>
+        <v>88034.75</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3209</v>
+        <v>13.3599</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41864.53</v>
+        <v>41881.42</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41797.39</v>
+        <v>41814.26</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41830.96</v>
+        <v>41847.84</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3209</v>
+        <v>13.3599</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13054.77</v>
+        <v>13060.04</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12910.98</v>
+        <v>12916.19</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12982.88</v>
+        <v>12988.11</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3209</v>
+        <v>13.3599</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4530.82</v>
+        <v>4532.65</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4420.22</v>
+        <v>4422</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4475.52</v>
+        <v>4477.33</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-03
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3532</v>
+        <v>13.3361</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150780.02</v>
+        <v>150788.13</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152680.92</v>
+        <v>152689.13</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151730.47</v>
+        <v>151738.63</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3532</v>
+        <v>13.3361</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115412.3</v>
+        <v>115418.5</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116196.99</v>
+        <v>116203.24</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115804.64</v>
+        <v>115810.87</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3532</v>
+        <v>13.3361</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82291.67</v>
+        <v>82296.10000000001</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82804.45</v>
+        <v>82808.89999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82548.06</v>
+        <v>82552.5</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3532</v>
+        <v>13.3361</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58311.85</v>
+        <v>58314.99</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57869.92</v>
+        <v>57873.03</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58090.89</v>
+        <v>58094.01</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3532</v>
+        <v>13.3361</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37667.15</v>
+        <v>37669.17</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37975.27</v>
+        <v>37977.32</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37821.21</v>
+        <v>37823.24</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3532</v>
+        <v>13.3361</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17131.72</v>
+        <v>17132.64</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17019.22</v>
+        <v>17020.14</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17075.47</v>
+        <v>17076.39</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3471</v>
+        <v>13.321</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163818.05</v>
+        <v>163834.51</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162939.03</v>
+        <v>162955.41</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163378.54</v>
+        <v>163394.96</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3471</v>
+        <v>13.321</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123027.86</v>
+        <v>123040.22</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121290.26</v>
+        <v>121302.45</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122159.06</v>
+        <v>122171.33</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3471</v>
+        <v>13.321</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87895.75999999999</v>
+        <v>87904.59</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86807.34</v>
+        <v>86816.06</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87351.55</v>
+        <v>87360.33</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3471</v>
+        <v>13.321</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66954.53</v>
+        <v>66961.25999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66483.86</v>
+        <v>66490.53999999999</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66719.2</v>
+        <v>66725.89999999999</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3471</v>
+        <v>13.321</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52305.97</v>
+        <v>52311.23</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50426.14</v>
+        <v>50431.21</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51366.06</v>
+        <v>51371.22</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3471</v>
+        <v>13.321</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39650.76</v>
+        <v>39654.74</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40630.55</v>
+        <v>40634.63</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40140.65</v>
+        <v>40144.69</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.347</v>
+        <v>13.3123</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168674.32</v>
+        <v>168701.36</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170228.09</v>
+        <v>170255.38</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>169451.21</v>
+        <v>169478.37</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.347</v>
+        <v>13.3123</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121590.69</v>
+        <v>121610.18</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120137.42</v>
+        <v>120156.68</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120864.06</v>
+        <v>120883.43</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.347</v>
+        <v>13.3123</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83291.53999999999</v>
+        <v>83304.89999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82976.95</v>
+        <v>82990.25</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83134.25</v>
+        <v>83147.57000000001</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.347</v>
+        <v>13.3123</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55492.82</v>
+        <v>55501.72</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55799.01</v>
+        <v>55807.96</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55645.92</v>
+        <v>55654.84</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.347</v>
+        <v>13.3123</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33492.75</v>
+        <v>33498.12</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33100.73</v>
+        <v>33106.04</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33296.74</v>
+        <v>33302.08</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.347</v>
+        <v>13.3123</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17388.01</v>
+        <v>17390.8</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18077.36</v>
+        <v>18080.26</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17732.69</v>
+        <v>17735.53</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3647</v>
+        <v>13.3249</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130352.34</v>
+        <v>130380.28</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130447.85</v>
+        <v>130475.81</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130400.1</v>
+        <v>130428.04</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3647</v>
+        <v>13.3249</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90275.83</v>
+        <v>90295.17</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88875</v>
+        <v>88894.05</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89575.42</v>
+        <v>89594.61</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3647</v>
+        <v>13.3249</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56743.43</v>
+        <v>56755.59</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57033.01</v>
+        <v>57045.23</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56888.22</v>
+        <v>56900.41</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3647</v>
+        <v>13.3249</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30040.01</v>
+        <v>30046.45</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30242.21</v>
+        <v>30248.69</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30141.11</v>
+        <v>30147.57</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3647</v>
+        <v>13.3249</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6889.92</v>
+        <v>6891.4</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6888.61</v>
+        <v>6890.08</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6889.27</v>
+        <v>6890.74</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3647</v>
+        <v>13.3249</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3828.35</v>
+        <v>3829.17</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3738.05</v>
+        <v>3738.85</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3783.2</v>
+        <v>3784.01</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3816</v>
+        <v>13.337</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110053.4</v>
+        <v>110083.46</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110536.21</v>
+        <v>110566.4</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110294.8</v>
+        <v>110324.93</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3816</v>
+        <v>13.337</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77178.99000000001</v>
+        <v>77200.06</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76629.89</v>
+        <v>76650.82000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76904.44</v>
+        <v>76925.44</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3816</v>
+        <v>13.337</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46701.1</v>
+        <v>46713.86</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47817.66</v>
+        <v>47830.73</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47259.38</v>
+        <v>47272.29</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3816</v>
+        <v>13.337</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29013.48</v>
+        <v>29021.4</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28905.35</v>
+        <v>28913.24</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28959.41</v>
+        <v>28967.32</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3816</v>
+        <v>13.337</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14232.74</v>
+        <v>14236.62</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14356.13</v>
+        <v>14360.05</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14294.43</v>
+        <v>14298.34</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3816</v>
+        <v>13.337</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6598.3</v>
+        <v>6600.1</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6435.29</v>
+        <v>6437.05</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6516.8</v>
+        <v>6518.58</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.3992</v>
+        <v>13.3496</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50088.99</v>
+        <v>50106.13</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49753.65</v>
+        <v>49770.68</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49921.32</v>
+        <v>49938.41</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.3992</v>
+        <v>13.3496</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44064.93</v>
+        <v>44080.02</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44260.56</v>
+        <v>44275.71</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44162.75</v>
+        <v>44177.87</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.3992</v>
+        <v>13.3496</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32248.9</v>
+        <v>32259.94</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32592.34</v>
+        <v>32603.5</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32420.62</v>
+        <v>32431.72</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.3992</v>
+        <v>13.3496</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22675.13</v>
+        <v>22682.89</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22830.85</v>
+        <v>22838.67</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22752.99</v>
+        <v>22760.78</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.3992</v>
+        <v>13.3496</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14574.02</v>
+        <v>14579.01</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14781.42</v>
+        <v>14786.48</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14677.72</v>
+        <v>14682.75</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.3992</v>
+        <v>13.3496</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8375.700000000001</v>
+        <v>8378.57</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8431.200000000001</v>
+        <v>8434.08</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8403.450000000001</v>
+        <v>8406.33</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4177</v>
+        <v>13.3628</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49277.64</v>
+        <v>49298.48</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48552.4</v>
+        <v>48572.94</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48915.02</v>
+        <v>48935.71</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4177</v>
+        <v>13.3628</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44128.82</v>
+        <v>44147.49</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43789.82</v>
+        <v>43808.35</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43959.32</v>
+        <v>43977.92</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4177</v>
+        <v>13.3628</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31869.85</v>
+        <v>31883.33</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31296.94</v>
+        <v>31310.18</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31583.39</v>
+        <v>31596.75</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4177</v>
+        <v>13.3628</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23753.61</v>
+        <v>23763.66</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23647.7</v>
+        <v>23657.71</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23700.66</v>
+        <v>23710.68</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4177</v>
+        <v>13.3628</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18634.4</v>
+        <v>18642.28</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18447.14</v>
+        <v>18454.94</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18540.77</v>
+        <v>18548.61</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4177</v>
+        <v>13.3628</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15672.8</v>
+        <v>15679.44</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15616.85</v>
+        <v>15623.45</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15644.83</v>
+        <v>15651.44</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4346</v>
+        <v>13.3748</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109473.32</v>
+        <v>109528.51</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110027.72</v>
+        <v>110083.19</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109750.52</v>
+        <v>109805.85</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4346</v>
+        <v>13.3748</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78504.08</v>
+        <v>78543.66</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78821.42999999999</v>
+        <v>78861.17</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78662.75999999999</v>
+        <v>78702.42</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4346</v>
+        <v>13.3748</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51282.22</v>
+        <v>51308.08</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50846.69</v>
+        <v>50872.32</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51064.46</v>
+        <v>51090.2</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4346</v>
+        <v>13.3748</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29483.79</v>
+        <v>29498.65</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29271.35</v>
+        <v>29286.1</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29377.57</v>
+        <v>29392.38</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4346</v>
+        <v>13.3748</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16755.34</v>
+        <v>16763.79</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16689.13</v>
+        <v>16697.54</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16722.23</v>
+        <v>16730.67</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4346</v>
+        <v>13.3748</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6793.23</v>
+        <v>6796.66</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6578.27</v>
+        <v>6581.59</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6685.75</v>
+        <v>6689.12</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.4219</v>
+        <v>13.4439</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>405958.97</v>
+        <v>405958.34</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>400936.25</v>
+        <v>400935.63</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>403447.61</v>
+        <v>403446.99</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.4219</v>
+        <v>13.4439</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>304765.37</v>
+        <v>304764.9</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>305753.79</v>
+        <v>305753.32</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>305259.58</v>
+        <v>305259.11</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.4219</v>
+        <v>13.4439</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>213245.27</v>
+        <v>213244.94</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>213116.62</v>
+        <v>213116.3</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>213180.95</v>
+        <v>213180.62</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.4219</v>
+        <v>13.4439</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129640.71</v>
+        <v>129640.51</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129926.45</v>
+        <v>129926.25</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129783.58</v>
+        <v>129783.38</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.4219</v>
+        <v>13.4439</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62838.53</v>
+        <v>62838.43</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62544.97</v>
+        <v>62544.87</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62691.75</v>
+        <v>62691.65</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.4219</v>
+        <v>13.4439</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>32092.67</v>
+        <v>32092.62</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32116.91</v>
+        <v>32116.86</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>32104.79</v>
+        <v>32104.74</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.415</v>
+        <v>13.4343</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>409536.45</v>
+        <v>409529.56</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>410086.92</v>
+        <v>410080.01</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>409811.69</v>
+        <v>409804.79</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.415</v>
+        <v>13.4343</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>303994.55</v>
+        <v>303989.43</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>302096.44</v>
+        <v>302091.35</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>303045.5</v>
+        <v>303040.39</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.415</v>
+        <v>13.4343</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206199.78</v>
+        <v>206196.31</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206270.32</v>
+        <v>206266.84</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206235.05</v>
+        <v>206231.58</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.415</v>
+        <v>13.4343</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124778.65</v>
+        <v>124776.55</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125298.91</v>
+        <v>125296.8</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125038.78</v>
+        <v>125036.67</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.415</v>
+        <v>13.4343</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49831.03</v>
+        <v>49830.19</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49771.65</v>
+        <v>49770.81</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49801.34</v>
+        <v>49800.5</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.415</v>
+        <v>13.4343</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5481.25</v>
+        <v>5481.16</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5517.4</v>
+        <v>5517.31</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5499.33</v>
+        <v>5499.23</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3823</v>
+        <v>13.3881</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171043.16</v>
+        <v>171041.59</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171070.51</v>
+        <v>171068.95</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171056.84</v>
+        <v>171055.27</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3823</v>
+        <v>13.3881</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112403.76</v>
+        <v>112402.73</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112012.73</v>
+        <v>112011.7</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112208.24</v>
+        <v>112207.21</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3823</v>
+        <v>13.3881</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62951.06</v>
+        <v>62950.49</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63308.13</v>
+        <v>63307.55</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63129.6</v>
+        <v>63129.02</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3823</v>
+        <v>13.3881</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26949.96</v>
+        <v>26949.71</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27150.74</v>
+        <v>27150.49</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27050.35</v>
+        <v>27050.1</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3823</v>
+        <v>13.3881</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6343.73</v>
+        <v>6343.68</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6496.23</v>
+        <v>6496.17</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6419.98</v>
+        <v>6419.92</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3823</v>
+        <v>13.3881</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3757.09</v>
+        <v>3757.06</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3750.57</v>
+        <v>3750.54</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3753.83</v>
+        <v>3753.8</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.3527</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191321.51</v>
+        <v>191324.76</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192255.7</v>
+        <v>192258.98</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191788.6</v>
+        <v>191791.87</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.3527</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138712.14</v>
+        <v>138714.5</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139680.12</v>
+        <v>139682.5</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139196.13</v>
+        <v>139198.5</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.3527</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87679.97</v>
+        <v>87681.46000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88389.53</v>
+        <v>88391.03999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88034.75</v>
+        <v>88036.25</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.3527</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41881.42</v>
+        <v>41882.14</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41814.26</v>
+        <v>41814.97</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41847.84</v>
+        <v>41848.55</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.3527</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13060.04</v>
+        <v>13060.26</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12916.19</v>
+        <v>12916.41</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12988.11</v>
+        <v>12988.34</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.3527</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4532.65</v>
+        <v>4532.73</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4422</v>
+        <v>4422.08</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4477.33</v>
+        <v>4477.4</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-06
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3361</v>
+        <v>13.1628</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>150788.13</v>
+        <v>151018.68</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152689.13</v>
+        <v>152922.59</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151738.63</v>
+        <v>151970.63</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3361</v>
+        <v>13.1628</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115418.5</v>
+        <v>115594.97</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116203.24</v>
+        <v>116380.91</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115810.87</v>
+        <v>115987.94</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3361</v>
+        <v>13.1628</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82296.10000000001</v>
+        <v>82421.92</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82808.89999999999</v>
+        <v>82935.50999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82552.5</v>
+        <v>82678.72</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3361</v>
+        <v>13.1628</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58314.99</v>
+        <v>58404.15</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57873.03</v>
+        <v>57961.52</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58094.01</v>
+        <v>58182.83</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3361</v>
+        <v>13.1628</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37669.17</v>
+        <v>37726.77</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37977.32</v>
+        <v>38035.38</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37823.24</v>
+        <v>37881.07</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3361</v>
+        <v>13.1628</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17132.64</v>
+        <v>17158.84</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17020.14</v>
+        <v>17046.16</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17076.39</v>
+        <v>17102.5</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.321</v>
+        <v>13.0686</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>163834.51</v>
+        <v>164154.01</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>162955.41</v>
+        <v>163273.19</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163394.96</v>
+        <v>163713.6</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.321</v>
+        <v>13.0686</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123040.22</v>
+        <v>123280.16</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121302.45</v>
+        <v>121539.01</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122171.33</v>
+        <v>122409.59</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.321</v>
+        <v>13.0686</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87904.59</v>
+        <v>88076.00999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86816.06</v>
+        <v>86985.37</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87360.33</v>
+        <v>87530.69</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.321</v>
+        <v>13.0686</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66961.25999999999</v>
+        <v>67091.85000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66490.53999999999</v>
+        <v>66620.2</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66725.89999999999</v>
+        <v>66856.02</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.321</v>
+        <v>13.0686</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52311.23</v>
+        <v>52413.24</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50431.21</v>
+        <v>50529.56</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51371.22</v>
+        <v>51471.4</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.321</v>
+        <v>13.0686</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39654.74</v>
+        <v>39732.07</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40634.63</v>
+        <v>40713.87</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40144.69</v>
+        <v>40222.97</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3123</v>
+        <v>12.9741</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>168701.36</v>
+        <v>169129.44</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170255.38</v>
+        <v>170687.41</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>169478.37</v>
+        <v>169908.42</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3123</v>
+        <v>12.9741</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121610.18</v>
+        <v>121918.77</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120156.68</v>
+        <v>120461.58</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>120883.43</v>
+        <v>121190.18</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3123</v>
+        <v>12.9741</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83304.89999999999</v>
+        <v>83516.28</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82990.25</v>
+        <v>83200.84</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83147.57000000001</v>
+        <v>83358.56</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3123</v>
+        <v>12.9741</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55501.72</v>
+        <v>55642.56</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55807.96</v>
+        <v>55949.57</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55654.84</v>
+        <v>55796.06</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3123</v>
+        <v>12.9741</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33498.12</v>
+        <v>33583.12</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33106.04</v>
+        <v>33190.04</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33302.08</v>
+        <v>33386.58</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3123</v>
+        <v>12.9741</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17390.8</v>
+        <v>17434.93</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18080.26</v>
+        <v>18126.14</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17735.53</v>
+        <v>17780.53</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3249</v>
+        <v>12.921</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130380.28</v>
+        <v>130791.19</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130475.81</v>
+        <v>130887.02</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130428.04</v>
+        <v>130839.1</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3249</v>
+        <v>12.921</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90295.17</v>
+        <v>90579.75</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88894.05</v>
+        <v>89174.21000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89594.61</v>
+        <v>89876.98</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3249</v>
+        <v>12.921</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56755.59</v>
+        <v>56934.46</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57045.23</v>
+        <v>57225.02</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56900.41</v>
+        <v>57079.74</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3249</v>
+        <v>12.921</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30046.45</v>
+        <v>30141.14</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30248.69</v>
+        <v>30344.02</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30147.57</v>
+        <v>30242.58</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3249</v>
+        <v>12.921</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6891.4</v>
+        <v>6913.12</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6890.08</v>
+        <v>6911.8</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6890.74</v>
+        <v>6912.46</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3249</v>
+        <v>12.921</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3829.17</v>
+        <v>3841.23</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3738.85</v>
+        <v>3750.63</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3784.01</v>
+        <v>3795.93</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.337</v>
+        <v>12.8703</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110083.46</v>
+        <v>110505.44</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110566.4</v>
+        <v>110990.23</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110324.93</v>
+        <v>110747.84</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.337</v>
+        <v>12.8703</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77200.06</v>
+        <v>77496</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76650.82000000001</v>
+        <v>76944.64999999999</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76925.44</v>
+        <v>77220.32000000001</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.337</v>
+        <v>12.8703</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46713.86</v>
+        <v>46892.93</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47830.73</v>
+        <v>48014.07</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47272.29</v>
+        <v>47453.5</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.337</v>
+        <v>12.8703</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29021.4</v>
+        <v>29132.65</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28913.24</v>
+        <v>29024.08</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28967.32</v>
+        <v>29078.36</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.337</v>
+        <v>12.8703</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14236.62</v>
+        <v>14291.2</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14360.05</v>
+        <v>14415.1</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14298.34</v>
+        <v>14353.15</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.337</v>
+        <v>12.8703</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6600.1</v>
+        <v>6625.4</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6437.05</v>
+        <v>6461.73</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6518.58</v>
+        <v>6543.57</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.3496</v>
+        <v>12.8173</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50106.13</v>
+        <v>50339.01</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49770.68</v>
+        <v>50002</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49938.41</v>
+        <v>50170.51</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.3496</v>
+        <v>12.8173</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44080.02</v>
+        <v>44284.89</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44275.71</v>
+        <v>44481.5</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44177.87</v>
+        <v>44383.19</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.3496</v>
+        <v>12.8173</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32259.94</v>
+        <v>32409.88</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32603.5</v>
+        <v>32755.03</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32431.72</v>
+        <v>32582.46</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.3496</v>
+        <v>12.8173</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22682.89</v>
+        <v>22788.31</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22838.67</v>
+        <v>22944.82</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22760.78</v>
+        <v>22866.56</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.3496</v>
+        <v>12.8173</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14579.01</v>
+        <v>14646.77</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14786.48</v>
+        <v>14855.2</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14682.75</v>
+        <v>14750.99</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.3496</v>
+        <v>12.8173</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8378.57</v>
+        <v>8417.51</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8434.08</v>
+        <v>8473.280000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8406.33</v>
+        <v>8445.4</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.3628</v>
+        <v>12.7618</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49298.48</v>
+        <v>49575.01</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48572.94</v>
+        <v>48845.39</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48935.71</v>
+        <v>49210.2</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.3628</v>
+        <v>12.7618</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44147.49</v>
+        <v>44395.12</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43808.35</v>
+        <v>44054.08</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43977.92</v>
+        <v>44224.6</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.3628</v>
+        <v>12.7618</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31883.33</v>
+        <v>32062.17</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31310.18</v>
+        <v>31485.8</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31596.75</v>
+        <v>31773.99</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.3628</v>
+        <v>12.7618</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23763.66</v>
+        <v>23896.95</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23657.71</v>
+        <v>23790.41</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23710.68</v>
+        <v>23843.68</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.3628</v>
+        <v>12.7618</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18642.28</v>
+        <v>18746.85</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18454.94</v>
+        <v>18558.46</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18548.61</v>
+        <v>18652.66</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.3628</v>
+        <v>12.7618</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15679.44</v>
+        <v>15767.38</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15623.45</v>
+        <v>15711.09</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15651.44</v>
+        <v>15739.24</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.3748</v>
+        <v>12.7112</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109528.51</v>
+        <v>110249.84</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110083.19</v>
+        <v>110808.16</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109805.85</v>
+        <v>110529</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.3748</v>
+        <v>12.7112</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78543.66</v>
+        <v>79060.92999999999</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78861.17</v>
+        <v>79380.53</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78702.42</v>
+        <v>79220.73</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.3748</v>
+        <v>12.7112</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51308.08</v>
+        <v>51645.98</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50872.32</v>
+        <v>51207.35</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51090.2</v>
+        <v>51426.67</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.3748</v>
+        <v>12.7112</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29498.65</v>
+        <v>29692.92</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29286.1</v>
+        <v>29478.97</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29392.38</v>
+        <v>29585.95</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.3748</v>
+        <v>12.7112</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16763.79</v>
+        <v>16874.19</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16697.54</v>
+        <v>16807.51</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16730.67</v>
+        <v>16840.85</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.3748</v>
+        <v>12.7112</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6796.66</v>
+        <v>6841.42</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6581.59</v>
+        <v>6624.94</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6689.12</v>
+        <v>6733.18</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5587,11 +5587,11 @@
       </c>
       <c r="B52" s="50" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2027-10-06</t>
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.4439</v>
+        <v>12.677</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>405958.34</v>
+        <v>359111.98</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>400935.63</v>
+        <v>354668.87</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>403446.99</v>
+        <v>356890.43</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5640,11 +5640,11 @@
       </c>
       <c r="B53" s="50" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2027-10-06</t>
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.4439</v>
+        <v>12.677</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>304764.9</v>
+        <v>269595.96</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>305753.32</v>
+        <v>270470.31</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>305259.11</v>
+        <v>270033.14</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5693,11 +5693,11 @@
       </c>
       <c r="B54" s="50" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2027-10-06</t>
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.4439</v>
+        <v>12.677</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>213244.94</v>
+        <v>188637.12</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>213116.3</v>
+        <v>188523.32</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>213180.62</v>
+        <v>188580.22</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5746,11 +5746,11 @@
       </c>
       <c r="B55" s="50" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2027-10-06</t>
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.4439</v>
+        <v>12.677</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>129640.51</v>
+        <v>114680.39</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>129926.25</v>
+        <v>114933.16</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>129783.38</v>
+        <v>114806.77</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5799,11 +5799,11 @@
       </c>
       <c r="B56" s="50" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2027-10-06</t>
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.4439</v>
+        <v>12.677</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62838.43</v>
+        <v>55587.07</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62544.87</v>
+        <v>55327.38</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62691.65</v>
+        <v>55457.23</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5852,11 +5852,11 @@
       </c>
       <c r="B57" s="50" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2027-10-06</t>
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.4439</v>
+        <v>12.677</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>32092.62</v>
+        <v>28389.23</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>32116.86</v>
+        <v>28410.67</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>32104.74</v>
+        <v>28399.95</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4343</v>
+        <v>13.5455</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>409529.56</v>
+        <v>409902.79</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>410080.01</v>
+        <v>410453.75</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>409804.79</v>
+        <v>410178.27</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4343</v>
+        <v>13.5455</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>303989.43</v>
+        <v>304266.48</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>302091.35</v>
+        <v>302366.67</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>303040.39</v>
+        <v>303316.58</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4343</v>
+        <v>13.5455</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206196.31</v>
+        <v>206384.23</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206266.84</v>
+        <v>206454.83</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206231.58</v>
+        <v>206419.53</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4343</v>
+        <v>13.5455</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124776.55</v>
+        <v>124890.27</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125296.8</v>
+        <v>125410.99</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125036.67</v>
+        <v>125150.63</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4343</v>
+        <v>13.5455</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49830.19</v>
+        <v>49875.61</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49770.81</v>
+        <v>49816.17</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49800.5</v>
+        <v>49845.89</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4343</v>
+        <v>13.5455</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5481.16</v>
+        <v>5486.15</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5517.31</v>
+        <v>5522.33</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5499.23</v>
+        <v>5504.24</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3881</v>
+        <v>13.4046</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171041.59</v>
+        <v>171207.99</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171068.95</v>
+        <v>171235.38</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171055.27</v>
+        <v>171221.68</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3881</v>
+        <v>13.4046</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112402.73</v>
+        <v>112512.08</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112011.7</v>
+        <v>112120.68</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112207.21</v>
+        <v>112316.38</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3881</v>
+        <v>13.4046</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62950.49</v>
+        <v>63011.73</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63307.55</v>
+        <v>63369.14</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63129.02</v>
+        <v>63190.43</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3881</v>
+        <v>13.4046</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26949.71</v>
+        <v>26975.93</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27150.49</v>
+        <v>27176.9</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27050.1</v>
+        <v>27076.42</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3881</v>
+        <v>13.4046</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6343.68</v>
+        <v>6349.85</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6496.17</v>
+        <v>6502.49</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6419.92</v>
+        <v>6426.17</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3881</v>
+        <v>13.4046</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3757.06</v>
+        <v>3760.71</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3750.54</v>
+        <v>3754.19</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3753.8</v>
+        <v>3757.45</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3527</v>
+        <v>13.2666</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191324.76</v>
+        <v>191553.32</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192258.98</v>
+        <v>192488.65</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>191791.87</v>
+        <v>192020.98</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3527</v>
+        <v>13.2666</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138714.5</v>
+        <v>138880.21</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139682.5</v>
+        <v>139849.36</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139198.5</v>
+        <v>139364.78</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3527</v>
+        <v>13.2666</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87681.46000000001</v>
+        <v>87786.21000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88391.03999999999</v>
+        <v>88496.63</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88036.25</v>
+        <v>88141.42</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3527</v>
+        <v>13.2666</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41882.14</v>
+        <v>41932.17</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41814.97</v>
+        <v>41864.92</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41848.55</v>
+        <v>41898.54</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3527</v>
+        <v>13.2666</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13060.26</v>
+        <v>13075.86</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12916.41</v>
+        <v>12931.84</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12988.34</v>
+        <v>13003.85</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3527</v>
+        <v>13.2666</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4532.73</v>
+        <v>4538.14</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4422.08</v>
+        <v>4427.36</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4477.4</v>
+        <v>4482.75</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-07
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.1628</v>
+        <v>13.2053</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151018.68</v>
+        <v>151073.24</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152922.59</v>
+        <v>152977.84</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>151970.63</v>
+        <v>152025.54</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.1628</v>
+        <v>13.2053</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115594.97</v>
+        <v>115636.74</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116380.91</v>
+        <v>116422.95</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>115987.94</v>
+        <v>116029.85</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.1628</v>
+        <v>13.2053</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82421.92</v>
+        <v>82451.7</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82935.50999999999</v>
+        <v>82965.48</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82678.72</v>
+        <v>82708.59</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.1628</v>
+        <v>13.2053</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58404.15</v>
+        <v>58425.25</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57961.52</v>
+        <v>57982.46</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58182.83</v>
+        <v>58203.86</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.1628</v>
+        <v>13.2053</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37726.77</v>
+        <v>37740.4</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38035.38</v>
+        <v>38049.12</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37881.07</v>
+        <v>37894.76</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.1628</v>
+        <v>13.2053</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17158.84</v>
+        <v>17165.04</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17046.16</v>
+        <v>17052.32</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17102.5</v>
+        <v>17108.68</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.0686</v>
+        <v>13.099</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164154.01</v>
+        <v>164215.24</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163273.19</v>
+        <v>163334.09</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163713.6</v>
+        <v>163774.67</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.0686</v>
+        <v>13.099</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123280.16</v>
+        <v>123326.15</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121539.01</v>
+        <v>121584.34</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122409.59</v>
+        <v>122455.24</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.0686</v>
+        <v>13.099</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88076.00999999999</v>
+        <v>88108.87</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86985.37</v>
+        <v>87017.81</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87530.69</v>
+        <v>87563.34</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.0686</v>
+        <v>13.099</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67091.85000000001</v>
+        <v>67116.87</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66620.2</v>
+        <v>66645.05</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66856.02</v>
+        <v>66880.96000000001</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.0686</v>
+        <v>13.099</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52413.24</v>
+        <v>52432.79</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50529.56</v>
+        <v>50548.4</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51471.4</v>
+        <v>51490.6</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.0686</v>
+        <v>13.099</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39732.07</v>
+        <v>39746.89</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40713.87</v>
+        <v>40729.06</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40222.97</v>
+        <v>40237.98</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>12.9741</v>
+        <v>12.9893</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169129.44</v>
+        <v>169199.64</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170687.41</v>
+        <v>170758.26</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>169908.42</v>
+        <v>169978.95</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>12.9741</v>
+        <v>12.9893</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121918.77</v>
+        <v>121969.38</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120461.58</v>
+        <v>120511.58</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121190.18</v>
+        <v>121240.48</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>12.9741</v>
+        <v>12.9893</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83516.28</v>
+        <v>83550.95</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83200.84</v>
+        <v>83235.37</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83358.56</v>
+        <v>83393.16</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>12.9741</v>
+        <v>12.9893</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55642.56</v>
+        <v>55665.65</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55949.57</v>
+        <v>55972.8</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55796.06</v>
+        <v>55819.22</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>12.9741</v>
+        <v>12.9893</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33583.12</v>
+        <v>33597.06</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33190.04</v>
+        <v>33203.82</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33386.58</v>
+        <v>33400.44</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>12.9741</v>
+        <v>12.9893</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17434.93</v>
+        <v>17442.17</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18126.14</v>
+        <v>18133.66</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17780.53</v>
+        <v>17787.91</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>12.921</v>
+        <v>12.9248</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130791.19</v>
+        <v>130851.65</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130887.02</v>
+        <v>130947.53</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130839.1</v>
+        <v>130899.59</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>12.921</v>
+        <v>12.9248</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90579.75</v>
+        <v>90621.62</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89174.21000000001</v>
+        <v>89215.44</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89876.98</v>
+        <v>89918.53</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>12.921</v>
+        <v>12.9248</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56934.46</v>
+        <v>56960.78</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57225.02</v>
+        <v>57251.47</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57079.74</v>
+        <v>57106.12</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>12.921</v>
+        <v>12.9248</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30141.14</v>
+        <v>30155.08</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30344.02</v>
+        <v>30358.05</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30242.58</v>
+        <v>30256.57</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>12.921</v>
+        <v>12.9248</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6913.12</v>
+        <v>6916.31</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6911.8</v>
+        <v>6914.99</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6912.46</v>
+        <v>6915.65</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>12.921</v>
+        <v>12.9248</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3841.23</v>
+        <v>3843.01</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3750.63</v>
+        <v>3752.37</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3795.93</v>
+        <v>3797.69</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>12.8703</v>
+        <v>12.8632</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110505.44</v>
+        <v>110563.34</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110990.23</v>
+        <v>111048.39</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110747.84</v>
+        <v>110805.86</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>12.8703</v>
+        <v>12.8632</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77496</v>
+        <v>77536.60000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76944.64999999999</v>
+        <v>76984.96000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77220.32000000001</v>
+        <v>77260.78</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>12.8703</v>
+        <v>12.8632</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46892.93</v>
+        <v>46917.49</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48014.07</v>
+        <v>48039.23</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47453.5</v>
+        <v>47478.36</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>12.8703</v>
+        <v>12.8632</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29132.65</v>
+        <v>29147.91</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29024.08</v>
+        <v>29039.29</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29078.36</v>
+        <v>29093.6</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>12.8703</v>
+        <v>12.8632</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14291.2</v>
+        <v>14298.68</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14415.1</v>
+        <v>14422.65</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14353.15</v>
+        <v>14360.67</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>12.8703</v>
+        <v>12.8632</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6625.4</v>
+        <v>6628.88</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6461.73</v>
+        <v>6465.11</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6543.57</v>
+        <v>6546.99</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.8173</v>
+        <v>12.7986</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50339.01</v>
+        <v>50369.52</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50002</v>
+        <v>50032.3</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50170.51</v>
+        <v>50200.91</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.8173</v>
+        <v>12.7986</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44284.89</v>
+        <v>44311.73</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44481.5</v>
+        <v>44508.45</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44383.19</v>
+        <v>44410.09</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.8173</v>
+        <v>12.7986</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32409.88</v>
+        <v>32429.52</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32755.03</v>
+        <v>32774.88</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32582.46</v>
+        <v>32602.2</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.8173</v>
+        <v>12.7986</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22788.31</v>
+        <v>22802.12</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22944.82</v>
+        <v>22958.72</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22866.56</v>
+        <v>22880.42</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.8173</v>
+        <v>12.7986</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14646.77</v>
+        <v>14655.65</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14855.2</v>
+        <v>14864.21</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14750.99</v>
+        <v>14759.93</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.8173</v>
+        <v>12.7986</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8417.51</v>
+        <v>8422.610000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8473.280000000001</v>
+        <v>8478.42</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8445.4</v>
+        <v>8450.51</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.7618</v>
+        <v>12.7312</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49575.01</v>
+        <v>49610.25</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48845.39</v>
+        <v>48880.12</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49210.2</v>
+        <v>49245.18</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.7618</v>
+        <v>12.7312</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44395.12</v>
+        <v>44426.68</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44054.08</v>
+        <v>44085.4</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44224.6</v>
+        <v>44256.04</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.7618</v>
+        <v>12.7312</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32062.17</v>
+        <v>32084.97</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31485.8</v>
+        <v>31508.18</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31773.99</v>
+        <v>31796.58</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.7618</v>
+        <v>12.7312</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23896.95</v>
+        <v>23913.94</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23790.41</v>
+        <v>23807.32</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23843.68</v>
+        <v>23860.63</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.7618</v>
+        <v>12.7312</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18746.85</v>
+        <v>18760.18</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18558.46</v>
+        <v>18571.65</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18652.66</v>
+        <v>18665.92</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.7618</v>
+        <v>12.7312</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15767.38</v>
+        <v>15778.59</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15711.09</v>
+        <v>15722.26</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15739.24</v>
+        <v>15750.43</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.7112</v>
+        <v>12.6696</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110249.84</v>
+        <v>110340.65</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110808.16</v>
+        <v>110899.44</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110529</v>
+        <v>110620.05</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.7112</v>
+        <v>12.6696</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79060.92999999999</v>
+        <v>79126.05</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79380.53</v>
+        <v>79445.92</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79220.73</v>
+        <v>79285.98</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.7112</v>
+        <v>12.6696</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51645.98</v>
+        <v>51688.52</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51207.35</v>
+        <v>51249.54</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51426.67</v>
+        <v>51469.03</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.7112</v>
+        <v>12.6696</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29692.92</v>
+        <v>29717.38</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29478.97</v>
+        <v>29503.26</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29585.95</v>
+        <v>29610.32</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.7112</v>
+        <v>12.6696</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16874.19</v>
+        <v>16888.09</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16807.51</v>
+        <v>16821.35</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16840.85</v>
+        <v>16854.72</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.7112</v>
+        <v>12.6696</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6841.42</v>
+        <v>6847.06</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6624.94</v>
+        <v>6630.39</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6733.18</v>
+        <v>6738.72</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.677</v>
+        <v>12.6241</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>359111.98</v>
+        <v>359456.03</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>354668.87</v>
+        <v>355008.67</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>356890.43</v>
+        <v>357232.35</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.677</v>
+        <v>12.6241</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>269595.96</v>
+        <v>269854.25</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>270470.31</v>
+        <v>270729.45</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270033.14</v>
+        <v>270291.85</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.677</v>
+        <v>12.6241</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>188637.12</v>
+        <v>188817.85</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>188523.32</v>
+        <v>188703.94</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>188580.22</v>
+        <v>188760.9</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.677</v>
+        <v>12.6241</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114680.39</v>
+        <v>114790.26</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>114933.16</v>
+        <v>115043.27</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>114806.77</v>
+        <v>114916.77</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.677</v>
+        <v>12.6241</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55587.07</v>
+        <v>55640.32</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55327.38</v>
+        <v>55380.39</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55457.23</v>
+        <v>55510.36</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.677</v>
+        <v>12.6241</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28389.23</v>
+        <v>28416.43</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28410.67</v>
+        <v>28437.89</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28399.95</v>
+        <v>28427.16</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5455</v>
+        <v>13.6278</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>409902.79</v>
+        <v>410083.55</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>410453.75</v>
+        <v>410634.76</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>410178.27</v>
+        <v>410359.16</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5455</v>
+        <v>13.6278</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>304266.48</v>
+        <v>304400.66</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>302366.67</v>
+        <v>302500.01</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>303316.58</v>
+        <v>303450.34</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5455</v>
+        <v>13.6278</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206384.23</v>
+        <v>206475.24</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206454.83</v>
+        <v>206545.88</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206419.53</v>
+        <v>206510.56</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5455</v>
+        <v>13.6278</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124890.27</v>
+        <v>124945.34</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125410.99</v>
+        <v>125466.29</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125150.63</v>
+        <v>125205.82</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5455</v>
+        <v>13.6278</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49875.61</v>
+        <v>49897.6</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49816.17</v>
+        <v>49838.14</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49845.89</v>
+        <v>49867.87</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5455</v>
+        <v>13.6278</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5486.15</v>
+        <v>5488.57</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5522.33</v>
+        <v>5524.77</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5504.24</v>
+        <v>5506.67</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4046</v>
+        <v>13.4751</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171207.99</v>
+        <v>171275.74</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171235.38</v>
+        <v>171303.13</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171221.68</v>
+        <v>171289.43</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4046</v>
+        <v>13.4751</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112512.08</v>
+        <v>112556.6</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112120.68</v>
+        <v>112165.04</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112316.38</v>
+        <v>112360.82</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4046</v>
+        <v>13.4751</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63011.73</v>
+        <v>63036.66</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63369.14</v>
+        <v>63394.21</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63190.43</v>
+        <v>63215.44</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4046</v>
+        <v>13.4751</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26975.93</v>
+        <v>26986.61</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27176.9</v>
+        <v>27187.66</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27076.42</v>
+        <v>27087.13</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4046</v>
+        <v>13.4751</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6349.85</v>
+        <v>6352.36</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6502.49</v>
+        <v>6505.06</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6426.17</v>
+        <v>6428.71</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4046</v>
+        <v>13.4751</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3760.71</v>
+        <v>3762.2</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3754.19</v>
+        <v>3755.67</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3757.45</v>
+        <v>3758.94</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.2666</v>
+        <v>13.3222</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191553.32</v>
+        <v>191623.77</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192488.65</v>
+        <v>192559.44</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192020.98</v>
+        <v>192091.61</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.2666</v>
+        <v>13.3222</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138880.21</v>
+        <v>138931.29</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139849.36</v>
+        <v>139900.8</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139364.78</v>
+        <v>139416.04</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.2666</v>
+        <v>13.3222</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87786.21000000001</v>
+        <v>87818.49000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88496.63</v>
+        <v>88529.17</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88141.42</v>
+        <v>88173.83</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.2666</v>
+        <v>13.3222</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41932.17</v>
+        <v>41947.59</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41864.92</v>
+        <v>41880.32</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41898.54</v>
+        <v>41913.95</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.2666</v>
+        <v>13.3222</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13075.86</v>
+        <v>13080.67</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12931.84</v>
+        <v>12936.59</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13003.85</v>
+        <v>13008.63</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.2666</v>
+        <v>13.3222</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4538.14</v>
+        <v>4539.81</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4427.36</v>
+        <v>4428.99</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4482.75</v>
+        <v>4484.4</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-08
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2053</v>
+        <v>13.2362</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151073.24</v>
+        <v>151133.55</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>152977.84</v>
+        <v>153038.91</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152025.54</v>
+        <v>152086.23</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2053</v>
+        <v>13.2362</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115636.74</v>
+        <v>115682.9</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116422.95</v>
+        <v>116469.43</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116029.85</v>
+        <v>116076.17</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2053</v>
+        <v>13.2362</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82451.7</v>
+        <v>82484.62</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82965.48</v>
+        <v>82998.60000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82708.59</v>
+        <v>82741.61</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2053</v>
+        <v>13.2362</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58425.25</v>
+        <v>58448.58</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57982.46</v>
+        <v>58005.61</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58203.86</v>
+        <v>58227.09</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2053</v>
+        <v>13.2362</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37740.4</v>
+        <v>37755.46</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38049.12</v>
+        <v>38064.31</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37894.76</v>
+        <v>37909.89</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2053</v>
+        <v>13.2362</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17165.04</v>
+        <v>17171.89</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17052.32</v>
+        <v>17059.13</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17108.68</v>
+        <v>17115.51</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.099</v>
+        <v>13.1252</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164215.24</v>
+        <v>164279.5</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163334.09</v>
+        <v>163398.01</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163774.67</v>
+        <v>163838.76</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.099</v>
+        <v>13.1252</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123326.15</v>
+        <v>123374.41</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121584.34</v>
+        <v>121631.92</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122455.24</v>
+        <v>122503.16</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.099</v>
+        <v>13.1252</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88108.87</v>
+        <v>88143.35000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87017.81</v>
+        <v>87051.87</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87563.34</v>
+        <v>87597.61</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.099</v>
+        <v>13.1252</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67116.87</v>
+        <v>67143.14</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66645.05</v>
+        <v>66671.13</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66880.96000000001</v>
+        <v>66907.13</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.099</v>
+        <v>13.1252</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52432.79</v>
+        <v>52453.31</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50548.4</v>
+        <v>50568.18</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51490.6</v>
+        <v>51510.75</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.099</v>
+        <v>13.1252</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39746.89</v>
+        <v>39762.45</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40729.06</v>
+        <v>40745</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40237.98</v>
+        <v>40253.72</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>12.9893</v>
+        <v>13.008</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169199.64</v>
+        <v>169267.46</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170758.26</v>
+        <v>170826.7</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>169978.95</v>
+        <v>170047.08</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>12.9893</v>
+        <v>13.008</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>121969.38</v>
+        <v>122018.27</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120511.58</v>
+        <v>120559.89</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121240.48</v>
+        <v>121289.08</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>12.9893</v>
+        <v>13.008</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83550.95</v>
+        <v>83584.44</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83235.37</v>
+        <v>83268.74000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83393.16</v>
+        <v>83426.59</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>12.9893</v>
+        <v>13.008</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55665.65</v>
+        <v>55687.96</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55972.8</v>
+        <v>55995.23</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55819.22</v>
+        <v>55841.6</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>12.9893</v>
+        <v>13.008</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33597.06</v>
+        <v>33610.53</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33203.82</v>
+        <v>33217.13</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33400.44</v>
+        <v>33413.83</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>12.9893</v>
+        <v>13.008</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17442.17</v>
+        <v>17449.16</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18133.66</v>
+        <v>18140.93</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17787.91</v>
+        <v>17795.04</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>12.9248</v>
+        <v>12.9393</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130851.65</v>
+        <v>130904.76</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>130947.53</v>
+        <v>131000.68</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130899.59</v>
+        <v>130952.72</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>12.9248</v>
+        <v>12.9393</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90621.62</v>
+        <v>90658.41</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89215.44</v>
+        <v>89251.64999999999</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89918.53</v>
+        <v>89955.03</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>12.9248</v>
+        <v>12.9393</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56960.78</v>
+        <v>56983.9</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57251.47</v>
+        <v>57274.71</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57106.12</v>
+        <v>57129.3</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>12.9248</v>
+        <v>12.9393</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30155.08</v>
+        <v>30167.32</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30358.05</v>
+        <v>30370.37</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30256.57</v>
+        <v>30268.85</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>12.9248</v>
+        <v>12.9393</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6916.31</v>
+        <v>6919.12</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6914.99</v>
+        <v>6917.8</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6915.65</v>
+        <v>6918.46</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>12.9248</v>
+        <v>12.9393</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3843.01</v>
+        <v>3844.57</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3752.37</v>
+        <v>3753.89</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3797.69</v>
+        <v>3799.23</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>12.8632</v>
+        <v>12.8737</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110563.34</v>
+        <v>110609.42</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111048.39</v>
+        <v>111094.66</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110805.86</v>
+        <v>110852.04</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>12.8632</v>
+        <v>12.8737</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77536.60000000001</v>
+        <v>77568.91</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76984.96000000001</v>
+        <v>77017.03999999999</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77260.78</v>
+        <v>77292.98</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>12.8632</v>
+        <v>12.8737</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46917.49</v>
+        <v>46937.05</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48039.23</v>
+        <v>48059.25</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47478.36</v>
+        <v>47498.15</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>12.8632</v>
+        <v>12.8737</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29147.91</v>
+        <v>29160.06</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29039.29</v>
+        <v>29051.39</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29093.6</v>
+        <v>29105.72</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>12.8632</v>
+        <v>12.8737</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14298.68</v>
+        <v>14304.64</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14422.65</v>
+        <v>14428.66</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14360.67</v>
+        <v>14366.65</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>12.8632</v>
+        <v>12.8737</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6628.88</v>
+        <v>6631.64</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6465.11</v>
+        <v>6467.81</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6546.99</v>
+        <v>6549.72</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.7986</v>
+        <v>12.8051</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50369.52</v>
+        <v>50391.4</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50032.3</v>
+        <v>50054.04</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50200.91</v>
+        <v>50222.72</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.7986</v>
+        <v>12.8051</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44311.73</v>
+        <v>44330.97</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44508.45</v>
+        <v>44527.78</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44410.09</v>
+        <v>44429.38</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.7986</v>
+        <v>12.8051</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32429.52</v>
+        <v>32443.6</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32774.88</v>
+        <v>32789.12</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32602.2</v>
+        <v>32616.36</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.7986</v>
+        <v>12.8051</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22802.12</v>
+        <v>22812.03</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22958.72</v>
+        <v>22968.69</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22880.42</v>
+        <v>22890.36</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.7986</v>
+        <v>12.8051</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14655.65</v>
+        <v>14662.02</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14864.21</v>
+        <v>14870.66</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14759.93</v>
+        <v>14766.34</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.7986</v>
+        <v>12.8051</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8422.610000000001</v>
+        <v>8426.27</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8478.42</v>
+        <v>8482.1</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8450.51</v>
+        <v>8454.18</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.7312</v>
+        <v>12.7333</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49610.25</v>
+        <v>49633.05</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48880.12</v>
+        <v>48902.58</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49245.18</v>
+        <v>49267.82</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.7312</v>
+        <v>12.7333</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44426.68</v>
+        <v>44447.1</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44085.4</v>
+        <v>44105.66</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44256.04</v>
+        <v>44276.38</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.7312</v>
+        <v>12.7333</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32084.97</v>
+        <v>32099.71</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31508.18</v>
+        <v>31522.67</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31796.58</v>
+        <v>31811.19</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.7312</v>
+        <v>12.7333</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23913.94</v>
+        <v>23924.93</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23807.32</v>
+        <v>23818.26</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23860.63</v>
+        <v>23871.6</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.7312</v>
+        <v>12.7333</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18760.18</v>
+        <v>18768.8</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18571.65</v>
+        <v>18580.19</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18665.92</v>
+        <v>18674.5</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.7312</v>
+        <v>12.7333</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15778.59</v>
+        <v>15785.85</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15722.26</v>
+        <v>15729.48</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15750.43</v>
+        <v>15757.66</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.6696</v>
+        <v>12.6677</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110340.65</v>
+        <v>110394.6</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110899.44</v>
+        <v>110953.66</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110620.05</v>
+        <v>110674.13</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.6696</v>
+        <v>12.6677</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79126.05</v>
+        <v>79164.74000000001</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79445.92</v>
+        <v>79484.75999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79285.98</v>
+        <v>79324.75</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.6696</v>
+        <v>12.6677</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51688.52</v>
+        <v>51713.79</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51249.54</v>
+        <v>51274.59</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51469.03</v>
+        <v>51494.19</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.6696</v>
+        <v>12.6677</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29717.38</v>
+        <v>29731.91</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29503.26</v>
+        <v>29517.68</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29610.32</v>
+        <v>29624.8</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.6696</v>
+        <v>12.6677</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16888.09</v>
+        <v>16896.34</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16821.35</v>
+        <v>16829.58</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16854.72</v>
+        <v>16862.96</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.6696</v>
+        <v>12.6677</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6847.06</v>
+        <v>6850.4</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6630.39</v>
+        <v>6633.63</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6738.72</v>
+        <v>6742.02</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.6241</v>
+        <v>12.6167</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>359456.03</v>
+        <v>359649.94</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355008.67</v>
+        <v>355200.18</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357232.35</v>
+        <v>357425.06</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.6241</v>
+        <v>12.6167</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>269854.25</v>
+        <v>269999.82</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>270729.45</v>
+        <v>270875.49</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270291.85</v>
+        <v>270437.65</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.6241</v>
+        <v>12.6167</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>188817.85</v>
+        <v>188919.7</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>188703.94</v>
+        <v>188805.73</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>188760.9</v>
+        <v>188862.72</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.6241</v>
+        <v>12.6167</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114790.26</v>
+        <v>114852.18</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115043.27</v>
+        <v>115105.33</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>114916.77</v>
+        <v>114978.76</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.6241</v>
+        <v>12.6167</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55640.32</v>
+        <v>55670.34</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55380.39</v>
+        <v>55410.27</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55510.36</v>
+        <v>55540.3</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.6241</v>
+        <v>12.6167</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28416.43</v>
+        <v>28431.76</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28437.89</v>
+        <v>28453.23</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28427.16</v>
+        <v>28442.5</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.6278</v>
+        <v>13.6764</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>410083.55</v>
+        <v>410276.88</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>410634.76</v>
+        <v>410828.34</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>410359.16</v>
+        <v>410552.61</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.6278</v>
+        <v>13.6764</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>304400.66</v>
+        <v>304544.16</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>302500.01</v>
+        <v>302642.62</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>303450.34</v>
+        <v>303593.39</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.6278</v>
+        <v>13.6764</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206475.24</v>
+        <v>206572.58</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206545.88</v>
+        <v>206643.25</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206510.56</v>
+        <v>206607.91</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.6278</v>
+        <v>13.6764</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>124945.34</v>
+        <v>125004.25</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125466.29</v>
+        <v>125525.44</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125205.82</v>
+        <v>125264.84</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.6278</v>
+        <v>13.6764</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49897.6</v>
+        <v>49921.12</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49838.14</v>
+        <v>49861.64</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49867.87</v>
+        <v>49891.38</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.6278</v>
+        <v>13.6764</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5488.57</v>
+        <v>5491.16</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5524.77</v>
+        <v>5527.37</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5506.67</v>
+        <v>5509.27</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4751</v>
+        <v>13.519</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171275.74</v>
+        <v>171350.9</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171303.13</v>
+        <v>171378.31</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171289.43</v>
+        <v>171364.6</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4751</v>
+        <v>13.519</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112556.6</v>
+        <v>112605.99</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112165.04</v>
+        <v>112214.26</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112360.82</v>
+        <v>112410.13</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4751</v>
+        <v>13.519</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63036.66</v>
+        <v>63064.33</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63394.21</v>
+        <v>63422.03</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63215.44</v>
+        <v>63243.18</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4751</v>
+        <v>13.519</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26986.61</v>
+        <v>26998.45</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27187.66</v>
+        <v>27199.59</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27087.13</v>
+        <v>27099.02</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4751</v>
+        <v>13.519</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6352.36</v>
+        <v>6355.15</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6505.06</v>
+        <v>6507.92</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6428.71</v>
+        <v>6431.53</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4751</v>
+        <v>13.519</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3762.2</v>
+        <v>3763.85</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3755.67</v>
+        <v>3757.32</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3758.94</v>
+        <v>3760.59</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3222</v>
+        <v>13.3583</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191623.77</v>
+        <v>191703.4</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192559.44</v>
+        <v>192639.46</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192091.61</v>
+        <v>192171.43</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3222</v>
+        <v>13.3583</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138931.29</v>
+        <v>138989.02</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139900.8</v>
+        <v>139958.93</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139416.04</v>
+        <v>139473.97</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3222</v>
+        <v>13.3583</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87818.49000000001</v>
+        <v>87854.98</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88529.17</v>
+        <v>88565.96000000001</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88173.83</v>
+        <v>88210.47</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3222</v>
+        <v>13.3583</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41947.59</v>
+        <v>41965.02</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41880.32</v>
+        <v>41897.72</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41913.95</v>
+        <v>41931.37</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3222</v>
+        <v>13.3583</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13080.67</v>
+        <v>13086.11</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12936.59</v>
+        <v>12941.97</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13008.63</v>
+        <v>13014.04</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3222</v>
+        <v>13.3583</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4539.81</v>
+        <v>4541.7</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4428.99</v>
+        <v>4430.83</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4484.4</v>
+        <v>4486.26</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-11
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2362</v>
+        <v>13.2337</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151133.55</v>
+        <v>151209.22</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153038.91</v>
+        <v>153115.53</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152086.23</v>
+        <v>152162.37</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2362</v>
+        <v>13.2337</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115682.9</v>
+        <v>115740.82</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116469.43</v>
+        <v>116527.75</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116076.17</v>
+        <v>116134.28</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2362</v>
+        <v>13.2337</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82484.62</v>
+        <v>82525.91</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82998.60000000001</v>
+        <v>83040.14999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82741.61</v>
+        <v>82783.03</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2362</v>
+        <v>13.2337</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58448.58</v>
+        <v>58477.84</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58005.61</v>
+        <v>58034.65</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58227.09</v>
+        <v>58256.24</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2362</v>
+        <v>13.2337</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37755.46</v>
+        <v>37774.37</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38064.31</v>
+        <v>38083.37</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37909.89</v>
+        <v>37928.87</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2362</v>
+        <v>13.2337</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17171.89</v>
+        <v>17180.49</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17059.13</v>
+        <v>17067.67</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17115.51</v>
+        <v>17124.08</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.1252</v>
+        <v>13.1236</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164279.5</v>
+        <v>164360.9</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163398.01</v>
+        <v>163478.97</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163838.76</v>
+        <v>163919.93</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.1252</v>
+        <v>13.1236</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123374.41</v>
+        <v>123435.54</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121631.92</v>
+        <v>121692.19</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122503.16</v>
+        <v>122563.86</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.1252</v>
+        <v>13.1236</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88143.35000000001</v>
+        <v>88187.02</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87051.87</v>
+        <v>87095</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87597.61</v>
+        <v>87641.00999999999</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.1252</v>
+        <v>13.1236</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67143.14</v>
+        <v>67176.39999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66671.13</v>
+        <v>66704.16</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66907.13</v>
+        <v>66940.28</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.1252</v>
+        <v>13.1236</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52453.31</v>
+        <v>52479.3</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50568.18</v>
+        <v>50593.24</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51510.75</v>
+        <v>51536.27</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.1252</v>
+        <v>13.1236</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39762.45</v>
+        <v>39782.15</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40745</v>
+        <v>40765.19</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40253.72</v>
+        <v>40273.67</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.008</v>
+        <v>13.0045</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169267.46</v>
+        <v>169352.24</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170826.7</v>
+        <v>170912.25</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170047.08</v>
+        <v>170132.25</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.008</v>
+        <v>13.0045</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122018.27</v>
+        <v>122079.38</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120559.89</v>
+        <v>120620.27</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121289.08</v>
+        <v>121349.82</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.008</v>
+        <v>13.0045</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83584.44</v>
+        <v>83626.3</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83268.74000000001</v>
+        <v>83310.44</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83426.59</v>
+        <v>83468.37</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.008</v>
+        <v>13.0045</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55687.96</v>
+        <v>55715.85</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55995.23</v>
+        <v>56023.28</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55841.6</v>
+        <v>55869.57</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.008</v>
+        <v>13.0045</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33610.53</v>
+        <v>33627.36</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33217.13</v>
+        <v>33233.76</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33413.83</v>
+        <v>33430.56</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.008</v>
+        <v>13.0045</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17449.16</v>
+        <v>17457.9</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18140.93</v>
+        <v>18150.01</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17795.04</v>
+        <v>17803.96</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>12.9393</v>
+        <v>12.9296</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130904.76</v>
+        <v>130974.6</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131000.68</v>
+        <v>131070.57</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>130952.72</v>
+        <v>131022.58</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>12.9393</v>
+        <v>12.9296</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90658.41</v>
+        <v>90706.77</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89251.64999999999</v>
+        <v>89299.25999999999</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>89955.03</v>
+        <v>90003.02</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>12.9393</v>
+        <v>12.9296</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56983.9</v>
+        <v>57014.3</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57274.71</v>
+        <v>57305.27</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57129.3</v>
+        <v>57159.78</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>12.9393</v>
+        <v>12.9296</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30167.32</v>
+        <v>30183.41</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30370.37</v>
+        <v>30386.58</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30268.85</v>
+        <v>30284.99</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>12.9393</v>
+        <v>12.9296</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6919.12</v>
+        <v>6922.81</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6917.8</v>
+        <v>6921.49</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6918.46</v>
+        <v>6922.15</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>12.9393</v>
+        <v>12.9296</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3844.57</v>
+        <v>3846.62</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3753.89</v>
+        <v>3755.89</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3799.23</v>
+        <v>3801.26</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>12.8737</v>
+        <v>12.8582</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110609.42</v>
+        <v>110672.86</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111094.66</v>
+        <v>111158.39</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110852.04</v>
+        <v>110915.63</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>12.8737</v>
+        <v>12.8582</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77568.91</v>
+        <v>77613.41</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77017.03999999999</v>
+        <v>77061.22</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77292.98</v>
+        <v>77337.31</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>12.8737</v>
+        <v>12.8582</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46937.05</v>
+        <v>46963.97</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48059.25</v>
+        <v>48086.82</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47498.15</v>
+        <v>47525.39</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>12.8737</v>
+        <v>12.8582</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29160.06</v>
+        <v>29176.79</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29051.39</v>
+        <v>29068.05</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29105.72</v>
+        <v>29122.42</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>12.8737</v>
+        <v>12.8582</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14304.64</v>
+        <v>14312.85</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14428.66</v>
+        <v>14436.94</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14366.65</v>
+        <v>14374.89</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>12.8737</v>
+        <v>12.8582</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6631.64</v>
+        <v>6635.44</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6467.81</v>
+        <v>6471.52</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6549.72</v>
+        <v>6553.48</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.8051</v>
+        <v>12.7833</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50391.4</v>
+        <v>50422.9</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50054.04</v>
+        <v>50085.32</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50222.72</v>
+        <v>50254.11</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.8051</v>
+        <v>12.7833</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44330.97</v>
+        <v>44358.68</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44527.78</v>
+        <v>44555.62</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44429.38</v>
+        <v>44457.15</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.8051</v>
+        <v>12.7833</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32443.6</v>
+        <v>32463.88</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32789.12</v>
+        <v>32809.61</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32616.36</v>
+        <v>32636.75</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.8051</v>
+        <v>12.7833</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22812.03</v>
+        <v>22826.29</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22968.69</v>
+        <v>22983.05</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22890.36</v>
+        <v>22904.67</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.8051</v>
+        <v>12.7833</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14662.02</v>
+        <v>14671.18</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14870.66</v>
+        <v>14879.96</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14766.34</v>
+        <v>14775.57</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.8051</v>
+        <v>12.7833</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8426.27</v>
+        <v>8431.540000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8482.1</v>
+        <v>8487.4</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8454.18</v>
+        <v>8459.469999999999</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.7333</v>
+        <v>12.7051</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49633.05</v>
+        <v>49667.26</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48902.58</v>
+        <v>48936.29</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49267.82</v>
+        <v>49301.77</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.7333</v>
+        <v>12.7051</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44447.1</v>
+        <v>44477.73</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44105.66</v>
+        <v>44136.06</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44276.38</v>
+        <v>44306.89</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.7333</v>
+        <v>12.7051</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32099.71</v>
+        <v>32121.84</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31522.67</v>
+        <v>31544.39</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31811.19</v>
+        <v>31833.11</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.7333</v>
+        <v>12.7051</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23924.93</v>
+        <v>23941.42</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23818.26</v>
+        <v>23834.68</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23871.6</v>
+        <v>23888.05</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.7333</v>
+        <v>12.7051</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18768.8</v>
+        <v>18781.74</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18580.19</v>
+        <v>18592.99</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18674.5</v>
+        <v>18687.37</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.7333</v>
+        <v>12.7051</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15785.85</v>
+        <v>15796.73</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15729.48</v>
+        <v>15740.32</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15757.66</v>
+        <v>15768.52</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.6677</v>
+        <v>12.6336</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110394.6</v>
+        <v>110478.16</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110953.66</v>
+        <v>111037.64</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110674.13</v>
+        <v>110757.9</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.6677</v>
+        <v>12.6336</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79164.74000000001</v>
+        <v>79224.66</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79484.75999999999</v>
+        <v>79544.92</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79324.75</v>
+        <v>79384.78999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.6677</v>
+        <v>12.6336</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51713.79</v>
+        <v>51752.94</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51274.59</v>
+        <v>51313.4</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51494.19</v>
+        <v>51533.17</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.6677</v>
+        <v>12.6336</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29731.91</v>
+        <v>29754.42</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29517.68</v>
+        <v>29540.02</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29624.8</v>
+        <v>29647.22</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.6677</v>
+        <v>12.6336</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16896.34</v>
+        <v>16909.13</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16829.58</v>
+        <v>16842.32</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16862.96</v>
+        <v>16875.73</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.6677</v>
+        <v>12.6336</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6850.4</v>
+        <v>6855.59</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6633.63</v>
+        <v>6638.65</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6742.02</v>
+        <v>6747.12</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.6167</v>
+        <v>12.5727</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>359649.94</v>
+        <v>359963.63</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355200.18</v>
+        <v>355509.99</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357425.06</v>
+        <v>357736.81</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.6167</v>
+        <v>12.5727</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>269999.82</v>
+        <v>270235.31</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>270875.49</v>
+        <v>271111.74</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270437.65</v>
+        <v>270673.53</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.6167</v>
+        <v>12.5727</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>188919.7</v>
+        <v>189084.48</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>188805.73</v>
+        <v>188970.41</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>188862.72</v>
+        <v>189027.45</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.6167</v>
+        <v>12.5727</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114852.18</v>
+        <v>114952.36</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115105.33</v>
+        <v>115205.73</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>114978.76</v>
+        <v>115079.04</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.6167</v>
+        <v>12.5727</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55670.34</v>
+        <v>55718.89</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55410.27</v>
+        <v>55458.59</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55540.3</v>
+        <v>55588.74</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.6167</v>
+        <v>12.5727</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28431.76</v>
+        <v>28456.56</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28453.23</v>
+        <v>28478.05</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28442.5</v>
+        <v>28467.3</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.6764</v>
+        <v>13.6532</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>410276.88</v>
+        <v>410492.28</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>410828.34</v>
+        <v>411044.03</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>410552.61</v>
+        <v>410768.15</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.6764</v>
+        <v>13.6532</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>304544.16</v>
+        <v>304704.05</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>302642.62</v>
+        <v>302801.51</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>303593.39</v>
+        <v>303752.78</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.6764</v>
+        <v>13.6532</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206572.58</v>
+        <v>206681.03</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206643.25</v>
+        <v>206751.74</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206607.91</v>
+        <v>206716.38</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.6764</v>
+        <v>13.6532</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125004.25</v>
+        <v>125069.87</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125525.44</v>
+        <v>125591.35</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125264.84</v>
+        <v>125330.61</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.6764</v>
+        <v>13.6532</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49921.12</v>
+        <v>49947.33</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49861.64</v>
+        <v>49887.82</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49891.38</v>
+        <v>49917.57</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.6764</v>
+        <v>13.6532</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5491.16</v>
+        <v>5494.04</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5527.37</v>
+        <v>5530.28</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5509.27</v>
+        <v>5512.16</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5114</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171350.9</v>
+        <v>171438.95</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171378.31</v>
+        <v>171466.37</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171364.6</v>
+        <v>171452.66</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5114</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112605.99</v>
+        <v>112663.86</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112214.26</v>
+        <v>112271.93</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112410.13</v>
+        <v>112467.89</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5114</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63064.33</v>
+        <v>63096.73</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63422.03</v>
+        <v>63454.62</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63243.18</v>
+        <v>63275.68</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5114</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26998.45</v>
+        <v>27012.32</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27199.59</v>
+        <v>27213.56</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27099.02</v>
+        <v>27112.94</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5114</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6355.15</v>
+        <v>6358.41</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6507.92</v>
+        <v>6511.26</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6431.53</v>
+        <v>6434.84</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5114</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3763.85</v>
+        <v>3765.79</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3757.32</v>
+        <v>3759.25</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3760.59</v>
+        <v>3762.52</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3583</v>
+        <v>13.3549</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191703.4</v>
+        <v>191800.22</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192639.46</v>
+        <v>192736.75</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192171.43</v>
+        <v>192268.49</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3583</v>
+        <v>13.3549</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>138989.02</v>
+        <v>139059.22</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>139958.93</v>
+        <v>140029.62</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139473.97</v>
+        <v>139544.42</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3583</v>
+        <v>13.3549</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87854.98</v>
+        <v>87899.36</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88565.96000000001</v>
+        <v>88610.69</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88210.47</v>
+        <v>88255.03</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3583</v>
+        <v>13.3549</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41965.02</v>
+        <v>41986.22</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41897.72</v>
+        <v>41918.88</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41931.37</v>
+        <v>41952.55</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3583</v>
+        <v>13.3549</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13086.11</v>
+        <v>13092.72</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12941.97</v>
+        <v>12948.51</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13014.04</v>
+        <v>13020.61</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3583</v>
+        <v>13.3549</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4541.7</v>
+        <v>4543.99</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4430.83</v>
+        <v>4433.07</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4486.26</v>
+        <v>4488.53</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-12
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2337</v>
+        <v>13.2392</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151209.22</v>
+        <v>151281.36</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153115.53</v>
+        <v>153188.58</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152162.37</v>
+        <v>152234.97</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2337</v>
+        <v>13.2392</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115740.82</v>
+        <v>115796.04</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116527.75</v>
+        <v>116583.34</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116134.28</v>
+        <v>116189.69</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2337</v>
+        <v>13.2392</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82525.91</v>
+        <v>82565.28999999999</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83040.14999999999</v>
+        <v>83079.77</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82783.03</v>
+        <v>82822.53</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2337</v>
+        <v>13.2392</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58477.84</v>
+        <v>58505.74</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58034.65</v>
+        <v>58062.33</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58256.24</v>
+        <v>58284.04</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2337</v>
+        <v>13.2392</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37774.37</v>
+        <v>37792.39</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38083.37</v>
+        <v>38101.54</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37928.87</v>
+        <v>37946.96</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2337</v>
+        <v>13.2392</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17180.49</v>
+        <v>17188.68</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17067.67</v>
+        <v>17075.81</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17124.08</v>
+        <v>17132.25</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.1236</v>
+        <v>13.1291</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164360.9</v>
+        <v>164438.04</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163478.97</v>
+        <v>163555.69</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163919.93</v>
+        <v>163996.87</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.1236</v>
+        <v>13.1291</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123435.54</v>
+        <v>123493.47</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121692.19</v>
+        <v>121749.3</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122563.86</v>
+        <v>122621.39</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.1236</v>
+        <v>13.1291</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88187.02</v>
+        <v>88228.41</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87095</v>
+        <v>87135.87</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87641.00999999999</v>
+        <v>87682.14</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.1236</v>
+        <v>13.1291</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67176.39999999999</v>
+        <v>67207.92999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66704.16</v>
+        <v>66735.47</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66940.28</v>
+        <v>66971.7</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.1236</v>
+        <v>13.1291</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52479.3</v>
+        <v>52503.93</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50593.24</v>
+        <v>50616.98</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51536.27</v>
+        <v>51560.46</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.1236</v>
+        <v>13.1291</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39782.15</v>
+        <v>39800.82</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40765.19</v>
+        <v>40784.32</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40273.67</v>
+        <v>40292.57</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.0045</v>
+        <v>13.0079</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169352.24</v>
+        <v>169431.87</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170912.25</v>
+        <v>170992.62</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170132.25</v>
+        <v>170212.24</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.0045</v>
+        <v>13.0079</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122079.38</v>
+        <v>122136.78</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120620.27</v>
+        <v>120676.98</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121349.82</v>
+        <v>121406.88</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.0045</v>
+        <v>13.0079</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83626.3</v>
+        <v>83665.62</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83310.44</v>
+        <v>83349.61</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83468.37</v>
+        <v>83507.62</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.0045</v>
+        <v>13.0079</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55715.85</v>
+        <v>55742.05</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56023.28</v>
+        <v>56049.62</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55869.57</v>
+        <v>55895.84</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.0045</v>
+        <v>13.0079</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33627.36</v>
+        <v>33643.17</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33233.76</v>
+        <v>33249.39</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33430.56</v>
+        <v>33446.28</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.0045</v>
+        <v>13.0079</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17457.9</v>
+        <v>17466.1</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18150.01</v>
+        <v>18158.55</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17803.96</v>
+        <v>17812.33</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>12.9296</v>
+        <v>12.933</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>130974.6</v>
+        <v>131035.49</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131070.57</v>
+        <v>131131.5</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131022.58</v>
+        <v>131083.5</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>12.9296</v>
+        <v>12.933</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90706.77</v>
+        <v>90748.94</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89299.25999999999</v>
+        <v>89340.78</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90003.02</v>
+        <v>90044.86</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>12.9296</v>
+        <v>12.933</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57014.3</v>
+        <v>57040.81</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57305.27</v>
+        <v>57331.91</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57159.78</v>
+        <v>57186.36</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>12.9296</v>
+        <v>12.933</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30183.41</v>
+        <v>30197.44</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30386.58</v>
+        <v>30400.7</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30284.99</v>
+        <v>30299.07</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>12.9296</v>
+        <v>12.933</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6922.81</v>
+        <v>6926.03</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6921.49</v>
+        <v>6924.71</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6922.15</v>
+        <v>6925.37</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>12.9296</v>
+        <v>12.933</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3846.62</v>
+        <v>3848.41</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3755.89</v>
+        <v>3757.64</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3801.26</v>
+        <v>3803.02</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>12.8582</v>
+        <v>12.8616</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110672.86</v>
+        <v>110723.76</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111158.39</v>
+        <v>111209.51</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110915.63</v>
+        <v>110966.64</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>12.8582</v>
+        <v>12.8616</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77613.41</v>
+        <v>77649.10000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77061.22</v>
+        <v>77096.66</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77337.31</v>
+        <v>77372.88</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>12.8582</v>
+        <v>12.8616</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46963.97</v>
+        <v>46985.57</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48086.82</v>
+        <v>48108.93</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47525.39</v>
+        <v>47547.25</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>12.8582</v>
+        <v>12.8616</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29176.79</v>
+        <v>29190.2</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29068.05</v>
+        <v>29081.42</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29122.42</v>
+        <v>29135.81</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>12.8582</v>
+        <v>12.8616</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14312.85</v>
+        <v>14319.43</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14436.94</v>
+        <v>14443.58</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14374.89</v>
+        <v>14381.5</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>12.8582</v>
+        <v>12.8616</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6635.44</v>
+        <v>6638.49</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6471.52</v>
+        <v>6474.49</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6553.48</v>
+        <v>6556.49</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.7833</v>
+        <v>12.7867</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50422.9</v>
+        <v>50445.82</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50085.32</v>
+        <v>50108.09</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50254.11</v>
+        <v>50276.96</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.7833</v>
+        <v>12.7867</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44358.68</v>
+        <v>44378.85</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44555.62</v>
+        <v>44575.87</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44457.15</v>
+        <v>44477.36</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.7833</v>
+        <v>12.7867</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32463.88</v>
+        <v>32478.64</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32809.61</v>
+        <v>32824.53</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32636.75</v>
+        <v>32651.59</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.7833</v>
+        <v>12.7867</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22826.29</v>
+        <v>22836.66</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22983.05</v>
+        <v>22993.5</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22904.67</v>
+        <v>22915.08</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.7833</v>
+        <v>12.7867</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14671.18</v>
+        <v>14677.85</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14879.96</v>
+        <v>14886.72</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14775.57</v>
+        <v>14782.29</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.7833</v>
+        <v>12.7867</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8431.540000000001</v>
+        <v>8435.370000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8487.4</v>
+        <v>8491.26</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8459.469999999999</v>
+        <v>8463.32</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.7051</v>
+        <v>12.7085</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49667.26</v>
+        <v>49689.57</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48936.29</v>
+        <v>48958.26</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49301.77</v>
+        <v>49323.91</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.7051</v>
+        <v>12.7085</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44477.73</v>
+        <v>44497.71</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44136.06</v>
+        <v>44155.88</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44306.89</v>
+        <v>44326.79</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.7051</v>
+        <v>12.7085</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32121.84</v>
+        <v>32136.26</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31544.39</v>
+        <v>31558.56</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31833.11</v>
+        <v>31847.41</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.7051</v>
+        <v>12.7085</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23941.42</v>
+        <v>23952.17</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23834.68</v>
+        <v>23845.38</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23888.05</v>
+        <v>23898.78</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.7051</v>
+        <v>12.7085</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18781.74</v>
+        <v>18790.17</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18592.99</v>
+        <v>18601.34</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18687.37</v>
+        <v>18695.76</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.7051</v>
+        <v>12.7085</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15796.73</v>
+        <v>15803.82</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15740.32</v>
+        <v>15747.39</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15768.52</v>
+        <v>15775.61</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.6336</v>
+        <v>12.637</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110478.16</v>
+        <v>110527.21</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111037.64</v>
+        <v>111086.95</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110757.9</v>
+        <v>110807.08</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.6336</v>
+        <v>12.637</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79224.66</v>
+        <v>79259.84</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79544.92</v>
+        <v>79580.24000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79384.78999999999</v>
+        <v>79420.03999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.6336</v>
+        <v>12.637</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51752.94</v>
+        <v>51775.92</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51313.4</v>
+        <v>51336.19</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51533.17</v>
+        <v>51556.05</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.6336</v>
+        <v>12.637</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29754.42</v>
+        <v>29767.63</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29540.02</v>
+        <v>29553.14</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29647.22</v>
+        <v>29660.38</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.6336</v>
+        <v>12.637</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16909.13</v>
+        <v>16916.64</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16842.32</v>
+        <v>16849.79</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16875.73</v>
+        <v>16883.22</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.6336</v>
+        <v>12.637</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6855.59</v>
+        <v>6858.63</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6638.65</v>
+        <v>6641.6</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6747.12</v>
+        <v>6750.12</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.5727</v>
+        <v>12.5738</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>359963.63</v>
+        <v>360129.29</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355509.99</v>
+        <v>355673.6</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357736.81</v>
+        <v>357901.45</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.5727</v>
+        <v>12.5738</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270235.31</v>
+        <v>270359.68</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271111.74</v>
+        <v>271236.52</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270673.53</v>
+        <v>270798.1</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.5727</v>
+        <v>12.5738</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189084.48</v>
+        <v>189171.5</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>188970.41</v>
+        <v>189057.38</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189027.45</v>
+        <v>189114.44</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.5727</v>
+        <v>12.5738</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114952.36</v>
+        <v>115005.26</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115205.73</v>
+        <v>115258.75</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115079.04</v>
+        <v>115132</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.5727</v>
+        <v>12.5738</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55718.89</v>
+        <v>55744.54</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55458.59</v>
+        <v>55484.12</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55588.74</v>
+        <v>55614.33</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.5727</v>
+        <v>12.5738</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28456.56</v>
+        <v>28469.66</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28478.05</v>
+        <v>28491.16</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28467.3</v>
+        <v>28480.41</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>410492.28</v>
+        <v>410700.81</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>411044.03</v>
+        <v>411252.84</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>410768.15</v>
+        <v>410976.82</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>304704.05</v>
+        <v>304858.84</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>302801.51</v>
+        <v>302955.33</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>303752.78</v>
+        <v>303907.08</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206681.03</v>
+        <v>206786.02</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206751.74</v>
+        <v>206856.76</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206716.38</v>
+        <v>206821.39</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125069.87</v>
+        <v>125133.41</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125591.35</v>
+        <v>125655.14</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125330.61</v>
+        <v>125394.28</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49947.33</v>
+        <v>49972.71</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49887.82</v>
+        <v>49913.16</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49917.57</v>
+        <v>49942.93</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5494.04</v>
+        <v>5496.84</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5530.28</v>
+        <v>5533.08</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5512.16</v>
+        <v>5514.96</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5114</v>
+        <v>13.5189</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171438.95</v>
+        <v>171523.45</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171466.37</v>
+        <v>171550.88</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171452.66</v>
+        <v>171537.16</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5114</v>
+        <v>13.5189</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112663.86</v>
+        <v>112719.38</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112271.93</v>
+        <v>112327.26</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112467.89</v>
+        <v>112523.32</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5114</v>
+        <v>13.5189</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63096.73</v>
+        <v>63127.83</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63454.62</v>
+        <v>63485.9</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63275.68</v>
+        <v>63306.86</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5114</v>
+        <v>13.5189</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27012.32</v>
+        <v>27025.64</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27213.56</v>
+        <v>27226.98</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27112.94</v>
+        <v>27126.31</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5114</v>
+        <v>13.5189</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6358.41</v>
+        <v>6361.55</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6511.26</v>
+        <v>6514.47</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6434.84</v>
+        <v>6438.01</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5114</v>
+        <v>13.5189</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3765.79</v>
+        <v>3767.64</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3759.25</v>
+        <v>3761.11</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3762.52</v>
+        <v>3764.37</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3549</v>
+        <v>13.3616</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191800.22</v>
+        <v>191892.84</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192736.75</v>
+        <v>192829.83</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192268.49</v>
+        <v>192361.34</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3549</v>
+        <v>13.3616</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139059.22</v>
+        <v>139126.37</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140029.62</v>
+        <v>140097.24</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139544.42</v>
+        <v>139611.81</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3549</v>
+        <v>13.3616</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87899.36</v>
+        <v>87941.8</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88610.69</v>
+        <v>88653.48</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88255.03</v>
+        <v>88297.64</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3549</v>
+        <v>13.3616</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41986.22</v>
+        <v>42006.49</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41918.88</v>
+        <v>41939.13</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41952.55</v>
+        <v>41972.81</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3549</v>
+        <v>13.3616</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13092.72</v>
+        <v>13099.04</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12948.51</v>
+        <v>12954.76</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13020.61</v>
+        <v>13026.9</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3549</v>
+        <v>13.3616</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4543.99</v>
+        <v>4546.19</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4433.07</v>
+        <v>4435.21</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4488.53</v>
+        <v>4490.7</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-13
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2392</v>
+        <v>13.2447</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151281.36</v>
+        <v>151353.59</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153188.58</v>
+        <v>153261.73</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152234.97</v>
+        <v>152307.66</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2392</v>
+        <v>13.2447</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115796.04</v>
+        <v>115851.33</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116583.34</v>
+        <v>116639.01</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116189.69</v>
+        <v>116245.17</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2392</v>
+        <v>13.2447</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82565.28999999999</v>
+        <v>82604.71000000001</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83079.77</v>
+        <v>83119.44</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82822.53</v>
+        <v>82862.08</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2392</v>
+        <v>13.2447</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58505.74</v>
+        <v>58533.68</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58062.33</v>
+        <v>58090.06</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58284.04</v>
+        <v>58311.87</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2392</v>
+        <v>13.2447</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37792.39</v>
+        <v>37810.43</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38101.54</v>
+        <v>38119.73</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37946.96</v>
+        <v>37965.08</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2392</v>
+        <v>13.2447</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17188.68</v>
+        <v>17196.89</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17075.81</v>
+        <v>17083.96</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17132.25</v>
+        <v>17140.43</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.1291</v>
+        <v>13.1346</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164438.04</v>
+        <v>164515.28</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163555.69</v>
+        <v>163632.52</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>163996.87</v>
+        <v>164073.9</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.1291</v>
+        <v>13.1346</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123493.47</v>
+        <v>123551.48</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121749.3</v>
+        <v>121806.49</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122621.39</v>
+        <v>122678.98</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.1291</v>
+        <v>13.1346</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88228.41</v>
+        <v>88269.85000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87135.87</v>
+        <v>87176.8</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87682.14</v>
+        <v>87723.33</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.1291</v>
+        <v>13.1346</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67207.92999999999</v>
+        <v>67239.5</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66735.47</v>
+        <v>66766.82000000001</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66971.7</v>
+        <v>67003.16</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.1291</v>
+        <v>13.1346</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52503.93</v>
+        <v>52528.59</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50616.98</v>
+        <v>50640.76</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51560.46</v>
+        <v>51584.68</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.1291</v>
+        <v>13.1346</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39800.82</v>
+        <v>39819.52</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40784.32</v>
+        <v>40803.48</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40292.57</v>
+        <v>40311.5</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.0079</v>
+        <v>13.0134</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169431.87</v>
+        <v>169510.01</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>170992.62</v>
+        <v>171071.48</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170212.24</v>
+        <v>170290.75</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.0079</v>
+        <v>13.0134</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122136.78</v>
+        <v>122193.11</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120676.98</v>
+        <v>120732.64</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121406.88</v>
+        <v>121462.87</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.0079</v>
+        <v>13.0134</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83665.62</v>
+        <v>83704.21000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83349.61</v>
+        <v>83388.05</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83507.62</v>
+        <v>83546.13</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.0079</v>
+        <v>13.0134</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55742.05</v>
+        <v>55767.76</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56049.62</v>
+        <v>56075.47</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55895.84</v>
+        <v>55921.61</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.0079</v>
+        <v>13.0134</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33643.17</v>
+        <v>33658.69</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33249.39</v>
+        <v>33264.73</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33446.28</v>
+        <v>33461.71</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.0079</v>
+        <v>13.0134</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17466.1</v>
+        <v>17474.16</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18158.55</v>
+        <v>18166.92</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17812.33</v>
+        <v>17820.54</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>12.933</v>
+        <v>12.9364</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131035.49</v>
+        <v>131096.45</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131131.5</v>
+        <v>131192.5</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131083.5</v>
+        <v>131144.47</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>12.933</v>
+        <v>12.9364</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90748.94</v>
+        <v>90791.16</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89340.78</v>
+        <v>89382.34</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90044.86</v>
+        <v>90086.75</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>12.933</v>
+        <v>12.9364</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57040.81</v>
+        <v>57067.34</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57331.91</v>
+        <v>57358.58</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57186.36</v>
+        <v>57212.96</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>12.933</v>
+        <v>12.9364</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30197.44</v>
+        <v>30211.49</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30400.7</v>
+        <v>30414.85</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30299.07</v>
+        <v>30313.17</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>12.933</v>
+        <v>12.9364</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6926.03</v>
+        <v>6929.25</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6924.71</v>
+        <v>6927.93</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6925.37</v>
+        <v>6928.59</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>12.933</v>
+        <v>12.9364</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3848.41</v>
+        <v>3850.2</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3757.64</v>
+        <v>3759.39</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3803.02</v>
+        <v>3804.79</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>12.8616</v>
+        <v>12.865</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110723.76</v>
+        <v>110774.71</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111209.51</v>
+        <v>111260.68</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110966.64</v>
+        <v>111017.7</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>12.8616</v>
+        <v>12.865</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77649.10000000001</v>
+        <v>77684.83</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77096.66</v>
+        <v>77132.13</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77372.88</v>
+        <v>77408.48</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>12.8616</v>
+        <v>12.865</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46985.57</v>
+        <v>47007.19</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48108.93</v>
+        <v>48131.07</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47547.25</v>
+        <v>47569.13</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>12.8616</v>
+        <v>12.865</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29190.2</v>
+        <v>29203.64</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29081.42</v>
+        <v>29094.8</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29135.81</v>
+        <v>29149.22</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>12.8616</v>
+        <v>12.865</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14319.43</v>
+        <v>14326.02</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14443.58</v>
+        <v>14450.22</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14381.5</v>
+        <v>14388.12</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>12.8616</v>
+        <v>12.865</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6638.49</v>
+        <v>6641.55</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6474.49</v>
+        <v>6477.47</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6556.49</v>
+        <v>6559.51</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.7867</v>
+        <v>12.7901</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50445.82</v>
+        <v>50468.76</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50108.09</v>
+        <v>50130.88</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50276.96</v>
+        <v>50299.82</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.7867</v>
+        <v>12.7901</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44378.85</v>
+        <v>44399.03</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44575.87</v>
+        <v>44596.15</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44477.36</v>
+        <v>44497.59</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.7867</v>
+        <v>12.7901</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32478.64</v>
+        <v>32493.42</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32824.53</v>
+        <v>32839.46</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32651.59</v>
+        <v>32666.44</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.7867</v>
+        <v>12.7901</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22836.66</v>
+        <v>22847.05</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22993.5</v>
+        <v>23003.96</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22915.08</v>
+        <v>22925.5</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.7867</v>
+        <v>12.7901</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14677.85</v>
+        <v>14684.53</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14886.72</v>
+        <v>14893.49</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14782.29</v>
+        <v>14789.01</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.7867</v>
+        <v>12.7901</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8435.370000000001</v>
+        <v>8439.209999999999</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8491.26</v>
+        <v>8495.120000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8463.32</v>
+        <v>8467.16</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.7085</v>
+        <v>12.7119</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49689.57</v>
+        <v>49711.89</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48958.26</v>
+        <v>48980.26</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49323.91</v>
+        <v>49346.08</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.7085</v>
+        <v>12.7119</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44497.71</v>
+        <v>44517.7</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44155.88</v>
+        <v>44175.72</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44326.79</v>
+        <v>44346.71</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.7085</v>
+        <v>12.7119</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32136.26</v>
+        <v>32150.7</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31558.56</v>
+        <v>31572.74</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31847.41</v>
+        <v>31861.72</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.7085</v>
+        <v>12.7119</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23952.17</v>
+        <v>23962.94</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23845.38</v>
+        <v>23856.1</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23898.78</v>
+        <v>23909.52</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.7085</v>
+        <v>12.7119</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18790.17</v>
+        <v>18798.62</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18601.34</v>
+        <v>18609.7</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18695.76</v>
+        <v>18704.16</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.7085</v>
+        <v>12.7119</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15803.82</v>
+        <v>15810.92</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15747.39</v>
+        <v>15754.47</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15775.61</v>
+        <v>15782.69</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.637</v>
+        <v>12.6404</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110527.21</v>
+        <v>110576.32</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111086.95</v>
+        <v>111136.3</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110807.08</v>
+        <v>110856.31</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.637</v>
+        <v>12.6404</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79259.84</v>
+        <v>79295.05</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79580.24000000001</v>
+        <v>79615.60000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79420.03999999999</v>
+        <v>79455.32000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.637</v>
+        <v>12.6404</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51775.92</v>
+        <v>51798.92</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51336.19</v>
+        <v>51358.99</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51556.05</v>
+        <v>51578.96</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.637</v>
+        <v>12.6404</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29767.63</v>
+        <v>29780.85</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29553.14</v>
+        <v>29566.27</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29660.38</v>
+        <v>29673.56</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.637</v>
+        <v>12.6404</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16916.64</v>
+        <v>16924.16</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16849.79</v>
+        <v>16857.28</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16883.22</v>
+        <v>16890.72</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.637</v>
+        <v>12.6404</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6858.63</v>
+        <v>6861.68</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6641.6</v>
+        <v>6644.55</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6750.12</v>
+        <v>6753.12</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.5738</v>
+        <v>12.5749</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360129.29</v>
+        <v>360295.06</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355673.6</v>
+        <v>355837.32</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357901.45</v>
+        <v>358066.19</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.5738</v>
+        <v>12.5749</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270359.68</v>
+        <v>270484.13</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271236.52</v>
+        <v>271361.37</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270798.1</v>
+        <v>270922.75</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.5738</v>
+        <v>12.5749</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189171.5</v>
+        <v>189258.58</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189057.38</v>
+        <v>189144.4</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189114.44</v>
+        <v>189201.49</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.5738</v>
+        <v>12.5749</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>115005.26</v>
+        <v>115058.2</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115258.75</v>
+        <v>115311.8</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115132</v>
+        <v>115185</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.5738</v>
+        <v>12.5749</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55744.54</v>
+        <v>55770.2</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55484.12</v>
+        <v>55509.66</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55614.33</v>
+        <v>55639.93</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.5738</v>
+        <v>12.5749</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28469.66</v>
+        <v>28482.76</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28491.16</v>
+        <v>28504.27</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28480.41</v>
+        <v>28493.52</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>410700.81</v>
+        <v>410909.44</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>411252.84</v>
+        <v>411461.75</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>410976.82</v>
+        <v>411185.59</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>304858.84</v>
+        <v>305013.7</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>302955.33</v>
+        <v>303109.23</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>303907.08</v>
+        <v>304061.47</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206786.02</v>
+        <v>206891.07</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206856.76</v>
+        <v>206961.85</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206821.39</v>
+        <v>206926.46</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125133.41</v>
+        <v>125196.98</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125655.14</v>
+        <v>125718.98</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125394.28</v>
+        <v>125457.98</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49972.71</v>
+        <v>49998.09</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49913.16</v>
+        <v>49938.51</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49942.93</v>
+        <v>49968.3</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5496.84</v>
+        <v>5499.63</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5533.08</v>
+        <v>5535.9</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5514.96</v>
+        <v>5517.76</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5189</v>
+        <v>13.5263</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171523.45</v>
+        <v>171608.07</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171550.88</v>
+        <v>171635.52</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171537.16</v>
+        <v>171621.8</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5189</v>
+        <v>13.5263</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112719.38</v>
+        <v>112775</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112327.26</v>
+        <v>112382.68</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112523.32</v>
+        <v>112578.84</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5189</v>
+        <v>13.5263</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63127.83</v>
+        <v>63158.98</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63485.9</v>
+        <v>63517.22</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63306.86</v>
+        <v>63338.1</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5189</v>
+        <v>13.5263</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27025.64</v>
+        <v>27038.97</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27226.98</v>
+        <v>27240.41</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27126.31</v>
+        <v>27139.69</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5189</v>
+        <v>13.5263</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6361.55</v>
+        <v>6364.69</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6514.47</v>
+        <v>6517.68</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6438.01</v>
+        <v>6441.19</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5189</v>
+        <v>13.5263</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3767.64</v>
+        <v>3769.5</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3761.11</v>
+        <v>3762.96</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3764.37</v>
+        <v>3766.23</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.3684</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191892.84</v>
+        <v>191985.6</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192829.83</v>
+        <v>192923.04</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192361.34</v>
+        <v>192454.32</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.3684</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139126.37</v>
+        <v>139193.62</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140097.24</v>
+        <v>140164.96</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139611.81</v>
+        <v>139679.29</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.3684</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87941.8</v>
+        <v>87984.32000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88653.48</v>
+        <v>88696.34</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88297.64</v>
+        <v>88340.33</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.3684</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42006.49</v>
+        <v>42026.8</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41939.13</v>
+        <v>41959.4</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41972.81</v>
+        <v>41993.1</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.3684</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13099.04</v>
+        <v>13105.37</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12954.76</v>
+        <v>12961.02</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13026.9</v>
+        <v>13033.2</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3616</v>
+        <v>13.3684</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4546.19</v>
+        <v>4548.38</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4435.21</v>
+        <v>4437.35</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4490.7</v>
+        <v>4492.87</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-14
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2447</v>
+        <v>13.2956</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151353.59</v>
+        <v>151406.17</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153261.73</v>
+        <v>153314.97</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152307.66</v>
+        <v>152360.57</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2447</v>
+        <v>13.2956</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115851.33</v>
+        <v>115891.58</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116639.01</v>
+        <v>116679.53</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116245.17</v>
+        <v>116285.55</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2447</v>
+        <v>13.2956</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82604.71000000001</v>
+        <v>82633.41</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83119.44</v>
+        <v>83148.32000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82862.08</v>
+        <v>82890.86</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2447</v>
+        <v>13.2956</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58533.68</v>
+        <v>58554.01</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58090.06</v>
+        <v>58110.24</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58311.87</v>
+        <v>58332.13</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2447</v>
+        <v>13.2956</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37810.43</v>
+        <v>37823.57</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38119.73</v>
+        <v>38132.98</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37965.08</v>
+        <v>37978.27</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2447</v>
+        <v>13.2956</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17196.89</v>
+        <v>17202.86</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17083.96</v>
+        <v>17089.9</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17140.43</v>
+        <v>17146.38</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.1346</v>
+        <v>13.2016</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164515.28</v>
+        <v>164556.43</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163632.52</v>
+        <v>163673.45</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164073.9</v>
+        <v>164114.94</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.1346</v>
+        <v>13.2016</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123551.48</v>
+        <v>123582.38</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121806.49</v>
+        <v>121836.96</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122678.98</v>
+        <v>122709.67</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.1346</v>
+        <v>13.2016</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88269.85000000001</v>
+        <v>88291.92999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87176.8</v>
+        <v>87198.61</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87723.33</v>
+        <v>87745.27</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.1346</v>
+        <v>13.2016</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67239.5</v>
+        <v>67256.32000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66766.82000000001</v>
+        <v>66783.52</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67003.16</v>
+        <v>67019.92</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.1346</v>
+        <v>13.2016</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52528.59</v>
+        <v>52541.73</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50640.76</v>
+        <v>50653.43</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51584.68</v>
+        <v>51597.58</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.1346</v>
+        <v>13.2016</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39819.52</v>
+        <v>39829.48</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40803.48</v>
+        <v>40813.68</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40311.5</v>
+        <v>40321.58</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.0134</v>
+        <v>13.0981</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169510.01</v>
+        <v>169529.81</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171071.48</v>
+        <v>171091.47</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170290.75</v>
+        <v>170310.64</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.0134</v>
+        <v>13.0981</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122193.11</v>
+        <v>122207.38</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120732.64</v>
+        <v>120746.74</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121462.87</v>
+        <v>121477.06</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.0134</v>
+        <v>13.0981</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83704.21000000001</v>
+        <v>83713.99000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83388.05</v>
+        <v>83397.8</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83546.13</v>
+        <v>83555.89</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.0134</v>
+        <v>13.0981</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55767.76</v>
+        <v>55774.28</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56075.47</v>
+        <v>56082.02</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55921.61</v>
+        <v>55928.15</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.0134</v>
+        <v>13.0981</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33658.69</v>
+        <v>33662.62</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33264.73</v>
+        <v>33268.61</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33461.71</v>
+        <v>33465.62</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.0134</v>
+        <v>13.0981</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17474.16</v>
+        <v>17476.2</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18166.92</v>
+        <v>18169.05</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17820.54</v>
+        <v>17822.62</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>12.9364</v>
+        <v>13.0317</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131096.45</v>
+        <v>131095.72</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131192.5</v>
+        <v>131191.78</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131144.47</v>
+        <v>131143.75</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>12.9364</v>
+        <v>13.0317</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90791.16</v>
+        <v>90790.66</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89382.34</v>
+        <v>89381.85000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90086.75</v>
+        <v>90086.25</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>12.9364</v>
+        <v>13.0317</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57067.34</v>
+        <v>57067.03</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57358.58</v>
+        <v>57358.26</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57212.96</v>
+        <v>57212.64</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>12.9364</v>
+        <v>13.0317</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30211.49</v>
+        <v>30211.33</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30414.85</v>
+        <v>30414.68</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30313.17</v>
+        <v>30313</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>12.9364</v>
+        <v>13.0317</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6929.25</v>
+        <v>6929.21</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6927.93</v>
+        <v>6927.89</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6928.59</v>
+        <v>6928.55</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>12.9364</v>
+        <v>13.0317</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3850.2</v>
+        <v>3850.18</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3759.39</v>
+        <v>3759.37</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3804.79</v>
+        <v>3804.77</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>12.865</v>
+        <v>12.9718</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110774.71</v>
+        <v>110758.49</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111260.68</v>
+        <v>111244.39</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111017.7</v>
+        <v>111001.44</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>12.865</v>
+        <v>12.9718</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77684.83</v>
+        <v>77673.45</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77132.13</v>
+        <v>77120.84</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77408.48</v>
+        <v>77397.14999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>12.865</v>
+        <v>12.9718</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47007.19</v>
+        <v>47000.3</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48131.07</v>
+        <v>48124.02</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47569.13</v>
+        <v>47562.16</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>12.865</v>
+        <v>12.9718</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29203.64</v>
+        <v>29199.36</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29094.8</v>
+        <v>29090.54</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29149.22</v>
+        <v>29144.95</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>12.865</v>
+        <v>12.9718</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14326.02</v>
+        <v>14323.92</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14450.22</v>
+        <v>14448.11</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14388.12</v>
+        <v>14386.01</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>12.865</v>
+        <v>12.9718</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6641.55</v>
+        <v>6640.58</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6477.47</v>
+        <v>6476.52</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6559.51</v>
+        <v>6558.55</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.7901</v>
+        <v>12.9091</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50468.76</v>
+        <v>50452.99</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50130.88</v>
+        <v>50115.21</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50299.82</v>
+        <v>50284.1</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.7901</v>
+        <v>12.9091</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44399.03</v>
+        <v>44385.16</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44596.15</v>
+        <v>44582.21</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44497.59</v>
+        <v>44483.68</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.7901</v>
+        <v>12.9091</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32493.42</v>
+        <v>32483.26</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32839.46</v>
+        <v>32829.19</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32666.44</v>
+        <v>32656.23</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.7901</v>
+        <v>12.9091</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22847.05</v>
+        <v>22839.91</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>23003.96</v>
+        <v>22996.77</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22925.5</v>
+        <v>22918.34</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.7901</v>
+        <v>12.9091</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14684.53</v>
+        <v>14679.94</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14893.49</v>
+        <v>14888.84</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14789.01</v>
+        <v>14784.39</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.7901</v>
+        <v>12.9091</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8439.209999999999</v>
+        <v>8436.57</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8495.120000000001</v>
+        <v>8492.469999999999</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8467.16</v>
+        <v>8464.52</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.7119</v>
+        <v>12.8435</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49711.89</v>
+        <v>49686.71</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48980.26</v>
+        <v>48955.45</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49346.08</v>
+        <v>49321.08</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.7119</v>
+        <v>12.8435</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44517.7</v>
+        <v>44495.15</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44175.72</v>
+        <v>44153.34</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44346.71</v>
+        <v>44324.25</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.7119</v>
+        <v>12.8435</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32150.7</v>
+        <v>32134.42</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31572.74</v>
+        <v>31556.75</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31861.72</v>
+        <v>31845.58</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.7119</v>
+        <v>12.8435</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23962.94</v>
+        <v>23950.8</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23856.1</v>
+        <v>23844.01</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23909.52</v>
+        <v>23897.41</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.7119</v>
+        <v>12.8435</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18798.62</v>
+        <v>18789.1</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18609.7</v>
+        <v>18600.28</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18704.16</v>
+        <v>18694.69</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.7119</v>
+        <v>12.8435</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15810.92</v>
+        <v>15802.91</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15754.47</v>
+        <v>15746.49</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15782.69</v>
+        <v>15774.7</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.6404</v>
+        <v>12.7836</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110576.32</v>
+        <v>110498.74</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111136.3</v>
+        <v>111058.33</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110856.31</v>
+        <v>110778.53</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.6404</v>
+        <v>12.7836</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79295.05</v>
+        <v>79239.42</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79615.60000000001</v>
+        <v>79559.74000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79455.32000000001</v>
+        <v>79399.58</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.6404</v>
+        <v>12.7836</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51798.92</v>
+        <v>51762.58</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51358.99</v>
+        <v>51322.96</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51578.96</v>
+        <v>51542.77</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.6404</v>
+        <v>12.7836</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29780.85</v>
+        <v>29759.96</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29566.27</v>
+        <v>29545.53</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29673.56</v>
+        <v>29652.74</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.6404</v>
+        <v>12.7836</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16924.16</v>
+        <v>16912.28</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16857.28</v>
+        <v>16845.45</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16890.72</v>
+        <v>16878.87</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.6404</v>
+        <v>12.7836</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6861.68</v>
+        <v>6856.87</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6644.55</v>
+        <v>6639.89</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6753.12</v>
+        <v>6748.38</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.5749</v>
+        <v>12.727</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360295.06</v>
+        <v>359972.31</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355837.32</v>
+        <v>355518.56</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>358066.19</v>
+        <v>357745.44</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.5749</v>
+        <v>12.727</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270484.13</v>
+        <v>270241.83</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271361.37</v>
+        <v>271118.29</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270922.75</v>
+        <v>270680.06</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.5749</v>
+        <v>12.727</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189258.58</v>
+        <v>189089.04</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189144.4</v>
+        <v>188974.97</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189201.49</v>
+        <v>189032.01</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.5749</v>
+        <v>12.727</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>115058.2</v>
+        <v>114955.13</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115311.8</v>
+        <v>115208.51</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115185</v>
+        <v>115081.82</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.5749</v>
+        <v>12.727</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55770.2</v>
+        <v>55720.24</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55509.66</v>
+        <v>55459.93</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55639.93</v>
+        <v>55590.09</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.5749</v>
+        <v>12.727</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28482.76</v>
+        <v>28457.25</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28504.27</v>
+        <v>28478.74</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28493.52</v>
+        <v>28467.99</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.6532</v>
+        <v>13.6415</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>410909.44</v>
+        <v>411121.03</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>411461.75</v>
+        <v>411673.63</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>411185.59</v>
+        <v>411397.33</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.6532</v>
+        <v>13.6415</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>305013.7</v>
+        <v>305170.77</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>303109.23</v>
+        <v>303265.31</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>304061.47</v>
+        <v>304218.04</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.6532</v>
+        <v>13.6415</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206891.07</v>
+        <v>206997.61</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>206961.85</v>
+        <v>207068.42</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>206926.46</v>
+        <v>207033.01</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.6532</v>
+        <v>13.6415</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125196.98</v>
+        <v>125261.44</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125718.98</v>
+        <v>125783.71</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125457.98</v>
+        <v>125522.58</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.6532</v>
+        <v>13.6415</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49998.09</v>
+        <v>50023.84</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49938.51</v>
+        <v>49964.23</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49968.3</v>
+        <v>49994.03</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.6532</v>
+        <v>13.6415</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5499.63</v>
+        <v>5502.46</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5535.9</v>
+        <v>5538.75</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5517.76</v>
+        <v>5520.6</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5263</v>
+        <v>13.5388</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171608.07</v>
+        <v>171691.72</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171635.52</v>
+        <v>171719.18</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171621.8</v>
+        <v>171705.45</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5263</v>
+        <v>13.5388</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112775</v>
+        <v>112829.97</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112382.68</v>
+        <v>112437.46</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112578.84</v>
+        <v>112633.72</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5263</v>
+        <v>13.5388</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63158.98</v>
+        <v>63189.76</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63517.22</v>
+        <v>63548.18</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63338.1</v>
+        <v>63368.97</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5263</v>
+        <v>13.5388</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27038.97</v>
+        <v>27052.15</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27240.41</v>
+        <v>27253.69</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27139.69</v>
+        <v>27152.92</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5263</v>
+        <v>13.5388</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6364.69</v>
+        <v>6367.79</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6517.68</v>
+        <v>6520.86</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6441.19</v>
+        <v>6444.33</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5263</v>
+        <v>13.5388</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3769.5</v>
+        <v>3771.34</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3762.96</v>
+        <v>3764.8</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3766.23</v>
+        <v>3768.07</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3684</v>
+        <v>13.4024</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>191985.6</v>
+        <v>192067.5</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>192923.04</v>
+        <v>193005.34</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192454.32</v>
+        <v>192536.42</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3684</v>
+        <v>13.4024</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139193.62</v>
+        <v>139253</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140164.96</v>
+        <v>140224.76</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139679.29</v>
+        <v>139738.88</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3684</v>
+        <v>13.4024</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87984.32000000001</v>
+        <v>88021.85000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88696.34</v>
+        <v>88734.17999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88340.33</v>
+        <v>88378.00999999999</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3684</v>
+        <v>13.4024</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42026.8</v>
+        <v>42044.73</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41959.4</v>
+        <v>41977.3</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41993.1</v>
+        <v>42011.01</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3684</v>
+        <v>13.4024</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13105.37</v>
+        <v>13110.96</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12961.02</v>
+        <v>12966.55</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13033.2</v>
+        <v>13038.76</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3684</v>
+        <v>13.4024</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4548.38</v>
+        <v>4550.32</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4437.35</v>
+        <v>4439.25</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4492.87</v>
+        <v>4494.79</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-15
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2956</v>
+        <v>13.3213</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151406.17</v>
+        <v>151470.18</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153314.97</v>
+        <v>153379.79</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152360.57</v>
+        <v>152424.99</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2956</v>
+        <v>13.3213</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115891.58</v>
+        <v>115940.57</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116679.53</v>
+        <v>116728.86</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116285.55</v>
+        <v>116334.72</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2956</v>
+        <v>13.3213</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82633.41</v>
+        <v>82668.34</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83148.32000000001</v>
+        <v>83183.47</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82890.86</v>
+        <v>82925.91</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2956</v>
+        <v>13.3213</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58554.01</v>
+        <v>58578.77</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58110.24</v>
+        <v>58134.81</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58332.13</v>
+        <v>58356.79</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2956</v>
+        <v>13.3213</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37823.57</v>
+        <v>37839.56</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38132.98</v>
+        <v>38149.1</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37978.27</v>
+        <v>37994.33</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2956</v>
+        <v>13.3213</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17202.86</v>
+        <v>17210.14</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17089.9</v>
+        <v>17097.12</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17146.38</v>
+        <v>17153.63</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.2016</v>
+        <v>13.2258</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164556.43</v>
+        <v>164623.33</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163673.45</v>
+        <v>163739.99</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164114.94</v>
+        <v>164181.66</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.2016</v>
+        <v>13.2258</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123582.38</v>
+        <v>123632.62</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121836.96</v>
+        <v>121886.49</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122709.67</v>
+        <v>122759.55</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.2016</v>
+        <v>13.2258</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88291.92999999999</v>
+        <v>88327.82000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87198.61</v>
+        <v>87234.06</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87745.27</v>
+        <v>87780.94</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.2016</v>
+        <v>13.2258</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67256.32000000001</v>
+        <v>67283.66</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66783.52</v>
+        <v>66810.67</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67019.92</v>
+        <v>67047.16</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.2016</v>
+        <v>13.2258</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52541.73</v>
+        <v>52563.09</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50653.43</v>
+        <v>50674.02</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51597.58</v>
+        <v>51618.55</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.2016</v>
+        <v>13.2258</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39829.48</v>
+        <v>39845.67</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40813.68</v>
+        <v>40830.27</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40321.58</v>
+        <v>40337.97</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.0981</v>
+        <v>13.1207</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169529.81</v>
+        <v>169596.08</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171091.47</v>
+        <v>171158.35</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170310.64</v>
+        <v>170377.22</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.0981</v>
+        <v>13.1207</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122207.38</v>
+        <v>122255.16</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120746.74</v>
+        <v>120793.94</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121477.06</v>
+        <v>121524.55</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.0981</v>
+        <v>13.1207</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83713.99000000001</v>
+        <v>83746.71000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83397.8</v>
+        <v>83430.39999999999</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83555.89</v>
+        <v>83588.55</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.0981</v>
+        <v>13.1207</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55774.28</v>
+        <v>55796.08</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56082.02</v>
+        <v>56103.94</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55928.15</v>
+        <v>55950.01</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.0981</v>
+        <v>13.1207</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33662.62</v>
+        <v>33675.78</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33268.61</v>
+        <v>33281.62</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33465.62</v>
+        <v>33478.7</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.0981</v>
+        <v>13.1207</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17476.2</v>
+        <v>17483.03</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18169.05</v>
+        <v>18176.15</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17822.62</v>
+        <v>17829.59</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.0317</v>
+        <v>13.051</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131095.72</v>
+        <v>131146.56</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131191.78</v>
+        <v>131242.65</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131143.75</v>
+        <v>131194.61</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.0317</v>
+        <v>13.051</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90790.66</v>
+        <v>90825.86</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89381.85000000001</v>
+        <v>89416.50999999999</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90086.25</v>
+        <v>90121.19</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.0317</v>
+        <v>13.051</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57067.03</v>
+        <v>57089.16</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57358.26</v>
+        <v>57380.5</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57212.64</v>
+        <v>57234.83</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.0317</v>
+        <v>13.051</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30211.33</v>
+        <v>30223.04</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30414.68</v>
+        <v>30426.47</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30313</v>
+        <v>30324.76</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.0317</v>
+        <v>13.051</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6929.21</v>
+        <v>6931.9</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6927.89</v>
+        <v>6930.58</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6928.55</v>
+        <v>6931.24</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.0317</v>
+        <v>13.051</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3850.18</v>
+        <v>3851.67</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3759.37</v>
+        <v>3760.82</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3804.77</v>
+        <v>3806.25</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>12.9718</v>
+        <v>12.9898</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110758.49</v>
+        <v>110800.49</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111244.39</v>
+        <v>111286.58</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111001.44</v>
+        <v>111043.53</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>12.9718</v>
+        <v>12.9898</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77673.45</v>
+        <v>77702.91</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77120.84</v>
+        <v>77150.09</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77397.14999999999</v>
+        <v>77426.5</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>12.9718</v>
+        <v>12.9898</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47000.3</v>
+        <v>47018.13</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48124.02</v>
+        <v>48142.27</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47562.16</v>
+        <v>47580.2</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>12.9718</v>
+        <v>12.9898</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29199.36</v>
+        <v>29210.43</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29090.54</v>
+        <v>29101.57</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29144.95</v>
+        <v>29156</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>12.9718</v>
+        <v>12.9898</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14323.92</v>
+        <v>14329.35</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14448.11</v>
+        <v>14453.59</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14386.01</v>
+        <v>14391.47</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>12.9718</v>
+        <v>12.9898</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6640.58</v>
+        <v>6643.09</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6476.52</v>
+        <v>6478.98</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6558.55</v>
+        <v>6561.04</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.9091</v>
+        <v>12.9256</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50452.99</v>
+        <v>50471.78</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50115.21</v>
+        <v>50133.88</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50284.1</v>
+        <v>50302.83</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.9091</v>
+        <v>12.9256</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44385.16</v>
+        <v>44401.69</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44582.21</v>
+        <v>44598.81</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44483.68</v>
+        <v>44500.25</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.9091</v>
+        <v>12.9256</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32483.26</v>
+        <v>32495.36</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32829.19</v>
+        <v>32841.42</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32656.23</v>
+        <v>32668.39</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.9091</v>
+        <v>12.9256</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22839.91</v>
+        <v>22848.41</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22996.77</v>
+        <v>23005.33</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22918.34</v>
+        <v>22926.87</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.9091</v>
+        <v>12.9256</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14679.94</v>
+        <v>14685.4</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14888.84</v>
+        <v>14894.38</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14784.39</v>
+        <v>14789.89</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.9091</v>
+        <v>12.9256</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8436.57</v>
+        <v>8439.709999999999</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8492.469999999999</v>
+        <v>8495.629999999999</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8464.52</v>
+        <v>8467.67</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.8435</v>
+        <v>12.8586</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49686.71</v>
+        <v>49704.98</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48955.45</v>
+        <v>48973.45</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49321.08</v>
+        <v>49339.22</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.8435</v>
+        <v>12.8586</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44495.15</v>
+        <v>44511.51</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44153.34</v>
+        <v>44169.58</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44324.25</v>
+        <v>44340.54</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.8435</v>
+        <v>12.8586</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32134.42</v>
+        <v>32146.23</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31556.75</v>
+        <v>31568.35</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31845.58</v>
+        <v>31857.29</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.8435</v>
+        <v>12.8586</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23950.8</v>
+        <v>23959.6</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23844.01</v>
+        <v>23852.78</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23897.41</v>
+        <v>23906.19</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.8435</v>
+        <v>12.8586</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18789.1</v>
+        <v>18796</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18600.28</v>
+        <v>18607.11</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18694.69</v>
+        <v>18701.56</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.8435</v>
+        <v>12.8586</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15802.91</v>
+        <v>15808.72</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15746.49</v>
+        <v>15752.28</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15774.7</v>
+        <v>15780.5</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.7836</v>
+        <v>12.7973</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110498.74</v>
+        <v>110539.11</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111058.33</v>
+        <v>111098.9</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110778.53</v>
+        <v>110819</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.7836</v>
+        <v>12.7973</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79239.42</v>
+        <v>79268.36</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79559.74000000001</v>
+        <v>79588.81</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79399.58</v>
+        <v>79428.59</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.7836</v>
+        <v>12.7973</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51762.58</v>
+        <v>51781.49</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51322.96</v>
+        <v>51341.71</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51542.77</v>
+        <v>51561.6</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.7836</v>
+        <v>12.7973</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29759.96</v>
+        <v>29770.83</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29545.53</v>
+        <v>29556.32</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29652.74</v>
+        <v>29663.58</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.7836</v>
+        <v>12.7973</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16912.28</v>
+        <v>16918.46</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16845.45</v>
+        <v>16851.61</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16878.87</v>
+        <v>16885.03</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.7836</v>
+        <v>12.7973</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6856.87</v>
+        <v>6859.37</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6639.89</v>
+        <v>6642.32</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6748.38</v>
+        <v>6750.84</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.727</v>
+        <v>12.7373</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>359972.31</v>
+        <v>360110.1</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355518.56</v>
+        <v>355654.65</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357745.44</v>
+        <v>357882.38</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.727</v>
+        <v>12.7373</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270241.83</v>
+        <v>270345.28</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271118.29</v>
+        <v>271222.07</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270680.06</v>
+        <v>270783.67</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.727</v>
+        <v>12.7373</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189089.04</v>
+        <v>189161.42</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>188974.97</v>
+        <v>189047.31</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189032.01</v>
+        <v>189104.37</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.727</v>
+        <v>12.7373</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114955.13</v>
+        <v>114999.14</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115208.51</v>
+        <v>115252.61</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115081.82</v>
+        <v>115125.87</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.727</v>
+        <v>12.7373</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55720.24</v>
+        <v>55741.57</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55459.93</v>
+        <v>55481.16</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55590.09</v>
+        <v>55611.36</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.727</v>
+        <v>12.7373</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28457.25</v>
+        <v>28468.14</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28478.74</v>
+        <v>28489.64</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28467.99</v>
+        <v>28478.89</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.6415</v>
+        <v>13.6663</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>411121.03</v>
+        <v>411324.01</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>411673.63</v>
+        <v>411876.88</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>411397.33</v>
+        <v>411600.45</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.6415</v>
+        <v>13.6663</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>305170.77</v>
+        <v>305321.44</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>303265.31</v>
+        <v>303415.04</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>304218.04</v>
+        <v>304368.24</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.6415</v>
+        <v>13.6663</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>206997.61</v>
+        <v>207099.81</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207068.42</v>
+        <v>207170.65</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207033.01</v>
+        <v>207135.23</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.6415</v>
+        <v>13.6663</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125261.44</v>
+        <v>125323.29</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125783.71</v>
+        <v>125845.82</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125522.58</v>
+        <v>125584.55</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.6415</v>
+        <v>13.6663</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50023.84</v>
+        <v>50048.54</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49964.23</v>
+        <v>49988.9</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49994.03</v>
+        <v>50018.72</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.6415</v>
+        <v>13.6663</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5502.46</v>
+        <v>5505.18</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5538.75</v>
+        <v>5541.48</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5520.6</v>
+        <v>5523.33</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5388</v>
+        <v>13.5691</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171691.72</v>
+        <v>171771.71</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171719.18</v>
+        <v>171799.18</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171705.45</v>
+        <v>171785.45</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5388</v>
+        <v>13.5691</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112829.97</v>
+        <v>112882.53</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112437.46</v>
+        <v>112489.84</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112633.72</v>
+        <v>112686.19</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5388</v>
+        <v>13.5691</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63189.76</v>
+        <v>63219.2</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63548.18</v>
+        <v>63577.79</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63368.97</v>
+        <v>63398.49</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5388</v>
+        <v>13.5691</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27052.15</v>
+        <v>27064.75</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27253.69</v>
+        <v>27266.39</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27152.92</v>
+        <v>27165.57</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5388</v>
+        <v>13.5691</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6367.79</v>
+        <v>6370.76</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6520.86</v>
+        <v>6523.9</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6444.33</v>
+        <v>6447.33</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5388</v>
+        <v>13.5691</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3771.34</v>
+        <v>3773.1</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3764.8</v>
+        <v>3766.55</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3768.07</v>
+        <v>3769.82</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4024</v>
+        <v>13.4306</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192067.5</v>
+        <v>192152.18</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193005.34</v>
+        <v>193090.44</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192536.42</v>
+        <v>192621.31</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4024</v>
+        <v>13.4306</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139253</v>
+        <v>139314.4</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140224.76</v>
+        <v>140286.58</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139738.88</v>
+        <v>139800.49</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4024</v>
+        <v>13.4306</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88021.85000000001</v>
+        <v>88060.66</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88734.17999999999</v>
+        <v>88773.3</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88378.00999999999</v>
+        <v>88416.98</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4024</v>
+        <v>13.4306</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42044.73</v>
+        <v>42063.26</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41977.3</v>
+        <v>41995.81</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42011.01</v>
+        <v>42029.53</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4024</v>
+        <v>13.4306</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13110.96</v>
+        <v>13116.74</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12966.55</v>
+        <v>12972.27</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13038.76</v>
+        <v>13044.51</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4024</v>
+        <v>13.4306</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4550.32</v>
+        <v>4552.33</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4439.25</v>
+        <v>4441.2</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4494.79</v>
+        <v>4496.77</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-16
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3213</v>
+        <v>13.4059</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151470.18</v>
+        <v>151509.44</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153379.79</v>
+        <v>153419.54</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152424.99</v>
+        <v>152464.49</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3213</v>
+        <v>13.4059</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115940.57</v>
+        <v>115970.62</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116728.86</v>
+        <v>116759.11</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116334.72</v>
+        <v>116364.87</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3213</v>
+        <v>13.4059</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82668.34</v>
+        <v>82689.77</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83183.47</v>
+        <v>83205.03</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82925.91</v>
+        <v>82947.39999999999</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3213</v>
+        <v>13.4059</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58578.77</v>
+        <v>58593.95</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58134.81</v>
+        <v>58149.88</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58356.79</v>
+        <v>58371.91</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3213</v>
+        <v>13.4059</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37839.56</v>
+        <v>37849.37</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38149.1</v>
+        <v>38158.99</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37994.33</v>
+        <v>38004.18</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3213</v>
+        <v>13.4059</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17210.14</v>
+        <v>17214.6</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17097.12</v>
+        <v>17101.56</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17153.63</v>
+        <v>17158.08</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.2258</v>
+        <v>13.3231</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164623.33</v>
+        <v>164648.32</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163739.99</v>
+        <v>163764.85</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164181.66</v>
+        <v>164206.58</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.2258</v>
+        <v>13.3231</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123632.62</v>
+        <v>123651.39</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121886.49</v>
+        <v>121904.99</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122759.55</v>
+        <v>122778.19</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.2258</v>
+        <v>13.3231</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88327.82000000001</v>
+        <v>88341.23</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87234.06</v>
+        <v>87247.3</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87780.94</v>
+        <v>87794.27</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.2258</v>
+        <v>13.3231</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67283.66</v>
+        <v>67293.88</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66810.67</v>
+        <v>66820.81</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67047.16</v>
+        <v>67057.34</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.2258</v>
+        <v>13.3231</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52563.09</v>
+        <v>52571.07</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50674.02</v>
+        <v>50681.71</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51618.55</v>
+        <v>51626.39</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.2258</v>
+        <v>13.3231</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39845.67</v>
+        <v>39851.72</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40830.27</v>
+        <v>40836.47</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40337.97</v>
+        <v>40344.1</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.1207</v>
+        <v>13.2321</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169596.08</v>
+        <v>169598.29</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171158.35</v>
+        <v>171160.57</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170377.22</v>
+        <v>170379.43</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.1207</v>
+        <v>13.2321</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122255.16</v>
+        <v>122256.74</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120793.94</v>
+        <v>120795.51</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121524.55</v>
+        <v>121526.13</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.1207</v>
+        <v>13.2321</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83746.71000000001</v>
+        <v>83747.8</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83430.39999999999</v>
+        <v>83431.48</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83588.55</v>
+        <v>83589.64</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.1207</v>
+        <v>13.2321</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55796.08</v>
+        <v>55796.8</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56103.94</v>
+        <v>56104.67</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55950.01</v>
+        <v>55950.74</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.1207</v>
+        <v>13.2321</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33675.78</v>
+        <v>33676.22</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33281.62</v>
+        <v>33282.05</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33478.7</v>
+        <v>33479.13</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.1207</v>
+        <v>13.2321</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17483.03</v>
+        <v>17483.26</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18176.15</v>
+        <v>18176.38</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17829.59</v>
+        <v>17829.82</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.051</v>
+        <v>13.1699</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131146.56</v>
+        <v>131131.6</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131242.65</v>
+        <v>131227.68</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131194.61</v>
+        <v>131179.64</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.051</v>
+        <v>13.1699</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90825.86</v>
+        <v>90815.5</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89416.50999999999</v>
+        <v>89406.3</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90121.19</v>
+        <v>90110.89999999999</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.051</v>
+        <v>13.1699</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57089.16</v>
+        <v>57082.64</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57380.5</v>
+        <v>57373.96</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57234.83</v>
+        <v>57228.3</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.051</v>
+        <v>13.1699</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30223.04</v>
+        <v>30219.59</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30426.47</v>
+        <v>30423</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30324.76</v>
+        <v>30321.3</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.051</v>
+        <v>13.1699</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6931.9</v>
+        <v>6931.11</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6930.58</v>
+        <v>6929.79</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6931.24</v>
+        <v>6930.45</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.051</v>
+        <v>13.1699</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3851.67</v>
+        <v>3851.23</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3760.82</v>
+        <v>3760.39</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3806.25</v>
+        <v>3805.81</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>12.9898</v>
+        <v>13.1168</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110800.49</v>
+        <v>110772.68</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111286.58</v>
+        <v>111258.64</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111043.53</v>
+        <v>111015.66</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>12.9898</v>
+        <v>13.1168</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77702.91</v>
+        <v>77683.39999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77150.09</v>
+        <v>77130.72</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77426.5</v>
+        <v>77407.06</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>12.9898</v>
+        <v>13.1168</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47018.13</v>
+        <v>47006.33</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48142.27</v>
+        <v>48130.19</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47580.2</v>
+        <v>47568.26</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>12.9898</v>
+        <v>13.1168</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29210.43</v>
+        <v>29203.1</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29101.57</v>
+        <v>29094.27</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29156</v>
+        <v>29148.68</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>12.9898</v>
+        <v>13.1168</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14329.35</v>
+        <v>14325.76</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14453.59</v>
+        <v>14449.96</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14391.47</v>
+        <v>14387.86</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>12.9898</v>
+        <v>13.1168</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6643.09</v>
+        <v>6641.43</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6478.98</v>
+        <v>6477.35</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6561.04</v>
+        <v>6559.39</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.9256</v>
+        <v>13.0611</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50471.78</v>
+        <v>50451.22</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50133.88</v>
+        <v>50113.45</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50302.83</v>
+        <v>50282.34</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.9256</v>
+        <v>13.0611</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44401.69</v>
+        <v>44383.6</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44598.81</v>
+        <v>44580.64</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44500.25</v>
+        <v>44482.12</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.9256</v>
+        <v>13.0611</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32495.36</v>
+        <v>32482.12</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32841.42</v>
+        <v>32828.04</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32668.39</v>
+        <v>32655.08</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.9256</v>
+        <v>13.0611</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22848.41</v>
+        <v>22839.11</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>23005.33</v>
+        <v>22995.96</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22926.87</v>
+        <v>22917.53</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.9256</v>
+        <v>13.0611</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14685.4</v>
+        <v>14679.42</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14894.38</v>
+        <v>14888.31</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14789.89</v>
+        <v>14783.87</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.9256</v>
+        <v>13.0611</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8439.709999999999</v>
+        <v>8436.27</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8495.629999999999</v>
+        <v>8492.17</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8467.67</v>
+        <v>8464.219999999999</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.8586</v>
+        <v>13.0029</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49704.98</v>
+        <v>49675.9</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48973.45</v>
+        <v>48944.8</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49339.22</v>
+        <v>49310.35</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.8586</v>
+        <v>13.0029</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44511.51</v>
+        <v>44485.47</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44169.58</v>
+        <v>44143.74</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44340.54</v>
+        <v>44314.6</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.8586</v>
+        <v>13.0029</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32146.23</v>
+        <v>32127.43</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31568.35</v>
+        <v>31549.88</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31857.29</v>
+        <v>31838.65</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.8586</v>
+        <v>13.0029</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23959.6</v>
+        <v>23945.59</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23852.78</v>
+        <v>23838.83</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23906.19</v>
+        <v>23892.21</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.8586</v>
+        <v>13.0029</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18796</v>
+        <v>18785.01</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18607.11</v>
+        <v>18596.23</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18701.56</v>
+        <v>18690.62</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.8586</v>
+        <v>13.0029</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15808.72</v>
+        <v>15799.47</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15752.28</v>
+        <v>15743.06</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15780.5</v>
+        <v>15771.27</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.7973</v>
+        <v>12.9497</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110539.11</v>
+        <v>110455.12</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111098.9</v>
+        <v>111014.49</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110819</v>
+        <v>110734.8</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.7973</v>
+        <v>12.9497</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79268.36</v>
+        <v>79208.14</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79588.81</v>
+        <v>79528.34</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79428.59</v>
+        <v>79368.24000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.7973</v>
+        <v>12.9497</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51781.49</v>
+        <v>51742.14</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51341.71</v>
+        <v>51302.7</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51561.6</v>
+        <v>51522.42</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.7973</v>
+        <v>12.9497</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29770.83</v>
+        <v>29748.21</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29556.32</v>
+        <v>29533.86</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29663.58</v>
+        <v>29641.04</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.7973</v>
+        <v>12.9497</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16918.46</v>
+        <v>16905.61</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16851.61</v>
+        <v>16838.8</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16885.03</v>
+        <v>16872.21</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.7973</v>
+        <v>12.9497</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6859.37</v>
+        <v>6854.16</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6642.32</v>
+        <v>6637.27</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6750.84</v>
+        <v>6745.71</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.7373</v>
+        <v>12.8959</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360110.1</v>
+        <v>359773.44</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355654.65</v>
+        <v>355322.15</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357882.38</v>
+        <v>357547.79</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.7373</v>
+        <v>12.8959</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270345.28</v>
+        <v>270092.53</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271222.07</v>
+        <v>270968.5</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270783.67</v>
+        <v>270530.52</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.7373</v>
+        <v>12.8959</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189161.42</v>
+        <v>188984.58</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189047.31</v>
+        <v>188870.57</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189104.37</v>
+        <v>188927.57</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.7373</v>
+        <v>12.8959</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114999.14</v>
+        <v>114891.62</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115252.61</v>
+        <v>115144.86</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115125.87</v>
+        <v>115018.24</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.7373</v>
+        <v>12.8959</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55741.57</v>
+        <v>55689.46</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55481.16</v>
+        <v>55429.29</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55611.36</v>
+        <v>55559.37</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.7373</v>
+        <v>12.8959</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28468.14</v>
+        <v>28441.52</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28489.64</v>
+        <v>28463</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28478.89</v>
+        <v>28452.26</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.6663</v>
+        <v>13.7007</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>411324.01</v>
+        <v>411525.74</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>411876.88</v>
+        <v>412078.88</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>411600.45</v>
+        <v>411802.31</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.6663</v>
+        <v>13.7007</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>305321.44</v>
+        <v>305471.18</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>303415.04</v>
+        <v>303563.84</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>304368.24</v>
+        <v>304517.51</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.6663</v>
+        <v>13.7007</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207099.81</v>
+        <v>207201.37</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207170.65</v>
+        <v>207272.26</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207135.23</v>
+        <v>207236.81</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.6663</v>
+        <v>13.7007</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125323.29</v>
+        <v>125384.75</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125845.82</v>
+        <v>125907.53</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125584.55</v>
+        <v>125646.14</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.6663</v>
+        <v>13.7007</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50048.54</v>
+        <v>50073.08</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49988.9</v>
+        <v>50013.41</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50018.72</v>
+        <v>50043.25</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.6663</v>
+        <v>13.7007</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5505.18</v>
+        <v>5507.88</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5541.48</v>
+        <v>5544.2</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5523.33</v>
+        <v>5526.04</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5691</v>
+        <v>13.6222</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171771.71</v>
+        <v>171847.31</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171799.18</v>
+        <v>171874.79</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171785.45</v>
+        <v>171861.05</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5691</v>
+        <v>13.6222</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112882.53</v>
+        <v>112932.22</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112489.84</v>
+        <v>112539.35</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112686.19</v>
+        <v>112735.78</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5691</v>
+        <v>13.6222</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63219.2</v>
+        <v>63247.03</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63577.79</v>
+        <v>63605.77</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63398.49</v>
+        <v>63426.4</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5691</v>
+        <v>13.6222</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27064.75</v>
+        <v>27076.66</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27266.39</v>
+        <v>27278.39</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27165.57</v>
+        <v>27177.53</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5691</v>
+        <v>13.6222</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6370.76</v>
+        <v>6373.56</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6523.9</v>
+        <v>6526.77</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6447.33</v>
+        <v>6450.17</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5691</v>
+        <v>13.6222</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3773.1</v>
+        <v>3774.76</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3766.55</v>
+        <v>3768.21</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3769.82</v>
+        <v>3771.48</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4306</v>
+        <v>13.5017</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192152.18</v>
+        <v>192220.59</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193090.44</v>
+        <v>193159.18</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192621.31</v>
+        <v>192689.89</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4306</v>
+        <v>13.5017</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139314.4</v>
+        <v>139364</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140286.58</v>
+        <v>140336.53</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139800.49</v>
+        <v>139850.26</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4306</v>
+        <v>13.5017</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88060.66</v>
+        <v>88092.00999999999</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88773.3</v>
+        <v>88804.89999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88416.98</v>
+        <v>88448.46000000001</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4306</v>
+        <v>13.5017</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42063.26</v>
+        <v>42078.24</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41995.81</v>
+        <v>42010.76</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42029.53</v>
+        <v>42044.5</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4306</v>
+        <v>13.5017</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13116.74</v>
+        <v>13121.41</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12972.27</v>
+        <v>12976.89</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13044.51</v>
+        <v>13049.15</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4306</v>
+        <v>13.5017</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4552.33</v>
+        <v>4553.95</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4441.2</v>
+        <v>4442.78</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4496.77</v>
+        <v>4498.37</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-17
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.4059</v>
+        <v>13.3491</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151509.44</v>
+        <v>151533.55</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153419.54</v>
+        <v>153443.96</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152464.49</v>
+        <v>152488.75</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.4059</v>
+        <v>13.3491</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115970.62</v>
+        <v>115989.08</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116759.11</v>
+        <v>116777.69</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116364.87</v>
+        <v>116383.39</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.4059</v>
+        <v>13.3491</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82689.77</v>
+        <v>82702.92999999999</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83205.03</v>
+        <v>83218.27</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82947.39999999999</v>
+        <v>82960.60000000001</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.4059</v>
+        <v>13.3491</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58593.95</v>
+        <v>58603.27</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58149.88</v>
+        <v>58159.13</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58371.91</v>
+        <v>58381.2</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.4059</v>
+        <v>13.3491</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37849.37</v>
+        <v>37855.39</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38158.99</v>
+        <v>38165.06</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38004.18</v>
+        <v>38010.22</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.4059</v>
+        <v>13.3491</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17214.6</v>
+        <v>17217.34</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17101.56</v>
+        <v>17104.28</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17158.08</v>
+        <v>17160.81</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3231</v>
+        <v>13.2791</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164648.32</v>
+        <v>164673.71</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163764.85</v>
+        <v>163790.1</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164206.58</v>
+        <v>164231.91</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3231</v>
+        <v>13.2791</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123651.39</v>
+        <v>123670.46</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121904.99</v>
+        <v>121923.79</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122778.19</v>
+        <v>122797.13</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3231</v>
+        <v>13.2791</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88341.23</v>
+        <v>88354.86</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87247.3</v>
+        <v>87260.75999999999</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87794.27</v>
+        <v>87807.81</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3231</v>
+        <v>13.2791</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67293.88</v>
+        <v>67304.25</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66820.81</v>
+        <v>66831.12</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67057.34</v>
+        <v>67067.69</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3231</v>
+        <v>13.2791</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52571.07</v>
+        <v>52579.18</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50681.71</v>
+        <v>50689.53</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51626.39</v>
+        <v>51634.35</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3231</v>
+        <v>13.2791</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39851.72</v>
+        <v>39857.86</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40836.47</v>
+        <v>40842.77</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40344.1</v>
+        <v>40350.32</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.2321</v>
+        <v>13.2021</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169598.29</v>
+        <v>169620.01</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171160.57</v>
+        <v>171182.5</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170379.43</v>
+        <v>170401.26</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.2321</v>
+        <v>13.2021</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122256.74</v>
+        <v>122272.4</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120795.51</v>
+        <v>120810.99</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121526.13</v>
+        <v>121541.7</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.2321</v>
+        <v>13.2021</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83747.8</v>
+        <v>83758.53</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83431.48</v>
+        <v>83442.17</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83589.64</v>
+        <v>83600.35000000001</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.2321</v>
+        <v>13.2021</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55796.8</v>
+        <v>55803.95</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56104.67</v>
+        <v>56111.86</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55950.74</v>
+        <v>55957.9</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.2321</v>
+        <v>13.2021</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33676.22</v>
+        <v>33680.53</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33282.05</v>
+        <v>33286.31</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33479.13</v>
+        <v>33483.42</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.2321</v>
+        <v>13.2021</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17483.26</v>
+        <v>17485.5</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18176.38</v>
+        <v>18178.71</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17829.82</v>
+        <v>17832.11</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.1699</v>
+        <v>13.1503</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131131.6</v>
+        <v>131144.61</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131227.68</v>
+        <v>131240.7</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131179.64</v>
+        <v>131192.66</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.1699</v>
+        <v>13.1503</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90815.5</v>
+        <v>90824.50999999999</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89406.3</v>
+        <v>89415.17999999999</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90110.89999999999</v>
+        <v>90119.85000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.1699</v>
+        <v>13.1503</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57082.64</v>
+        <v>57088.31</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57373.96</v>
+        <v>57379.65</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57228.3</v>
+        <v>57233.98</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.1699</v>
+        <v>13.1503</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30219.59</v>
+        <v>30222.59</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30423</v>
+        <v>30426.02</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30321.3</v>
+        <v>30324.31</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.1699</v>
+        <v>13.1503</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6931.11</v>
+        <v>6931.8</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6929.79</v>
+        <v>6930.48</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6930.45</v>
+        <v>6931.14</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.1699</v>
+        <v>13.1503</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3851.23</v>
+        <v>3851.61</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3760.39</v>
+        <v>3760.77</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3805.81</v>
+        <v>3806.19</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.1168</v>
+        <v>13.1062</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110772.68</v>
+        <v>110779.49</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111258.64</v>
+        <v>111265.48</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111015.66</v>
+        <v>111022.48</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.1168</v>
+        <v>13.1062</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77683.39999999999</v>
+        <v>77688.17999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77130.72</v>
+        <v>77135.46000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77407.06</v>
+        <v>77411.82000000001</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.1168</v>
+        <v>13.1062</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47006.33</v>
+        <v>47009.22</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48130.19</v>
+        <v>48133.15</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47568.26</v>
+        <v>47571.18</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.1168</v>
+        <v>13.1062</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29203.1</v>
+        <v>29204.9</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29094.27</v>
+        <v>29096.06</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29148.68</v>
+        <v>29150.48</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.1168</v>
+        <v>13.1062</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14325.76</v>
+        <v>14326.64</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14449.96</v>
+        <v>14450.85</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14387.86</v>
+        <v>14388.74</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.1168</v>
+        <v>13.1062</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6641.43</v>
+        <v>6641.84</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6477.35</v>
+        <v>6477.75</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6559.39</v>
+        <v>6559.79</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.0611</v>
+        <v>13.06</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50451.22</v>
+        <v>50451.6</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50113.45</v>
+        <v>50113.84</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50282.34</v>
+        <v>50282.72</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.0611</v>
+        <v>13.06</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44383.6</v>
+        <v>44383.94</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44580.64</v>
+        <v>44580.98</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44482.12</v>
+        <v>44482.46</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.0611</v>
+        <v>13.06</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32482.12</v>
+        <v>32482.37</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32828.04</v>
+        <v>32828.29</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32655.08</v>
+        <v>32655.33</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.0611</v>
+        <v>13.06</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22839.11</v>
+        <v>22839.28</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22995.96</v>
+        <v>22996.13</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22917.53</v>
+        <v>22917.71</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.0611</v>
+        <v>13.06</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14679.42</v>
+        <v>14679.53</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14888.31</v>
+        <v>14888.43</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14783.87</v>
+        <v>14783.98</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.0611</v>
+        <v>13.06</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8436.27</v>
+        <v>8436.34</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8492.17</v>
+        <v>8492.23</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8464.219999999999</v>
+        <v>8464.290000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.0029</v>
+        <v>13.0116</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49675.9</v>
+        <v>49672.7</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48944.8</v>
+        <v>48941.65</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49310.35</v>
+        <v>49307.18</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.0029</v>
+        <v>13.0116</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44485.47</v>
+        <v>44482.61</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44143.74</v>
+        <v>44140.89</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44314.6</v>
+        <v>44311.75</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.0029</v>
+        <v>13.0116</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32127.43</v>
+        <v>32125.36</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31549.88</v>
+        <v>31547.85</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31838.65</v>
+        <v>31836.6</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.0029</v>
+        <v>13.0116</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23945.59</v>
+        <v>23944.05</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23838.83</v>
+        <v>23837.29</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23892.21</v>
+        <v>23890.67</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.0029</v>
+        <v>13.0116</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18785.01</v>
+        <v>18783.8</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18596.23</v>
+        <v>18595.03</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18690.62</v>
+        <v>18689.41</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.0029</v>
+        <v>13.0116</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15799.47</v>
+        <v>15798.46</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15743.06</v>
+        <v>15742.05</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15771.27</v>
+        <v>15770.25</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.9497</v>
+        <v>12.9675</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110455.12</v>
+        <v>110439.2</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111014.49</v>
+        <v>110998.48</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110734.8</v>
+        <v>110718.84</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.9497</v>
+        <v>12.9675</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79208.14</v>
+        <v>79196.72</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79528.34</v>
+        <v>79516.87</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79368.24000000001</v>
+        <v>79356.78999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.9497</v>
+        <v>12.9675</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51742.14</v>
+        <v>51734.68</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51302.7</v>
+        <v>51295.31</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51522.42</v>
+        <v>51515</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.9497</v>
+        <v>12.9675</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29748.21</v>
+        <v>29743.92</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29533.86</v>
+        <v>29529.61</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29641.04</v>
+        <v>29636.76</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.9497</v>
+        <v>12.9675</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16905.61</v>
+        <v>16903.17</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16838.8</v>
+        <v>16836.38</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16872.21</v>
+        <v>16869.77</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.9497</v>
+        <v>12.9675</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6854.16</v>
+        <v>6853.17</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6637.27</v>
+        <v>6636.31</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6745.71</v>
+        <v>6744.74</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.8959</v>
+        <v>12.9229</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>359773.44</v>
+        <v>359687.12</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355322.15</v>
+        <v>355236.9</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357547.79</v>
+        <v>357462.01</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.8959</v>
+        <v>12.9229</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270092.53</v>
+        <v>270027.73</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>270968.5</v>
+        <v>270903.49</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270530.52</v>
+        <v>270465.61</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.8959</v>
+        <v>12.9229</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>188984.58</v>
+        <v>188939.23</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>188870.57</v>
+        <v>188825.25</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>188927.57</v>
+        <v>188882.24</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.8959</v>
+        <v>12.9229</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114891.62</v>
+        <v>114864.06</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115144.86</v>
+        <v>115117.23</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115018.24</v>
+        <v>114990.64</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.8959</v>
+        <v>12.9229</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55689.46</v>
+        <v>55676.09</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55429.29</v>
+        <v>55415.99</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55559.37</v>
+        <v>55546.04</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.8959</v>
+        <v>12.9229</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28441.52</v>
+        <v>28434.7</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28463</v>
+        <v>28456.17</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28452.26</v>
+        <v>28445.44</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.7007</v>
+        <v>13.5995</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>411525.74</v>
+        <v>411547.55</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>412078.88</v>
+        <v>412100.72</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>411802.31</v>
+        <v>411824.13</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.7007</v>
+        <v>13.5995</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>305471.18</v>
+        <v>305487.37</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>303563.84</v>
+        <v>303579.94</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>304517.51</v>
+        <v>304533.65</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.7007</v>
+        <v>13.5995</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207201.37</v>
+        <v>207212.36</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207272.26</v>
+        <v>207283.24</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207236.81</v>
+        <v>207247.8</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.7007</v>
+        <v>13.5995</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125384.75</v>
+        <v>125391.4</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125907.53</v>
+        <v>125914.21</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125646.14</v>
+        <v>125652.8</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.7007</v>
+        <v>13.5995</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50073.08</v>
+        <v>50075.74</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50013.41</v>
+        <v>50016.06</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50043.25</v>
+        <v>50045.9</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.7007</v>
+        <v>13.5995</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5507.88</v>
+        <v>5508.17</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5544.2</v>
+        <v>5544.49</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5526.04</v>
+        <v>5526.33</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.6222</v>
+        <v>13.5326</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171847.31</v>
+        <v>171866.12</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171874.79</v>
+        <v>171893.61</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171861.05</v>
+        <v>171879.87</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.6222</v>
+        <v>13.5326</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112932.22</v>
+        <v>112944.58</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112539.35</v>
+        <v>112551.67</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112735.78</v>
+        <v>112748.13</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.6222</v>
+        <v>13.5326</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63247.03</v>
+        <v>63253.95</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63605.77</v>
+        <v>63612.73</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63426.4</v>
+        <v>63433.34</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.6222</v>
+        <v>13.5326</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27076.66</v>
+        <v>27079.63</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27278.39</v>
+        <v>27281.37</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27177.53</v>
+        <v>27180.5</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.6222</v>
+        <v>13.5326</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6373.56</v>
+        <v>6374.26</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6526.77</v>
+        <v>6527.49</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6450.17</v>
+        <v>6450.87</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.6222</v>
+        <v>13.5326</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3774.76</v>
+        <v>3775.17</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3768.21</v>
+        <v>3768.62</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3771.48</v>
+        <v>3771.89</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.5017</v>
+        <v>13.4302</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192220.59</v>
+        <v>192248.48</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193159.18</v>
+        <v>193187.2</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192689.89</v>
+        <v>192717.84</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.5017</v>
+        <v>13.4302</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139364</v>
+        <v>139384.21</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140336.53</v>
+        <v>140356.88</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139850.26</v>
+        <v>139870.55</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.5017</v>
+        <v>13.4302</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88092.00999999999</v>
+        <v>88104.78999999999</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88804.89999999999</v>
+        <v>88817.78999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88448.46000000001</v>
+        <v>88461.28999999999</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.5017</v>
+        <v>13.4302</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42078.24</v>
+        <v>42084.34</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42010.76</v>
+        <v>42016.85</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42044.5</v>
+        <v>42050.6</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.5017</v>
+        <v>13.4302</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13121.41</v>
+        <v>13123.32</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12976.89</v>
+        <v>12978.77</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13049.15</v>
+        <v>13051.04</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.5017</v>
+        <v>13.4302</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4553.95</v>
+        <v>4554.61</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4442.78</v>
+        <v>4443.43</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4498.37</v>
+        <v>4499.02</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-20
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3491</v>
+        <v>13.3244</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151533.55</v>
+        <v>151694.55</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153443.96</v>
+        <v>153606.99</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152488.75</v>
+        <v>152650.77</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3491</v>
+        <v>13.3244</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>115989.08</v>
+        <v>116112.31</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116777.69</v>
+        <v>116901.76</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116383.39</v>
+        <v>116507.04</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3491</v>
+        <v>13.3244</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82702.92999999999</v>
+        <v>82790.8</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83218.27</v>
+        <v>83306.69</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>82960.60000000001</v>
+        <v>83048.74000000001</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3491</v>
+        <v>13.3244</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58603.27</v>
+        <v>58665.54</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58159.13</v>
+        <v>58220.92</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58381.2</v>
+        <v>58443.23</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3491</v>
+        <v>13.3244</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37855.39</v>
+        <v>37895.61</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38165.06</v>
+        <v>38205.61</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38010.22</v>
+        <v>38050.61</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3491</v>
+        <v>13.3244</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17217.34</v>
+        <v>17235.63</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17104.28</v>
+        <v>17122.45</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17160.81</v>
+        <v>17179.04</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.2791</v>
+        <v>13.2535</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164673.71</v>
+        <v>164851.25</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163790.1</v>
+        <v>163966.68</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164231.91</v>
+        <v>164408.96</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.2791</v>
+        <v>13.2535</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123670.46</v>
+        <v>123803.79</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>121923.79</v>
+        <v>122055.24</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122797.13</v>
+        <v>122929.51</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.2791</v>
+        <v>13.2535</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88354.86</v>
+        <v>88450.11</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87260.75999999999</v>
+        <v>87354.83</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87807.81</v>
+        <v>87902.47</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.2791</v>
+        <v>13.2535</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67304.25</v>
+        <v>67376.81</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66831.12</v>
+        <v>66903.17</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67067.69</v>
+        <v>67139.99000000001</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.2791</v>
+        <v>13.2535</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52579.18</v>
+        <v>52635.86</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50689.53</v>
+        <v>50744.18</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51634.35</v>
+        <v>51690.02</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.2791</v>
+        <v>13.2535</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39857.86</v>
+        <v>39900.83</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40842.77</v>
+        <v>40886.8</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40350.32</v>
+        <v>40393.82</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.2021</v>
+        <v>13.1755</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169620.01</v>
+        <v>169806.05</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171182.5</v>
+        <v>171370.24</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170401.26</v>
+        <v>170588.15</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.2021</v>
+        <v>13.1755</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122272.4</v>
+        <v>122406.51</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120810.99</v>
+        <v>120943.49</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121541.7</v>
+        <v>121675</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.2021</v>
+        <v>13.1755</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83758.53</v>
+        <v>83850.39</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83442.17</v>
+        <v>83533.69</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83600.35000000001</v>
+        <v>83692.03999999999</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.2021</v>
+        <v>13.1755</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55803.95</v>
+        <v>55865.16</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56111.86</v>
+        <v>56173.4</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55957.9</v>
+        <v>56019.28</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.2021</v>
+        <v>13.1755</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33680.53</v>
+        <v>33717.47</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33286.31</v>
+        <v>33322.82</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33483.42</v>
+        <v>33520.14</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.2021</v>
+        <v>13.1755</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17485.5</v>
+        <v>17504.68</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18178.71</v>
+        <v>18198.65</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17832.11</v>
+        <v>17851.66</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.1503</v>
+        <v>13.1208</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131144.61</v>
+        <v>131292.52</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131240.7</v>
+        <v>131388.72</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131192.66</v>
+        <v>131340.62</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.1503</v>
+        <v>13.1208</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90824.50999999999</v>
+        <v>90926.95</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89415.17999999999</v>
+        <v>89516.02</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90119.85000000001</v>
+        <v>90221.49000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.1503</v>
+        <v>13.1208</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57088.31</v>
+        <v>57152.69</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57379.65</v>
+        <v>57444.37</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57233.98</v>
+        <v>57298.53</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.1503</v>
+        <v>13.1208</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30222.59</v>
+        <v>30256.68</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30426.02</v>
+        <v>30460.34</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30324.31</v>
+        <v>30358.51</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.1503</v>
+        <v>13.1208</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6931.8</v>
+        <v>6939.62</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6930.48</v>
+        <v>6938.29</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6931.14</v>
+        <v>6938.95</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.1503</v>
+        <v>13.1208</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3851.61</v>
+        <v>3855.96</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3760.77</v>
+        <v>3765.01</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3806.19</v>
+        <v>3810.48</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.1062</v>
+        <v>13.0771</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110779.49</v>
+        <v>110906.29</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111265.48</v>
+        <v>111392.83</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111022.48</v>
+        <v>111149.56</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.1062</v>
+        <v>13.0771</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77688.17999999999</v>
+        <v>77777.10000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77135.46000000001</v>
+        <v>77223.75</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77411.82000000001</v>
+        <v>77500.42999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.1062</v>
+        <v>13.0771</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47009.22</v>
+        <v>47063.02</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48133.15</v>
+        <v>48188.24</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47571.18</v>
+        <v>47625.63</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.1062</v>
+        <v>13.0771</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29204.9</v>
+        <v>29238.32</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29096.06</v>
+        <v>29129.36</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29150.48</v>
+        <v>29183.84</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.1062</v>
+        <v>13.0771</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14326.64</v>
+        <v>14343.04</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14450.85</v>
+        <v>14467.39</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14388.74</v>
+        <v>14405.21</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.1062</v>
+        <v>13.0771</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6641.84</v>
+        <v>6649.44</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6477.75</v>
+        <v>6485.17</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6559.79</v>
+        <v>6567.3</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.06</v>
+        <v>13.0312</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50451.6</v>
+        <v>50510.21</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50113.84</v>
+        <v>50172.05</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50282.72</v>
+        <v>50341.13</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.06</v>
+        <v>13.0312</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44383.94</v>
+        <v>44435.49</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44580.98</v>
+        <v>44632.77</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44482.46</v>
+        <v>44534.13</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.06</v>
+        <v>13.0312</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32482.37</v>
+        <v>32520.1</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32828.29</v>
+        <v>32866.43</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32655.33</v>
+        <v>32693.26</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.06</v>
+        <v>13.0312</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22839.28</v>
+        <v>22865.81</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22996.13</v>
+        <v>23022.85</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22917.71</v>
+        <v>22944.33</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.06</v>
+        <v>13.0312</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14679.53</v>
+        <v>14696.58</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14888.43</v>
+        <v>14905.72</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14783.98</v>
+        <v>14801.15</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.06</v>
+        <v>13.0312</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8436.34</v>
+        <v>8446.139999999999</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8492.23</v>
+        <v>8502.1</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8464.290000000001</v>
+        <v>8474.120000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.0116</v>
+        <v>12.9832</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49672.7</v>
+        <v>49731.26</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48941.65</v>
+        <v>48999.35</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49307.18</v>
+        <v>49365.31</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.0116</v>
+        <v>12.9832</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44482.61</v>
+        <v>44535.05</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44140.89</v>
+        <v>44192.93</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44311.75</v>
+        <v>44363.99</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.0116</v>
+        <v>12.9832</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32125.36</v>
+        <v>32163.23</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31547.85</v>
+        <v>31585.04</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31836.6</v>
+        <v>31874.14</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.0116</v>
+        <v>12.9832</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23944.05</v>
+        <v>23972.27</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23837.29</v>
+        <v>23865.39</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23890.67</v>
+        <v>23918.83</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.0116</v>
+        <v>12.9832</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18783.8</v>
+        <v>18805.94</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18595.03</v>
+        <v>18616.95</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18689.41</v>
+        <v>18711.45</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.0116</v>
+        <v>12.9832</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15798.46</v>
+        <v>15817.08</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15742.05</v>
+        <v>15760.61</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15770.25</v>
+        <v>15788.84</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.9675</v>
+        <v>12.9395</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110439.2</v>
+        <v>110571.08</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110998.48</v>
+        <v>111131.04</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110718.84</v>
+        <v>110851.06</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.9675</v>
+        <v>12.9395</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79196.72</v>
+        <v>79291.28999999999</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79516.87</v>
+        <v>79611.83</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79356.78999999999</v>
+        <v>79451.56</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.9675</v>
+        <v>12.9395</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51734.68</v>
+        <v>51796.46</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51295.31</v>
+        <v>51356.56</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51515</v>
+        <v>51576.51</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.9675</v>
+        <v>12.9395</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29743.92</v>
+        <v>29779.44</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29529.61</v>
+        <v>29564.87</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29636.76</v>
+        <v>29672.16</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.9675</v>
+        <v>12.9395</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16903.17</v>
+        <v>16923.36</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16836.38</v>
+        <v>16856.48</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16869.77</v>
+        <v>16889.92</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.9675</v>
+        <v>12.9395</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6853.17</v>
+        <v>6861.35</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6636.31</v>
+        <v>6644.24</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6744.74</v>
+        <v>6752.8</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.9229</v>
+        <v>12.8936</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>359687.12</v>
+        <v>360127.25</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355236.9</v>
+        <v>355671.58</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357462.01</v>
+        <v>357899.41</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.9229</v>
+        <v>12.8936</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270027.73</v>
+        <v>270358.15</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>270903.49</v>
+        <v>271234.98</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270465.61</v>
+        <v>270796.56</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.9229</v>
+        <v>12.8936</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>188939.23</v>
+        <v>189170.43</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>188825.25</v>
+        <v>189056.31</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>188882.24</v>
+        <v>189113.37</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.9229</v>
+        <v>12.8936</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114864.06</v>
+        <v>115004.61</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115117.23</v>
+        <v>115258.09</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>114990.64</v>
+        <v>115131.35</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.9229</v>
+        <v>12.8936</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55676.09</v>
+        <v>55744.22</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55415.99</v>
+        <v>55483.8</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55546.04</v>
+        <v>55614.01</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.9229</v>
+        <v>12.8936</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28434.7</v>
+        <v>28469.49</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28456.17</v>
+        <v>28490.99</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28445.44</v>
+        <v>28480.24</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5995</v>
+        <v>13.5725</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>411547.55</v>
+        <v>411969.29</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>412100.72</v>
+        <v>412523.02</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>411824.13</v>
+        <v>412246.16</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5995</v>
+        <v>13.5725</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>305487.37</v>
+        <v>305800.42</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>303579.94</v>
+        <v>303891.03</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>304533.65</v>
+        <v>304845.73</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5995</v>
+        <v>13.5725</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207212.36</v>
+        <v>207424.7</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207283.24</v>
+        <v>207495.66</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207247.8</v>
+        <v>207460.18</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5995</v>
+        <v>13.5725</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125391.4</v>
+        <v>125519.89</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>125914.21</v>
+        <v>126043.24</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125652.8</v>
+        <v>125781.57</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5995</v>
+        <v>13.5725</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50075.74</v>
+        <v>50127.05</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50016.06</v>
+        <v>50067.32</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50045.9</v>
+        <v>50097.18</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5995</v>
+        <v>13.5725</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5508.17</v>
+        <v>5513.81</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5544.49</v>
+        <v>5550.17</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5526.33</v>
+        <v>5531.99</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5326</v>
+        <v>13.5139</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>171866.12</v>
+        <v>172043.06</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>171893.61</v>
+        <v>172070.57</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>171879.87</v>
+        <v>172056.82</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5326</v>
+        <v>13.5139</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>112944.58</v>
+        <v>113060.86</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112551.67</v>
+        <v>112667.54</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112748.13</v>
+        <v>112864.2</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5326</v>
+        <v>13.5139</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63253.95</v>
+        <v>63319.07</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63612.73</v>
+        <v>63678.22</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63433.34</v>
+        <v>63498.64</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5326</v>
+        <v>13.5139</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27079.63</v>
+        <v>27107.51</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27281.37</v>
+        <v>27309.46</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27180.5</v>
+        <v>27208.48</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5326</v>
+        <v>13.5139</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6374.26</v>
+        <v>6380.82</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6527.49</v>
+        <v>6534.21</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6450.87</v>
+        <v>6457.51</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5326</v>
+        <v>13.5139</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3775.17</v>
+        <v>3779.06</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3768.62</v>
+        <v>3772.5</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3771.89</v>
+        <v>3775.78</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4302</v>
+        <v>13.4084</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192248.48</v>
+        <v>192449.07</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193187.2</v>
+        <v>193388.77</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192717.84</v>
+        <v>192918.92</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4302</v>
+        <v>13.4084</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139384.21</v>
+        <v>139529.65</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140356.88</v>
+        <v>140503.33</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>139870.55</v>
+        <v>140016.49</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4302</v>
+        <v>13.4084</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88104.78999999999</v>
+        <v>88196.72</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88817.78999999999</v>
+        <v>88910.46000000001</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88461.28999999999</v>
+        <v>88553.59</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4302</v>
+        <v>13.4084</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42084.34</v>
+        <v>42128.25</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42016.85</v>
+        <v>42060.69</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42050.6</v>
+        <v>42094.47</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4302</v>
+        <v>13.4084</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13123.32</v>
+        <v>13137.01</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12978.77</v>
+        <v>12992.31</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13051.04</v>
+        <v>13064.66</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4302</v>
+        <v>13.4084</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4554.61</v>
+        <v>4559.36</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4443.43</v>
+        <v>4448.06</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4499.02</v>
+        <v>4503.71</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-21
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3244</v>
+        <v>13.3032</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151694.55</v>
+        <v>151778.54</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153606.99</v>
+        <v>153692.03</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152650.77</v>
+        <v>152735.29</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3244</v>
+        <v>13.3032</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116112.31</v>
+        <v>116176.6</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116901.76</v>
+        <v>116966.49</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116507.04</v>
+        <v>116571.55</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3244</v>
+        <v>13.3032</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82790.8</v>
+        <v>82836.64</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83306.69</v>
+        <v>83352.81</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83048.74000000001</v>
+        <v>83094.72</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3244</v>
+        <v>13.3032</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58665.54</v>
+        <v>58698.02</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58220.92</v>
+        <v>58253.16</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58443.23</v>
+        <v>58475.59</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3244</v>
+        <v>13.3032</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37895.61</v>
+        <v>37916.59</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38205.61</v>
+        <v>38226.76</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38050.61</v>
+        <v>38071.68</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3244</v>
+        <v>13.3032</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17235.63</v>
+        <v>17245.17</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17122.45</v>
+        <v>17131.93</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17179.04</v>
+        <v>17188.55</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.2535</v>
+        <v>13.2225</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164851.25</v>
+        <v>164950.05</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>163966.68</v>
+        <v>164064.96</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164408.96</v>
+        <v>164507.5</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.2535</v>
+        <v>13.2225</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123803.79</v>
+        <v>123877.99</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122055.24</v>
+        <v>122128.39</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122929.51</v>
+        <v>123003.19</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.2535</v>
+        <v>13.2225</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88450.11</v>
+        <v>88503.12</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87354.83</v>
+        <v>87407.19</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87902.47</v>
+        <v>87955.16</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.2535</v>
+        <v>13.2225</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67376.81</v>
+        <v>67417.2</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66903.17</v>
+        <v>66943.27</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67139.99000000001</v>
+        <v>67180.23</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.2535</v>
+        <v>13.2225</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52635.86</v>
+        <v>52667.41</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50744.18</v>
+        <v>50774.59</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51690.02</v>
+        <v>51721</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.2535</v>
+        <v>13.2225</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39900.83</v>
+        <v>39924.75</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40886.8</v>
+        <v>40911.31</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40393.82</v>
+        <v>40418.03</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.1755</v>
+        <v>13.1337</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169806.05</v>
+        <v>169919.06</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171370.24</v>
+        <v>171484.3</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170588.15</v>
+        <v>170701.68</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.1755</v>
+        <v>13.1337</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122406.51</v>
+        <v>122487.97</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120943.49</v>
+        <v>121023.98</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121675</v>
+        <v>121755.98</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.1755</v>
+        <v>13.1337</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83850.39</v>
+        <v>83906.2</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83533.69</v>
+        <v>83589.28</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83692.03999999999</v>
+        <v>83747.74000000001</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.1755</v>
+        <v>13.1337</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55865.16</v>
+        <v>55902.33</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56173.4</v>
+        <v>56210.79</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56019.28</v>
+        <v>56056.56</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.1755</v>
+        <v>13.1337</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33717.47</v>
+        <v>33739.91</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33322.82</v>
+        <v>33345</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33520.14</v>
+        <v>33542.45</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.1755</v>
+        <v>13.1337</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17504.68</v>
+        <v>17516.33</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18198.65</v>
+        <v>18210.76</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17851.66</v>
+        <v>17863.55</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.1208</v>
+        <v>13.069</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131292.52</v>
+        <v>131390.45</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131388.72</v>
+        <v>131486.73</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131340.62</v>
+        <v>131438.59</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.1208</v>
+        <v>13.069</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90926.95</v>
+        <v>90994.77</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89516.02</v>
+        <v>89582.8</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90221.49000000001</v>
+        <v>90288.78</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.1208</v>
+        <v>13.069</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57152.69</v>
+        <v>57195.32</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57444.37</v>
+        <v>57487.21</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57298.53</v>
+        <v>57341.27</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.1208</v>
+        <v>13.069</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30256.68</v>
+        <v>30279.25</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30460.34</v>
+        <v>30483.06</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30358.51</v>
+        <v>30381.15</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.1208</v>
+        <v>13.069</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6939.62</v>
+        <v>6944.79</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6938.29</v>
+        <v>6943.47</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6938.95</v>
+        <v>6944.13</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.1208</v>
+        <v>13.069</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3855.96</v>
+        <v>3858.83</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3765.01</v>
+        <v>3767.82</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3810.48</v>
+        <v>3813.33</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.0771</v>
+        <v>13.0179</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110906.29</v>
+        <v>110997.7</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111392.83</v>
+        <v>111484.65</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111149.56</v>
+        <v>111241.18</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.0771</v>
+        <v>13.0179</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77777.10000000001</v>
+        <v>77841.21000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77223.75</v>
+        <v>77287.39999999999</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77500.42999999999</v>
+        <v>77564.31</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.0771</v>
+        <v>13.0179</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47063.02</v>
+        <v>47101.82</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48188.24</v>
+        <v>48227.96</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47625.63</v>
+        <v>47664.89</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.0771</v>
+        <v>13.0179</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29238.32</v>
+        <v>29262.42</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29129.36</v>
+        <v>29153.37</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29183.84</v>
+        <v>29207.9</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.0771</v>
+        <v>13.0179</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14343.04</v>
+        <v>14354.86</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14467.39</v>
+        <v>14479.31</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14405.21</v>
+        <v>14417.08</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.0771</v>
+        <v>13.0179</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6649.44</v>
+        <v>6654.92</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6485.17</v>
+        <v>6490.51</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6567.3</v>
+        <v>6572.71</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.0312</v>
+        <v>12.9644</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50510.21</v>
+        <v>50556.58</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50172.05</v>
+        <v>50218.11</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50341.13</v>
+        <v>50387.34</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.0312</v>
+        <v>12.9644</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44435.49</v>
+        <v>44476.29</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44632.77</v>
+        <v>44673.74</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44534.13</v>
+        <v>44575.01</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.0312</v>
+        <v>12.9644</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32520.1</v>
+        <v>32549.95</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32866.43</v>
+        <v>32896.6</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32693.26</v>
+        <v>32723.27</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.0312</v>
+        <v>12.9644</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22865.81</v>
+        <v>22886.8</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>23022.85</v>
+        <v>23043.98</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22944.33</v>
+        <v>22965.39</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.0312</v>
+        <v>12.9644</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14696.58</v>
+        <v>14710.08</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14905.72</v>
+        <v>14919.41</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14801.15</v>
+        <v>14814.74</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.0312</v>
+        <v>12.9644</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8446.139999999999</v>
+        <v>8453.889999999999</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8502.1</v>
+        <v>8509.9</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8474.120000000001</v>
+        <v>8481.9</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.9832</v>
+        <v>12.9085</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49731.26</v>
+        <v>49782.42</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48999.35</v>
+        <v>49049.76</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49365.31</v>
+        <v>49416.09</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.9832</v>
+        <v>12.9085</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44535.05</v>
+        <v>44580.86</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44192.93</v>
+        <v>44238.4</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44363.99</v>
+        <v>44409.63</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.9832</v>
+        <v>12.9085</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32163.23</v>
+        <v>32196.32</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31585.04</v>
+        <v>31617.53</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31874.14</v>
+        <v>31906.93</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.9832</v>
+        <v>12.9085</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23972.27</v>
+        <v>23996.94</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23865.39</v>
+        <v>23889.94</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23918.83</v>
+        <v>23943.44</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.9832</v>
+        <v>12.9085</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18805.94</v>
+        <v>18825.29</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18616.95</v>
+        <v>18636.11</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18711.45</v>
+        <v>18730.7</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.9832</v>
+        <v>12.9085</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15817.08</v>
+        <v>15833.35</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15760.61</v>
+        <v>15776.82</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15788.84</v>
+        <v>15805.09</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.9395</v>
+        <v>12.8574</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110571.08</v>
+        <v>110697.27</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111131.04</v>
+        <v>111257.86</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110851.06</v>
+        <v>110977.57</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.9395</v>
+        <v>12.8574</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79291.28999999999</v>
+        <v>79381.78</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79611.83</v>
+        <v>79702.69</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79451.56</v>
+        <v>79542.23</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.9395</v>
+        <v>12.8574</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51796.46</v>
+        <v>51855.58</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51356.56</v>
+        <v>51415.17</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51576.51</v>
+        <v>51635.37</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.9395</v>
+        <v>12.8574</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29779.44</v>
+        <v>29813.43</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29564.87</v>
+        <v>29598.61</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29672.16</v>
+        <v>29706.02</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.9395</v>
+        <v>12.8574</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16923.36</v>
+        <v>16942.67</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16856.48</v>
+        <v>16875.72</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16889.92</v>
+        <v>16909.19</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.9395</v>
+        <v>12.8574</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6861.35</v>
+        <v>6869.19</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6644.24</v>
+        <v>6651.82</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6752.8</v>
+        <v>6760.5</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.8936</v>
+        <v>12.8039</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360127.25</v>
+        <v>360584.89</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>355671.58</v>
+        <v>356123.57</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>357899.41</v>
+        <v>358354.23</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.8936</v>
+        <v>12.8039</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270358.15</v>
+        <v>270701.72</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271234.98</v>
+        <v>271579.66</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>270796.56</v>
+        <v>271140.69</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.8936</v>
+        <v>12.8039</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189170.43</v>
+        <v>189410.83</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189056.31</v>
+        <v>189296.56</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189113.37</v>
+        <v>189353.69</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.8936</v>
+        <v>12.8039</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>115004.61</v>
+        <v>115150.76</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115258.09</v>
+        <v>115404.56</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115131.35</v>
+        <v>115277.66</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.8936</v>
+        <v>12.8039</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55744.22</v>
+        <v>55815.06</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55483.8</v>
+        <v>55554.31</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55614.01</v>
+        <v>55684.69</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.8936</v>
+        <v>12.8039</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28469.49</v>
+        <v>28505.67</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28490.99</v>
+        <v>28527.2</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28480.24</v>
+        <v>28516.44</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5725</v>
+        <v>13.5794</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>411969.29</v>
+        <v>412176.21</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>412523.02</v>
+        <v>412730.23</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>412246.16</v>
+        <v>412453.22</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5725</v>
+        <v>13.5794</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>305800.42</v>
+        <v>305954.02</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>303891.03</v>
+        <v>304043.67</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>304845.73</v>
+        <v>304998.84</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5725</v>
+        <v>13.5794</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207424.7</v>
+        <v>207528.88</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207495.66</v>
+        <v>207599.88</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207460.18</v>
+        <v>207564.38</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5725</v>
+        <v>13.5794</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125519.89</v>
+        <v>125582.94</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126043.24</v>
+        <v>126106.55</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125781.57</v>
+        <v>125844.74</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5725</v>
+        <v>13.5794</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50127.05</v>
+        <v>50152.23</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50067.32</v>
+        <v>50092.47</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50097.18</v>
+        <v>50122.35</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5725</v>
+        <v>13.5794</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5513.81</v>
+        <v>5516.58</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5550.17</v>
+        <v>5552.96</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5531.99</v>
+        <v>5534.77</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.519</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172043.06</v>
+        <v>172128.64</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172070.57</v>
+        <v>172156.17</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172056.82</v>
+        <v>172142.4</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.519</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113060.86</v>
+        <v>113117.1</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112667.54</v>
+        <v>112723.59</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112864.2</v>
+        <v>112920.34</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.519</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63319.07</v>
+        <v>63350.57</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63678.22</v>
+        <v>63709.9</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63498.64</v>
+        <v>63530.23</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.519</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27107.51</v>
+        <v>27120.99</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27309.46</v>
+        <v>27323.04</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27208.48</v>
+        <v>27222.02</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.519</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6380.82</v>
+        <v>6383.99</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6534.21</v>
+        <v>6537.46</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6457.51</v>
+        <v>6460.72</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.519</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3779.06</v>
+        <v>3780.94</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3772.5</v>
+        <v>3774.38</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3775.78</v>
+        <v>3777.66</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4084</v>
+        <v>13.3994</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192449.07</v>
+        <v>192548.5</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193388.77</v>
+        <v>193488.68</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>192918.92</v>
+        <v>193018.59</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4084</v>
+        <v>13.3994</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139529.65</v>
+        <v>139601.73</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140503.33</v>
+        <v>140575.92</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140016.49</v>
+        <v>140088.83</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4084</v>
+        <v>13.3994</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88196.72</v>
+        <v>88242.28</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88910.46000000001</v>
+        <v>88956.39</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88553.59</v>
+        <v>88599.34</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4084</v>
+        <v>13.3994</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42128.25</v>
+        <v>42150.02</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42060.69</v>
+        <v>42082.42</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42094.47</v>
+        <v>42116.22</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4084</v>
+        <v>13.3994</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13137.01</v>
+        <v>13143.8</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12992.31</v>
+        <v>12999.02</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13064.66</v>
+        <v>13071.41</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4084</v>
+        <v>13.3994</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4559.36</v>
+        <v>4561.72</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4448.06</v>
+        <v>4450.36</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4503.71</v>
+        <v>4506.04</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-22
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3032</v>
+        <v>13.2997</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151778.54</v>
+        <v>151855.19</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153692.03</v>
+        <v>153769.65</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152735.29</v>
+        <v>152812.42</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3032</v>
+        <v>13.2997</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116176.6</v>
+        <v>116235.27</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>116966.49</v>
+        <v>117025.56</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116571.55</v>
+        <v>116630.41</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3032</v>
+        <v>13.2997</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82836.64</v>
+        <v>82878.47</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83352.81</v>
+        <v>83394.89999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83094.72</v>
+        <v>83136.69</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3032</v>
+        <v>13.2997</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58698.02</v>
+        <v>58727.66</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58253.16</v>
+        <v>58282.57</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58475.59</v>
+        <v>58505.12</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3032</v>
+        <v>13.2997</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37916.59</v>
+        <v>37935.74</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38226.76</v>
+        <v>38246.07</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38071.68</v>
+        <v>38090.9</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3032</v>
+        <v>13.2997</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17245.17</v>
+        <v>17253.88</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17131.93</v>
+        <v>17140.58</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17188.55</v>
+        <v>17197.23</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.2225</v>
+        <v>13.22</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164950.05</v>
+        <v>165032.77</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164064.96</v>
+        <v>164147.23</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164507.5</v>
+        <v>164590</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.2225</v>
+        <v>13.22</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123877.99</v>
+        <v>123940.11</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122128.39</v>
+        <v>122189.64</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>123003.19</v>
+        <v>123064.88</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.2225</v>
+        <v>13.22</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88503.12</v>
+        <v>88547.50999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87407.19</v>
+        <v>87451.02</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87955.16</v>
+        <v>87999.25999999999</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.2225</v>
+        <v>13.22</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67417.2</v>
+        <v>67451.00999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66943.27</v>
+        <v>66976.84</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67180.23</v>
+        <v>67213.92</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.2225</v>
+        <v>13.22</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52667.41</v>
+        <v>52693.82</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50774.59</v>
+        <v>50800.05</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51721</v>
+        <v>51746.94</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.2225</v>
+        <v>13.22</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39924.75</v>
+        <v>39944.77</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40911.31</v>
+        <v>40931.83</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40418.03</v>
+        <v>40438.3</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.1337</v>
+        <v>13.1322</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169919.06</v>
+        <v>170003.36</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171484.3</v>
+        <v>171569.38</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170701.68</v>
+        <v>170786.37</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.1337</v>
+        <v>13.1322</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122487.97</v>
+        <v>122548.75</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>121023.98</v>
+        <v>121084.03</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121755.98</v>
+        <v>121816.39</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.1337</v>
+        <v>13.1322</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83906.2</v>
+        <v>83947.83</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83589.28</v>
+        <v>83630.75</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83747.74000000001</v>
+        <v>83789.28999999999</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.1337</v>
+        <v>13.1322</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55902.33</v>
+        <v>55930.07</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56210.79</v>
+        <v>56238.67</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56056.56</v>
+        <v>56084.37</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.1337</v>
+        <v>13.1322</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33739.91</v>
+        <v>33756.65</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33345</v>
+        <v>33361.54</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33542.45</v>
+        <v>33559.1</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.1337</v>
+        <v>13.1322</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17516.33</v>
+        <v>17525.02</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18210.76</v>
+        <v>18219.8</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17863.55</v>
+        <v>17872.41</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.069</v>
+        <v>13.0663</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131390.45</v>
+        <v>131456.27</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131486.73</v>
+        <v>131552.59</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131438.59</v>
+        <v>131504.43</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.069</v>
+        <v>13.0663</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90994.77</v>
+        <v>91040.35000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89582.8</v>
+        <v>89627.67</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90288.78</v>
+        <v>90334.00999999999</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.069</v>
+        <v>13.0663</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57195.32</v>
+        <v>57223.97</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57487.21</v>
+        <v>57516.01</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57341.27</v>
+        <v>57369.99</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.069</v>
+        <v>13.0663</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30279.25</v>
+        <v>30294.41</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30483.06</v>
+        <v>30498.33</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30381.15</v>
+        <v>30396.37</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.069</v>
+        <v>13.0663</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6944.79</v>
+        <v>6948.27</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6943.47</v>
+        <v>6946.95</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6944.13</v>
+        <v>6947.61</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.069</v>
+        <v>13.0663</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3858.83</v>
+        <v>3860.77</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3767.82</v>
+        <v>3769.71</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3813.33</v>
+        <v>3815.24</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.0179</v>
+        <v>13.0153</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110997.7</v>
+        <v>111053.29</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111484.65</v>
+        <v>111540.48</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111241.18</v>
+        <v>111296.88</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.0179</v>
+        <v>13.0153</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77841.21000000001</v>
+        <v>77880.19</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77287.39999999999</v>
+        <v>77326.11</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77564.31</v>
+        <v>77603.14999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.0179</v>
+        <v>13.0153</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47101.82</v>
+        <v>47125.4</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48227.96</v>
+        <v>48252.11</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47664.89</v>
+        <v>47688.76</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.0179</v>
+        <v>13.0153</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29262.42</v>
+        <v>29277.08</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29153.37</v>
+        <v>29167.97</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29207.9</v>
+        <v>29222.52</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.0179</v>
+        <v>13.0153</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14354.86</v>
+        <v>14362.05</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14479.31</v>
+        <v>14486.56</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14417.08</v>
+        <v>14424.3</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.0179</v>
+        <v>13.0153</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6654.92</v>
+        <v>6658.25</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6490.51</v>
+        <v>6493.76</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6572.71</v>
+        <v>6576.01</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.9644</v>
+        <v>12.9618</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50556.58</v>
+        <v>50581.88</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50218.11</v>
+        <v>50243.24</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50387.34</v>
+        <v>50412.56</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.9644</v>
+        <v>12.9618</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44476.29</v>
+        <v>44498.55</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44673.74</v>
+        <v>44696.1</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44575.01</v>
+        <v>44597.32</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.9644</v>
+        <v>12.9618</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32549.95</v>
+        <v>32566.24</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32896.6</v>
+        <v>32913.06</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32723.27</v>
+        <v>32739.65</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.9644</v>
+        <v>12.9618</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22886.8</v>
+        <v>22898.26</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>23043.98</v>
+        <v>23055.51</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22965.39</v>
+        <v>22976.89</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.9644</v>
+        <v>12.9618</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14710.08</v>
+        <v>14717.44</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14919.41</v>
+        <v>14926.87</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14814.74</v>
+        <v>14822.16</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.9644</v>
+        <v>12.9618</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8453.889999999999</v>
+        <v>8458.120000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8509.9</v>
+        <v>8514.16</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8481.9</v>
+        <v>8486.139999999999</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.9085</v>
+        <v>12.906</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49782.42</v>
+        <v>49807.32</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>49049.76</v>
+        <v>49074.29</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49416.09</v>
+        <v>49440.8</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.9085</v>
+        <v>12.906</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44580.86</v>
+        <v>44603.16</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44238.4</v>
+        <v>44260.52</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44409.63</v>
+        <v>44431.84</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.9085</v>
+        <v>12.906</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32196.32</v>
+        <v>32212.42</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31617.53</v>
+        <v>31633.35</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31906.93</v>
+        <v>31922.88</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.9085</v>
+        <v>12.906</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23996.94</v>
+        <v>24008.94</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23889.94</v>
+        <v>23901.89</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23943.44</v>
+        <v>23955.41</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.9085</v>
+        <v>12.906</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18825.29</v>
+        <v>18834.7</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18636.11</v>
+        <v>18645.43</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18730.7</v>
+        <v>18740.06</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.9085</v>
+        <v>12.906</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15833.35</v>
+        <v>15841.27</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15776.82</v>
+        <v>15784.71</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15805.09</v>
+        <v>15812.99</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.8574</v>
+        <v>12.8549</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110697.27</v>
+        <v>110752.58</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111257.86</v>
+        <v>111313.45</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110977.57</v>
+        <v>111033.01</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.8574</v>
+        <v>12.8549</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79381.78</v>
+        <v>79421.45</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79702.69</v>
+        <v>79742.50999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79542.23</v>
+        <v>79581.98</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.8574</v>
+        <v>12.8549</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51855.58</v>
+        <v>51881.49</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51415.17</v>
+        <v>51440.86</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51635.37</v>
+        <v>51661.17</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.8574</v>
+        <v>12.8549</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29813.43</v>
+        <v>29828.32</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29598.61</v>
+        <v>29613.4</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29706.02</v>
+        <v>29720.86</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.8574</v>
+        <v>12.8549</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16942.67</v>
+        <v>16951.13</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16875.72</v>
+        <v>16884.15</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16909.19</v>
+        <v>16917.64</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.8574</v>
+        <v>12.8549</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6869.19</v>
+        <v>6872.62</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6651.82</v>
+        <v>6655.14</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6760.5</v>
+        <v>6763.88</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.8039</v>
+        <v>12.8015</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360584.89</v>
+        <v>360764.84</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>356123.57</v>
+        <v>356301.29</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>358354.23</v>
+        <v>358533.07</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.8039</v>
+        <v>12.8015</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270701.72</v>
+        <v>270836.81</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271579.66</v>
+        <v>271715.19</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>271140.69</v>
+        <v>271276</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.8039</v>
+        <v>12.8015</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189410.83</v>
+        <v>189505.35</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189296.56</v>
+        <v>189391.03</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189353.69</v>
+        <v>189448.19</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.8039</v>
+        <v>12.8015</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>115150.76</v>
+        <v>115208.22</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115404.56</v>
+        <v>115462.15</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115277.66</v>
+        <v>115335.19</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.8039</v>
+        <v>12.8015</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55815.06</v>
+        <v>55842.92</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55554.31</v>
+        <v>55582.04</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55684.69</v>
+        <v>55712.48</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.8039</v>
+        <v>12.8015</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28505.67</v>
+        <v>28519.9</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28527.2</v>
+        <v>28541.44</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28516.44</v>
+        <v>28530.67</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5794</v>
+        <v>13.5679</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>412176.21</v>
+        <v>412386.35</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>412730.23</v>
+        <v>412940.65</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>412453.22</v>
+        <v>412663.5</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5794</v>
+        <v>13.5679</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>305954.02</v>
+        <v>306110</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>304043.67</v>
+        <v>304198.68</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>304998.84</v>
+        <v>305154.34</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5794</v>
+        <v>13.5679</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207528.88</v>
+        <v>207634.69</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207599.88</v>
+        <v>207705.72</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207564.38</v>
+        <v>207670.21</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5794</v>
+        <v>13.5679</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125582.94</v>
+        <v>125646.97</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126106.55</v>
+        <v>126170.84</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125844.74</v>
+        <v>125908.9</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5794</v>
+        <v>13.5679</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50152.23</v>
+        <v>50177.8</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50092.47</v>
+        <v>50118.01</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50122.35</v>
+        <v>50147.9</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5794</v>
+        <v>13.5679</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5516.58</v>
+        <v>5519.4</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5552.96</v>
+        <v>5555.79</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5534.77</v>
+        <v>5537.59</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5139</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172128.64</v>
+        <v>172216.22</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172156.17</v>
+        <v>172243.77</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172142.4</v>
+        <v>172229.99</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5139</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113117.1</v>
+        <v>113174.65</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112723.59</v>
+        <v>112780.94</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112920.34</v>
+        <v>112977.8</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5139</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63350.57</v>
+        <v>63382.8</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63709.9</v>
+        <v>63742.31</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63530.23</v>
+        <v>63562.56</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5139</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27120.99</v>
+        <v>27134.79</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27323.04</v>
+        <v>27336.95</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27222.02</v>
+        <v>27235.87</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5139</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6383.99</v>
+        <v>6387.24</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6537.46</v>
+        <v>6540.78</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6460.72</v>
+        <v>6464.01</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.519</v>
+        <v>13.5139</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3780.94</v>
+        <v>3782.86</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3774.38</v>
+        <v>3776.3</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3777.66</v>
+        <v>3779.58</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3994</v>
+        <v>13.3957</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192548.5</v>
+        <v>192645.98</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193488.68</v>
+        <v>193586.64</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193018.59</v>
+        <v>193116.31</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3994</v>
+        <v>13.3957</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139601.73</v>
+        <v>139672.41</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140575.92</v>
+        <v>140647.09</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140088.83</v>
+        <v>140159.75</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3994</v>
+        <v>13.3957</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88242.28</v>
+        <v>88286.96000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>88956.39</v>
+        <v>89001.42999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88599.34</v>
+        <v>88644.19</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3994</v>
+        <v>13.3957</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42150.02</v>
+        <v>42171.36</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42082.42</v>
+        <v>42103.73</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42116.22</v>
+        <v>42137.54</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3994</v>
+        <v>13.3957</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13143.8</v>
+        <v>13150.45</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12999.02</v>
+        <v>13005.6</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13071.41</v>
+        <v>13078.03</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3994</v>
+        <v>13.3957</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4561.72</v>
+        <v>4564.03</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4450.36</v>
+        <v>4452.62</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4506.04</v>
+        <v>4508.32</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-23
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2997</v>
+        <v>13.3306</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151855.19</v>
+        <v>151918.15</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153769.65</v>
+        <v>153833.4</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152812.42</v>
+        <v>152875.78</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2997</v>
+        <v>13.3306</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116235.27</v>
+        <v>116283.46</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>117025.56</v>
+        <v>117074.08</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116630.41</v>
+        <v>116678.77</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2997</v>
+        <v>13.3306</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82878.47</v>
+        <v>82912.83</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83394.89999999999</v>
+        <v>83429.48</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83136.69</v>
+        <v>83171.16</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2997</v>
+        <v>13.3306</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58727.66</v>
+        <v>58752.01</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58282.57</v>
+        <v>58306.74</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58505.12</v>
+        <v>58529.37</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2997</v>
+        <v>13.3306</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37935.74</v>
+        <v>37951.47</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38246.07</v>
+        <v>38261.92</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38090.9</v>
+        <v>38106.7</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2997</v>
+        <v>13.3306</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17253.88</v>
+        <v>17261.04</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17140.58</v>
+        <v>17147.69</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17197.23</v>
+        <v>17204.36</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.22</v>
+        <v>13.2623</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>165032.77</v>
+        <v>165090.81</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164147.23</v>
+        <v>164204.96</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164590</v>
+        <v>164647.89</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.22</v>
+        <v>13.2623</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123940.11</v>
+        <v>123983.7</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122189.64</v>
+        <v>122232.61</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>123064.88</v>
+        <v>123108.16</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.22</v>
+        <v>13.2623</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88547.50999999999</v>
+        <v>88578.64999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87451.02</v>
+        <v>87481.78</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87999.25999999999</v>
+        <v>88030.21000000001</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.22</v>
+        <v>13.2623</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67451.00999999999</v>
+        <v>67474.73</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66976.84</v>
+        <v>67000.39</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67213.92</v>
+        <v>67237.56</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.22</v>
+        <v>13.2623</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52693.82</v>
+        <v>52712.35</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50800.05</v>
+        <v>50817.92</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51746.94</v>
+        <v>51765.14</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.22</v>
+        <v>13.2623</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39944.77</v>
+        <v>39958.82</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40931.83</v>
+        <v>40946.22</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40438.3</v>
+        <v>40452.52</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.1322</v>
+        <v>13.1873</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>170003.36</v>
+        <v>170048.18</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171569.38</v>
+        <v>171614.61</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170786.37</v>
+        <v>170831.4</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.1322</v>
+        <v>13.1873</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122548.75</v>
+        <v>122581.06</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>121084.03</v>
+        <v>121115.95</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121816.39</v>
+        <v>121848.5</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.1322</v>
+        <v>13.1873</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83947.83</v>
+        <v>83969.96000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83630.75</v>
+        <v>83652.8</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83789.28999999999</v>
+        <v>83811.38</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.1322</v>
+        <v>13.1873</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55930.07</v>
+        <v>55944.82</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56238.67</v>
+        <v>56253.5</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56084.37</v>
+        <v>56099.16</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.1322</v>
+        <v>13.1873</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33756.65</v>
+        <v>33765.55</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33361.54</v>
+        <v>33370.34</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33559.1</v>
+        <v>33567.94</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.1322</v>
+        <v>13.1873</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17525.02</v>
+        <v>17529.64</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18219.8</v>
+        <v>18224.6</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17872.41</v>
+        <v>17877.12</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.0663</v>
+        <v>13.1292</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131456.27</v>
+        <v>131480.01</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131552.59</v>
+        <v>131576.35</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131504.43</v>
+        <v>131528.18</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.0663</v>
+        <v>13.1292</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>91040.35000000001</v>
+        <v>91056.78999999999</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89627.67</v>
+        <v>89643.85000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90334.00999999999</v>
+        <v>90350.32000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.0663</v>
+        <v>13.1292</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57223.97</v>
+        <v>57234.31</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57516.01</v>
+        <v>57526.4</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57369.99</v>
+        <v>57380.35</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.0663</v>
+        <v>13.1292</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30294.41</v>
+        <v>30299.88</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30498.33</v>
+        <v>30503.83</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30396.37</v>
+        <v>30401.86</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.0663</v>
+        <v>13.1292</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6948.27</v>
+        <v>6949.53</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6946.95</v>
+        <v>6948.2</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6947.61</v>
+        <v>6948.86</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.0663</v>
+        <v>13.1292</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3860.77</v>
+        <v>3861.46</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3769.71</v>
+        <v>3770.39</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3815.24</v>
+        <v>3815.93</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.0153</v>
+        <v>13.0849</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>111053.29</v>
+        <v>111063.78</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111540.48</v>
+        <v>111551.02</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111296.88</v>
+        <v>111307.4</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.0153</v>
+        <v>13.0849</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77880.19</v>
+        <v>77887.55</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77326.11</v>
+        <v>77333.41</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77603.14999999999</v>
+        <v>77610.48</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.0153</v>
+        <v>13.0849</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47125.4</v>
+        <v>47129.85</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48252.11</v>
+        <v>48256.67</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47688.76</v>
+        <v>47693.26</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.0153</v>
+        <v>13.0849</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29277.08</v>
+        <v>29279.84</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29167.97</v>
+        <v>29170.72</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29222.52</v>
+        <v>29225.28</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.0153</v>
+        <v>13.0849</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14362.05</v>
+        <v>14363.4</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14486.56</v>
+        <v>14487.93</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14424.3</v>
+        <v>14425.67</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.0153</v>
+        <v>13.0849</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6658.25</v>
+        <v>6658.88</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6493.76</v>
+        <v>6494.37</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6576.01</v>
+        <v>6576.63</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>12.9618</v>
+        <v>13.0385</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50581.88</v>
+        <v>50581.55</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50243.24</v>
+        <v>50242.92</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50412.56</v>
+        <v>50412.24</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>12.9618</v>
+        <v>13.0385</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44498.55</v>
+        <v>44498.26</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44696.1</v>
+        <v>44695.81</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44597.32</v>
+        <v>44597.03</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>12.9618</v>
+        <v>13.0385</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32566.24</v>
+        <v>32566.03</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32913.06</v>
+        <v>32912.85</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32739.65</v>
+        <v>32739.44</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>12.9618</v>
+        <v>13.0385</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22898.26</v>
+        <v>22898.11</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>23055.51</v>
+        <v>23055.37</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22976.89</v>
+        <v>22976.74</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>12.9618</v>
+        <v>13.0385</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14717.44</v>
+        <v>14717.34</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14926.87</v>
+        <v>14926.78</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14822.16</v>
+        <v>14822.06</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>12.9618</v>
+        <v>13.0385</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8458.120000000001</v>
+        <v>8458.07</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8514.16</v>
+        <v>8514.110000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8486.139999999999</v>
+        <v>8486.09</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.906</v>
+        <v>12.99</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49807.32</v>
+        <v>49801.16</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>49074.29</v>
+        <v>49068.21</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49440.8</v>
+        <v>49434.69</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.906</v>
+        <v>12.99</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44603.16</v>
+        <v>44597.64</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44260.52</v>
+        <v>44255.04</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44431.84</v>
+        <v>44426.34</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.906</v>
+        <v>12.99</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32212.42</v>
+        <v>32208.43</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31633.35</v>
+        <v>31629.43</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31922.88</v>
+        <v>31918.93</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.906</v>
+        <v>12.99</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>24008.94</v>
+        <v>24005.97</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23901.89</v>
+        <v>23898.93</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23955.41</v>
+        <v>23952.45</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.906</v>
+        <v>12.99</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18834.7</v>
+        <v>18832.37</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18645.43</v>
+        <v>18643.12</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18740.06</v>
+        <v>18737.75</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.906</v>
+        <v>12.99</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15841.27</v>
+        <v>15839.31</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15784.71</v>
+        <v>15782.76</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15812.99</v>
+        <v>15811.03</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.8549</v>
+        <v>12.9457</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110752.58</v>
+        <v>110725.85</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111313.45</v>
+        <v>111286.59</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>111033.01</v>
+        <v>111006.22</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.8549</v>
+        <v>12.9457</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79421.45</v>
+        <v>79402.28</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79742.50999999999</v>
+        <v>79723.27</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79581.98</v>
+        <v>79562.77</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.8549</v>
+        <v>12.9457</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51881.49</v>
+        <v>51868.97</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51440.86</v>
+        <v>51428.45</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51661.17</v>
+        <v>51648.71</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.8549</v>
+        <v>12.9457</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29828.32</v>
+        <v>29821.13</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29613.4</v>
+        <v>29606.25</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29720.86</v>
+        <v>29713.69</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.8549</v>
+        <v>12.9457</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16951.13</v>
+        <v>16947.04</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16884.15</v>
+        <v>16880.08</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16917.64</v>
+        <v>16913.56</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.8549</v>
+        <v>12.9457</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6872.62</v>
+        <v>6870.96</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6655.14</v>
+        <v>6653.54</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6763.88</v>
+        <v>6762.25</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.8015</v>
+        <v>12.8993</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360764.84</v>
+        <v>360629.48</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>356301.29</v>
+        <v>356167.6</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>358533.07</v>
+        <v>358398.54</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.8015</v>
+        <v>12.8993</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270836.81</v>
+        <v>270735.19</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271715.19</v>
+        <v>271613.24</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>271276</v>
+        <v>271174.22</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.8015</v>
+        <v>12.8993</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189505.35</v>
+        <v>189434.25</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189391.03</v>
+        <v>189319.97</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189448.19</v>
+        <v>189377.11</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.8015</v>
+        <v>12.8993</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>115208.22</v>
+        <v>115165</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115462.15</v>
+        <v>115418.83</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115335.19</v>
+        <v>115291.91</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.8015</v>
+        <v>12.8993</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55842.92</v>
+        <v>55821.96</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55582.04</v>
+        <v>55561.18</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55712.48</v>
+        <v>55691.57</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.8015</v>
+        <v>12.8993</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28519.9</v>
+        <v>28509.2</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28541.44</v>
+        <v>28530.73</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28530.67</v>
+        <v>28519.96</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5679</v>
+        <v>13.5554</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>412386.35</v>
+        <v>412596.42</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>412940.65</v>
+        <v>413150.99</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>412663.5</v>
+        <v>412873.7</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5679</v>
+        <v>13.5554</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>306110</v>
+        <v>306265.93</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>304198.68</v>
+        <v>304353.64</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>305154.34</v>
+        <v>305309.78</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5679</v>
+        <v>13.5554</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207634.69</v>
+        <v>207740.46</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207705.72</v>
+        <v>207811.52</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207670.21</v>
+        <v>207775.99</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5679</v>
+        <v>13.5554</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125646.97</v>
+        <v>125710.97</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126170.84</v>
+        <v>126235.11</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125908.9</v>
+        <v>125973.04</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5679</v>
+        <v>13.5554</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50177.8</v>
+        <v>50203.36</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50118.01</v>
+        <v>50143.53</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50147.9</v>
+        <v>50173.45</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5679</v>
+        <v>13.5554</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5519.4</v>
+        <v>5522.21</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5555.79</v>
+        <v>5558.62</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5537.59</v>
+        <v>5540.41</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.5141</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172216.22</v>
+        <v>172302.82</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172243.77</v>
+        <v>172330.38</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172229.99</v>
+        <v>172316.6</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.5141</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113174.65</v>
+        <v>113231.57</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112780.94</v>
+        <v>112837.66</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>112977.8</v>
+        <v>113034.61</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.5141</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63382.8</v>
+        <v>63414.68</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63742.31</v>
+        <v>63774.37</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63562.56</v>
+        <v>63594.52</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.5141</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27134.79</v>
+        <v>27148.44</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27336.95</v>
+        <v>27350.69</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27235.87</v>
+        <v>27249.56</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.5141</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6387.24</v>
+        <v>6390.45</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6540.78</v>
+        <v>6544.07</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6464.01</v>
+        <v>6467.26</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5139</v>
+        <v>13.5141</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3782.86</v>
+        <v>3784.76</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3776.3</v>
+        <v>3778.2</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3779.58</v>
+        <v>3781.48</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3957</v>
+        <v>13.4132</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192645.98</v>
+        <v>192735.84</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193586.64</v>
+        <v>193676.95</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193116.31</v>
+        <v>193206.4</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3957</v>
+        <v>13.4132</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139672.41</v>
+        <v>139737.56</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140647.09</v>
+        <v>140712.7</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140159.75</v>
+        <v>140225.13</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3957</v>
+        <v>13.4132</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88286.96000000001</v>
+        <v>88328.14</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>89001.42999999999</v>
+        <v>89042.95</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88644.19</v>
+        <v>88685.53999999999</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3957</v>
+        <v>13.4132</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42171.36</v>
+        <v>42191.03</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42103.73</v>
+        <v>42123.37</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42137.54</v>
+        <v>42157.2</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3957</v>
+        <v>13.4132</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13150.45</v>
+        <v>13156.59</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>13005.6</v>
+        <v>13011.67</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13078.03</v>
+        <v>13084.13</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3957</v>
+        <v>13.4132</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4564.03</v>
+        <v>4566.16</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4452.62</v>
+        <v>4454.69</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4508.32</v>
+        <v>4510.43</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-24
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3306</v>
+        <v>13.2952</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151918.15</v>
+        <v>151932.24</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153833.4</v>
+        <v>153847.68</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152875.78</v>
+        <v>152889.96</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3306</v>
+        <v>13.2952</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116283.46</v>
+        <v>116294.25</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>117074.08</v>
+        <v>117084.94</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116678.77</v>
+        <v>116689.6</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3306</v>
+        <v>13.2952</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82912.83</v>
+        <v>82920.52</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83429.48</v>
+        <v>83437.22</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83171.16</v>
+        <v>83178.87</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3306</v>
+        <v>13.2952</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58752.01</v>
+        <v>58757.46</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58306.74</v>
+        <v>58312.15</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58529.37</v>
+        <v>58534.8</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3306</v>
+        <v>13.2952</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37951.47</v>
+        <v>37954.99</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38261.92</v>
+        <v>38265.47</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38106.7</v>
+        <v>38110.23</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3306</v>
+        <v>13.2952</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17261.04</v>
+        <v>17262.64</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17147.69</v>
+        <v>17149.28</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17204.36</v>
+        <v>17205.96</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.2623</v>
+        <v>13.227</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>165090.81</v>
+        <v>165110.24</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164204.96</v>
+        <v>164224.29</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164647.89</v>
+        <v>164667.26</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.2623</v>
+        <v>13.227</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123983.7</v>
+        <v>123998.29</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122232.61</v>
+        <v>122247</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>123108.16</v>
+        <v>123122.64</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.2623</v>
+        <v>13.227</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88578.64999999999</v>
+        <v>88589.07000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87481.78</v>
+        <v>87492.07000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>88030.21000000001</v>
+        <v>88040.57000000001</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.2623</v>
+        <v>13.227</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67474.73</v>
+        <v>67482.67</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>67000.39</v>
+        <v>67008.28</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67237.56</v>
+        <v>67245.47</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.2623</v>
+        <v>13.227</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52712.35</v>
+        <v>52718.56</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50817.92</v>
+        <v>50823.9</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51765.14</v>
+        <v>51771.23</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.2623</v>
+        <v>13.227</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39958.82</v>
+        <v>39963.52</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40946.22</v>
+        <v>40951.04</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40452.52</v>
+        <v>40457.28</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.1873</v>
+        <v>13.1519</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>170048.18</v>
+        <v>170072.87</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171614.61</v>
+        <v>171639.53</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170831.4</v>
+        <v>170856.2</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.1873</v>
+        <v>13.1519</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122581.06</v>
+        <v>122598.85</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>121115.95</v>
+        <v>121133.53</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121848.5</v>
+        <v>121866.19</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.1873</v>
+        <v>13.1519</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83969.96000000001</v>
+        <v>83982.14999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83652.8</v>
+        <v>83664.95</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83811.38</v>
+        <v>83823.55</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.1873</v>
+        <v>13.1519</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55944.82</v>
+        <v>55952.94</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56253.5</v>
+        <v>56261.67</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56099.16</v>
+        <v>56107.3</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.1873</v>
+        <v>13.1519</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33765.55</v>
+        <v>33770.45</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33370.34</v>
+        <v>33375.18</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33567.94</v>
+        <v>33572.82</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.1873</v>
+        <v>13.1519</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17529.64</v>
+        <v>17532.18</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18224.6</v>
+        <v>18227.25</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17877.12</v>
+        <v>17879.72</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.1292</v>
+        <v>13.0939</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131480.01</v>
+        <v>131502.61</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131576.35</v>
+        <v>131598.97</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131528.18</v>
+        <v>131550.79</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.1292</v>
+        <v>13.0939</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>91056.78999999999</v>
+        <v>91072.45</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89643.85000000001</v>
+        <v>89659.27</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90350.32000000001</v>
+        <v>90365.86</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.1292</v>
+        <v>13.0939</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57234.31</v>
+        <v>57244.15</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57526.4</v>
+        <v>57536.29</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57380.35</v>
+        <v>57390.22</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.1292</v>
+        <v>13.0939</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30299.88</v>
+        <v>30305.09</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30503.83</v>
+        <v>30509.08</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30401.86</v>
+        <v>30407.09</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.1292</v>
+        <v>13.0939</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6949.53</v>
+        <v>6950.72</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6948.2</v>
+        <v>6949.4</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6948.86</v>
+        <v>6950.06</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.1292</v>
+        <v>13.0939</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3861.46</v>
+        <v>3862.13</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3770.39</v>
+        <v>3771.03</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3815.93</v>
+        <v>3816.58</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.0849</v>
+        <v>13.0499</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>111063.78</v>
+        <v>111085.62</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111551.02</v>
+        <v>111572.96</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111307.4</v>
+        <v>111329.29</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.0849</v>
+        <v>13.0499</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77887.55</v>
+        <v>77902.87</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77333.41</v>
+        <v>77348.62</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77610.48</v>
+        <v>77625.75</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.0849</v>
+        <v>13.0499</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47129.85</v>
+        <v>47139.12</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48256.67</v>
+        <v>48266.16</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47693.26</v>
+        <v>47702.64</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.0849</v>
+        <v>13.0499</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29279.84</v>
+        <v>29285.6</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29170.72</v>
+        <v>29176.46</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29225.28</v>
+        <v>29231.03</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.0849</v>
+        <v>13.0499</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14363.4</v>
+        <v>14366.23</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14487.93</v>
+        <v>14490.78</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14425.67</v>
+        <v>14428.5</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.0849</v>
+        <v>13.0499</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6658.88</v>
+        <v>6660.19</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6494.37</v>
+        <v>6495.65</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6576.63</v>
+        <v>6577.92</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.0385</v>
+        <v>13.0037</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50581.55</v>
+        <v>50592.79</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50242.92</v>
+        <v>50254.08</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50412.24</v>
+        <v>50423.44</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.0385</v>
+        <v>13.0037</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44498.26</v>
+        <v>44508.15</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44695.81</v>
+        <v>44705.75</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44597.03</v>
+        <v>44606.95</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.0385</v>
+        <v>13.0037</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32566.03</v>
+        <v>32573.27</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32912.85</v>
+        <v>32920.16</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32739.44</v>
+        <v>32746.72</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.0385</v>
+        <v>13.0037</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22898.11</v>
+        <v>22903.2</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>23055.37</v>
+        <v>23060.49</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22976.74</v>
+        <v>22981.84</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.0385</v>
+        <v>13.0037</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14717.34</v>
+        <v>14720.61</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14926.78</v>
+        <v>14930.09</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14822.06</v>
+        <v>14825.35</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.0385</v>
+        <v>13.0037</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8458.07</v>
+        <v>8459.950000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8514.110000000001</v>
+        <v>8516</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8486.09</v>
+        <v>8487.969999999999</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.99</v>
+        <v>12.9555</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49801.16</v>
+        <v>49813.54</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>49068.21</v>
+        <v>49080.41</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49434.69</v>
+        <v>49446.98</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.99</v>
+        <v>12.9555</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44597.64</v>
+        <v>44608.73</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44255.04</v>
+        <v>44266.04</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44426.34</v>
+        <v>44437.39</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.99</v>
+        <v>12.9555</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32208.43</v>
+        <v>32216.44</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31629.43</v>
+        <v>31637.3</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31918.93</v>
+        <v>31926.87</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.99</v>
+        <v>12.9555</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>24005.97</v>
+        <v>24011.93</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23898.93</v>
+        <v>23904.87</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23952.45</v>
+        <v>23958.4</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.99</v>
+        <v>12.9555</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18832.37</v>
+        <v>18837.05</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18643.12</v>
+        <v>18647.75</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18737.75</v>
+        <v>18742.4</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.99</v>
+        <v>12.9555</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15839.31</v>
+        <v>15843.25</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15782.76</v>
+        <v>15786.68</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15811.03</v>
+        <v>15814.97</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.9457</v>
+        <v>12.9114</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110725.85</v>
+        <v>110756.01</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111286.59</v>
+        <v>111316.9</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>111006.22</v>
+        <v>111036.45</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.9457</v>
+        <v>12.9114</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79402.28</v>
+        <v>79423.91</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79723.27</v>
+        <v>79744.98</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79562.77</v>
+        <v>79584.44</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.9457</v>
+        <v>12.9114</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51868.97</v>
+        <v>51883.09</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51428.45</v>
+        <v>51442.46</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51648.71</v>
+        <v>51662.77</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.9457</v>
+        <v>12.9114</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29821.13</v>
+        <v>29829.25</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29606.25</v>
+        <v>29614.32</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29713.69</v>
+        <v>29721.78</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.9457</v>
+        <v>12.9114</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16947.04</v>
+        <v>16951.66</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16880.08</v>
+        <v>16884.67</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16913.56</v>
+        <v>16918.17</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.9457</v>
+        <v>12.9114</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6870.96</v>
+        <v>6872.83</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6653.54</v>
+        <v>6655.35</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6762.25</v>
+        <v>6764.09</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.8993</v>
+        <v>12.8653</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360629.48</v>
+        <v>360736.53</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>356167.6</v>
+        <v>356273.33</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>358398.54</v>
+        <v>358504.93</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.8993</v>
+        <v>12.8653</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270735.19</v>
+        <v>270815.56</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271613.24</v>
+        <v>271693.87</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>271174.22</v>
+        <v>271254.72</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.8993</v>
+        <v>12.8653</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189434.25</v>
+        <v>189490.48</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189319.97</v>
+        <v>189376.17</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189377.11</v>
+        <v>189433.32</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.8993</v>
+        <v>12.8653</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>115165</v>
+        <v>115199.18</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115418.83</v>
+        <v>115453.09</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115291.91</v>
+        <v>115326.14</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.8993</v>
+        <v>12.8653</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55821.96</v>
+        <v>55838.53</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55561.18</v>
+        <v>55577.67</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55691.57</v>
+        <v>55708.1</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.8993</v>
+        <v>12.8653</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28509.2</v>
+        <v>28517.66</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28530.73</v>
+        <v>28539.2</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28519.96</v>
+        <v>28528.43</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5554</v>
+        <v>13.5205</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>412596.42</v>
+        <v>412601.45</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>413150.99</v>
+        <v>413156.03</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>412873.7</v>
+        <v>412878.74</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5554</v>
+        <v>13.5205</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>306265.93</v>
+        <v>306269.67</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>304353.64</v>
+        <v>304357.35</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>305309.78</v>
+        <v>305313.51</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5554</v>
+        <v>13.5205</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207740.46</v>
+        <v>207742.99</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207811.52</v>
+        <v>207814.06</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207775.99</v>
+        <v>207778.52</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5554</v>
+        <v>13.5205</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125710.97</v>
+        <v>125712.5</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126235.11</v>
+        <v>126236.65</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125973.04</v>
+        <v>125974.58</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5554</v>
+        <v>13.5205</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50203.36</v>
+        <v>50203.97</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50143.53</v>
+        <v>50144.15</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50173.45</v>
+        <v>50174.06</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5554</v>
+        <v>13.5205</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5522.21</v>
+        <v>5522.27</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5558.62</v>
+        <v>5558.69</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5540.41</v>
+        <v>5540.48</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5141</v>
+        <v>13.4791</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172302.82</v>
+        <v>172309.16</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172330.38</v>
+        <v>172336.72</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172316.6</v>
+        <v>172322.94</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5141</v>
+        <v>13.4791</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113231.57</v>
+        <v>113235.73</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112837.66</v>
+        <v>112841.81</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>113034.61</v>
+        <v>113038.77</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5141</v>
+        <v>13.4791</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63414.68</v>
+        <v>63417.01</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63774.37</v>
+        <v>63776.71</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63594.52</v>
+        <v>63596.86</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5141</v>
+        <v>13.4791</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27148.44</v>
+        <v>27149.43</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27350.69</v>
+        <v>27351.7</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27249.56</v>
+        <v>27250.57</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5141</v>
+        <v>13.4791</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6390.45</v>
+        <v>6390.69</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6544.07</v>
+        <v>6544.31</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6467.26</v>
+        <v>6467.5</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5141</v>
+        <v>13.4791</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3784.76</v>
+        <v>3784.9</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3778.2</v>
+        <v>3778.33</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3781.48</v>
+        <v>3781.62</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4132</v>
+        <v>13.3779</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192735.84</v>
+        <v>192748.45</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193676.95</v>
+        <v>193689.61</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193206.4</v>
+        <v>193219.03</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4132</v>
+        <v>13.3779</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139737.56</v>
+        <v>139746.7</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140712.7</v>
+        <v>140721.9</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140225.13</v>
+        <v>140234.3</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4132</v>
+        <v>13.3779</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88328.14</v>
+        <v>88333.92</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>89042.95</v>
+        <v>89048.77</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88685.53999999999</v>
+        <v>88691.34</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4132</v>
+        <v>13.3779</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42191.03</v>
+        <v>42193.79</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42123.37</v>
+        <v>42126.12</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42157.2</v>
+        <v>42159.96</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4132</v>
+        <v>13.3779</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13156.59</v>
+        <v>13157.45</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>13011.67</v>
+        <v>13012.52</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13084.13</v>
+        <v>13084.98</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4132</v>
+        <v>13.3779</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4566.16</v>
+        <v>4566.46</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4454.69</v>
+        <v>4454.98</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4510.43</v>
+        <v>4510.72</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-26
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2952</v>
+        <v>13.2987</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151932.24</v>
+        <v>152006.18</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153847.68</v>
+        <v>153922.54</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152889.96</v>
+        <v>152964.36</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2952</v>
+        <v>13.2987</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116294.25</v>
+        <v>116350.84</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>117084.94</v>
+        <v>117141.92</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116689.6</v>
+        <v>116746.38</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2952</v>
+        <v>13.2987</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82920.52</v>
+        <v>82960.87</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83437.22</v>
+        <v>83477.82000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83178.87</v>
+        <v>83219.35000000001</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2952</v>
+        <v>13.2987</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58757.46</v>
+        <v>58786.05</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58312.15</v>
+        <v>58340.52</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58534.8</v>
+        <v>58563.29</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2952</v>
+        <v>13.2987</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37954.99</v>
+        <v>37973.46</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38265.47</v>
+        <v>38284.09</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38110.23</v>
+        <v>38128.78</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2952</v>
+        <v>13.2987</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17262.64</v>
+        <v>17271.04</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17149.28</v>
+        <v>17157.62</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17205.96</v>
+        <v>17214.33</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.227</v>
+        <v>13.2304</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>165110.24</v>
+        <v>165189.8</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164224.29</v>
+        <v>164303.42</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164667.26</v>
+        <v>164746.61</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.227</v>
+        <v>13.2304</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123998.29</v>
+        <v>124058.04</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122247</v>
+        <v>122305.9</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>123122.64</v>
+        <v>123181.97</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.227</v>
+        <v>13.2304</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88589.07000000001</v>
+        <v>88631.75999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87492.07000000001</v>
+        <v>87534.23</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>88040.57000000001</v>
+        <v>88082.99000000001</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.227</v>
+        <v>13.2304</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67482.67</v>
+        <v>67515.17999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>67008.28</v>
+        <v>67040.56</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67245.47</v>
+        <v>67277.87</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.227</v>
+        <v>13.2304</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52718.56</v>
+        <v>52743.96</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50823.9</v>
+        <v>50848.39</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51771.23</v>
+        <v>51796.17</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.227</v>
+        <v>13.2304</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39963.52</v>
+        <v>39982.78</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40951.04</v>
+        <v>40970.77</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40457.28</v>
+        <v>40476.77</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.1519</v>
+        <v>13.1553</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>170072.87</v>
+        <v>170153.92</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171639.53</v>
+        <v>171721.32</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170856.2</v>
+        <v>170937.62</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.1519</v>
+        <v>13.1553</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122598.85</v>
+        <v>122657.28</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>121133.53</v>
+        <v>121191.26</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121866.19</v>
+        <v>121924.27</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.1519</v>
+        <v>13.1553</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83982.14999999999</v>
+        <v>84022.17</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83664.95</v>
+        <v>83704.82000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83823.55</v>
+        <v>83863.49000000001</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.1519</v>
+        <v>13.1553</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55952.94</v>
+        <v>55979.6</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56261.67</v>
+        <v>56288.48</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56107.3</v>
+        <v>56134.04</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.1519</v>
+        <v>13.1553</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33770.45</v>
+        <v>33786.54</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33375.18</v>
+        <v>33391.09</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33572.82</v>
+        <v>33588.82</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.1519</v>
+        <v>13.1553</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17532.18</v>
+        <v>17540.54</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18227.25</v>
+        <v>18235.93</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17879.72</v>
+        <v>17888.24</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.0939</v>
+        <v>13.096</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131502.61</v>
+        <v>131565.51</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131598.97</v>
+        <v>131661.91</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131550.79</v>
+        <v>131613.71</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.0939</v>
+        <v>13.096</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>91072.45</v>
+        <v>91116.00999999999</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89659.27</v>
+        <v>89702.14999999999</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90365.86</v>
+        <v>90409.08</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.0939</v>
+        <v>13.096</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57244.15</v>
+        <v>57271.53</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57536.29</v>
+        <v>57563.8</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57390.22</v>
+        <v>57417.66</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.0939</v>
+        <v>13.096</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30305.09</v>
+        <v>30319.59</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30509.08</v>
+        <v>30523.67</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30407.09</v>
+        <v>30421.63</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.0939</v>
+        <v>13.096</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6950.72</v>
+        <v>6954.05</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6949.4</v>
+        <v>6952.72</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6950.06</v>
+        <v>6953.38</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.0939</v>
+        <v>13.096</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3862.13</v>
+        <v>3863.98</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3771.03</v>
+        <v>3772.84</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3816.58</v>
+        <v>3818.41</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.0499</v>
+        <v>13.052</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>111085.62</v>
+        <v>111138.4</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111572.96</v>
+        <v>111625.97</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111329.29</v>
+        <v>111382.19</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.0499</v>
+        <v>13.052</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77902.87</v>
+        <v>77939.88</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77348.62</v>
+        <v>77385.37</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77625.75</v>
+        <v>77662.63</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.0499</v>
+        <v>13.052</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47139.12</v>
+        <v>47161.52</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48266.16</v>
+        <v>48289.09</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47702.64</v>
+        <v>47725.31</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.0499</v>
+        <v>13.052</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29285.6</v>
+        <v>29299.52</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29176.46</v>
+        <v>29190.32</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29231.03</v>
+        <v>29244.92</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.0499</v>
+        <v>13.052</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14366.23</v>
+        <v>14373.05</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14490.78</v>
+        <v>14497.66</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14428.5</v>
+        <v>14435.36</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.0499</v>
+        <v>13.052</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6660.19</v>
+        <v>6663.35</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6495.65</v>
+        <v>6498.74</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6577.92</v>
+        <v>6581.05</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.0037</v>
+        <v>13.0058</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50592.79</v>
+        <v>50616.67</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50254.08</v>
+        <v>50277.8</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50423.44</v>
+        <v>50447.23</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.0037</v>
+        <v>13.0058</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44508.15</v>
+        <v>44529.15</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44705.75</v>
+        <v>44726.84</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44606.95</v>
+        <v>44628</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.0037</v>
+        <v>13.0058</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32573.27</v>
+        <v>32588.64</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32920.16</v>
+        <v>32935.7</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32746.72</v>
+        <v>32762.17</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.0037</v>
+        <v>13.0058</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22903.2</v>
+        <v>22914.01</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>23060.49</v>
+        <v>23071.37</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22981.84</v>
+        <v>22992.69</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.0037</v>
+        <v>13.0058</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14720.61</v>
+        <v>14727.56</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14930.09</v>
+        <v>14937.14</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14825.35</v>
+        <v>14832.35</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.0037</v>
+        <v>13.0058</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8459.950000000001</v>
+        <v>8463.940000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8516</v>
+        <v>8520.02</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8487.969999999999</v>
+        <v>8491.98</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.9555</v>
+        <v>12.9576</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49813.54</v>
+        <v>49836.88</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>49080.41</v>
+        <v>49103.41</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49446.98</v>
+        <v>49470.14</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.9555</v>
+        <v>12.9576</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44608.73</v>
+        <v>44629.63</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44266.04</v>
+        <v>44286.78</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44437.39</v>
+        <v>44458.2</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.9555</v>
+        <v>12.9576</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32216.44</v>
+        <v>32231.53</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31637.3</v>
+        <v>31652.12</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31926.87</v>
+        <v>31941.83</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.9555</v>
+        <v>12.9576</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>24011.93</v>
+        <v>24023.18</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23904.87</v>
+        <v>23916.07</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23958.4</v>
+        <v>23969.63</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.9555</v>
+        <v>12.9576</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18837.05</v>
+        <v>18845.88</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18647.75</v>
+        <v>18656.49</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18742.4</v>
+        <v>18751.18</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.9555</v>
+        <v>12.9576</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15843.25</v>
+        <v>15850.67</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15786.68</v>
+        <v>15794.08</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15814.97</v>
+        <v>15822.38</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.9114</v>
+        <v>12.9135</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110756.01</v>
+        <v>110807.56</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111316.9</v>
+        <v>111368.71</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>111036.45</v>
+        <v>111088.13</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.9114</v>
+        <v>12.9135</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79423.91</v>
+        <v>79460.87</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79744.98</v>
+        <v>79782.09</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79584.44</v>
+        <v>79621.48</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.9114</v>
+        <v>12.9135</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51883.09</v>
+        <v>51907.24</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51442.46</v>
+        <v>51466.4</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51662.77</v>
+        <v>51686.82</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.9114</v>
+        <v>12.9135</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29829.25</v>
+        <v>29843.13</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29614.32</v>
+        <v>29628.1</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29721.78</v>
+        <v>29735.61</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.9114</v>
+        <v>12.9135</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16951.66</v>
+        <v>16959.55</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16884.67</v>
+        <v>16892.53</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16918.17</v>
+        <v>16926.04</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.9114</v>
+        <v>12.9135</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6872.83</v>
+        <v>6876.03</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6655.35</v>
+        <v>6658.45</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6764.09</v>
+        <v>6767.24</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.8653</v>
+        <v>12.8674</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360736.53</v>
+        <v>360903.25</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>356273.33</v>
+        <v>356437.98</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>358504.93</v>
+        <v>358670.62</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.8653</v>
+        <v>12.8674</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270815.56</v>
+        <v>270940.72</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271693.87</v>
+        <v>271819.44</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>271254.72</v>
+        <v>271380.08</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.8653</v>
+        <v>12.8674</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189490.48</v>
+        <v>189578.05</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189376.17</v>
+        <v>189463.69</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189433.32</v>
+        <v>189520.87</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.8653</v>
+        <v>12.8674</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>115199.18</v>
+        <v>115252.42</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115453.09</v>
+        <v>115506.45</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115326.14</v>
+        <v>115379.44</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.8653</v>
+        <v>12.8674</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55838.53</v>
+        <v>55864.34</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55577.67</v>
+        <v>55603.36</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55708.1</v>
+        <v>55733.85</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.8653</v>
+        <v>12.8674</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28517.66</v>
+        <v>28530.84</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28539.2</v>
+        <v>28552.39</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28528.43</v>
+        <v>28541.61</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>412601.45</v>
+        <v>412809.13</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>413156.03</v>
+        <v>413364</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>412878.74</v>
+        <v>413086.57</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>306269.67</v>
+        <v>306423.83</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>304357.35</v>
+        <v>304510.55</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>305313.51</v>
+        <v>305467.19</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207742.99</v>
+        <v>207847.56</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207814.06</v>
+        <v>207918.66</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207778.52</v>
+        <v>207883.11</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125712.5</v>
+        <v>125775.78</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126236.65</v>
+        <v>126300.19</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>125974.58</v>
+        <v>126037.99</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50203.97</v>
+        <v>50229.24</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50144.15</v>
+        <v>50169.39</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50174.06</v>
+        <v>50199.31</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5522.27</v>
+        <v>5525.05</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5558.69</v>
+        <v>5561.49</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5540.48</v>
+        <v>5543.27</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4791</v>
+        <v>13.4837</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172309.16</v>
+        <v>172394.83</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172336.72</v>
+        <v>172422.41</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172322.94</v>
+        <v>172408.62</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4791</v>
+        <v>13.4837</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113235.73</v>
+        <v>113292.03</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112841.81</v>
+        <v>112897.91</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>113038.77</v>
+        <v>113094.97</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4791</v>
+        <v>13.4837</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63417.01</v>
+        <v>63448.54</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63776.71</v>
+        <v>63808.42</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63596.86</v>
+        <v>63628.48</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4791</v>
+        <v>13.4837</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27149.43</v>
+        <v>27162.93</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27351.7</v>
+        <v>27365.3</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27250.57</v>
+        <v>27264.12</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4791</v>
+        <v>13.4837</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6390.69</v>
+        <v>6393.87</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6544.31</v>
+        <v>6547.57</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6467.5</v>
+        <v>6470.72</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4791</v>
+        <v>13.4837</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3784.9</v>
+        <v>3786.78</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3778.33</v>
+        <v>3780.21</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3781.62</v>
+        <v>3783.5</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3779</v>
+        <v>13.3821</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192748.45</v>
+        <v>192843.04</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193689.61</v>
+        <v>193784.67</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193219.03</v>
+        <v>193313.85</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3779</v>
+        <v>13.3821</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139746.7</v>
+        <v>139815.28</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140721.9</v>
+        <v>140790.96</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140234.3</v>
+        <v>140303.12</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3779</v>
+        <v>13.3821</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88333.92</v>
+        <v>88377.27</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>89048.77</v>
+        <v>89092.47</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88691.34</v>
+        <v>88734.87</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3779</v>
+        <v>13.3821</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42193.79</v>
+        <v>42214.5</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42126.12</v>
+        <v>42146.8</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42159.96</v>
+        <v>42180.65</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3779</v>
+        <v>13.3821</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13157.45</v>
+        <v>13163.9</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>13012.52</v>
+        <v>13018.91</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13084.98</v>
+        <v>13091.41</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3779</v>
+        <v>13.3821</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4566.46</v>
+        <v>4568.7</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4454.98</v>
+        <v>4457.17</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4510.72</v>
+        <v>4512.93</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-27
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.2987</v>
+        <v>13.7219</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>152006.18</v>
+        <v>151917.32</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153922.54</v>
+        <v>153832.56</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152964.36</v>
+        <v>152874.94</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.2987</v>
+        <v>13.7219</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116350.84</v>
+        <v>116282.83</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>117141.92</v>
+        <v>117073.44</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116746.38</v>
+        <v>116678.13</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.2987</v>
+        <v>13.7219</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82960.87</v>
+        <v>82912.38</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83477.82000000001</v>
+        <v>83429.03</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83219.35000000001</v>
+        <v>83170.7</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.2987</v>
+        <v>13.7219</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58786.05</v>
+        <v>58751.69</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58340.52</v>
+        <v>58306.42</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58563.29</v>
+        <v>58529.05</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.2987</v>
+        <v>13.7219</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37973.46</v>
+        <v>37951.26</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38284.09</v>
+        <v>38261.71</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38128.78</v>
+        <v>38106.49</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.2987</v>
+        <v>13.7219</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17271.04</v>
+        <v>17260.94</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17157.62</v>
+        <v>17147.59</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17214.33</v>
+        <v>17204.27</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.2304</v>
+        <v>13.8442</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>165189.8</v>
+        <v>164941.87</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164303.42</v>
+        <v>164056.82</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164746.61</v>
+        <v>164499.35</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.2304</v>
+        <v>13.8442</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>124058.04</v>
+        <v>123871.85</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122305.9</v>
+        <v>122122.33</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>123181.97</v>
+        <v>122997.09</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.2304</v>
+        <v>13.8442</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88631.75999999999</v>
+        <v>88498.73</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87534.23</v>
+        <v>87402.85000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>88082.99000000001</v>
+        <v>87950.78999999999</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.2304</v>
+        <v>13.8442</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67515.17999999999</v>
+        <v>67413.85000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>67040.56</v>
+        <v>66939.95</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67277.87</v>
+        <v>67176.89999999999</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.2304</v>
+        <v>13.8442</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52743.96</v>
+        <v>52664.8</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50848.39</v>
+        <v>50772.07</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51796.17</v>
+        <v>51718.43</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.2304</v>
+        <v>13.8442</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39982.78</v>
+        <v>39922.77</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40970.77</v>
+        <v>40909.28</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40476.77</v>
+        <v>40416.02</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.1553</v>
+        <v>13.9787</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>170153.92</v>
+        <v>169675.1</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171721.32</v>
+        <v>171238.09</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170937.62</v>
+        <v>170456.6</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.1553</v>
+        <v>13.9787</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122657.28</v>
+        <v>122312.12</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>121191.26</v>
+        <v>120850.22</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121924.27</v>
+        <v>121581.17</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.1553</v>
+        <v>13.9787</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>84022.17</v>
+        <v>83785.73</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83704.82000000001</v>
+        <v>83469.27</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83863.49000000001</v>
+        <v>83627.5</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.1553</v>
+        <v>13.9787</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55979.6</v>
+        <v>55822.08</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56288.48</v>
+        <v>56130.08</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56134.04</v>
+        <v>55976.08</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.1553</v>
+        <v>13.9787</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33786.54</v>
+        <v>33691.47</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33391.09</v>
+        <v>33297.12</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33588.82</v>
+        <v>33494.3</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.1553</v>
+        <v>13.9787</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17540.54</v>
+        <v>17491.18</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18235.93</v>
+        <v>18184.62</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17888.24</v>
+        <v>17837.9</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.096</v>
+        <v>14.0948</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131565.51</v>
+        <v>131002.11</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131661.91</v>
+        <v>131098.09</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131613.71</v>
+        <v>131050.1</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.096</v>
+        <v>14.0948</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>91116.00999999999</v>
+        <v>90725.82000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89702.14999999999</v>
+        <v>89318.02</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90409.08</v>
+        <v>90021.92</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.096</v>
+        <v>14.0948</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57271.53</v>
+        <v>57026.27</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57563.8</v>
+        <v>57317.3</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57417.66</v>
+        <v>57171.79</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.096</v>
+        <v>14.0948</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30319.59</v>
+        <v>30189.75</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30523.67</v>
+        <v>30392.96</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30421.63</v>
+        <v>30291.35</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.096</v>
+        <v>14.0948</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6954.05</v>
+        <v>6924.27</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6952.72</v>
+        <v>6922.95</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6953.38</v>
+        <v>6923.61</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.096</v>
+        <v>14.0948</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3863.98</v>
+        <v>3847.43</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3772.84</v>
+        <v>3756.68</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3818.41</v>
+        <v>3802.06</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.052</v>
+        <v>14.188</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>111138.4</v>
+        <v>110497.62</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111625.97</v>
+        <v>110982.37</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111382.19</v>
+        <v>110740</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.052</v>
+        <v>14.188</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77939.88</v>
+        <v>77490.50999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77385.37</v>
+        <v>76939.2</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77662.63</v>
+        <v>77214.85000000001</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.052</v>
+        <v>14.188</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47161.52</v>
+        <v>46889.6</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48289.09</v>
+        <v>48010.67</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47725.31</v>
+        <v>47450.14</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.052</v>
+        <v>14.188</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29299.52</v>
+        <v>29130.59</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29190.32</v>
+        <v>29022.02</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29244.92</v>
+        <v>29076.3</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.052</v>
+        <v>14.188</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14373.05</v>
+        <v>14290.18</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14497.66</v>
+        <v>14414.08</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14435.36</v>
+        <v>14352.13</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.052</v>
+        <v>14.188</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6663.35</v>
+        <v>6624.94</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6498.74</v>
+        <v>6461.27</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6581.05</v>
+        <v>6543.1</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.0058</v>
+        <v>14.2858</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50616.67</v>
+        <v>50235.47</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50277.8</v>
+        <v>49899.15</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50447.23</v>
+        <v>50067.31</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.0058</v>
+        <v>14.2858</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44529.15</v>
+        <v>44193.8</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44726.84</v>
+        <v>44390</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44628</v>
+        <v>44291.9</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.0058</v>
+        <v>14.2858</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32588.64</v>
+        <v>32343.21</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32935.7</v>
+        <v>32687.66</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32762.17</v>
+        <v>32515.44</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.0058</v>
+        <v>14.2858</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22914.01</v>
+        <v>22741.44</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>23071.37</v>
+        <v>22897.62</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22992.69</v>
+        <v>22819.53</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.0058</v>
+        <v>14.2858</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14727.56</v>
+        <v>14616.65</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14937.14</v>
+        <v>14824.65</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14832.35</v>
+        <v>14720.65</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.0058</v>
+        <v>14.2858</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8463.940000000001</v>
+        <v>8400.200000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8520.02</v>
+        <v>8455.85</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8491.98</v>
+        <v>8428.030000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>12.9576</v>
+        <v>14.3879</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49836.88</v>
+        <v>49358.12</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>49103.41</v>
+        <v>48631.69</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49470.14</v>
+        <v>48994.9</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>12.9576</v>
+        <v>14.3879</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44629.63</v>
+        <v>44200.89</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44286.78</v>
+        <v>43861.34</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44458.2</v>
+        <v>44031.11</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>12.9576</v>
+        <v>14.3879</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32231.53</v>
+        <v>31921.9</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31652.12</v>
+        <v>31348.05</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31941.83</v>
+        <v>31634.98</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>12.9576</v>
+        <v>14.3879</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>24023.18</v>
+        <v>23792.4</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23916.07</v>
+        <v>23686.32</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23969.63</v>
+        <v>23739.36</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>12.9576</v>
+        <v>14.3879</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18845.88</v>
+        <v>18664.84</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18656.49</v>
+        <v>18477.27</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18751.18</v>
+        <v>18571.05</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>12.9576</v>
+        <v>14.3879</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15850.67</v>
+        <v>15698.4</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15794.08</v>
+        <v>15642.35</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15822.38</v>
+        <v>15670.38</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>12.9135</v>
+        <v>14.4812</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>110807.56</v>
+        <v>109510.51</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>111368.71</v>
+        <v>110065.09</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>111088.13</v>
+        <v>109787.8</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>12.9135</v>
+        <v>14.4812</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>79460.87</v>
+        <v>78530.75</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79782.09</v>
+        <v>78848.21000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79621.48</v>
+        <v>78689.48</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>12.9135</v>
+        <v>14.4812</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51907.24</v>
+        <v>51299.64</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51466.4</v>
+        <v>50863.96</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51686.82</v>
+        <v>51081.8</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>12.9135</v>
+        <v>14.4812</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29843.13</v>
+        <v>29493.8</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29628.1</v>
+        <v>29281.29</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29735.61</v>
+        <v>29387.55</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>12.9135</v>
+        <v>14.4812</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16959.55</v>
+        <v>16761.03</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16892.53</v>
+        <v>16694.8</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16926.04</v>
+        <v>16727.91</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>12.9135</v>
+        <v>14.4812</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6876.03</v>
+        <v>6795.54</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6658.45</v>
+        <v>6580.51</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6767.24</v>
+        <v>6688.03</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>12.8674</v>
+        <v>14.5789</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>360903.25</v>
+        <v>355810.43</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>356437.98</v>
+        <v>351408.17</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>358670.62</v>
+        <v>353609.3</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>12.8674</v>
+        <v>14.5789</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>270940.72</v>
+        <v>267117.38</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>271819.44</v>
+        <v>267983.7</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>271380.08</v>
+        <v>267550.54</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>12.8674</v>
+        <v>14.5789</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>189578.05</v>
+        <v>186902.86</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>189463.69</v>
+        <v>186790.1</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>189520.87</v>
+        <v>186846.48</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>12.8674</v>
+        <v>14.5789</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>115252.42</v>
+        <v>113626.06</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>115506.45</v>
+        <v>113876.5</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>115379.44</v>
+        <v>113751.28</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>12.8674</v>
+        <v>14.5789</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55864.34</v>
+        <v>55076.02</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55603.36</v>
+        <v>54818.72</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55733.85</v>
+        <v>54947.37</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>12.8674</v>
+        <v>14.5789</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28530.84</v>
+        <v>28128.23</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28552.39</v>
+        <v>28149.47</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28541.61</v>
+        <v>28138.85</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5205</v>
+        <v>13.354</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>412809.13</v>
+        <v>413036.17</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>413364</v>
+        <v>413591.34</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>413086.57</v>
+        <v>413313.75</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5205</v>
+        <v>13.354</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>306423.83</v>
+        <v>306592.35</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>304510.55</v>
+        <v>304678.02</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>305467.19</v>
+        <v>305635.19</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5205</v>
+        <v>13.354</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207847.56</v>
+        <v>207961.87</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>207918.66</v>
+        <v>208033.01</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207883.11</v>
+        <v>207997.44</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5205</v>
+        <v>13.354</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125775.78</v>
+        <v>125844.95</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126300.19</v>
+        <v>126369.66</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>126037.99</v>
+        <v>126107.3</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5205</v>
+        <v>13.354</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50229.24</v>
+        <v>50256.87</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50169.39</v>
+        <v>50196.98</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50199.31</v>
+        <v>50226.92</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5205</v>
+        <v>13.354</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5525.05</v>
+        <v>5528.09</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5561.49</v>
+        <v>5564.55</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5543.27</v>
+        <v>5546.32</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4837</v>
+        <v>13.407</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172394.83</v>
+        <v>172494.34</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172422.41</v>
+        <v>172521.93</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172408.62</v>
+        <v>172508.14</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4837</v>
+        <v>13.407</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113292.03</v>
+        <v>113357.43</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112897.91</v>
+        <v>112963.08</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>113094.97</v>
+        <v>113160.25</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4837</v>
+        <v>13.407</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63448.54</v>
+        <v>63485.16</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63808.42</v>
+        <v>63845.25</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63628.48</v>
+        <v>63665.21</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4837</v>
+        <v>13.407</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27162.93</v>
+        <v>27178.61</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27365.3</v>
+        <v>27381.09</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27264.12</v>
+        <v>27279.85</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4837</v>
+        <v>13.407</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6393.87</v>
+        <v>6397.56</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6547.57</v>
+        <v>6551.35</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6470.72</v>
+        <v>6474.45</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4837</v>
+        <v>13.407</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3786.78</v>
+        <v>3788.97</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3780.21</v>
+        <v>3782.4</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3783.5</v>
+        <v>3785.68</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3821</v>
+        <v>13.5763</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192843.04</v>
+        <v>192872.36</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193784.67</v>
+        <v>193814.13</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193313.85</v>
+        <v>193343.25</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3821</v>
+        <v>13.5763</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139815.28</v>
+        <v>139836.54</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140790.96</v>
+        <v>140812.37</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140303.12</v>
+        <v>140324.46</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3821</v>
+        <v>13.5763</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88377.27</v>
+        <v>88390.71000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>89092.47</v>
+        <v>89106.02</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88734.87</v>
+        <v>88748.36</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3821</v>
+        <v>13.5763</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42214.5</v>
+        <v>42220.92</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42146.8</v>
+        <v>42153.2</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42180.65</v>
+        <v>42187.06</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3821</v>
+        <v>13.5763</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13163.9</v>
+        <v>13165.91</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>13018.91</v>
+        <v>13020.89</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13091.41</v>
+        <v>13093.4</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3821</v>
+        <v>13.5763</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4568.7</v>
+        <v>4569.39</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4457.17</v>
+        <v>4457.85</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4512.93</v>
+        <v>4513.62</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-28
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.7219</v>
+        <v>13.5955</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>151917.32</v>
+        <v>152043.18</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153832.56</v>
+        <v>153960.01</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>152874.94</v>
+        <v>153001.6</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.7219</v>
+        <v>13.5955</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116282.83</v>
+        <v>116379.17</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>117073.44</v>
+        <v>117170.43</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116678.13</v>
+        <v>116774.8</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.7219</v>
+        <v>13.5955</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82912.38</v>
+        <v>82981.07000000001</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83429.03</v>
+        <v>83498.14999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83170.7</v>
+        <v>83239.61</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.7219</v>
+        <v>13.5955</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58751.69</v>
+        <v>58800.36</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58306.42</v>
+        <v>58354.73</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58529.05</v>
+        <v>58577.55</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.7219</v>
+        <v>13.5955</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37951.26</v>
+        <v>37982.7</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38261.71</v>
+        <v>38293.41</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38106.49</v>
+        <v>38138.06</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.7219</v>
+        <v>13.5955</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17260.94</v>
+        <v>17275.24</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17147.59</v>
+        <v>17161.8</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17204.27</v>
+        <v>17218.52</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.8442</v>
+        <v>13.6776</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>164941.87</v>
+        <v>165114.99</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164056.82</v>
+        <v>164229.01</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164499.35</v>
+        <v>164672</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.8442</v>
+        <v>13.6776</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>123871.85</v>
+        <v>124001.86</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122122.33</v>
+        <v>122250.51</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>122997.09</v>
+        <v>123126.18</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.8442</v>
+        <v>13.6776</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88498.73</v>
+        <v>88591.62</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87402.85000000001</v>
+        <v>87494.59</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>87950.78999999999</v>
+        <v>88043.10000000001</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.8442</v>
+        <v>13.6776</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67413.85000000001</v>
+        <v>67484.61</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>66939.95</v>
+        <v>67010.2</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67176.89999999999</v>
+        <v>67247.41</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.8442</v>
+        <v>13.6776</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52664.8</v>
+        <v>52720.07</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50772.07</v>
+        <v>50825.36</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51718.43</v>
+        <v>51772.72</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.8442</v>
+        <v>13.6776</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39922.77</v>
+        <v>39964.67</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40909.28</v>
+        <v>40952.22</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40416.02</v>
+        <v>40458.44</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.9787</v>
+        <v>13.768</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169675.1</v>
+        <v>169905.35</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171238.09</v>
+        <v>171470.46</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170456.6</v>
+        <v>170687.91</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.9787</v>
+        <v>13.768</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122312.12</v>
+        <v>122478.09</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>120850.22</v>
+        <v>121014.22</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121581.17</v>
+        <v>121746.16</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.9787</v>
+        <v>13.768</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83785.73</v>
+        <v>83899.42999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83469.27</v>
+        <v>83582.53999999999</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83627.5</v>
+        <v>83740.98</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.9787</v>
+        <v>13.768</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55822.08</v>
+        <v>55897.83</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56130.08</v>
+        <v>56206.25</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55976.08</v>
+        <v>56052.04</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.9787</v>
+        <v>13.768</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33691.47</v>
+        <v>33737.19</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33297.12</v>
+        <v>33342.31</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33494.3</v>
+        <v>33539.75</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.9787</v>
+        <v>13.768</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17491.18</v>
+        <v>17514.91</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18184.62</v>
+        <v>18209.29</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17837.9</v>
+        <v>17862.1</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>14.0948</v>
+        <v>13.8495</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131002.11</v>
+        <v>131222.98</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131098.09</v>
+        <v>131319.13</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131050.1</v>
+        <v>131271.06</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>14.0948</v>
+        <v>13.8495</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90725.82000000001</v>
+        <v>90878.78999999999</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89318.02</v>
+        <v>89468.61</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90021.92</v>
+        <v>90173.7</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>14.0948</v>
+        <v>13.8495</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57026.27</v>
+        <v>57122.42</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57317.3</v>
+        <v>57413.94</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57171.79</v>
+        <v>57268.18</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>14.0948</v>
+        <v>13.8495</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30189.75</v>
+        <v>30240.65</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30392.96</v>
+        <v>30444.2</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30291.35</v>
+        <v>30342.43</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>14.0948</v>
+        <v>13.8495</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6924.27</v>
+        <v>6935.94</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6922.95</v>
+        <v>6934.62</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6923.61</v>
+        <v>6935.28</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>14.0948</v>
+        <v>13.8495</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3847.43</v>
+        <v>3853.92</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3756.68</v>
+        <v>3763.02</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3802.06</v>
+        <v>3808.47</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>14.188</v>
+        <v>13.9171</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110497.62</v>
+        <v>110719.55</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>110982.37</v>
+        <v>111205.28</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110740</v>
+        <v>110962.41</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>14.188</v>
+        <v>13.9171</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77490.50999999999</v>
+        <v>77646.14999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76939.2</v>
+        <v>77093.73</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77214.85000000001</v>
+        <v>77369.94</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>14.188</v>
+        <v>13.9171</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46889.6</v>
+        <v>46983.78</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48010.67</v>
+        <v>48107.1</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47450.14</v>
+        <v>47545.44</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>14.188</v>
+        <v>13.9171</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29130.59</v>
+        <v>29189.09</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29022.02</v>
+        <v>29080.31</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29076.3</v>
+        <v>29134.7</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>14.188</v>
+        <v>13.9171</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14290.18</v>
+        <v>14318.89</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14414.08</v>
+        <v>14443.03</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14352.13</v>
+        <v>14380.96</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>14.188</v>
+        <v>13.9171</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6624.94</v>
+        <v>6638.24</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6461.27</v>
+        <v>6474.25</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6543.1</v>
+        <v>6556.24</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>14.2858</v>
+        <v>13.988</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50235.47</v>
+        <v>50355.34</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49899.15</v>
+        <v>50018.22</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50067.31</v>
+        <v>50186.78</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>14.2858</v>
+        <v>13.988</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44193.8</v>
+        <v>44299.25</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44390</v>
+        <v>44495.92</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44291.9</v>
+        <v>44397.59</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>14.2858</v>
+        <v>13.988</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32343.21</v>
+        <v>32420.39</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32687.66</v>
+        <v>32765.66</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32515.44</v>
+        <v>32593.02</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>14.2858</v>
+        <v>13.988</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22741.44</v>
+        <v>22795.7</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22897.62</v>
+        <v>22952.26</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22819.53</v>
+        <v>22873.98</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>14.2858</v>
+        <v>13.988</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14616.65</v>
+        <v>14651.52</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14824.65</v>
+        <v>14860.02</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14720.65</v>
+        <v>14755.77</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>14.2858</v>
+        <v>13.988</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8400.200000000001</v>
+        <v>8420.24</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8455.85</v>
+        <v>8476.030000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8428.030000000001</v>
+        <v>8448.139999999999</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>14.3879</v>
+        <v>14.062</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49358.12</v>
+        <v>49497.54</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48631.69</v>
+        <v>48769.06</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48994.9</v>
+        <v>49133.3</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>14.3879</v>
+        <v>14.062</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44200.89</v>
+        <v>44325.74</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43861.34</v>
+        <v>43985.23</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44031.11</v>
+        <v>44155.49</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>14.3879</v>
+        <v>14.062</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31921.9</v>
+        <v>32012.07</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31348.05</v>
+        <v>31436.6</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31634.98</v>
+        <v>31724.33</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>14.3879</v>
+        <v>14.062</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23792.4</v>
+        <v>23859.61</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23686.32</v>
+        <v>23753.23</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23739.36</v>
+        <v>23806.42</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>14.3879</v>
+        <v>14.062</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18664.84</v>
+        <v>18717.56</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18477.27</v>
+        <v>18529.46</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18571.05</v>
+        <v>18623.51</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>14.3879</v>
+        <v>14.062</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15698.4</v>
+        <v>15742.74</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15642.35</v>
+        <v>15686.54</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15670.38</v>
+        <v>15714.64</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>14.4812</v>
+        <v>14.1296</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109510.51</v>
+        <v>109867.95</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110065.09</v>
+        <v>110424.34</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>109787.8</v>
+        <v>110146.14</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>14.4812</v>
+        <v>14.1296</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78530.75</v>
+        <v>78787.07000000001</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78848.21000000001</v>
+        <v>79105.57000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78689.48</v>
+        <v>78946.32000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>14.4812</v>
+        <v>14.1296</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51299.64</v>
+        <v>51467.08</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50863.96</v>
+        <v>51029.98</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51081.8</v>
+        <v>51248.53</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>14.4812</v>
+        <v>14.1296</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29493.8</v>
+        <v>29590.07</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29281.29</v>
+        <v>29376.86</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29387.55</v>
+        <v>29483.47</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>14.4812</v>
+        <v>14.1296</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16761.03</v>
+        <v>16815.74</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16694.8</v>
+        <v>16749.29</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16727.91</v>
+        <v>16782.51</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>14.4812</v>
+        <v>14.1296</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6795.54</v>
+        <v>6817.72</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6580.51</v>
+        <v>6601.99</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6688.03</v>
+        <v>6709.85</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>14.5789</v>
+        <v>14.2005</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>355810.43</v>
+        <v>357149.68</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>351408.17</v>
+        <v>352730.86</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>353609.3</v>
+        <v>354940.27</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>14.5789</v>
+        <v>14.2005</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>267117.38</v>
+        <v>268122.8</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>267983.7</v>
+        <v>268992.38</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>267550.54</v>
+        <v>268557.59</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>14.5789</v>
+        <v>14.2005</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>186902.86</v>
+        <v>187606.35</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>186790.1</v>
+        <v>187493.17</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>186846.48</v>
+        <v>187549.76</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>14.5789</v>
+        <v>14.2005</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>113626.06</v>
+        <v>114053.74</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>113876.5</v>
+        <v>114305.13</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>113751.28</v>
+        <v>114179.44</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>14.5789</v>
+        <v>14.2005</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55076.02</v>
+        <v>55283.32</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>54818.72</v>
+        <v>55025.06</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>54947.37</v>
+        <v>55154.19</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>14.5789</v>
+        <v>14.2005</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28128.23</v>
+        <v>28234.11</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28149.47</v>
+        <v>28255.43</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28138.85</v>
+        <v>28244.77</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.354</v>
+        <v>13.3599</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>413036.17</v>
+        <v>413241.07</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>413591.34</v>
+        <v>413796.51</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>413313.75</v>
+        <v>413518.79</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.354</v>
+        <v>13.3599</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>306592.35</v>
+        <v>306744.45</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>304678.02</v>
+        <v>304829.17</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>305635.19</v>
+        <v>305786.81</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.354</v>
+        <v>13.3599</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>207961.87</v>
+        <v>208065.03</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>208033.01</v>
+        <v>208136.21</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>207997.44</v>
+        <v>208100.62</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.354</v>
+        <v>13.3599</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125844.95</v>
+        <v>125907.38</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126369.66</v>
+        <v>126432.34</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>126107.3</v>
+        <v>126169.86</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.354</v>
+        <v>13.3599</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50256.87</v>
+        <v>50281.8</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50196.98</v>
+        <v>50221.88</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50226.92</v>
+        <v>50251.84</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.354</v>
+        <v>13.3599</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5528.09</v>
+        <v>5530.83</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5564.55</v>
+        <v>5567.31</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5546.32</v>
+        <v>5549.07</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.407</v>
+        <v>13.3891</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172494.34</v>
+        <v>172583.4</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172521.93</v>
+        <v>172611</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172508.14</v>
+        <v>172597.2</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.407</v>
+        <v>13.3891</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113357.43</v>
+        <v>113415.95</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>112963.08</v>
+        <v>113021.4</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>113160.25</v>
+        <v>113218.67</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.407</v>
+        <v>13.3891</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63485.16</v>
+        <v>63517.94</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63845.25</v>
+        <v>63878.22</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63665.21</v>
+        <v>63698.08</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.407</v>
+        <v>13.3891</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27178.61</v>
+        <v>27192.64</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27381.09</v>
+        <v>27395.23</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27279.85</v>
+        <v>27293.94</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.407</v>
+        <v>13.3891</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6397.56</v>
+        <v>6400.86</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6551.35</v>
+        <v>6554.73</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6474.45</v>
+        <v>6477.79</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.407</v>
+        <v>13.3891</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3788.97</v>
+        <v>3790.93</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3782.4</v>
+        <v>3784.35</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3785.68</v>
+        <v>3787.64</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.5763</v>
+        <v>13.4988</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192872.36</v>
+        <v>192995.95</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193814.13</v>
+        <v>193938.32</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193343.25</v>
+        <v>193467.13</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.5763</v>
+        <v>13.4988</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139836.54</v>
+        <v>139926.14</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140812.37</v>
+        <v>140902.6</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140324.46</v>
+        <v>140414.37</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.5763</v>
+        <v>13.4988</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88390.71000000001</v>
+        <v>88447.34</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>89106.02</v>
+        <v>89163.11</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88748.36</v>
+        <v>88805.23</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.5763</v>
+        <v>13.4988</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42220.92</v>
+        <v>42247.97</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42153.2</v>
+        <v>42180.21</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42187.06</v>
+        <v>42214.09</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.5763</v>
+        <v>13.4988</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13165.91</v>
+        <v>13174.34</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>13020.89</v>
+        <v>13029.23</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13093.4</v>
+        <v>13101.79</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.5763</v>
+        <v>13.4988</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4569.39</v>
+        <v>4572.32</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4457.85</v>
+        <v>4460.7</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4513.62</v>
+        <v>4516.51</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-29
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.5955</v>
+        <v>13.6176</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>152043.18</v>
+        <v>152111.76</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>153960.01</v>
+        <v>154029.45</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>153001.6</v>
+        <v>153070.6</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.5955</v>
+        <v>13.6176</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116379.17</v>
+        <v>116431.66</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>117170.43</v>
+        <v>117223.28</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116774.8</v>
+        <v>116827.47</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.5955</v>
+        <v>13.6176</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>82981.07000000001</v>
+        <v>83018.5</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83498.14999999999</v>
+        <v>83535.81</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83239.61</v>
+        <v>83277.14999999999</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.5955</v>
+        <v>13.6176</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58800.36</v>
+        <v>58826.88</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58354.73</v>
+        <v>58381.05</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58577.55</v>
+        <v>58603.96</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.5955</v>
+        <v>13.6176</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37982.7</v>
+        <v>37999.83</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38293.41</v>
+        <v>38310.68</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38138.06</v>
+        <v>38155.26</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.5955</v>
+        <v>13.6176</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17275.24</v>
+        <v>17283.03</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17161.8</v>
+        <v>17169.54</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17218.52</v>
+        <v>17226.29</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.6776</v>
+        <v>13.6969</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>165114.99</v>
+        <v>165188.88</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164229.01</v>
+        <v>164302.51</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164672</v>
+        <v>164745.7</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.6776</v>
+        <v>13.6969</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>124001.86</v>
+        <v>124057.35</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122250.51</v>
+        <v>122305.22</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>123126.18</v>
+        <v>123181.29</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.6776</v>
+        <v>13.6969</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88591.62</v>
+        <v>88631.27</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87494.59</v>
+        <v>87533.75</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>88043.10000000001</v>
+        <v>88082.50999999999</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.6776</v>
+        <v>13.6969</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67484.61</v>
+        <v>67514.81</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>67010.2</v>
+        <v>67040.19</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67247.41</v>
+        <v>67277.5</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.6776</v>
+        <v>13.6969</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52720.07</v>
+        <v>52743.67</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50825.36</v>
+        <v>50848.11</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51772.72</v>
+        <v>51795.89</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.6776</v>
+        <v>13.6969</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39964.67</v>
+        <v>39982.56</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40952.22</v>
+        <v>40970.54</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40458.44</v>
+        <v>40476.55</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.768</v>
+        <v>13.7842</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169905.35</v>
+        <v>169981.52</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171470.46</v>
+        <v>171547.34</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170687.91</v>
+        <v>170764.43</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.768</v>
+        <v>13.7842</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122478.09</v>
+        <v>122533</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>121014.22</v>
+        <v>121068.47</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121746.16</v>
+        <v>121800.74</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.768</v>
+        <v>13.7842</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83899.42999999999</v>
+        <v>83937.03999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83582.53999999999</v>
+        <v>83620.00999999999</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83740.98</v>
+        <v>83778.53</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.768</v>
+        <v>13.7842</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55897.83</v>
+        <v>55922.89</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56206.25</v>
+        <v>56231.45</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56052.04</v>
+        <v>56077.17</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.768</v>
+        <v>13.7842</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33737.19</v>
+        <v>33752.31</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33342.31</v>
+        <v>33357.26</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33539.75</v>
+        <v>33554.78</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.768</v>
+        <v>13.7842</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17514.91</v>
+        <v>17522.77</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18209.29</v>
+        <v>18217.46</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17862.1</v>
+        <v>17870.11</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.8495</v>
+        <v>13.8651</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131222.98</v>
+        <v>131280.89</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131319.13</v>
+        <v>131377.08</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131271.06</v>
+        <v>131328.99</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.8495</v>
+        <v>13.8651</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90878.78999999999</v>
+        <v>90918.89999999999</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89468.61</v>
+        <v>89508.09</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90173.7</v>
+        <v>90213.49000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.8495</v>
+        <v>13.8651</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57122.42</v>
+        <v>57147.63</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57413.94</v>
+        <v>57439.28</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57268.18</v>
+        <v>57293.45</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.8495</v>
+        <v>13.8651</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30240.65</v>
+        <v>30254</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30444.2</v>
+        <v>30457.64</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30342.43</v>
+        <v>30355.82</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.8495</v>
+        <v>13.8651</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6935.94</v>
+        <v>6939</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6934.62</v>
+        <v>6937.68</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6935.28</v>
+        <v>6938.34</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.8495</v>
+        <v>13.8651</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3853.92</v>
+        <v>3855.62</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3763.02</v>
+        <v>3764.68</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3808.47</v>
+        <v>3810.15</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.9171</v>
+        <v>13.9338</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110719.55</v>
+        <v>110766.79</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111205.28</v>
+        <v>111252.73</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>110962.41</v>
+        <v>111009.76</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.9171</v>
+        <v>13.9338</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77646.14999999999</v>
+        <v>77679.27</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77093.73</v>
+        <v>77126.62</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77369.94</v>
+        <v>77402.95</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.9171</v>
+        <v>13.9338</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46983.78</v>
+        <v>47003.83</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48107.1</v>
+        <v>48127.63</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47545.44</v>
+        <v>47565.73</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.9171</v>
+        <v>13.9338</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29189.09</v>
+        <v>29201.55</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29080.31</v>
+        <v>29092.72</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29134.7</v>
+        <v>29147.13</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.9171</v>
+        <v>13.9338</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14318.89</v>
+        <v>14324.99</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14443.03</v>
+        <v>14449.19</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14380.96</v>
+        <v>14387.09</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.9171</v>
+        <v>13.9338</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6638.24</v>
+        <v>6641.07</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6474.25</v>
+        <v>6477.01</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6556.24</v>
+        <v>6559.04</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.988</v>
+        <v>14.0057</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50355.34</v>
+        <v>50375.97</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50018.22</v>
+        <v>50038.72</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50186.78</v>
+        <v>50207.34</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.988</v>
+        <v>14.0057</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44299.25</v>
+        <v>44317.4</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44495.92</v>
+        <v>44514.15</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44397.59</v>
+        <v>44415.78</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.988</v>
+        <v>14.0057</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32420.39</v>
+        <v>32433.67</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32765.66</v>
+        <v>32779.08</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32593.02</v>
+        <v>32606.38</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.988</v>
+        <v>14.0057</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22795.7</v>
+        <v>22805.04</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22952.26</v>
+        <v>22961.66</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22873.98</v>
+        <v>22883.35</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.988</v>
+        <v>14.0057</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14651.52</v>
+        <v>14657.53</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14860.02</v>
+        <v>14866.11</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14755.77</v>
+        <v>14761.82</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.988</v>
+        <v>14.0057</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8420.24</v>
+        <v>8423.690000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8476.030000000001</v>
+        <v>8479.5</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8448.139999999999</v>
+        <v>8451.6</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>14.062</v>
+        <v>14.0809</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49497.54</v>
+        <v>49516.85</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48769.06</v>
+        <v>48788.09</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49133.3</v>
+        <v>49152.47</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>14.062</v>
+        <v>14.0809</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44325.74</v>
+        <v>44343.04</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43985.23</v>
+        <v>44002.4</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44155.49</v>
+        <v>44172.72</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>14.062</v>
+        <v>14.0809</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32012.07</v>
+        <v>32024.56</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31436.6</v>
+        <v>31448.87</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31724.33</v>
+        <v>31736.71</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>14.062</v>
+        <v>14.0809</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23859.61</v>
+        <v>23868.92</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23753.23</v>
+        <v>23762.5</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23806.42</v>
+        <v>23815.71</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>14.062</v>
+        <v>14.0809</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18717.56</v>
+        <v>18724.86</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18529.46</v>
+        <v>18536.69</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18623.51</v>
+        <v>18630.78</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>14.062</v>
+        <v>14.0809</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15742.74</v>
+        <v>15748.89</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15686.54</v>
+        <v>15692.66</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15714.64</v>
+        <v>15720.77</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>14.1296</v>
+        <v>14.1495</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109867.95</v>
+        <v>109908.7</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110424.34</v>
+        <v>110465.3</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110146.14</v>
+        <v>110187</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>14.1296</v>
+        <v>14.1495</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78787.07000000001</v>
+        <v>78816.28999999999</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79105.57000000001</v>
+        <v>79134.91</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78946.32000000001</v>
+        <v>78975.60000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>14.1296</v>
+        <v>14.1495</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51467.08</v>
+        <v>51486.17</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51029.98</v>
+        <v>51048.91</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51248.53</v>
+        <v>51267.54</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>14.1296</v>
+        <v>14.1495</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29590.07</v>
+        <v>29601.05</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29376.86</v>
+        <v>29387.76</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29483.47</v>
+        <v>29494.4</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>14.1296</v>
+        <v>14.1495</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16815.74</v>
+        <v>16821.98</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16749.29</v>
+        <v>16755.5</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16782.51</v>
+        <v>16788.74</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>14.1296</v>
+        <v>14.1495</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6817.72</v>
+        <v>6820.25</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6601.99</v>
+        <v>6604.44</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6709.85</v>
+        <v>6712.34</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>14.2005</v>
+        <v>14.2214</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>357149.68</v>
+        <v>357274.35</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>352730.86</v>
+        <v>352853.98</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>354940.27</v>
+        <v>355064.17</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>14.2005</v>
+        <v>14.2214</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>268122.8</v>
+        <v>268216.4</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>268992.38</v>
+        <v>269086.28</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>268557.59</v>
+        <v>268651.34</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>14.2005</v>
+        <v>14.2214</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>187606.35</v>
+        <v>187671.84</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>187493.17</v>
+        <v>187558.62</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>187549.76</v>
+        <v>187615.23</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>14.2005</v>
+        <v>14.2214</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114053.74</v>
+        <v>114093.55</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>114305.13</v>
+        <v>114345.03</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>114179.44</v>
+        <v>114219.29</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>14.2005</v>
+        <v>14.2214</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55283.32</v>
+        <v>55302.62</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55025.06</v>
+        <v>55044.27</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55154.19</v>
+        <v>55173.44</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>14.2005</v>
+        <v>14.2214</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28234.11</v>
+        <v>28243.96</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28255.43</v>
+        <v>28265.29</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28244.77</v>
+        <v>28254.63</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.4004</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>413241.07</v>
+        <v>413443.23</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>413796.51</v>
+        <v>413998.95</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>413518.79</v>
+        <v>413721.09</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.4004</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>306744.45</v>
+        <v>306894.51</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>304829.17</v>
+        <v>304978.29</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>305786.81</v>
+        <v>305936.4</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.4004</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>208065.03</v>
+        <v>208166.82</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>208136.21</v>
+        <v>208238.04</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>208100.62</v>
+        <v>208202.43</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.4004</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125907.38</v>
+        <v>125968.98</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126432.34</v>
+        <v>126494.2</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>126169.86</v>
+        <v>126231.59</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.4004</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50281.8</v>
+        <v>50306.4</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50221.88</v>
+        <v>50246.45</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50251.84</v>
+        <v>50276.42</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.3599</v>
+        <v>13.4004</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5530.83</v>
+        <v>5533.54</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5567.31</v>
+        <v>5570.03</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5549.07</v>
+        <v>5551.79</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.3891</v>
+        <v>13.423</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172583.4</v>
+        <v>172664.15</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172611</v>
+        <v>172691.77</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172597.2</v>
+        <v>172677.96</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.3891</v>
+        <v>13.423</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113415.95</v>
+        <v>113469.02</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>113021.4</v>
+        <v>113074.29</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>113218.67</v>
+        <v>113271.65</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.3891</v>
+        <v>13.423</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63517.94</v>
+        <v>63547.66</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63878.22</v>
+        <v>63908.11</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63698.08</v>
+        <v>63727.88</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.3891</v>
+        <v>13.423</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27192.64</v>
+        <v>27205.37</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27395.23</v>
+        <v>27408.05</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27293.94</v>
+        <v>27306.71</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.3891</v>
+        <v>13.423</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6400.86</v>
+        <v>6403.86</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6554.73</v>
+        <v>6557.79</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6477.79</v>
+        <v>6480.82</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.3891</v>
+        <v>13.423</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3790.93</v>
+        <v>3792.7</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3784.35</v>
+        <v>3786.12</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3787.64</v>
+        <v>3789.41</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4988</v>
+        <v>13.5254</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>192995.95</v>
+        <v>193084.15</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>193938.32</v>
+        <v>194026.95</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193467.13</v>
+        <v>193555.55</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4988</v>
+        <v>13.5254</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139926.14</v>
+        <v>139990.09</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140902.6</v>
+        <v>140966.99</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140414.37</v>
+        <v>140478.54</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4988</v>
+        <v>13.5254</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88447.34</v>
+        <v>88487.75999999999</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>89163.11</v>
+        <v>89203.86</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88805.23</v>
+        <v>88845.81</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4988</v>
+        <v>13.5254</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42247.97</v>
+        <v>42267.28</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42180.21</v>
+        <v>42199.49</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42214.09</v>
+        <v>42233.38</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4988</v>
+        <v>13.5254</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13174.34</v>
+        <v>13180.36</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>13029.23</v>
+        <v>13035.18</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13101.79</v>
+        <v>13107.77</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4988</v>
+        <v>13.5254</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4572.32</v>
+        <v>4574.41</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4460.7</v>
+        <v>4462.74</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4516.51</v>
+        <v>4518.58</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-30
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.6176</v>
+        <v>13.6491</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>152111.76</v>
+        <v>152177.14</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>154029.45</v>
+        <v>154095.66</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>153070.6</v>
+        <v>153136.4</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.6176</v>
+        <v>13.6491</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116431.66</v>
+        <v>116481.7</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>117223.28</v>
+        <v>117273.66</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116827.47</v>
+        <v>116877.68</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.6176</v>
+        <v>13.6491</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>83018.5</v>
+        <v>83054.17999999999</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83535.81</v>
+        <v>83571.71000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83277.14999999999</v>
+        <v>83312.94</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.6176</v>
+        <v>13.6491</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58826.88</v>
+        <v>58852.17</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58381.05</v>
+        <v>58406.14</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58603.96</v>
+        <v>58629.15</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.6176</v>
+        <v>13.6491</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37999.83</v>
+        <v>38016.17</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38310.68</v>
+        <v>38327.15</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38155.26</v>
+        <v>38171.66</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.6176</v>
+        <v>13.6491</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17283.03</v>
+        <v>17290.46</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17169.54</v>
+        <v>17176.92</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17226.29</v>
+        <v>17233.69</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.6969</v>
+        <v>13.7147</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>165188.88</v>
+        <v>165263.81</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164302.51</v>
+        <v>164377.03</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164745.7</v>
+        <v>164820.42</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.6969</v>
+        <v>13.7147</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>124057.35</v>
+        <v>124113.62</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122305.22</v>
+        <v>122360.7</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>123181.29</v>
+        <v>123237.16</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.6969</v>
+        <v>13.7147</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88631.27</v>
+        <v>88671.47</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87533.75</v>
+        <v>87573.45</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>88082.50999999999</v>
+        <v>88122.46000000001</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.6969</v>
+        <v>13.7147</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67514.81</v>
+        <v>67545.42999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>67040.19</v>
+        <v>67070.60000000001</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67277.5</v>
+        <v>67308.02</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.6969</v>
+        <v>13.7147</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52743.67</v>
+        <v>52767.59</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50848.11</v>
+        <v>50871.17</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51795.89</v>
+        <v>51819.38</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.6969</v>
+        <v>13.7147</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39982.56</v>
+        <v>40000.69</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40970.54</v>
+        <v>40989.13</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40476.55</v>
+        <v>40494.91</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.7842</v>
+        <v>13.7869</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>169981.52</v>
+        <v>170066.8</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171547.34</v>
+        <v>171633.4</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170764.43</v>
+        <v>170850.1</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.7842</v>
+        <v>13.7869</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122533</v>
+        <v>122594.47</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>121068.47</v>
+        <v>121129.21</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121800.74</v>
+        <v>121861.84</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.7842</v>
+        <v>13.7869</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83937.03999999999</v>
+        <v>83979.14999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83620.00999999999</v>
+        <v>83661.96000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83778.53</v>
+        <v>83820.55</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.7842</v>
+        <v>13.7869</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55922.89</v>
+        <v>55950.94</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56231.45</v>
+        <v>56259.66</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56077.17</v>
+        <v>56105.3</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.7842</v>
+        <v>13.7869</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33752.31</v>
+        <v>33769.24</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33357.26</v>
+        <v>33373.99</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33554.78</v>
+        <v>33571.62</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.7842</v>
+        <v>13.7869</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17522.77</v>
+        <v>17531.56</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18217.46</v>
+        <v>18226.6</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17870.11</v>
+        <v>17879.08</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.8651</v>
+        <v>13.8569</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131280.89</v>
+        <v>131353.61</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131377.08</v>
+        <v>131449.86</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131328.99</v>
+        <v>131401.73</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.8651</v>
+        <v>13.8569</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90918.89999999999</v>
+        <v>90969.25999999999</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89508.09</v>
+        <v>89557.67999999999</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90213.49000000001</v>
+        <v>90263.47</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.8651</v>
+        <v>13.8569</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57147.63</v>
+        <v>57179.29</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57439.28</v>
+        <v>57471.09</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57293.45</v>
+        <v>57325.19</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.8651</v>
+        <v>13.8569</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30254</v>
+        <v>30270.76</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30457.64</v>
+        <v>30474.51</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30355.82</v>
+        <v>30372.63</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.8651</v>
+        <v>13.8569</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6939</v>
+        <v>6942.85</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6937.68</v>
+        <v>6941.52</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6938.34</v>
+        <v>6942.18</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.8651</v>
+        <v>13.8569</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3855.62</v>
+        <v>3857.75</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3764.68</v>
+        <v>3766.76</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3810.15</v>
+        <v>3812.26</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.9338</v>
+        <v>13.9198</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110766.79</v>
+        <v>110832.5</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111252.73</v>
+        <v>111318.72</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111009.76</v>
+        <v>111075.61</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.9338</v>
+        <v>13.9198</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77679.27</v>
+        <v>77725.35000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77126.62</v>
+        <v>77172.37</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77402.95</v>
+        <v>77448.86</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.9338</v>
+        <v>13.9198</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47003.83</v>
+        <v>47031.71</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48127.63</v>
+        <v>48156.18</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47565.73</v>
+        <v>47593.94</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.9338</v>
+        <v>13.9198</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29201.55</v>
+        <v>29218.87</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29092.72</v>
+        <v>29109.98</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29147.13</v>
+        <v>29164.42</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.9338</v>
+        <v>13.9198</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14324.99</v>
+        <v>14333.49</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14449.19</v>
+        <v>14457.76</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14387.09</v>
+        <v>14395.63</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.9338</v>
+        <v>13.9198</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6641.07</v>
+        <v>6645.01</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6477.01</v>
+        <v>6480.85</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6559.04</v>
+        <v>6562.93</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>14.0057</v>
+        <v>13.9857</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50375.97</v>
+        <v>50408.38</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50038.72</v>
+        <v>50070.9</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50207.34</v>
+        <v>50239.64</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>14.0057</v>
+        <v>13.9857</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44317.4</v>
+        <v>44345.91</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44514.15</v>
+        <v>44542.79</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44415.78</v>
+        <v>44444.35</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>14.0057</v>
+        <v>13.9857</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32433.67</v>
+        <v>32454.54</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32779.08</v>
+        <v>32800.17</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32606.38</v>
+        <v>32627.35</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>14.0057</v>
+        <v>13.9857</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22805.04</v>
+        <v>22819.71</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22961.66</v>
+        <v>22976.43</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22883.35</v>
+        <v>22898.07</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>14.0057</v>
+        <v>13.9857</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14657.53</v>
+        <v>14666.96</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14866.11</v>
+        <v>14875.67</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14761.82</v>
+        <v>14771.32</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>14.0057</v>
+        <v>13.9857</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8423.690000000001</v>
+        <v>8429.110000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8479.5</v>
+        <v>8484.959999999999</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8451.6</v>
+        <v>8457.030000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>14.0809</v>
+        <v>14.0547</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49516.85</v>
+        <v>49551.78</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48788.09</v>
+        <v>48822.51</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49152.47</v>
+        <v>49187.15</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>14.0809</v>
+        <v>14.0547</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44343.04</v>
+        <v>44374.32</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44002.4</v>
+        <v>44033.44</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44172.72</v>
+        <v>44203.88</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>14.0809</v>
+        <v>14.0547</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32024.56</v>
+        <v>32047.15</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31448.87</v>
+        <v>31471.05</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31736.71</v>
+        <v>31759.1</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>14.0809</v>
+        <v>14.0547</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23868.92</v>
+        <v>23885.76</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23762.5</v>
+        <v>23779.26</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23815.71</v>
+        <v>23832.51</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>14.0809</v>
+        <v>14.0547</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18724.86</v>
+        <v>18738.07</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18536.69</v>
+        <v>18549.76</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18630.78</v>
+        <v>18643.92</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>14.0809</v>
+        <v>14.0547</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15748.89</v>
+        <v>15760</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15692.66</v>
+        <v>15703.73</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15720.77</v>
+        <v>15731.86</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>14.1495</v>
+        <v>14.1176</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109908.7</v>
+        <v>109993.41</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110465.3</v>
+        <v>110550.44</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110187</v>
+        <v>110271.93</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>14.1495</v>
+        <v>14.1176</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78816.28999999999</v>
+        <v>78877.03999999999</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79134.91</v>
+        <v>79195.89999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78975.60000000001</v>
+        <v>79036.47</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>14.1495</v>
+        <v>14.1176</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51486.17</v>
+        <v>51525.86</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51048.91</v>
+        <v>51088.26</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51267.54</v>
+        <v>51307.06</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>14.1495</v>
+        <v>14.1176</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29601.05</v>
+        <v>29623.86</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29387.76</v>
+        <v>29410.41</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29494.4</v>
+        <v>29517.14</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>14.1495</v>
+        <v>14.1176</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16821.98</v>
+        <v>16834.94</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16755.5</v>
+        <v>16768.42</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16788.74</v>
+        <v>16801.68</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>14.1495</v>
+        <v>14.1176</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6820.25</v>
+        <v>6825.51</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6604.44</v>
+        <v>6609.53</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6712.34</v>
+        <v>6717.52</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>14.2214</v>
+        <v>14.1835</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>357274.35</v>
+        <v>357577.39</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>352853.98</v>
+        <v>353153.27</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>355064.17</v>
+        <v>355365.33</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>14.2214</v>
+        <v>14.1835</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>268216.4</v>
+        <v>268443.89</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>269086.28</v>
+        <v>269314.52</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>268651.34</v>
+        <v>268879.21</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>14.2214</v>
+        <v>14.1835</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>187671.84</v>
+        <v>187831.02</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>187558.62</v>
+        <v>187717.71</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>187615.23</v>
+        <v>187774.36</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>14.2214</v>
+        <v>14.1835</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114093.55</v>
+        <v>114190.33</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>114345.03</v>
+        <v>114442.02</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>114219.29</v>
+        <v>114316.17</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>14.2214</v>
+        <v>14.1835</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55302.62</v>
+        <v>55349.53</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55044.27</v>
+        <v>55090.95</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55173.44</v>
+        <v>55220.24</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>14.2214</v>
+        <v>14.1835</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28243.96</v>
+        <v>28267.92</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28265.29</v>
+        <v>28289.27</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28254.63</v>
+        <v>28278.59</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4004</v>
+        <v>13.4836</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>413443.23</v>
+        <v>413643.59</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>413998.95</v>
+        <v>414199.57</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>413721.09</v>
+        <v>413921.58</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4004</v>
+        <v>13.4836</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>306894.51</v>
+        <v>307043.23</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>304978.29</v>
+        <v>305126.08</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>305936.4</v>
+        <v>306084.66</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4004</v>
+        <v>13.4836</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>208166.82</v>
+        <v>208267.7</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>208238.04</v>
+        <v>208338.95</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>208202.43</v>
+        <v>208303.32</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4004</v>
+        <v>13.4836</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>125968.98</v>
+        <v>126030.02</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126494.2</v>
+        <v>126555.5</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>126231.59</v>
+        <v>126292.76</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4004</v>
+        <v>13.4836</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50306.4</v>
+        <v>50330.77</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50246.45</v>
+        <v>50270.8</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50276.42</v>
+        <v>50300.79</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4004</v>
+        <v>13.4836</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5533.54</v>
+        <v>5536.22</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5570.03</v>
+        <v>5572.73</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5551.79</v>
+        <v>5554.48</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.423</v>
+        <v>13.4972</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172664.15</v>
+        <v>172739.26</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172691.77</v>
+        <v>172766.89</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172677.96</v>
+        <v>172753.07</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.423</v>
+        <v>13.4972</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113469.02</v>
+        <v>113518.37</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>113074.29</v>
+        <v>113123.47</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>113271.65</v>
+        <v>113320.92</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.423</v>
+        <v>13.4972</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63547.66</v>
+        <v>63575.3</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63908.11</v>
+        <v>63935.9</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63727.88</v>
+        <v>63755.6</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.423</v>
+        <v>13.4972</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27205.37</v>
+        <v>27217.2</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27408.05</v>
+        <v>27419.97</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27306.71</v>
+        <v>27318.59</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.423</v>
+        <v>13.4972</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6403.86</v>
+        <v>6406.64</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6557.79</v>
+        <v>6560.65</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6480.82</v>
+        <v>6483.64</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.423</v>
+        <v>13.4972</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3792.7</v>
+        <v>3794.35</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3786.12</v>
+        <v>3787.77</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3789.41</v>
+        <v>3791.06</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.5254</v>
+        <v>13.5755</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>193084.15</v>
+        <v>193165.16</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>194026.95</v>
+        <v>194108.36</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193555.55</v>
+        <v>193636.76</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.5254</v>
+        <v>13.5755</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>139990.09</v>
+        <v>140048.82</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>140966.99</v>
+        <v>141026.13</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140478.54</v>
+        <v>140537.48</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.5254</v>
+        <v>13.5755</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88487.75999999999</v>
+        <v>88524.89</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>89203.86</v>
+        <v>89241.28999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88845.81</v>
+        <v>88883.09</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.5254</v>
+        <v>13.5755</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42267.28</v>
+        <v>42285.01</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42199.49</v>
+        <v>42217.2</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42233.38</v>
+        <v>42251.1</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.5254</v>
+        <v>13.5755</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13180.36</v>
+        <v>13185.89</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>13035.18</v>
+        <v>13040.65</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13107.77</v>
+        <v>13113.27</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.5254</v>
+        <v>13.5755</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4574.41</v>
+        <v>4576.33</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4462.74</v>
+        <v>4464.62</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4518.58</v>
+        <v>4520.47</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-10-31
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.6491</v>
+        <v>13.6554</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>152177.14</v>
+        <v>152174.78</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>154095.66</v>
+        <v>154093.27</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>153136.4</v>
+        <v>153134.02</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.6491</v>
+        <v>13.6554</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>116481.7</v>
+        <v>116479.89</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>117273.66</v>
+        <v>117271.84</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>116877.68</v>
+        <v>116875.87</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.6491</v>
+        <v>13.6554</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>83054.17999999999</v>
+        <v>83052.89</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>83571.71000000001</v>
+        <v>83570.41</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>83312.94</v>
+        <v>83311.64999999999</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.6491</v>
+        <v>13.6554</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>58852.17</v>
+        <v>58851.26</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>58406.14</v>
+        <v>58405.23</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>58629.15</v>
+        <v>58628.24</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.6491</v>
+        <v>13.6554</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>38016.17</v>
+        <v>38015.58</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>38327.15</v>
+        <v>38326.56</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>38171.66</v>
+        <v>38171.07</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.6491</v>
+        <v>13.6554</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17290.46</v>
+        <v>17290.19</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>17176.92</v>
+        <v>17176.66</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>17233.69</v>
+        <v>17233.42</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.7147</v>
+        <v>13.7372</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>165263.81</v>
+        <v>165252.14</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>164377.03</v>
+        <v>164365.43</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>164820.42</v>
+        <v>164808.79</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.7147</v>
+        <v>13.7372</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>124113.62</v>
+        <v>124104.86</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>122360.7</v>
+        <v>122352.06</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>123237.16</v>
+        <v>123228.46</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.7147</v>
+        <v>13.7372</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>88671.47</v>
+        <v>88665.21000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>87573.45</v>
+        <v>87567.27</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>88122.46000000001</v>
+        <v>88116.24000000001</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.7147</v>
+        <v>13.7372</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>67545.42999999999</v>
+        <v>67540.67</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>67070.60000000001</v>
+        <v>67065.87</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>67308.02</v>
+        <v>67303.27</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.7147</v>
+        <v>13.7372</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>52767.59</v>
+        <v>52763.87</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50871.17</v>
+        <v>50867.58</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>51819.38</v>
+        <v>51815.72</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.7147</v>
+        <v>13.7372</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>40000.69</v>
+        <v>39997.87</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40989.13</v>
+        <v>40986.24</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>40494.91</v>
+        <v>40492.05</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.7869</v>
+        <v>13.8272</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>170066.8</v>
+        <v>170040.09</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>171633.4</v>
+        <v>171606.45</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>170850.1</v>
+        <v>170823.27</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.7869</v>
+        <v>13.8272</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>122594.47</v>
+        <v>122575.22</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>121129.21</v>
+        <v>121110.19</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>121861.84</v>
+        <v>121842.7</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.7869</v>
+        <v>13.8272</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>83979.14999999999</v>
+        <v>83965.96000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>83661.96000000001</v>
+        <v>83648.82000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>83820.55</v>
+        <v>83807.39</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.7869</v>
+        <v>13.8272</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55950.94</v>
+        <v>55942.15</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>56259.66</v>
+        <v>56250.82</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>56105.3</v>
+        <v>56096.49</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.7869</v>
+        <v>13.8272</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33769.24</v>
+        <v>33763.94</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>33373.99</v>
+        <v>33368.75</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33571.62</v>
+        <v>33566.35</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.7869</v>
+        <v>13.8272</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17531.56</v>
+        <v>17528.8</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>18226.6</v>
+        <v>18223.73</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17879.08</v>
+        <v>17876.27</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.8569</v>
+        <v>13.9124</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>131353.61</v>
+        <v>131319.58</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>131449.86</v>
+        <v>131415.8</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>131401.73</v>
+        <v>131367.69</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.8569</v>
+        <v>13.9124</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>90969.25999999999</v>
+        <v>90945.69</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>89557.67999999999</v>
+        <v>89534.47</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>90263.47</v>
+        <v>90240.08</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.8569</v>
+        <v>13.9124</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>57179.29</v>
+        <v>57164.47</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>57471.09</v>
+        <v>57456.21</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>57325.19</v>
+        <v>57310.34</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.8569</v>
+        <v>13.9124</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>30270.76</v>
+        <v>30262.91</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30474.51</v>
+        <v>30466.61</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>30372.63</v>
+        <v>30364.76</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.8569</v>
+        <v>13.9124</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6942.85</v>
+        <v>6941.05</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6941.52</v>
+        <v>6939.72</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6942.18</v>
+        <v>6940.38</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.8569</v>
+        <v>13.9124</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3857.75</v>
+        <v>3856.75</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3766.76</v>
+        <v>3765.79</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3812.26</v>
+        <v>3811.27</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.9198</v>
+        <v>13.9858</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>110832.5</v>
+        <v>110793.03</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>111318.72</v>
+        <v>111279.09</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>111075.61</v>
+        <v>111036.06</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.9198</v>
+        <v>13.9858</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>77725.35000000001</v>
+        <v>77697.67999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>77172.37</v>
+        <v>77144.89</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>77448.86</v>
+        <v>77421.28999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.9198</v>
+        <v>13.9858</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>47031.71</v>
+        <v>47014.96</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>48156.18</v>
+        <v>48139.03</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>47593.94</v>
+        <v>47577</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.9198</v>
+        <v>13.9858</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>29218.87</v>
+        <v>29208.47</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>29109.98</v>
+        <v>29099.61</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>29164.42</v>
+        <v>29154.04</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.9198</v>
+        <v>13.9858</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14333.49</v>
+        <v>14328.39</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14457.76</v>
+        <v>14452.61</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14395.63</v>
+        <v>14390.5</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.9198</v>
+        <v>13.9858</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6645.01</v>
+        <v>6642.65</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6480.85</v>
+        <v>6478.54</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6562.93</v>
+        <v>6560.6</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.9857</v>
+        <v>14.0627</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>50408.38</v>
+        <v>50384.49</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>50070.9</v>
+        <v>50047.17</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>50239.64</v>
+        <v>50215.83</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.9857</v>
+        <v>14.0627</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>44345.91</v>
+        <v>44324.9</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>44542.79</v>
+        <v>44521.68</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>44444.35</v>
+        <v>44423.29</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.9857</v>
+        <v>14.0627</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>32454.54</v>
+        <v>32439.16</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32800.17</v>
+        <v>32784.62</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32627.35</v>
+        <v>32611.89</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.9857</v>
+        <v>14.0627</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22819.71</v>
+        <v>22808.9</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22976.43</v>
+        <v>22965.54</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22898.07</v>
+        <v>22887.22</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.9857</v>
+        <v>14.0627</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14666.96</v>
+        <v>14660.01</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14875.67</v>
+        <v>14868.62</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14771.32</v>
+        <v>14764.31</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.9857</v>
+        <v>14.0627</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8429.110000000001</v>
+        <v>8425.120000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8484.959999999999</v>
+        <v>8480.940000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8457.030000000001</v>
+        <v>8453.030000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>14.0547</v>
+        <v>14.1431</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>49551.78</v>
+        <v>49521.31</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48822.51</v>
+        <v>48792.48</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>49187.15</v>
+        <v>49156.9</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>14.0547</v>
+        <v>14.1431</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>44374.32</v>
+        <v>44347.03</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>44033.44</v>
+        <v>44006.36</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>44203.88</v>
+        <v>44176.69</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>14.0547</v>
+        <v>14.1431</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>32047.15</v>
+        <v>32027.44</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31471.05</v>
+        <v>31451.7</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31759.1</v>
+        <v>31739.57</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>14.0547</v>
+        <v>14.1431</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23885.76</v>
+        <v>23871.07</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23779.26</v>
+        <v>23764.64</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23832.51</v>
+        <v>23817.85</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>14.0547</v>
+        <v>14.1431</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18738.07</v>
+        <v>18726.55</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18549.76</v>
+        <v>18538.36</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18643.92</v>
+        <v>18632.45</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>14.0547</v>
+        <v>14.1431</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15760</v>
+        <v>15750.3</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15703.73</v>
+        <v>15694.07</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15731.86</v>
+        <v>15722.19</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>14.1176</v>
+        <v>14.2165</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>109993.41</v>
+        <v>109909.86</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>110550.44</v>
+        <v>110466.47</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>110271.93</v>
+        <v>110188.16</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>14.1176</v>
+        <v>14.2165</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>78877.03999999999</v>
+        <v>78817.13</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>79195.89999999999</v>
+        <v>79135.75</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>79036.47</v>
+        <v>78976.44</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>14.1176</v>
+        <v>14.2165</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>51525.86</v>
+        <v>51486.72</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>51088.26</v>
+        <v>51049.45</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>51307.06</v>
+        <v>51268.08</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>14.1176</v>
+        <v>14.2165</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29623.86</v>
+        <v>29601.36</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29410.41</v>
+        <v>29388.07</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29517.14</v>
+        <v>29494.72</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>14.1176</v>
+        <v>14.2165</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16834.94</v>
+        <v>16822.15</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16768.42</v>
+        <v>16755.68</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16801.68</v>
+        <v>16788.92</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>14.1176</v>
+        <v>14.2165</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6825.51</v>
+        <v>6820.32</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6609.53</v>
+        <v>6604.51</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6717.52</v>
+        <v>6712.41</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>14.1835</v>
+        <v>14.2934</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>357577.39</v>
+        <v>357245.81</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>353153.27</v>
+        <v>352825.79</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>355365.33</v>
+        <v>355035.8</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>14.1835</v>
+        <v>14.2934</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>268443.89</v>
+        <v>268194.97</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>269314.52</v>
+        <v>269064.78</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>268879.21</v>
+        <v>268629.87</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>14.1835</v>
+        <v>14.2934</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>187831.02</v>
+        <v>187656.85</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>187717.71</v>
+        <v>187543.64</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>187774.36</v>
+        <v>187600.24</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>14.1835</v>
+        <v>14.2934</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>114190.33</v>
+        <v>114084.44</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>114442.02</v>
+        <v>114335.89</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>114316.17</v>
+        <v>114210.17</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>14.1835</v>
+        <v>14.2934</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>55349.53</v>
+        <v>55298.2</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>55090.95</v>
+        <v>55039.87</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>55220.24</v>
+        <v>55169.04</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>14.1835</v>
+        <v>14.2934</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>28267.92</v>
+        <v>28241.7</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>28289.27</v>
+        <v>28263.03</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>28278.59</v>
+        <v>28252.37</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.4836</v>
+        <v>13.441</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>413643.59</v>
+        <v>413646.67</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>414199.57</v>
+        <v>414202.66</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>413921.58</v>
+        <v>413924.66</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.4836</v>
+        <v>13.441</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>307043.23</v>
+        <v>307045.52</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>305126.08</v>
+        <v>305128.36</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>306084.66</v>
+        <v>306086.94</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.4836</v>
+        <v>13.441</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>208267.7</v>
+        <v>208269.25</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>208338.95</v>
+        <v>208340.5</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>208303.32</v>
+        <v>208304.88</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.4836</v>
+        <v>13.441</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>126030.02</v>
+        <v>126030.96</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>126555.5</v>
+        <v>126556.44</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>126292.76</v>
+        <v>126293.7</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.4836</v>
+        <v>13.441</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>50330.77</v>
+        <v>50331.15</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>50270.8</v>
+        <v>50271.17</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>50300.79</v>
+        <v>50301.16</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.4836</v>
+        <v>13.441</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5536.22</v>
+        <v>5536.26</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5572.73</v>
+        <v>5572.77</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5554.48</v>
+        <v>5554.52</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4972</v>
+        <v>13.459</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>172739.26</v>
+        <v>172745.04</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>172766.89</v>
+        <v>172772.67</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>172753.07</v>
+        <v>172758.85</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4972</v>
+        <v>13.459</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>113518.37</v>
+        <v>113522.17</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>113123.47</v>
+        <v>113127.26</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>113320.92</v>
+        <v>113324.71</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4972</v>
+        <v>13.459</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>63575.3</v>
+        <v>63577.43</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>63935.9</v>
+        <v>63938.04</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>63755.6</v>
+        <v>63757.74</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4972</v>
+        <v>13.459</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>27217.2</v>
+        <v>27218.11</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>27419.97</v>
+        <v>27420.89</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>27318.59</v>
+        <v>27319.5</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4972</v>
+        <v>13.459</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6406.64</v>
+        <v>6406.86</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6560.65</v>
+        <v>6560.87</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6483.64</v>
+        <v>6483.86</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4972</v>
+        <v>13.459</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3794.35</v>
+        <v>3794.48</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3787.77</v>
+        <v>3787.89</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3791.06</v>
+        <v>3791.18</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.5755</v>
+        <v>13.5614</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>193165.16</v>
+        <v>193169.7</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>194108.36</v>
+        <v>194112.92</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>193636.76</v>
+        <v>193641.31</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.5755</v>
+        <v>13.5614</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>140048.82</v>
+        <v>140052.12</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>141026.13</v>
+        <v>141029.45</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>140537.48</v>
+        <v>140540.78</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.5755</v>
+        <v>13.5614</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>88524.89</v>
+        <v>88526.97</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>89241.28999999999</v>
+        <v>89243.39</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>88883.09</v>
+        <v>88885.17999999999</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.5755</v>
+        <v>13.5614</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>42285.01</v>
+        <v>42286</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>42217.2</v>
+        <v>42218.19</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>42251.1</v>
+        <v>42252.1</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.5755</v>
+        <v>13.5614</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>13185.89</v>
+        <v>13186.2</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>13040.65</v>
+        <v>13040.96</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>13113.27</v>
+        <v>13113.58</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.5755</v>
+        <v>13.5614</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4576.33</v>
+        <v>4576.44</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4464.62</v>
+        <v>4464.72</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4520.47</v>
+        <v>4520.58</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>